<commit_message>
weekly scan 2026-06-12: completed locally — 8-K sweep all 135 names, AVGO 📊 refresh (74.6→78.2), ORCL/UEC/P rule-9 refreshes, PSTG→P (Everpure) rename, $40B+ AI debt-financing week, pipeline all HOLD, model +3.52%
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/00-master/portfolio.xlsx
+++ b/00-master/portfolio.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sizing Rules" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Targets" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Positions" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reconciliation" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sizing Rules" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Targets" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Positions" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Reconciliation" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -678,7 +678,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-06-10 (refresh_targets.py — hysteresis pipeline)</t>
+          <t>2026-06-12 (refresh_targets.py — hysteresis pipeline)</t>
         </is>
       </c>
     </row>
@@ -1070,7 +1070,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Target Portfolio (refreshed 2026-06-10, live Watchlist scores)</t>
+          <t>Target Portfolio (refreshed 2026-06-12, live Watchlist scores)</t>
         </is>
       </c>
     </row>
@@ -1160,7 +1160,7 @@
       </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="n">
-        <v>8.99</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="J3" t="inlineStr"/>
     </row>
@@ -1176,7 +1176,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>79.84999999999999</v>
+        <v>80.09999999999999</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
       </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="n">
-        <v>7.41</v>
+        <v>7.37</v>
       </c>
       <c r="J4" t="inlineStr"/>
     </row>
@@ -1236,7 +1236,7 @@
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="n">
-        <v>7.32</v>
+        <v>7.17</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -1278,7 +1278,7 @@
       </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="n">
-        <v>7.25</v>
+        <v>7.1</v>
       </c>
       <c r="J6" t="inlineStr"/>
     </row>
@@ -1316,7 +1316,7 @@
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="n">
-        <v>7</v>
+        <v>6.85</v>
       </c>
       <c r="J7" t="inlineStr"/>
     </row>
@@ -1332,7 +1332,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>78.3</v>
+        <v>78.8</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -1354,7 +1354,7 @@
       </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="n">
-        <v>6.7</v>
+        <v>6.79</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
@@ -1365,16 +1365,16 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>AVGO</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
+          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>77.72</v>
+        <v>78.15000000000001</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -1396,7 +1396,7 @@
       </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="n">
-        <v>6.44</v>
+        <v>6.5</v>
       </c>
       <c r="J9" t="inlineStr"/>
     </row>
@@ -1412,7 +1412,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>77.5</v>
+        <v>77.88</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -1434,23 +1434,23 @@
       </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="n">
-        <v>6.34</v>
+        <v>6.38</v>
       </c>
       <c r="J10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>EME</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>76.65000000000001</v>
+        <v>77.72</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -1472,27 +1472,23 @@
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="n">
-        <v>5.95</v>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>Added 2026-05-25: score 75.2, DC construction, strong momentum (86.7).</t>
-        </is>
-      </c>
+        <v>6.31</v>
+      </c>
+      <c r="J11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ALAB</t>
+          <t>EME</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>76.48</v>
+        <v>76.65000000000001</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -1514,23 +1510,27 @@
       </c>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="n">
-        <v>5.87</v>
-      </c>
-      <c r="J12" t="inlineStr"/>
+        <v>5.83</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Added 2026-05-25: score 75.2, DC construction, strong momentum (86.7).</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>FIX</t>
+          <t>ALAB</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>76.34999999999999</v>
+        <v>76.48</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -1552,27 +1552,23 @@
       </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="n">
-        <v>5.82</v>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>Manually excluded 2026-05-18: $1,854 share price prevents reasonable position sizing below ~$50k portfolio. Conscious framework override. | Override removed 2026-06-09: fractional shares adopted, share-price constraint obsolete (Dom decision).</t>
-        </is>
-      </c>
+        <v>5.75</v>
+      </c>
+      <c r="J13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>FIX</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>76.25</v>
+        <v>76.34999999999999</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -1594,23 +1590,27 @@
       </c>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="n">
-        <v>5.77</v>
-      </c>
-      <c r="J14" t="inlineStr"/>
+        <v>5.7</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Manually excluded 2026-05-18: $1,854 share price prevents reasonable position sizing below ~$50k portfolio. Conscious framework override. | Override removed 2026-06-09: fractional shares adopted, share-price constraint obsolete (Dom decision).</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>PLTR</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications</t>
+          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>74.84999999999999</v>
+        <v>76.25</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -1632,23 +1632,23 @@
       </c>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="n">
-        <v>5.13</v>
+        <v>5.65</v>
       </c>
       <c r="J15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>AVGO</t>
+          <t>PLTR</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
+          <t>10 Models, Software &amp; Applications</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>74.59999999999999</v>
+        <v>74.84999999999999</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -1670,7 +1670,7 @@
       </c>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="n">
-        <v>5.02</v>
+        <v>5.03</v>
       </c>
       <c r="J16" t="inlineStr"/>
     </row>
@@ -1708,7 +1708,7 @@
       </c>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="n">
-        <v>4.68</v>
+        <v>4.58</v>
       </c>
       <c r="J17" t="inlineStr"/>
     </row>
@@ -1812,7 +1812,7 @@
       </c>
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="n">
-        <v>4.29</v>
+        <v>4.2</v>
       </c>
       <c r="J20" t="inlineStr"/>
     </row>
@@ -1931,11 +1931,7 @@
       <c r="E24" t="n">
         <v>22</v>
       </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>EXIT (resize, score 72.0 &lt; 73.0)</t>
-        </is>
-      </c>
+      <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
           <t>N</t>
@@ -2001,11 +1997,7 @@
       <c r="E26" t="n">
         <v>24</v>
       </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>EXIT (resize, score 71.7 &lt; 73.0)</t>
-        </is>
-      </c>
+      <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
           <t>N</t>
@@ -2098,11 +2090,7 @@
       <c r="E29" t="n">
         <v>27</v>
       </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>EXIT (resize, score 70.9 &lt; 73.0)</t>
-        </is>
-      </c>
+      <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr">
         <is>
           <t>N</t>
@@ -2114,16 +2102,16 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>PATH</t>
+          <t>KEYS</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI-powered automation</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>70.90000000000001</v>
+        <v>70.87</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
@@ -2145,16 +2133,16 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>KEYS</t>
+          <t>PATH</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
+          <t>10 Models, Software &amp; Applications / AI-powered automation</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>70.87</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -2257,11 +2245,7 @@
       <c r="E34" t="n">
         <v>32</v>
       </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>EXIT (resize, score 70.0 &lt; 73.0)</t>
-        </is>
-      </c>
+      <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr">
         <is>
           <t>N</t>
@@ -2286,7 +2270,7 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>69.58</v>
+        <v>69.95</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
@@ -2370,12 +2354,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>FN</t>
+          <t>TEL</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
+          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -2401,16 +2385,16 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>TEL</t>
+          <t>TLN</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
+          <t>01 Power Generation / Independent Power Producers (IPPs)</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>69.2</v>
+        <v>69.17</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -2432,7 +2416,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>TLN</t>
+          <t>VST</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2441,7 +2425,7 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>69.17</v>
+        <v>69.09999999999999</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -2463,16 +2447,16 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>VST</t>
+          <t>FN</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>01 Power Generation / Independent Power Producers (IPPs)</t>
+          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>69.09999999999999</v>
+        <v>68.95</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -2525,12 +2509,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>ASML</t>
+          <t>PWR</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -2556,7 +2540,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>KLAC</t>
+          <t>ASML</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2587,16 +2571,16 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>HTHIY</t>
+          <t>KLAC</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>68.22</v>
+        <v>68.3</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
@@ -2711,7 +2695,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>PWR</t>
+          <t>HTHIY</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2720,7 +2704,7 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>68.05</v>
+        <v>67.84999999999999</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
@@ -3397,16 +3381,16 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>SNPS</t>
+          <t>RMBS</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
+          <t>06 AI Compute Silicon / Memory (HBM is the bottleneck)</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>65.47</v>
+        <v>65.22</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
@@ -3459,16 +3443,16 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>FLEX</t>
+          <t>SNPS</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Contract manufacturing / ODMs</t>
+          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>64.84999999999999</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
@@ -3490,12 +3474,12 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>RMBS</t>
+          <t>FLEX</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Memory (HBM is the bottleneck)</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Contract manufacturing / ODMs</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -3676,16 +3660,16 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>KLIC</t>
+          <t>ORCL</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>63.08</v>
+        <v>63.35</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
@@ -3707,16 +3691,16 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>ORCL</t>
+          <t>KLIC</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>62.75</v>
+        <v>63.08</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
@@ -5219,7 +5203,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Portfolio: $13,800 | Prices as of 2026-06-10</t>
+          <t>Portfolio: $13,800 | Prices as of 2026-06-12</t>
         </is>
       </c>
     </row>
@@ -5275,14 +5259,14 @@
         <v>83.3</v>
       </c>
       <c r="C4" t="n">
-        <v>8.99</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="D4">
         <f>C4/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E4" t="n">
-        <v>202.34</v>
+        <v>206.8</v>
       </c>
       <c r="F4">
         <f>IF(E4="","",ROUND(D4/E4,4))</f>
@@ -5305,17 +5289,17 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>79.8</v>
+        <v>80.09999999999999</v>
       </c>
       <c r="C5" t="n">
-        <v>7.41</v>
+        <v>7.37</v>
       </c>
       <c r="D5">
         <f>C5/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E5" t="n">
-        <v>412.98</v>
+        <v>426.36</v>
       </c>
       <c r="F5">
         <f>IF(E5="","",ROUND(D5/E5,4))</f>
@@ -5341,14 +5325,14 @@
         <v>79.7</v>
       </c>
       <c r="C6" t="n">
-        <v>7.32</v>
+        <v>7.17</v>
       </c>
       <c r="D6">
         <f>C6/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E6" t="n">
-        <v>1670.92</v>
+        <v>1985.5</v>
       </c>
       <c r="F6">
         <f>IF(E6="","",ROUND(D6/E6,4))</f>
@@ -5374,14 +5358,14 @@
         <v>79.5</v>
       </c>
       <c r="C7" t="n">
-        <v>7.25</v>
+        <v>7.1</v>
       </c>
       <c r="D7">
         <f>C7/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E7" t="n">
-        <v>901.41</v>
+        <v>1001.28</v>
       </c>
       <c r="F7">
         <f>IF(E7="","",ROUND(D7/E7,4))</f>
@@ -5407,14 +5391,14 @@
         <v>79</v>
       </c>
       <c r="C8" t="n">
-        <v>7</v>
+        <v>6.85</v>
       </c>
       <c r="D8">
         <f>C8/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E8" t="n">
-        <v>575.47</v>
+        <v>572.49</v>
       </c>
       <c r="F8">
         <f>IF(E8="","",ROUND(D8/E8,4))</f>
@@ -5437,17 +5421,17 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>78.3</v>
+        <v>78.8</v>
       </c>
       <c r="C9" t="n">
-        <v>6.7</v>
+        <v>6.79</v>
       </c>
       <c r="D9">
         <f>C9/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E9" t="n">
-        <v>241.86</v>
+        <v>254.34</v>
       </c>
       <c r="F9">
         <f>IF(E9="","",ROUND(D9/E9,4))</f>
@@ -5466,21 +5450,21 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>AVGO</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>77.7</v>
+        <v>78.2</v>
       </c>
       <c r="C10" t="n">
-        <v>6.44</v>
+        <v>6.5</v>
       </c>
       <c r="D10">
         <f>C10/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E10" t="n">
-        <v>356.14</v>
+        <v>383.41</v>
       </c>
       <c r="F10">
         <f>IF(E10="","",ROUND(D10/E10,4))</f>
@@ -5503,17 +5487,17 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>77.5</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="C11" t="n">
-        <v>6.34</v>
+        <v>6.38</v>
       </c>
       <c r="D11">
         <f>C11/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E11" t="n">
-        <v>152.44</v>
+        <v>164.57</v>
       </c>
       <c r="F11">
         <f>IF(E11="","",ROUND(D11/E11,4))</f>
@@ -5532,21 +5516,21 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>EME</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>76.7</v>
+        <v>77.7</v>
       </c>
       <c r="C12" t="n">
-        <v>5.95</v>
+        <v>6.31</v>
       </c>
       <c r="D12">
         <f>C12/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E12" t="n">
-        <v>788.1799999999999</v>
+        <v>365.38</v>
       </c>
       <c r="F12">
         <f>IF(E12="","",ROUND(D12/E12,4))</f>
@@ -5565,21 +5549,21 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ALAB</t>
+          <t>EME</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>76.5</v>
+        <v>76.7</v>
       </c>
       <c r="C13" t="n">
-        <v>5.87</v>
+        <v>5.83</v>
       </c>
       <c r="D13">
         <f>C13/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E13" t="n">
-        <v>339.65</v>
+        <v>824.97</v>
       </c>
       <c r="F13">
         <f>IF(E13="","",ROUND(D13/E13,4))</f>
@@ -5598,21 +5582,21 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>FIX</t>
+          <t>ALAB</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>76.40000000000001</v>
+        <v>76.5</v>
       </c>
       <c r="C14" t="n">
-        <v>5.82</v>
+        <v>5.75</v>
       </c>
       <c r="D14">
         <f>C14/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E14" t="n">
-        <v>1741.8</v>
+        <v>381.78</v>
       </c>
       <c r="F14">
         <f>IF(E14="","",ROUND(D14/E14,4))</f>
@@ -5631,21 +5615,21 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>FIX</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>76.2</v>
+        <v>76.40000000000001</v>
       </c>
       <c r="C15" t="n">
-        <v>5.77</v>
+        <v>5.7</v>
       </c>
       <c r="D15">
         <f>C15/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E15" t="n">
-        <v>401.28</v>
+        <v>1886.54</v>
       </c>
       <c r="F15">
         <f>IF(E15="","",ROUND(D15/E15,4))</f>
@@ -5664,21 +5648,21 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>PLTR</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>74.8</v>
+        <v>76.2</v>
       </c>
       <c r="C16" t="n">
-        <v>5.13</v>
+        <v>5.65</v>
       </c>
       <c r="D16">
         <f>C16/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E16" t="n">
-        <v>131.47</v>
+        <v>389.13</v>
       </c>
       <c r="F16">
         <f>IF(E16="","",ROUND(D16/E16,4))</f>
@@ -5697,21 +5681,21 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>AVGO</t>
+          <t>PLTR</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>74.59999999999999</v>
+        <v>74.8</v>
       </c>
       <c r="C17" t="n">
-        <v>5.02</v>
+        <v>5.03</v>
       </c>
       <c r="D17">
         <f>C17/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E17" t="n">
-        <v>378.69</v>
+        <v>130.12</v>
       </c>
       <c r="F17">
         <f>IF(E17="","",ROUND(D17/E17,4))</f>
@@ -5737,14 +5721,14 @@
         <v>73.8</v>
       </c>
       <c r="C18" t="n">
-        <v>4.68</v>
+        <v>4.58</v>
       </c>
       <c r="D18">
         <f>C18/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E18" t="n">
-        <v>52.93</v>
+        <v>52.22</v>
       </c>
       <c r="F18">
         <f>IF(E18="","",ROUND(D18/E18,4))</f>
@@ -5770,14 +5754,14 @@
         <v>73</v>
       </c>
       <c r="C19" t="n">
-        <v>4.29</v>
+        <v>4.2</v>
       </c>
       <c r="D19">
         <f>C19/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E19" t="n">
-        <v>350.63</v>
+        <v>404.93</v>
       </c>
       <c r="F19">
         <f>IF(E19="","",ROUND(D19/E19,4))</f>

</xml_diff>

<commit_message>
rating session 2026-06-12: 8 portfolio names re-rated research-backed — 20 changes, TER EXIT PENDING (72.2)
13 cuts / 7 raises across AVGO TSM META MSFT GOOGL EME FIX TER, all logged
to Rating Audit with rationale+source+confidence. TER falls below exit
threshold on R2 geographic-concentration cut (Taiwan 41%+Korea 19%);
2-run confirm next weekly refresh. TSM +1.5 on momentum evidence.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/00-master/portfolio.xlsx
+++ b/00-master/portfolio.xlsx
@@ -1160,7 +1160,7 @@
       </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="n">
-        <v>8.800000000000001</v>
+        <v>8.93</v>
       </c>
       <c r="J3" t="inlineStr"/>
     </row>
@@ -1176,7 +1176,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>80.09999999999999</v>
+        <v>81.59999999999999</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
       </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="n">
-        <v>7.37</v>
+        <v>8.15</v>
       </c>
       <c r="J4" t="inlineStr"/>
     </row>
@@ -1236,7 +1236,7 @@
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="n">
-        <v>7.17</v>
+        <v>7.27</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -1278,23 +1278,23 @@
       </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="n">
-        <v>7.1</v>
+        <v>7.2</v>
       </c>
       <c r="J6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>META</t>
+          <t>CRDO</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
+          <t>07 Optical, Networking &amp; Interconnect / Connectivity ASICs</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>78.95</v>
+        <v>78.8</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -1316,23 +1316,27 @@
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="n">
-        <v>6.85</v>
-      </c>
-      <c r="J7" t="inlineStr"/>
+        <v>6.89</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Added 2026-05-25: score 78.4, ranked #4 in reweighted watchlist. Optical connectivity pure-play.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CRDO</t>
+          <t>META</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Connectivity ASICs</t>
+          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>78.8</v>
+        <v>78.5</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -1354,13 +1358,9 @@
       </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="n">
-        <v>6.79</v>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>Added 2026-05-25: score 78.4, ranked #4 in reweighted watchlist. Optical connectivity pure-play.</t>
-        </is>
-      </c>
+        <v>6.75</v>
+      </c>
+      <c r="J8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1374,7 +1374,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>78.15000000000001</v>
+        <v>78.45</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -1396,7 +1396,7 @@
       </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="n">
-        <v>6.5</v>
+        <v>6.73</v>
       </c>
       <c r="J9" t="inlineStr"/>
     </row>
@@ -1434,14 +1434,14 @@
       </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="n">
-        <v>6.38</v>
+        <v>6.47</v>
       </c>
       <c r="J10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1450,7 +1450,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>77.72</v>
+        <v>76.75</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -1472,23 +1472,23 @@
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="n">
-        <v>6.31</v>
+        <v>5.96</v>
       </c>
       <c r="J11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>EME</t>
+          <t>ALAB</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>76.65000000000001</v>
+        <v>76.48</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -1510,27 +1510,23 @@
       </c>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="n">
-        <v>5.83</v>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>Added 2026-05-25: score 75.2, DC construction, strong momentum (86.7).</t>
-        </is>
-      </c>
+        <v>5.84</v>
+      </c>
+      <c r="J12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ALAB</t>
+          <t>FIX</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>76.48</v>
+        <v>76.34999999999999</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -1552,23 +1548,27 @@
       </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="n">
-        <v>5.75</v>
-      </c>
-      <c r="J13" t="inlineStr"/>
+        <v>5.78</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Manually excluded 2026-05-18: $1,854 share price prevents reasonable position sizing below ~$50k portfolio. Conscious framework override. | Override removed 2026-06-09: fractional shares adopted, share-price constraint obsolete (Dom decision).</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>FIX</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>76.34999999999999</v>
+        <v>75.47</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -1590,27 +1590,23 @@
       </c>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="n">
-        <v>5.7</v>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>Manually excluded 2026-05-18: $1,854 share price prevents reasonable position sizing below ~$50k portfolio. Conscious framework override. | Override removed 2026-06-09: fractional shares adopted, share-price constraint obsolete (Dom decision).</t>
-        </is>
-      </c>
+        <v>5.38</v>
+      </c>
+      <c r="J14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>PLTR</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
+          <t>10 Models, Software &amp; Applications</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>76.25</v>
+        <v>74.84999999999999</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -1632,23 +1628,23 @@
       </c>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="n">
-        <v>5.65</v>
+        <v>5.1</v>
       </c>
       <c r="J15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>PLTR</t>
+          <t>EME</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>74.84999999999999</v>
+        <v>74.55</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -1670,9 +1666,13 @@
       </c>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="n">
-        <v>5.03</v>
-      </c>
-      <c r="J16" t="inlineStr"/>
+        <v>4.97</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Added 2026-05-25: score 75.2, DC construction, strong momentum (86.7).</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1708,7 +1708,7 @@
       </c>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="n">
-        <v>4.58</v>
+        <v>4.65</v>
       </c>
       <c r="J17" t="inlineStr"/>
     </row>
@@ -1781,16 +1781,16 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>TER</t>
+          <t>DELL</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>73</v>
+        <v>72.67</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -1800,35 +1800,28 @@
       <c r="E20" t="n">
         <v>18</v>
       </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>HOLD</t>
-        </is>
-      </c>
+      <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H20" t="inlineStr"/>
-      <c r="I20" t="n">
-        <v>4.2</v>
-      </c>
       <c r="J20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>DELL</t>
+          <t>MRVL</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling</t>
+          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>72.67</v>
+        <v>72.42</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -1850,16 +1843,16 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>MRVL</t>
+          <t>APH</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
+          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>72.42</v>
+        <v>72.28</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -1881,16 +1874,16 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>APH</t>
+          <t>TER</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>72.28</v>
+        <v>72.25</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -1900,13 +1893,20 @@
       <c r="E23" t="n">
         <v>21</v>
       </c>
-      <c r="F23" t="inlineStr"/>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>EXIT PENDING (score 72.2, since 2026-06-12)</t>
+        </is>
+      </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H23" t="inlineStr"/>
+      <c r="I23" t="n">
+        <v>3.93</v>
+      </c>
       <c r="J23" t="inlineStr"/>
     </row>
     <row r="24">
@@ -3943,16 +3943,16 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>PSTG</t>
+          <t>HPE</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>61.8</v>
+        <v>61.48</v>
       </c>
       <c r="D89" t="inlineStr">
         <is>
@@ -3974,16 +3974,16 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>HPE</t>
+          <t>CRWD</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling</t>
+          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>61.48</v>
+        <v>61.45</v>
       </c>
       <c r="D90" t="inlineStr">
         <is>
@@ -4005,16 +4005,16 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>CRWD</t>
+          <t>NXT</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
+          <t>01 Power Generation / Solar &amp; renewables equipment (behind-the-meter DC power)</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>61.45</v>
+        <v>61.42</v>
       </c>
       <c r="D91" t="inlineStr">
         <is>
@@ -4036,16 +4036,16 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>NXT</t>
+          <t>CMI</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>01 Power Generation / Solar &amp; renewables equipment (behind-the-meter DC power)</t>
+          <t>01 Power Generation / Distributed / on-site power</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>61.42</v>
+        <v>61.35</v>
       </c>
       <c r="D92" t="inlineStr">
         <is>
@@ -4067,16 +4067,16 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>CMI</t>
+          <t>EQIX</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>01 Power Generation / Distributed / on-site power</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>61.35</v>
+        <v>60.25</v>
       </c>
       <c r="D93" t="inlineStr">
         <is>
@@ -4098,12 +4098,12 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>EQIX</t>
+          <t>HUT</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -4129,12 +4129,12 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>HUT</t>
+          <t>TTMI</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
+          <t>04 Semiconductor Equipment &amp; Materials / PCB / substrates</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -4160,16 +4160,16 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>TTMI</t>
+          <t>COHR</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / PCB / substrates</t>
+          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>60.25</v>
+        <v>60.05</v>
       </c>
       <c r="D96" t="inlineStr">
         <is>
@@ -4191,16 +4191,16 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>COHR</t>
+          <t>BWXT</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
+          <t>01 Power Generation / Nuclear-specific</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>60.05</v>
+        <v>59.78</v>
       </c>
       <c r="D97" t="inlineStr">
         <is>
@@ -4222,16 +4222,16 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>BWXT</t>
+          <t>DUK</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>01 Power Generation / Nuclear-specific</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>59.78</v>
+        <v>59.65</v>
       </c>
       <c r="D98" t="inlineStr">
         <is>
@@ -4253,16 +4253,16 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>DUK</t>
+          <t>P</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>59.65</v>
+        <v>59.55</v>
       </c>
       <c r="D99" t="inlineStr">
         <is>
@@ -5259,14 +5259,14 @@
         <v>83.3</v>
       </c>
       <c r="C4" t="n">
-        <v>8.800000000000001</v>
+        <v>8.93</v>
       </c>
       <c r="D4">
         <f>C4/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E4" t="n">
-        <v>206.8</v>
+        <v>204.86</v>
       </c>
       <c r="F4">
         <f>IF(E4="","",ROUND(D4/E4,4))</f>
@@ -5289,17 +5289,17 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>80.09999999999999</v>
+        <v>81.59999999999999</v>
       </c>
       <c r="C5" t="n">
-        <v>7.37</v>
+        <v>8.15</v>
       </c>
       <c r="D5">
         <f>C5/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E5" t="n">
-        <v>426.36</v>
+        <v>424.62</v>
       </c>
       <c r="F5">
         <f>IF(E5="","",ROUND(D5/E5,4))</f>
@@ -5325,14 +5325,14 @@
         <v>79.7</v>
       </c>
       <c r="C6" t="n">
-        <v>7.17</v>
+        <v>7.27</v>
       </c>
       <c r="D6">
         <f>C6/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E6" t="n">
-        <v>1985.5</v>
+        <v>1991</v>
       </c>
       <c r="F6">
         <f>IF(E6="","",ROUND(D6/E6,4))</f>
@@ -5358,14 +5358,14 @@
         <v>79.5</v>
       </c>
       <c r="C7" t="n">
-        <v>7.1</v>
+        <v>7.2</v>
       </c>
       <c r="D7">
         <f>C7/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E7" t="n">
-        <v>1001.28</v>
+        <v>993.53</v>
       </c>
       <c r="F7">
         <f>IF(E7="","",ROUND(D7/E7,4))</f>
@@ -5384,21 +5384,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>META</t>
+          <t>CRDO</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>79</v>
+        <v>78.8</v>
       </c>
       <c r="C8" t="n">
-        <v>6.85</v>
+        <v>6.89</v>
       </c>
       <c r="D8">
         <f>C8/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E8" t="n">
-        <v>572.49</v>
+        <v>258.04</v>
       </c>
       <c r="F8">
         <f>IF(E8="","",ROUND(D8/E8,4))</f>
@@ -5417,21 +5417,21 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CRDO</t>
+          <t>META</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>78.8</v>
+        <v>78.5</v>
       </c>
       <c r="C9" t="n">
-        <v>6.79</v>
+        <v>6.75</v>
       </c>
       <c r="D9">
         <f>C9/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E9" t="n">
-        <v>254.34</v>
+        <v>570.88</v>
       </c>
       <c r="F9">
         <f>IF(E9="","",ROUND(D9/E9,4))</f>
@@ -5454,17 +5454,17 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>78.2</v>
+        <v>78.5</v>
       </c>
       <c r="C10" t="n">
-        <v>6.5</v>
+        <v>6.73</v>
       </c>
       <c r="D10">
         <f>C10/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E10" t="n">
-        <v>383.41</v>
+        <v>381.05</v>
       </c>
       <c r="F10">
         <f>IF(E10="","",ROUND(D10/E10,4))</f>
@@ -5490,14 +5490,14 @@
         <v>77.90000000000001</v>
       </c>
       <c r="C11" t="n">
-        <v>6.38</v>
+        <v>6.47</v>
       </c>
       <c r="D11">
         <f>C11/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E11" t="n">
-        <v>164.57</v>
+        <v>163.65</v>
       </c>
       <c r="F11">
         <f>IF(E11="","",ROUND(D11/E11,4))</f>
@@ -5516,21 +5516,21 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>77.7</v>
+        <v>76.8</v>
       </c>
       <c r="C12" t="n">
-        <v>6.31</v>
+        <v>5.96</v>
       </c>
       <c r="D12">
         <f>C12/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E12" t="n">
-        <v>365.38</v>
+        <v>387.56</v>
       </c>
       <c r="F12">
         <f>IF(E12="","",ROUND(D12/E12,4))</f>
@@ -5549,21 +5549,21 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>EME</t>
+          <t>ALAB</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>76.7</v>
+        <v>76.5</v>
       </c>
       <c r="C13" t="n">
-        <v>5.83</v>
+        <v>5.84</v>
       </c>
       <c r="D13">
         <f>C13/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E13" t="n">
-        <v>824.97</v>
+        <v>382.95</v>
       </c>
       <c r="F13">
         <f>IF(E13="","",ROUND(D13/E13,4))</f>
@@ -5582,21 +5582,21 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ALAB</t>
+          <t>FIX</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>76.5</v>
+        <v>76.40000000000001</v>
       </c>
       <c r="C14" t="n">
-        <v>5.75</v>
+        <v>5.78</v>
       </c>
       <c r="D14">
         <f>C14/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E14" t="n">
-        <v>381.78</v>
+        <v>1904.31</v>
       </c>
       <c r="F14">
         <f>IF(E14="","",ROUND(D14/E14,4))</f>
@@ -5615,21 +5615,21 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>FIX</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>76.40000000000001</v>
+        <v>75.5</v>
       </c>
       <c r="C15" t="n">
-        <v>5.7</v>
+        <v>5.38</v>
       </c>
       <c r="D15">
         <f>C15/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E15" t="n">
-        <v>1886.54</v>
+        <v>361.36</v>
       </c>
       <c r="F15">
         <f>IF(E15="","",ROUND(D15/E15,4))</f>
@@ -5648,21 +5648,21 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>PLTR</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>76.2</v>
+        <v>74.8</v>
       </c>
       <c r="C16" t="n">
-        <v>5.65</v>
+        <v>5.1</v>
       </c>
       <c r="D16">
         <f>C16/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E16" t="n">
-        <v>389.13</v>
+        <v>128.14</v>
       </c>
       <c r="F16">
         <f>IF(E16="","",ROUND(D16/E16,4))</f>
@@ -5681,21 +5681,21 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>PLTR</t>
+          <t>EME</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>74.8</v>
+        <v>74.5</v>
       </c>
       <c r="C17" t="n">
-        <v>5.03</v>
+        <v>4.97</v>
       </c>
       <c r="D17">
         <f>C17/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E17" t="n">
-        <v>130.12</v>
+        <v>823.29</v>
       </c>
       <c r="F17">
         <f>IF(E17="","",ROUND(D17/E17,4))</f>
@@ -5721,14 +5721,14 @@
         <v>73.8</v>
       </c>
       <c r="C18" t="n">
-        <v>4.58</v>
+        <v>4.65</v>
       </c>
       <c r="D18">
         <f>C18/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E18" t="n">
-        <v>52.22</v>
+        <v>51.97</v>
       </c>
       <c r="F18">
         <f>IF(E18="","",ROUND(D18/E18,4))</f>
@@ -5751,17 +5751,17 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>73</v>
+        <v>72.2</v>
       </c>
       <c r="C19" t="n">
-        <v>4.2</v>
+        <v>3.93</v>
       </c>
       <c r="D19">
         <f>C19/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E19" t="n">
-        <v>404.93</v>
+        <v>402.99</v>
       </c>
       <c r="F19">
         <f>IF(E19="","",ROUND(D19/E19,4))</f>

</xml_diff>

<commit_message>
rating session close: TER R2 override to 4 on peer calibration — TER 73.0 at-threshold HOLD, no exit pending; R2 rubric re-eval queued
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/00-master/portfolio.xlsx
+++ b/00-master/portfolio.xlsx
@@ -1160,7 +1160,7 @@
       </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="n">
-        <v>8.93</v>
+        <v>8.84</v>
       </c>
       <c r="J3" t="inlineStr"/>
     </row>
@@ -1198,7 +1198,7 @@
       </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="n">
-        <v>8.15</v>
+        <v>8.07</v>
       </c>
       <c r="J4" t="inlineStr"/>
     </row>
@@ -1236,7 +1236,7 @@
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="n">
-        <v>7.27</v>
+        <v>7.2</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -1278,7 +1278,7 @@
       </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="n">
-        <v>7.2</v>
+        <v>7.13</v>
       </c>
       <c r="J6" t="inlineStr"/>
     </row>
@@ -1316,7 +1316,7 @@
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="n">
-        <v>6.89</v>
+        <v>6.82</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -1358,7 +1358,7 @@
       </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="n">
-        <v>6.75</v>
+        <v>6.68</v>
       </c>
       <c r="J8" t="inlineStr"/>
     </row>
@@ -1396,7 +1396,7 @@
       </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="n">
-        <v>6.73</v>
+        <v>6.66</v>
       </c>
       <c r="J9" t="inlineStr"/>
     </row>
@@ -1434,7 +1434,7 @@
       </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="n">
-        <v>6.47</v>
+        <v>6.4</v>
       </c>
       <c r="J10" t="inlineStr"/>
     </row>
@@ -1472,7 +1472,7 @@
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="n">
-        <v>5.96</v>
+        <v>5.9</v>
       </c>
       <c r="J11" t="inlineStr"/>
     </row>
@@ -1510,7 +1510,7 @@
       </c>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="n">
-        <v>5.84</v>
+        <v>5.78</v>
       </c>
       <c r="J12" t="inlineStr"/>
     </row>
@@ -1548,7 +1548,7 @@
       </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="n">
-        <v>5.78</v>
+        <v>5.72</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
@@ -1568,7 +1568,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>75.47</v>
+        <v>76.22</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -1590,23 +1590,23 @@
       </c>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="n">
-        <v>5.38</v>
+        <v>5.66</v>
       </c>
       <c r="J14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>PLTR</t>
+          <t>EME</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>74.84999999999999</v>
+        <v>75.34999999999999</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -1628,23 +1628,27 @@
       </c>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="n">
-        <v>5.1</v>
-      </c>
-      <c r="J15" t="inlineStr"/>
+        <v>5.27</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Added 2026-05-25: score 75.2, DC construction, strong momentum (86.7).</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>EME</t>
+          <t>PLTR</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>10 Models, Software &amp; Applications</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>74.55</v>
+        <v>74.84999999999999</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -1666,13 +1670,9 @@
       </c>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="n">
-        <v>4.97</v>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>Added 2026-05-25: score 75.2, DC construction, strong momentum (86.7).</t>
-        </is>
-      </c>
+        <v>5.05</v>
+      </c>
+      <c r="J16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1708,7 +1708,7 @@
       </c>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="n">
-        <v>4.65</v>
+        <v>4.6</v>
       </c>
       <c r="J17" t="inlineStr"/>
     </row>
@@ -1781,16 +1781,16 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>DELL</t>
+          <t>TER</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>72.67</v>
+        <v>73</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -1800,28 +1800,35 @@
       <c r="E20" t="n">
         <v>18</v>
       </c>
-      <c r="F20" t="inlineStr"/>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H20" t="inlineStr"/>
+      <c r="I20" t="n">
+        <v>4.22</v>
+      </c>
       <c r="J20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>MRVL</t>
+          <t>DELL</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>72.42</v>
+        <v>72.67</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -1843,16 +1850,16 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>APH</t>
+          <t>MRVL</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
+          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>72.28</v>
+        <v>72.42</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -1874,16 +1881,16 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>TER</t>
+          <t>APH</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>72.25</v>
+        <v>72.28</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -1893,20 +1900,13 @@
       <c r="E23" t="n">
         <v>21</v>
       </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>EXIT PENDING (score 72.2, since 2026-06-12)</t>
-        </is>
-      </c>
+      <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H23" t="inlineStr"/>
-      <c r="I23" t="n">
-        <v>3.93</v>
-      </c>
       <c r="J23" t="inlineStr"/>
     </row>
     <row r="24">
@@ -5259,14 +5259,14 @@
         <v>83.3</v>
       </c>
       <c r="C4" t="n">
-        <v>8.93</v>
+        <v>8.84</v>
       </c>
       <c r="D4">
         <f>C4/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E4" t="n">
-        <v>204.86</v>
+        <v>204.82</v>
       </c>
       <c r="F4">
         <f>IF(E4="","",ROUND(D4/E4,4))</f>
@@ -5292,14 +5292,14 @@
         <v>81.59999999999999</v>
       </c>
       <c r="C5" t="n">
-        <v>8.15</v>
+        <v>8.07</v>
       </c>
       <c r="D5">
         <f>C5/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E5" t="n">
-        <v>424.62</v>
+        <v>424.61</v>
       </c>
       <c r="F5">
         <f>IF(E5="","",ROUND(D5/E5,4))</f>
@@ -5325,14 +5325,14 @@
         <v>79.7</v>
       </c>
       <c r="C6" t="n">
-        <v>7.27</v>
+        <v>7.2</v>
       </c>
       <c r="D6">
         <f>C6/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E6" t="n">
-        <v>1991</v>
+        <v>2008.88</v>
       </c>
       <c r="F6">
         <f>IF(E6="","",ROUND(D6/E6,4))</f>
@@ -5358,14 +5358,14 @@
         <v>79.5</v>
       </c>
       <c r="C7" t="n">
-        <v>7.2</v>
+        <v>7.13</v>
       </c>
       <c r="D7">
         <f>C7/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E7" t="n">
-        <v>993.53</v>
+        <v>997.28</v>
       </c>
       <c r="F7">
         <f>IF(E7="","",ROUND(D7/E7,4))</f>
@@ -5391,14 +5391,14 @@
         <v>78.8</v>
       </c>
       <c r="C8" t="n">
-        <v>6.89</v>
+        <v>6.82</v>
       </c>
       <c r="D8">
         <f>C8/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E8" t="n">
-        <v>258.04</v>
+        <v>255.44</v>
       </c>
       <c r="F8">
         <f>IF(E8="","",ROUND(D8/E8,4))</f>
@@ -5424,14 +5424,14 @@
         <v>78.5</v>
       </c>
       <c r="C9" t="n">
-        <v>6.75</v>
+        <v>6.68</v>
       </c>
       <c r="D9">
         <f>C9/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E9" t="n">
-        <v>570.88</v>
+        <v>569.72</v>
       </c>
       <c r="F9">
         <f>IF(E9="","",ROUND(D9/E9,4))</f>
@@ -5457,14 +5457,14 @@
         <v>78.5</v>
       </c>
       <c r="C10" t="n">
-        <v>6.73</v>
+        <v>6.66</v>
       </c>
       <c r="D10">
         <f>C10/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E10" t="n">
-        <v>381.05</v>
+        <v>380.82</v>
       </c>
       <c r="F10">
         <f>IF(E10="","",ROUND(D10/E10,4))</f>
@@ -5490,14 +5490,14 @@
         <v>77.90000000000001</v>
       </c>
       <c r="C11" t="n">
-        <v>6.47</v>
+        <v>6.4</v>
       </c>
       <c r="D11">
         <f>C11/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E11" t="n">
-        <v>163.65</v>
+        <v>163.57</v>
       </c>
       <c r="F11">
         <f>IF(E11="","",ROUND(D11/E11,4))</f>
@@ -5523,14 +5523,14 @@
         <v>76.8</v>
       </c>
       <c r="C12" t="n">
-        <v>5.96</v>
+        <v>5.9</v>
       </c>
       <c r="D12">
         <f>C12/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E12" t="n">
-        <v>387.56</v>
+        <v>387.42</v>
       </c>
       <c r="F12">
         <f>IF(E12="","",ROUND(D12/E12,4))</f>
@@ -5556,14 +5556,14 @@
         <v>76.5</v>
       </c>
       <c r="C13" t="n">
-        <v>5.84</v>
+        <v>5.78</v>
       </c>
       <c r="D13">
         <f>C13/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E13" t="n">
-        <v>382.95</v>
+        <v>380.24</v>
       </c>
       <c r="F13">
         <f>IF(E13="","",ROUND(D13/E13,4))</f>
@@ -5589,14 +5589,14 @@
         <v>76.40000000000001</v>
       </c>
       <c r="C14" t="n">
-        <v>5.78</v>
+        <v>5.72</v>
       </c>
       <c r="D14">
         <f>C14/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E14" t="n">
-        <v>1904.31</v>
+        <v>1907.38</v>
       </c>
       <c r="F14">
         <f>IF(E14="","",ROUND(D14/E14,4))</f>
@@ -5619,17 +5619,17 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>75.5</v>
+        <v>76.2</v>
       </c>
       <c r="C15" t="n">
-        <v>5.38</v>
+        <v>5.66</v>
       </c>
       <c r="D15">
         <f>C15/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E15" t="n">
-        <v>361.36</v>
+        <v>361.55</v>
       </c>
       <c r="F15">
         <f>IF(E15="","",ROUND(D15/E15,4))</f>
@@ -5648,21 +5648,21 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>PLTR</t>
+          <t>EME</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>74.8</v>
+        <v>75.3</v>
       </c>
       <c r="C16" t="n">
-        <v>5.1</v>
+        <v>5.27</v>
       </c>
       <c r="D16">
         <f>C16/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E16" t="n">
-        <v>128.14</v>
+        <v>822.67</v>
       </c>
       <c r="F16">
         <f>IF(E16="","",ROUND(D16/E16,4))</f>
@@ -5681,21 +5681,21 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>EME</t>
+          <t>PLTR</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>74.5</v>
+        <v>74.8</v>
       </c>
       <c r="C17" t="n">
-        <v>4.97</v>
+        <v>5.05</v>
       </c>
       <c r="D17">
         <f>C17/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E17" t="n">
-        <v>823.29</v>
+        <v>127.97</v>
       </c>
       <c r="F17">
         <f>IF(E17="","",ROUND(D17/E17,4))</f>
@@ -5721,14 +5721,14 @@
         <v>73.8</v>
       </c>
       <c r="C18" t="n">
-        <v>4.65</v>
+        <v>4.6</v>
       </c>
       <c r="D18">
         <f>C18/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E18" t="n">
-        <v>51.97</v>
+        <v>51.74</v>
       </c>
       <c r="F18">
         <f>IF(E18="","",ROUND(D18/E18,4))</f>
@@ -5751,17 +5751,17 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>72.2</v>
+        <v>73</v>
       </c>
       <c r="C19" t="n">
-        <v>3.93</v>
+        <v>4.22</v>
       </c>
       <c r="D19">
         <f>C19/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E19" t="n">
-        <v>402.99</v>
+        <v>403.04</v>
       </c>
       <c r="F19">
         <f>IF(E19="","",ROUND(D19/E19,4))</f>

</xml_diff>

<commit_message>
NVDA Q1 FY27 + MOD Q4 FY26 /earnings-update; fix yfinance levered-FCF garbage inputs for both
NVDA: $1T Blackwell+Rubin visibility, networking ~18% of rev, FCF margin
47% TTM (yfinance info.freeCashflow artifact corrected with statement
values). MOD: $4B chillers-only LTA detailed (CY27-29, <=$2B/yr, ~11%
customer prepaying $165M), DC FY27 guide raised to +60-80%, MOD 68.8.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/00-master/portfolio.xlsx
+++ b/00-master/portfolio.xlsx
@@ -1850,16 +1850,16 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>MRVL</t>
+          <t>APH</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
+          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>72.42</v>
+        <v>72.28</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -1881,16 +1881,16 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>APH</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
+          <t>10 Models, Software &amp; Applications</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>72.28</v>
+        <v>72</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -1907,21 +1907,25 @@
         </is>
       </c>
       <c r="H23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Added 2026-05-25: score 74.8, Quality 97, PEG 0.8. Enterprise SaaS with AI exposure.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications</t>
+          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>72</v>
+        <v>71.95</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -1938,25 +1942,21 @@
         </is>
       </c>
       <c r="H24" t="inlineStr"/>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>Added 2026-05-25: score 74.8, Quality 97, PEG 0.8. Enterprise SaaS with AI exposure.</t>
-        </is>
-      </c>
+      <c r="J24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>RRC</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
+          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>71.95</v>
+        <v>71.7</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -1978,16 +1978,16 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>RRC</t>
+          <t>LSCC</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
+          <t>06 AI Compute Silicon / Programmable logic</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>71.7</v>
+        <v>71.48</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -2009,16 +2009,16 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>LSCC</t>
+          <t>GEV</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Programmable logic</t>
+          <t>02 Grid Equipment</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>71.48</v>
+        <v>71.09999999999999</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -2040,16 +2040,16 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>GEV</t>
+          <t>EXE</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>02 Grid Equipment</t>
+          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>71.09999999999999</v>
+        <v>70.92</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -2071,16 +2071,16 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>EXE</t>
+          <t>KEYS</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>70.92</v>
+        <v>70.87</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -2102,16 +2102,16 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>KEYS</t>
+          <t>PATH</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
+          <t>10 Models, Software &amp; Applications / AI-powered automation</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>70.87</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
@@ -2133,16 +2133,16 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>PATH</t>
+          <t>LRCX</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI-powered automation</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>70.40000000000001</v>
+        <v>70.34999999999999</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -2164,16 +2164,16 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>LRCX</t>
+          <t>MPWR</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>06 AI Compute Silicon / Power management silicon</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>70.34999999999999</v>
+        <v>70.15000000000001</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -2195,16 +2195,16 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>MPWR</t>
+          <t>AR</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Power management silicon</t>
+          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>70.15000000000001</v>
+        <v>70</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -2221,25 +2221,29 @@
         </is>
       </c>
       <c r="H33" t="inlineStr"/>
-      <c r="J33" t="inlineStr"/>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>Added 2026-05-22 as substitute for CTRA (delisted). Pure score-driven pick: next-best ✓✓ at 75.62, same Layer 1 NG E&amp;P sub-category — preserves natural gas thesis concentration.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>ARM</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
+          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>70</v>
+        <v>69.95</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>✓✓</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="E34" t="n">
@@ -2252,25 +2256,21 @@
         </is>
       </c>
       <c r="H34" t="inlineStr"/>
-      <c r="J34" t="inlineStr">
-        <is>
-          <t>Added 2026-05-22 as substitute for CTRA (delisted). Pure score-driven pick: next-best ✓✓ at 75.62, same Layer 1 NG E&amp;P sub-category — preserves natural gas thesis concentration.</t>
-        </is>
-      </c>
+      <c r="J34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>ARM</t>
+          <t>CIEN</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
+          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>69.95</v>
+        <v>69.25</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
@@ -2292,12 +2292,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>CIEN</t>
+          <t>STX</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -2323,16 +2323,16 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>STX</t>
+          <t>TEL</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
+          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>69.25</v>
+        <v>69.2</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
@@ -2354,16 +2354,16 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>TEL</t>
+          <t>TLN</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
+          <t>01 Power Generation / Independent Power Producers (IPPs)</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>69.2</v>
+        <v>69.17</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -2385,7 +2385,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>TLN</t>
+          <t>VST</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2394,7 +2394,7 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>69.17</v>
+        <v>69.09999999999999</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -2416,16 +2416,16 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>VST</t>
+          <t>FN</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>01 Power Generation / Independent Power Producers (IPPs)</t>
+          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>69.09999999999999</v>
+        <v>68.95</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -2447,16 +2447,16 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>FN</t>
+          <t>MOD</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>68.95</v>
+        <v>68.8</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -3474,16 +3474,16 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>FLEX</t>
+          <t>MRVL</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Contract manufacturing / ODMs</t>
+          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>64.84999999999999</v>
+        <v>64.97</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
@@ -3505,16 +3505,16 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>CCJ</t>
+          <t>FLEX</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>01 Power Generation / Nuclear-specific</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Contract manufacturing / ODMs</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>64.28</v>
+        <v>64.84999999999999</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
@@ -3536,16 +3536,16 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>HUBB</t>
+          <t>CCJ</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>01 Power Generation / Nuclear-specific</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>63.92</v>
+        <v>64.28</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
@@ -3567,16 +3567,16 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>GNRC</t>
+          <t>HUBB</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>01 Power Generation / Distributed / on-site power</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>63.85</v>
+        <v>63.92</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
@@ -3598,16 +3598,16 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>NEE</t>
+          <t>GNRC</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>01 Power Generation / Distributed / on-site power</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>63.62</v>
+        <v>63.85</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
@@ -3629,16 +3629,16 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>SNOW</t>
+          <t>NEE</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>63.4</v>
+        <v>63.62</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
@@ -3660,16 +3660,16 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>ORCL</t>
+          <t>SNOW</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
+          <t>10 Models, Software &amp; Applications</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>63.35</v>
+        <v>63.4</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
@@ -3691,16 +3691,16 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>KLIC</t>
+          <t>ORCL</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>63.08</v>
+        <v>63.35</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
@@ -3722,16 +3722,16 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>IRM</t>
+          <t>KLIC</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>62.6</v>
+        <v>63.08</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
@@ -3753,12 +3753,12 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>NBIS</t>
+          <t>IRM</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Neoclouds (AI-native cloud providers)</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -3779,25 +3779,21 @@
         </is>
       </c>
       <c r="H83" t="inlineStr"/>
-      <c r="J83" t="inlineStr">
-        <is>
-          <t>Removed 2026-05-25: dropped to ✓ (65.5) after reweight. Value 7.5 penalized by higher Value weight.</t>
-        </is>
-      </c>
+      <c r="J83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>SMCI</t>
+          <t>NBIS</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling</t>
+          <t>09 Compute-as-a-Service / Neoclouds (AI-native cloud providers)</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>62.45</v>
+        <v>62.6</v>
       </c>
       <c r="D84" t="inlineStr">
         <is>
@@ -3814,21 +3810,25 @@
         </is>
       </c>
       <c r="H84" t="inlineStr"/>
-      <c r="J84" t="inlineStr"/>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>Removed 2026-05-25: dropped to ✓ (65.5) after reweight. Value 7.5 penalized by higher Value weight.</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>ETN</t>
+          <t>SMCI</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>62.35</v>
+        <v>62.45</v>
       </c>
       <c r="D85" t="inlineStr">
         <is>
@@ -3850,16 +3850,16 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>CRWV</t>
+          <t>ETN</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>09 Cloud - Neocloud</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>62.23</v>
+        <v>62.35</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
@@ -3881,16 +3881,16 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>KN</t>
+          <t>CRWV</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>04 Semi Equip - Materials</t>
+          <t>09 Cloud - Neocloud</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>62.15</v>
+        <v>62.23</v>
       </c>
       <c r="D87" t="inlineStr">
         <is>
@@ -3912,16 +3912,16 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>LITE</t>
+          <t>KN</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
+          <t>04 Semi Equip - Materials</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>62.08</v>
+        <v>62.15</v>
       </c>
       <c r="D88" t="inlineStr">
         <is>
@@ -3943,16 +3943,16 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>HPE</t>
+          <t>LITE</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling</t>
+          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>61.48</v>
+        <v>62.08</v>
       </c>
       <c r="D89" t="inlineStr">
         <is>
@@ -3974,16 +3974,16 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>CRWD</t>
+          <t>HPE</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>61.45</v>
+        <v>61.48</v>
       </c>
       <c r="D90" t="inlineStr">
         <is>
@@ -4005,16 +4005,16 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>NXT</t>
+          <t>CRWD</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>01 Power Generation / Solar &amp; renewables equipment (behind-the-meter DC power)</t>
+          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>61.42</v>
+        <v>61.45</v>
       </c>
       <c r="D91" t="inlineStr">
         <is>
@@ -4036,16 +4036,16 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>CMI</t>
+          <t>NXT</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>01 Power Generation / Distributed / on-site power</t>
+          <t>01 Power Generation / Solar &amp; renewables equipment (behind-the-meter DC power)</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>61.35</v>
+        <v>61.42</v>
       </c>
       <c r="D92" t="inlineStr">
         <is>
@@ -4067,16 +4067,16 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>EQIX</t>
+          <t>CMI</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>01 Power Generation / Distributed / on-site power</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>60.25</v>
+        <v>61.35</v>
       </c>
       <c r="D93" t="inlineStr">
         <is>
@@ -4098,12 +4098,12 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>HUT</t>
+          <t>EQIX</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -4129,12 +4129,12 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>TTMI</t>
+          <t>HUT</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / PCB / substrates</t>
+          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -4160,16 +4160,16 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>COHR</t>
+          <t>TTMI</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
+          <t>04 Semiconductor Equipment &amp; Materials / PCB / substrates</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>60.05</v>
+        <v>60.25</v>
       </c>
       <c r="D96" t="inlineStr">
         <is>
@@ -4191,16 +4191,16 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>BWXT</t>
+          <t>COHR</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>01 Power Generation / Nuclear-specific</t>
+          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>59.78</v>
+        <v>60.05</v>
       </c>
       <c r="D97" t="inlineStr">
         <is>
@@ -4222,16 +4222,16 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>DUK</t>
+          <t>BWXT</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>01 Power Generation / Nuclear-specific</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>59.65</v>
+        <v>59.78</v>
       </c>
       <c r="D98" t="inlineStr">
         <is>
@@ -4253,16 +4253,16 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>DUK</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>59.55</v>
+        <v>59.65</v>
       </c>
       <c r="D99" t="inlineStr">
         <is>
@@ -4284,16 +4284,16 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>GFS</t>
+          <t>P</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>05 Fabs &amp; Foundries</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>59.35</v>
+        <v>59.55</v>
       </c>
       <c r="D100" t="inlineStr">
         <is>
@@ -4315,16 +4315,16 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>AEP</t>
+          <t>GFS</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>05 Fabs &amp; Foundries</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>58.92</v>
+        <v>59.35</v>
       </c>
       <c r="D101" t="inlineStr">
         <is>
@@ -4346,16 +4346,16 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>MOD</t>
+          <t>AEP</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>58.85</v>
+        <v>58.92</v>
       </c>
       <c r="D102" t="inlineStr">
         <is>
@@ -5266,7 +5266,7 @@
         <v/>
       </c>
       <c r="E4" t="n">
-        <v>204.82</v>
+        <v>204.37</v>
       </c>
       <c r="F4">
         <f>IF(E4="","",ROUND(D4/E4,4))</f>
@@ -5299,7 +5299,7 @@
         <v/>
       </c>
       <c r="E5" t="n">
-        <v>424.61</v>
+        <v>423.1</v>
       </c>
       <c r="F5">
         <f>IF(E5="","",ROUND(D5/E5,4))</f>
@@ -5332,7 +5332,7 @@
         <v/>
       </c>
       <c r="E6" t="n">
-        <v>2008.88</v>
+        <v>1989.67</v>
       </c>
       <c r="F6">
         <f>IF(E6="","",ROUND(D6/E6,4))</f>
@@ -5365,7 +5365,7 @@
         <v/>
       </c>
       <c r="E7" t="n">
-        <v>997.28</v>
+        <v>989.1</v>
       </c>
       <c r="F7">
         <f>IF(E7="","",ROUND(D7/E7,4))</f>
@@ -5398,7 +5398,7 @@
         <v/>
       </c>
       <c r="E8" t="n">
-        <v>255.44</v>
+        <v>253.64</v>
       </c>
       <c r="F8">
         <f>IF(E8="","",ROUND(D8/E8,4))</f>
@@ -5431,7 +5431,7 @@
         <v/>
       </c>
       <c r="E9" t="n">
-        <v>569.72</v>
+        <v>565.2</v>
       </c>
       <c r="F9">
         <f>IF(E9="","",ROUND(D9/E9,4))</f>
@@ -5464,7 +5464,7 @@
         <v/>
       </c>
       <c r="E10" t="n">
-        <v>380.82</v>
+        <v>379.69</v>
       </c>
       <c r="F10">
         <f>IF(E10="","",ROUND(D10/E10,4))</f>
@@ -5497,7 +5497,7 @@
         <v/>
       </c>
       <c r="E11" t="n">
-        <v>163.57</v>
+        <v>164.14</v>
       </c>
       <c r="F11">
         <f>IF(E11="","",ROUND(D11/E11,4))</f>
@@ -5563,7 +5563,7 @@
         <v/>
       </c>
       <c r="E13" t="n">
-        <v>380.24</v>
+        <v>373.72</v>
       </c>
       <c r="F13">
         <f>IF(E13="","",ROUND(D13/E13,4))</f>
@@ -5596,7 +5596,7 @@
         <v/>
       </c>
       <c r="E14" t="n">
-        <v>1907.38</v>
+        <v>1905</v>
       </c>
       <c r="F14">
         <f>IF(E14="","",ROUND(D14/E14,4))</f>
@@ -5629,7 +5629,7 @@
         <v/>
       </c>
       <c r="E15" t="n">
-        <v>361.55</v>
+        <v>361.19</v>
       </c>
       <c r="F15">
         <f>IF(E15="","",ROUND(D15/E15,4))</f>
@@ -5662,7 +5662,7 @@
         <v/>
       </c>
       <c r="E16" t="n">
-        <v>822.67</v>
+        <v>821.85</v>
       </c>
       <c r="F16">
         <f>IF(E16="","",ROUND(D16/E16,4))</f>
@@ -5695,7 +5695,7 @@
         <v/>
       </c>
       <c r="E17" t="n">
-        <v>127.97</v>
+        <v>127.99</v>
       </c>
       <c r="F17">
         <f>IF(E17="","",ROUND(D17/E17,4))</f>
@@ -5728,7 +5728,7 @@
         <v/>
       </c>
       <c r="E18" t="n">
-        <v>51.74</v>
+        <v>51.93</v>
       </c>
       <c r="F18">
         <f>IF(E18="","",ROUND(D18/E18,4))</f>
@@ -5761,7 +5761,7 @@
         <v/>
       </c>
       <c r="E19" t="n">
-        <v>403.04</v>
+        <v>403.25</v>
       </c>
       <c r="F19">
         <f>IF(E19="","",ROUND(D19/E19,4))</f>

</xml_diff>

<commit_message>
fix(data): statement-based FCF across all inputs — yfinance info.freeCashflow is levered estimate
- batch_score.statement_fcf(): TTM OCF - |capex| from quarterly_cashflow,
  info field fallback-only with flag; yfinance_fundamentals.py same
- full watchlist re-pull: 127/135 updated (8 statement-unavailable kept+flagged)
- big corrections: NEE -66->+8.5 FCF mgn, CEG -15->+3.8, TSM Value 53->64
- TSM 83.8 now #1; VRT 74.5 at entry threshold (no cross); TER 73.0 HOLD
- removed superseded NVDA Q1-FY2027 reconstruction transcripts (approved)
- CLAUDE.md: yfinance FCF trap documented

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/00-master/portfolio.xlsx
+++ b/00-master/portfolio.xlsx
@@ -1129,16 +1129,16 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>NVDA</t>
+          <t>TSM</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / GPUs / merchant accelerators</t>
+          <t>05 Fabs &amp; Foundries</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>83.33</v>
+        <v>83.8</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -1160,23 +1160,23 @@
       </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="n">
-        <v>8.84</v>
+        <v>9.01</v>
       </c>
       <c r="J3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>TSM</t>
+          <t>NVDA</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>05 Fabs &amp; Foundries</t>
+          <t>06 AI Compute Silicon / GPUs / merchant accelerators</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>81.59999999999999</v>
+        <v>83.33</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
       </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="n">
-        <v>8.07</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="J4" t="inlineStr"/>
     </row>
@@ -1236,7 +1236,7 @@
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="n">
-        <v>7.2</v>
+        <v>7.16</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -1256,7 +1256,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>79.5</v>
+        <v>78.90000000000001</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -1278,23 +1278,23 @@
       </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="n">
-        <v>7.13</v>
+        <v>6.83</v>
       </c>
       <c r="J6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CRDO</t>
+          <t>META</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Connectivity ASICs</t>
+          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>78.8</v>
+        <v>78.5</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -1316,27 +1316,23 @@
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="n">
-        <v>6.82</v>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>Added 2026-05-25: score 78.4, ranked #4 in reweighted watchlist. Optical connectivity pure-play.</t>
-        </is>
-      </c>
+        <v>6.65</v>
+      </c>
+      <c r="J7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>META</t>
+          <t>AVGO</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
+          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>78.5</v>
+        <v>78.45</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -1358,23 +1354,23 @@
       </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="n">
-        <v>6.68</v>
+        <v>6.63</v>
       </c>
       <c r="J8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>AVGO</t>
+          <t>CRDO</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
+          <t>07 Optical, Networking &amp; Interconnect / Connectivity ASICs</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>78.45</v>
+        <v>78.3</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -1396,9 +1392,13 @@
       </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="n">
-        <v>6.66</v>
-      </c>
-      <c r="J9" t="inlineStr"/>
+        <v>6.56</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Added 2026-05-25: score 78.4, ranked #4 in reweighted watchlist. Optical connectivity pure-play.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1434,7 +1434,7 @@
       </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="n">
-        <v>6.4</v>
+        <v>6.37</v>
       </c>
       <c r="J10" t="inlineStr"/>
     </row>
@@ -1472,7 +1472,7 @@
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="n">
-        <v>5.9</v>
+        <v>5.87</v>
       </c>
       <c r="J11" t="inlineStr"/>
     </row>
@@ -1510,7 +1510,7 @@
       </c>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="n">
-        <v>5.78</v>
+        <v>5.75</v>
       </c>
       <c r="J12" t="inlineStr"/>
     </row>
@@ -1548,7 +1548,7 @@
       </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="n">
-        <v>5.72</v>
+        <v>5.69</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
@@ -1590,7 +1590,7 @@
       </c>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="n">
-        <v>5.66</v>
+        <v>5.64</v>
       </c>
       <c r="J14" t="inlineStr"/>
     </row>
@@ -1628,7 +1628,7 @@
       </c>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="n">
-        <v>5.27</v>
+        <v>5.25</v>
       </c>
       <c r="J15" t="inlineStr">
         <is>
@@ -1670,23 +1670,23 @@
       </c>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="n">
-        <v>5.05</v>
+        <v>5.02</v>
       </c>
       <c r="J16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>EQT</t>
+          <t>VRT</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
+          <t>03 DC Infrastructure</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>73.84999999999999</v>
+        <v>74.45</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -1696,35 +1696,28 @@
       <c r="E17" t="n">
         <v>15</v>
       </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>HOLD</t>
-        </is>
-      </c>
+      <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H17" t="inlineStr"/>
-      <c r="I17" t="n">
-        <v>4.6</v>
-      </c>
       <c r="J17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>VRT</t>
+          <t>EQT</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>03 DC Infrastructure</t>
+          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>73.7</v>
+        <v>73.84999999999999</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -1734,13 +1727,20 @@
       <c r="E18" t="n">
         <v>16</v>
       </c>
-      <c r="F18" t="inlineStr"/>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H18" t="inlineStr"/>
+      <c r="I18" t="n">
+        <v>4.58</v>
+      </c>
       <c r="J18" t="inlineStr"/>
     </row>
     <row r="19">
@@ -1812,23 +1812,23 @@
       </c>
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="n">
-        <v>4.22</v>
+        <v>4.2</v>
       </c>
       <c r="J20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>DELL</t>
+          <t>KEYS</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>72.67</v>
+        <v>72.47</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -1881,16 +1881,16 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>DELL</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>72</v>
+        <v>72.08</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -1907,25 +1907,21 @@
         </is>
       </c>
       <c r="H23" t="inlineStr"/>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>Added 2026-05-25: score 74.8, Quality 97, PEG 0.8. Enterprise SaaS with AI exposure.</t>
-        </is>
-      </c>
+      <c r="J23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
+          <t>10 Models, Software &amp; Applications</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>71.95</v>
+        <v>72</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -1942,21 +1938,25 @@
         </is>
       </c>
       <c r="H24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Added 2026-05-25: score 74.8, Quality 97, PEG 0.8. Enterprise SaaS with AI exposure.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>RRC</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
+          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>71.7</v>
+        <v>71.95</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -1978,16 +1978,16 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>LSCC</t>
+          <t>STX</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Programmable logic</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>71.48</v>
+        <v>71.84999999999999</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -2009,16 +2009,16 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>GEV</t>
+          <t>RRC</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>02 Grid Equipment</t>
+          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>71.09999999999999</v>
+        <v>71.7</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -2049,7 +2049,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>70.92</v>
+        <v>71.67</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -2071,16 +2071,16 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>KEYS</t>
+          <t>LSCC</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
+          <t>06 AI Compute Silicon / Programmable logic</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>70.87</v>
+        <v>71.48</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -2102,16 +2102,16 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>PATH</t>
+          <t>VST</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI-powered automation</t>
+          <t>01 Power Generation / Independent Power Producers (IPPs)</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>70.40000000000001</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
@@ -2133,16 +2133,16 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>LRCX</t>
+          <t>PATH</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>10 Models, Software &amp; Applications / AI-powered automation</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>70.34999999999999</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -2164,16 +2164,16 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>MPWR</t>
+          <t>GEV</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Power management silicon</t>
+          <t>02 Grid Equipment</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>70.15000000000001</v>
+        <v>70.34999999999999</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -2195,16 +2195,16 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>LRCX</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>70</v>
+        <v>70.34999999999999</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -2221,29 +2221,25 @@
         </is>
       </c>
       <c r="H33" t="inlineStr"/>
-      <c r="J33" t="inlineStr">
-        <is>
-          <t>Added 2026-05-22 as substitute for CTRA (delisted). Pure score-driven pick: next-best ✓✓ at 75.62, same Layer 1 NG E&amp;P sub-category — preserves natural gas thesis concentration.</t>
-        </is>
-      </c>
+      <c r="J33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>ARM</t>
+          <t>ABBNY</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>69.95</v>
+        <v>70.15000000000001</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>✓✓</t>
         </is>
       </c>
       <c r="E34" t="n">
@@ -2261,20 +2257,20 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>CIEN</t>
+          <t>MPWR</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
+          <t>06 AI Compute Silicon / Power management silicon</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>69.25</v>
+        <v>70.15000000000001</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>✓✓</t>
         </is>
       </c>
       <c r="E35" t="n">
@@ -2292,20 +2288,20 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>STX</t>
+          <t>AR</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
+          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>69.25</v>
+        <v>70</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>✓✓</t>
         </is>
       </c>
       <c r="E36" t="n">
@@ -2318,21 +2314,25 @@
         </is>
       </c>
       <c r="H36" t="inlineStr"/>
-      <c r="J36" t="inlineStr"/>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>Added 2026-05-22 as substitute for CTRA (delisted). Pure score-driven pick: next-best ✓✓ at 75.62, same Layer 1 NG E&amp;P sub-category — preserves natural gas thesis concentration.</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>TEL</t>
+          <t>CIEN</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
+          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>69.2</v>
+        <v>69.84999999999999</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
@@ -2354,16 +2354,16 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>TLN</t>
+          <t>PWR</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>01 Power Generation / Independent Power Producers (IPPs)</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>69.17</v>
+        <v>69.65000000000001</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -2385,16 +2385,16 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>VST</t>
+          <t>ARM</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>01 Power Generation / Independent Power Producers (IPPs)</t>
+          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>69.09999999999999</v>
+        <v>69.2</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -2416,16 +2416,16 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>FN</t>
+          <t>TEL</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
+          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>68.95</v>
+        <v>69.2</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -2447,16 +2447,16 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>MOD</t>
+          <t>CEG</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>01 Power - IPP / Nuclear</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>68.8</v>
+        <v>69.09999999999999</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -2478,16 +2478,16 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>GLW</t>
+          <t>UMC</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
+          <t>05 Fabs &amp; Foundries</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>68.8</v>
+        <v>69.05</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
@@ -2509,16 +2509,16 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>PWR</t>
+          <t>FN</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>68.3</v>
+        <v>68.95</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
@@ -2540,16 +2540,16 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>ASML</t>
+          <t>MOD</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>68.3</v>
+        <v>68.8</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -2571,16 +2571,16 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>KLAC</t>
+          <t>GLW</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>68.3</v>
+        <v>68.8</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
@@ -2602,16 +2602,16 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>AEIS</t>
+          <t>ASML</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>68.17</v>
+        <v>68.3</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -2633,7 +2633,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>AMAT</t>
+          <t>KLAC</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2642,7 +2642,7 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>68.15000000000001</v>
+        <v>68.3</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -2664,16 +2664,16 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>TT</t>
+          <t>AEIS</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>68.12</v>
+        <v>68.17</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -2695,16 +2695,16 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>HTHIY</t>
+          <t>AMAT</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>67.84999999999999</v>
+        <v>68.15000000000001</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
@@ -2726,16 +2726,16 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>NOW</t>
+          <t>TT</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>67.8</v>
+        <v>68.12</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
@@ -2757,16 +2757,16 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>DDOG</t>
+          <t>TLN</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI observability &amp; infrastructure software</t>
+          <t>01 Power Generation / Independent Power Producers (IPPs)</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>67.7</v>
+        <v>67.92</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
@@ -2783,25 +2783,21 @@
         </is>
       </c>
       <c r="H51" t="inlineStr"/>
-      <c r="J51" t="inlineStr">
-        <is>
-          <t>Added 2026-05-25: score 75.4, Quality 100, PEG 0.7. Beats 4 existing portfolio names.</t>
-        </is>
-      </c>
+      <c r="J51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>UMC</t>
+          <t>BESIY</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>05 Fabs &amp; Foundries</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>67.55</v>
+        <v>67.87</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
@@ -2823,7 +2819,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>ABBNY</t>
+          <t>HTHIY</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2832,7 +2828,7 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>67.45</v>
+        <v>67.84999999999999</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
@@ -2854,16 +2850,16 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>CDNS</t>
+          <t>NOW</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
+          <t>10 Models, Software &amp; Applications</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>67.40000000000001</v>
+        <v>67.8</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
@@ -2885,16 +2881,16 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>CSCO</t>
+          <t>DDOG</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
+          <t>10 Models, Software &amp; Applications / AI observability &amp; infrastructure software</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>67.40000000000001</v>
+        <v>67.7</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
@@ -2911,21 +2907,25 @@
         </is>
       </c>
       <c r="H55" t="inlineStr"/>
-      <c r="J55" t="inlineStr"/>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>Added 2026-05-25: score 75.4, Quality 100, PEG 0.7. Beats 4 existing portfolio names.</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>DLR</t>
+          <t>CDNS</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>67.2</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
@@ -2947,16 +2947,16 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>BESIY</t>
+          <t>CSCO</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>67.2</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
@@ -2978,16 +2978,16 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>CEG</t>
+          <t>FORM</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>01 Power - IPP / Nuclear</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>67.15000000000001</v>
+        <v>67.31999999999999</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
@@ -3009,16 +3009,16 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>SBGSY</t>
+          <t>DLR</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>67.05</v>
+        <v>67.2</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
@@ -3040,16 +3040,16 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>JCI</t>
+          <t>SBGSY</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>66.8</v>
+        <v>67.05</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
@@ -3071,16 +3071,16 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>POWL</t>
+          <t>JCI</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>66.75</v>
+        <v>66.8</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
@@ -3102,7 +3102,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>MTZ</t>
+          <t>POWL</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -3111,7 +3111,7 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>66.7</v>
+        <v>66.75</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
@@ -3133,7 +3133,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>NVT</t>
+          <t>MTZ</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -3142,7 +3142,7 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>66.55</v>
+        <v>66.7</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
@@ -3164,16 +3164,16 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>ONTO</t>
+          <t>NVT</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>66.09999999999999</v>
+        <v>66.55</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
@@ -3195,16 +3195,16 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>ENTG</t>
+          <t>NEE</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>66.05</v>
+        <v>66.33</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
@@ -3226,16 +3226,16 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>CCJ</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>01 Power - Distributed</t>
+          <t>01 Power Generation / Nuclear-specific</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>65.90000000000001</v>
+        <v>66.12</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
@@ -3257,16 +3257,16 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>AAON</t>
+          <t>ONTO</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>65.83</v>
+        <v>66.09999999999999</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
@@ -3288,16 +3288,16 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>FORM</t>
+          <t>TSEM</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
+          <t>05 Fabs &amp; Foundries</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>65.72</v>
+        <v>66.09999999999999</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
@@ -3319,7 +3319,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>MKSI</t>
+          <t>ENTG</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -3328,7 +3328,7 @@
         </is>
       </c>
       <c r="C69" t="n">
-        <v>65.7</v>
+        <v>66.05</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
@@ -3350,16 +3350,16 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>TSEM</t>
+          <t>RMBS</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>05 Fabs &amp; Foundries</t>
+          <t>06 AI Compute Silicon / Memory (HBM is the bottleneck)</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>65.5</v>
+        <v>65.97</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
@@ -3381,16 +3381,16 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>RMBS</t>
+          <t>AAON</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Memory (HBM is the bottleneck)</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>65.22</v>
+        <v>65.83</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
@@ -3412,16 +3412,16 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>PLAB</t>
+          <t>GNRC</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
+          <t>01 Power Generation / Distributed / on-site power</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>65.15000000000001</v>
+        <v>65.8</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
@@ -3443,16 +3443,16 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>SNPS</t>
+          <t>MKSI</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>65.09999999999999</v>
+        <v>65.7</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
@@ -3474,16 +3474,16 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>MRVL</t>
+          <t>HUBB</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>64.97</v>
+        <v>65.42</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
@@ -3505,16 +3505,16 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>FLEX</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Contract manufacturing / ODMs</t>
+          <t>01 Power - Distributed</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>64.84999999999999</v>
+        <v>65.15000000000001</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
@@ -3536,16 +3536,16 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>CCJ</t>
+          <t>PLAB</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>01 Power Generation / Nuclear-specific</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>64.28</v>
+        <v>65.15000000000001</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
@@ -3567,16 +3567,16 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>HUBB</t>
+          <t>SNPS</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>63.92</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
@@ -3598,16 +3598,16 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>GNRC</t>
+          <t>FLEX</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>01 Power Generation / Distributed / on-site power</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Contract manufacturing / ODMs</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>63.85</v>
+        <v>64.25</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
@@ -3629,16 +3629,16 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>NEE</t>
+          <t>ETN</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>63.62</v>
+        <v>63.85</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
@@ -3660,16 +3660,16 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>SNOW</t>
+          <t>MRVL</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications</t>
+          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>63.4</v>
+        <v>63.73</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
@@ -3691,16 +3691,16 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>ORCL</t>
+          <t>SNOW</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
+          <t>10 Models, Software &amp; Applications</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>63.35</v>
+        <v>63.4</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
@@ -3722,16 +3722,16 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>KLIC</t>
+          <t>ORCL</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>63.08</v>
+        <v>63.35</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
@@ -3753,16 +3753,16 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>IRM</t>
+          <t>NXT</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>01 Power Generation / Solar &amp; renewables equipment (behind-the-meter DC power)</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>62.6</v>
+        <v>63.17</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
@@ -3784,16 +3784,16 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>NBIS</t>
+          <t>KLIC</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Neoclouds (AI-native cloud providers)</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>62.6</v>
+        <v>63.08</v>
       </c>
       <c r="D84" t="inlineStr">
         <is>
@@ -3810,16 +3810,12 @@
         </is>
       </c>
       <c r="H84" t="inlineStr"/>
-      <c r="J84" t="inlineStr">
-        <is>
-          <t>Removed 2026-05-25: dropped to ✓ (65.5) after reweight. Value 7.5 penalized by higher Value weight.</t>
-        </is>
-      </c>
+      <c r="J84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>SMCI</t>
+          <t>HPE</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -3828,7 +3824,7 @@
         </is>
       </c>
       <c r="C85" t="n">
-        <v>62.45</v>
+        <v>62.98</v>
       </c>
       <c r="D85" t="inlineStr">
         <is>
@@ -3850,16 +3846,16 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>ETN</t>
+          <t>CMI</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>01 Power Generation / Distributed / on-site power</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>62.35</v>
+        <v>62.85</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
@@ -3881,16 +3877,16 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>CRWV</t>
+          <t>IRM</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>09 Cloud - Neocloud</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>62.23</v>
+        <v>62.6</v>
       </c>
       <c r="D87" t="inlineStr">
         <is>
@@ -3912,16 +3908,16 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>KN</t>
+          <t>NBIS</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>04 Semi Equip - Materials</t>
+          <t>09 Compute-as-a-Service / Neoclouds (AI-native cloud providers)</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>62.15</v>
+        <v>62.6</v>
       </c>
       <c r="D88" t="inlineStr">
         <is>
@@ -3938,21 +3934,25 @@
         </is>
       </c>
       <c r="H88" t="inlineStr"/>
-      <c r="J88" t="inlineStr"/>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>Removed 2026-05-25: dropped to ✓ (65.5) after reweight. Value 7.5 penalized by higher Value weight.</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>LITE</t>
+          <t>SMCI</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>62.08</v>
+        <v>62.45</v>
       </c>
       <c r="D89" t="inlineStr">
         <is>
@@ -3974,16 +3974,16 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>HPE</t>
+          <t>CRWV</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling</t>
+          <t>09 Cloud - Neocloud</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>61.48</v>
+        <v>62.23</v>
       </c>
       <c r="D90" t="inlineStr">
         <is>
@@ -4005,16 +4005,16 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>CRWD</t>
+          <t>KN</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
+          <t>04 Semi Equip - Materials</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>61.45</v>
+        <v>62.15</v>
       </c>
       <c r="D91" t="inlineStr">
         <is>
@@ -4036,16 +4036,16 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>NXT</t>
+          <t>LITE</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>01 Power Generation / Solar &amp; renewables equipment (behind-the-meter DC power)</t>
+          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>61.42</v>
+        <v>62.08</v>
       </c>
       <c r="D92" t="inlineStr">
         <is>
@@ -4067,16 +4067,16 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>CMI</t>
+          <t>CRWD</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>01 Power Generation / Distributed / on-site power</t>
+          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>61.35</v>
+        <v>61.45</v>
       </c>
       <c r="D93" t="inlineStr">
         <is>
@@ -4098,16 +4098,16 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>EQIX</t>
+          <t>BWXT</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>01 Power Generation / Nuclear-specific</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>60.25</v>
+        <v>61.12</v>
       </c>
       <c r="D94" t="inlineStr">
         <is>
@@ -4129,16 +4129,16 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>HUT</t>
+          <t>P</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>60.25</v>
+        <v>61.05</v>
       </c>
       <c r="D95" t="inlineStr">
         <is>
@@ -4160,12 +4160,12 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>TTMI</t>
+          <t>EQIX</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / PCB / substrates</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C96" t="n">
@@ -4191,16 +4191,16 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>COHR</t>
+          <t>HUT</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
+          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>60.05</v>
+        <v>60.25</v>
       </c>
       <c r="D97" t="inlineStr">
         <is>
@@ -4222,16 +4222,16 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>BWXT</t>
+          <t>TTMI</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>01 Power Generation / Nuclear-specific</t>
+          <t>04 Semiconductor Equipment &amp; Materials / PCB / substrates</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>59.78</v>
+        <v>60.25</v>
       </c>
       <c r="D98" t="inlineStr">
         <is>
@@ -4253,16 +4253,16 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>DUK</t>
+          <t>COHR</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>59.65</v>
+        <v>60.05</v>
       </c>
       <c r="D99" t="inlineStr">
         <is>
@@ -4284,16 +4284,16 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>DUK</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>59.55</v>
+        <v>59.65</v>
       </c>
       <c r="D100" t="inlineStr">
         <is>
@@ -5252,21 +5252,21 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>NVDA</t>
+          <t>TSM</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>83.3</v>
+        <v>83.8</v>
       </c>
       <c r="C4" t="n">
-        <v>8.84</v>
+        <v>9.01</v>
       </c>
       <c r="D4">
         <f>C4/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E4" t="n">
-        <v>204.37</v>
+        <v>424.35</v>
       </c>
       <c r="F4">
         <f>IF(E4="","",ROUND(D4/E4,4))</f>
@@ -5285,21 +5285,21 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>TSM</t>
+          <t>NVDA</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>81.59999999999999</v>
+        <v>83.3</v>
       </c>
       <c r="C5" t="n">
-        <v>8.07</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="D5">
         <f>C5/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E5" t="n">
-        <v>423.1</v>
+        <v>205.16</v>
       </c>
       <c r="F5">
         <f>IF(E5="","",ROUND(D5/E5,4))</f>
@@ -5325,14 +5325,14 @@
         <v>79.7</v>
       </c>
       <c r="C6" t="n">
-        <v>7.2</v>
+        <v>7.16</v>
       </c>
       <c r="D6">
         <f>C6/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E6" t="n">
-        <v>1989.67</v>
+        <v>1999.61</v>
       </c>
       <c r="F6">
         <f>IF(E6="","",ROUND(D6/E6,4))</f>
@@ -5355,17 +5355,17 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>79.5</v>
+        <v>78.90000000000001</v>
       </c>
       <c r="C7" t="n">
-        <v>7.13</v>
+        <v>6.83</v>
       </c>
       <c r="D7">
         <f>C7/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E7" t="n">
-        <v>989.1</v>
+        <v>996.5</v>
       </c>
       <c r="F7">
         <f>IF(E7="","",ROUND(D7/E7,4))</f>
@@ -5384,21 +5384,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CRDO</t>
+          <t>META</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>78.8</v>
+        <v>78.5</v>
       </c>
       <c r="C8" t="n">
-        <v>6.82</v>
+        <v>6.65</v>
       </c>
       <c r="D8">
         <f>C8/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E8" t="n">
-        <v>253.64</v>
+        <v>566.55</v>
       </c>
       <c r="F8">
         <f>IF(E8="","",ROUND(D8/E8,4))</f>
@@ -5417,21 +5417,21 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>META</t>
+          <t>AVGO</t>
         </is>
       </c>
       <c r="B9" t="n">
         <v>78.5</v>
       </c>
       <c r="C9" t="n">
-        <v>6.68</v>
+        <v>6.63</v>
       </c>
       <c r="D9">
         <f>C9/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E9" t="n">
-        <v>565.2</v>
+        <v>381.15</v>
       </c>
       <c r="F9">
         <f>IF(E9="","",ROUND(D9/E9,4))</f>
@@ -5450,21 +5450,21 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>AVGO</t>
+          <t>CRDO</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>78.5</v>
+        <v>78.3</v>
       </c>
       <c r="C10" t="n">
-        <v>6.66</v>
+        <v>6.56</v>
       </c>
       <c r="D10">
         <f>C10/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E10" t="n">
-        <v>379.69</v>
+        <v>253.99</v>
       </c>
       <c r="F10">
         <f>IF(E10="","",ROUND(D10/E10,4))</f>
@@ -5490,14 +5490,14 @@
         <v>77.90000000000001</v>
       </c>
       <c r="C11" t="n">
-        <v>6.4</v>
+        <v>6.37</v>
       </c>
       <c r="D11">
         <f>C11/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E11" t="n">
-        <v>164.14</v>
+        <v>164.58</v>
       </c>
       <c r="F11">
         <f>IF(E11="","",ROUND(D11/E11,4))</f>
@@ -5523,14 +5523,14 @@
         <v>76.8</v>
       </c>
       <c r="C12" t="n">
-        <v>5.9</v>
+        <v>5.87</v>
       </c>
       <c r="D12">
         <f>C12/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E12" t="n">
-        <v>387.42</v>
+        <v>388.41</v>
       </c>
       <c r="F12">
         <f>IF(E12="","",ROUND(D12/E12,4))</f>
@@ -5556,14 +5556,14 @@
         <v>76.5</v>
       </c>
       <c r="C13" t="n">
-        <v>5.78</v>
+        <v>5.75</v>
       </c>
       <c r="D13">
         <f>C13/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E13" t="n">
-        <v>373.72</v>
+        <v>373.28</v>
       </c>
       <c r="F13">
         <f>IF(E13="","",ROUND(D13/E13,4))</f>
@@ -5589,14 +5589,14 @@
         <v>76.40000000000001</v>
       </c>
       <c r="C14" t="n">
-        <v>5.72</v>
+        <v>5.69</v>
       </c>
       <c r="D14">
         <f>C14/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E14" t="n">
-        <v>1905</v>
+        <v>1898.74</v>
       </c>
       <c r="F14">
         <f>IF(E14="","",ROUND(D14/E14,4))</f>
@@ -5622,14 +5622,14 @@
         <v>76.2</v>
       </c>
       <c r="C15" t="n">
-        <v>5.66</v>
+        <v>5.64</v>
       </c>
       <c r="D15">
         <f>C15/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E15" t="n">
-        <v>361.19</v>
+        <v>361.67</v>
       </c>
       <c r="F15">
         <f>IF(E15="","",ROUND(D15/E15,4))</f>
@@ -5655,14 +5655,14 @@
         <v>75.3</v>
       </c>
       <c r="C16" t="n">
-        <v>5.27</v>
+        <v>5.25</v>
       </c>
       <c r="D16">
         <f>C16/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E16" t="n">
-        <v>821.85</v>
+        <v>823.0700000000001</v>
       </c>
       <c r="F16">
         <f>IF(E16="","",ROUND(D16/E16,4))</f>
@@ -5688,14 +5688,14 @@
         <v>74.8</v>
       </c>
       <c r="C17" t="n">
-        <v>5.05</v>
+        <v>5.02</v>
       </c>
       <c r="D17">
         <f>C17/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E17" t="n">
-        <v>127.99</v>
+        <v>128.13</v>
       </c>
       <c r="F17">
         <f>IF(E17="","",ROUND(D17/E17,4))</f>
@@ -5721,14 +5721,14 @@
         <v>73.8</v>
       </c>
       <c r="C18" t="n">
-        <v>4.6</v>
+        <v>4.58</v>
       </c>
       <c r="D18">
         <f>C18/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E18" t="n">
-        <v>51.93</v>
+        <v>51.88</v>
       </c>
       <c r="F18">
         <f>IF(E18="","",ROUND(D18/E18,4))</f>
@@ -5754,14 +5754,14 @@
         <v>73</v>
       </c>
       <c r="C19" t="n">
-        <v>4.22</v>
+        <v>4.2</v>
       </c>
       <c r="D19">
         <f>C19/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E19" t="n">
-        <v>403.25</v>
+        <v>403.95</v>
       </c>
       <c r="F19">
         <f>IF(E19="","",ROUND(D19/E19,4))</f>

</xml_diff>

<commit_message>
score: 12 QQQ-coverage names + R5 full-watchlist pass + refresh targets
QQQ-vs-model overlap analysis surfaced an application-layer coverage gap.
Scored 12 names (WDC, PANW, APP, ADBE, FTNT, ZS, INTU, WDAY, ADSK, TSLA,
AAPL; SPCX as a research stub). 8 clear ✓✓. Applied an agentic-AI-disruption
absolute-lens moat re-rate + the new R5 dimension across all 20 Layer-10
names (default 5 elsewhere). Refreshed portfolio.xlsx Targets from live
scores (model membership +APP/VRT/WDC/ZS; mechanical pipeline, rule 5).

- scoring workbook: 12 rows, R5 column, ~180 Rating Audit rows
- research map: new Layer-10 sub-layers + WDC; AAPL/SPCX map-gap flags
- 12 per-stock context briefings (satisfy rule-12 gate)

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NWTt2N82FwnTLjQEKo3QnL
</commit_message>
<xml_diff>
--- a/00-master/portfolio.xlsx
+++ b/00-master/portfolio.xlsx
@@ -678,7 +678,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-06-12 (refresh_targets.py — hysteresis pipeline)</t>
+          <t>2026-06-17 (refresh_targets.py — hysteresis pipeline)</t>
         </is>
       </c>
     </row>
@@ -1053,7 +1053,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J111"/>
+  <dimension ref="A1:J134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1070,7 +1070,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Target Portfolio (refreshed 2026-06-12, live Watchlist scores)</t>
+          <t>Target Portfolio (refreshed 2026-06-17, live Watchlist scores)</t>
         </is>
       </c>
     </row>
@@ -1138,7 +1138,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>83.8</v>
+        <v>84.7</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -1160,7 +1160,7 @@
       </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="n">
-        <v>9.01</v>
+        <v>7.36</v>
       </c>
       <c r="J3" t="inlineStr"/>
     </row>
@@ -1176,7 +1176,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>83.33</v>
+        <v>84.08</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
       </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="n">
-        <v>8.800000000000001</v>
+        <v>7.14</v>
       </c>
       <c r="J4" t="inlineStr"/>
     </row>
@@ -1214,7 +1214,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>79.65000000000001</v>
+        <v>80.09999999999999</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -1236,7 +1236,7 @@
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="n">
-        <v>7.16</v>
+        <v>5.76</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -1256,7 +1256,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>78.90000000000001</v>
+        <v>79.95</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -1278,7 +1278,7 @@
       </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="n">
-        <v>6.83</v>
+        <v>5.71</v>
       </c>
       <c r="J6" t="inlineStr"/>
     </row>
@@ -1294,7 +1294,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>78.5</v>
+        <v>79.40000000000001</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -1316,7 +1316,7 @@
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="n">
-        <v>6.65</v>
+        <v>5.51</v>
       </c>
       <c r="J7" t="inlineStr"/>
     </row>
@@ -1332,7 +1332,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>78.45</v>
+        <v>79.2</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -1354,7 +1354,7 @@
       </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="n">
-        <v>6.63</v>
+        <v>5.44</v>
       </c>
       <c r="J8" t="inlineStr"/>
     </row>
@@ -1370,7 +1370,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>78.3</v>
+        <v>78.90000000000001</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -1392,7 +1392,7 @@
       </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="n">
-        <v>6.56</v>
+        <v>5.34</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
@@ -1403,16 +1403,16 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ANET</t>
+          <t>APP</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
+          <t>10 Models, Software &amp; Applications / AI advertising</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>77.88</v>
+        <v>78.90000000000001</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -1424,7 +1424,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>HOLD</t>
+          <t>ENTER (score 78.9)</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1434,23 +1434,23 @@
       </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="n">
-        <v>6.37</v>
+        <v>5.34</v>
       </c>
       <c r="J10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>ANET</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
+          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>76.75</v>
+        <v>78.48</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -1472,23 +1472,23 @@
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="n">
-        <v>5.87</v>
+        <v>5.19</v>
       </c>
       <c r="J11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ALAB</t>
+          <t>WDC</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>76.48</v>
+        <v>78</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -1500,7 +1500,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>HOLD</t>
+          <t>ENTER (score 78.0)</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1510,23 +1510,23 @@
       </c>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="n">
-        <v>5.75</v>
+        <v>5.03</v>
       </c>
       <c r="J12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>FIX</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>76.34999999999999</v>
+        <v>77.2</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -1548,27 +1548,23 @@
       </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="n">
-        <v>5.69</v>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>Manually excluded 2026-05-18: $1,854 share price prevents reasonable position sizing below ~$50k portfolio. Conscious framework override. | Override removed 2026-06-09: fractional shares adopted, share-price constraint obsolete (Dom decision).</t>
-        </is>
-      </c>
+        <v>4.75</v>
+      </c>
+      <c r="J13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>ALAB</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
+          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>76.22</v>
+        <v>77.08</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -1590,23 +1586,23 @@
       </c>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="n">
-        <v>5.64</v>
+        <v>4.7</v>
       </c>
       <c r="J14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>EME</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>75.34999999999999</v>
+        <v>76.83</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -1628,27 +1624,23 @@
       </c>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="n">
-        <v>5.25</v>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>Added 2026-05-25: score 75.2, DC construction, strong momentum (86.7).</t>
-        </is>
-      </c>
+        <v>4.62</v>
+      </c>
+      <c r="J15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>PLTR</t>
+          <t>FIX</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>74.84999999999999</v>
+        <v>76.65000000000001</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -1670,23 +1662,27 @@
       </c>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="n">
-        <v>5.02</v>
-      </c>
-      <c r="J16" t="inlineStr"/>
+        <v>4.56</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Manually excluded 2026-05-18: $1,854 share price prevents reasonable position sizing below ~$50k portfolio. Conscious framework override. | Override removed 2026-06-09: fractional shares adopted, share-price constraint obsolete (Dom decision).</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>VRT</t>
+          <t>EME</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>03 DC Infrastructure</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>74.45</v>
+        <v>75.5</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -1696,28 +1692,39 @@
       <c r="E17" t="n">
         <v>15</v>
       </c>
-      <c r="F17" t="inlineStr"/>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
+      <c r="I17" t="n">
+        <v>4.16</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Added 2026-05-25: score 75.2, DC construction, strong momentum (86.7).</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>EQT</t>
+          <t>ZS</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
+          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>73.84999999999999</v>
+        <v>75.47</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -1729,7 +1736,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>HOLD</t>
+          <t>ENTER (score 75.5)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1739,23 +1746,23 @@
       </c>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="n">
-        <v>4.58</v>
+        <v>4.15</v>
       </c>
       <c r="J18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>PLTR</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / GPUs / merchant accelerators</t>
+          <t>10 Models, Software &amp; Applications</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>73.45</v>
+        <v>75.40000000000001</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -1765,32 +1772,35 @@
       <c r="E19" t="n">
         <v>17</v>
       </c>
-      <c r="F19" t="inlineStr"/>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H19" t="inlineStr"/>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>Removed 2026-05-25: score 74.1 fell below natural 17-name cutoff (ARM 74.2). First name out.</t>
-        </is>
-      </c>
+      <c r="I19" t="n">
+        <v>4.12</v>
+      </c>
+      <c r="J19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>TER</t>
+          <t>VRT</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>03 DC Infrastructure</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>73</v>
+        <v>75.05</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -1802,7 +1812,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>HOLD</t>
+          <t>ENTER (score 75.0)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1812,23 +1822,23 @@
       </c>
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="n">
-        <v>4.2</v>
+        <v>4</v>
       </c>
       <c r="J20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>KEYS</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
+          <t>06 AI Compute Silicon / GPUs / merchant accelerators</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>72.47</v>
+        <v>74.2</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -1845,21 +1855,25 @@
         </is>
       </c>
       <c r="H21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Removed 2026-05-25: score 74.1 fell below natural 17-name cutoff (ARM 74.2). First name out.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>APH</t>
+          <t>EQT</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
+          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>72.28</v>
+        <v>74.15000000000001</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -1869,28 +1883,35 @@
       <c r="E22" t="n">
         <v>20</v>
       </c>
-      <c r="F22" t="inlineStr"/>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H22" t="inlineStr"/>
+      <c r="I22" t="n">
+        <v>3.69</v>
+      </c>
       <c r="J22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>DELL</t>
+          <t>TER</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>72.08</v>
+        <v>73.45</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -1900,28 +1921,35 @@
       <c r="E23" t="n">
         <v>21</v>
       </c>
-      <c r="F23" t="inlineStr"/>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H23" t="inlineStr"/>
+      <c r="I23" t="n">
+        <v>3.44</v>
+      </c>
       <c r="J23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>KEYS</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>72</v>
+        <v>73.22</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -1938,25 +1966,21 @@
         </is>
       </c>
       <c r="H24" t="inlineStr"/>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>Added 2026-05-25: score 74.8, Quality 97, PEG 0.8. Enterprise SaaS with AI exposure.</t>
-        </is>
-      </c>
+      <c r="J24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>ADSK</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
+          <t>10 Models, Software &amp; Applications / Design &amp; engineering software</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>71.95</v>
+        <v>73.15000000000001</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -1987,7 +2011,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>71.84999999999999</v>
+        <v>72.75</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -2009,16 +2033,16 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>RRC</t>
+          <t>APH</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
+          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>71.7</v>
+        <v>72.72</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -2040,16 +2064,16 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>EXE</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
+          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>71.67</v>
+        <v>72.7</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -2071,16 +2095,16 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>LSCC</t>
+          <t>DELL</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Programmable logic</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>71.48</v>
+        <v>72.67</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -2102,16 +2126,16 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>VST</t>
+          <t>PANW</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>01 Power Generation / Independent Power Producers (IPPs)</t>
+          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>70.59999999999999</v>
+        <v>72.65000000000001</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
@@ -2133,16 +2157,16 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>PATH</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI-powered automation</t>
+          <t>10 Models, Software &amp; Applications</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>70.40000000000001</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -2159,21 +2183,25 @@
         </is>
       </c>
       <c r="H31" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>Added 2026-05-25: score 74.8, Quality 97, PEG 0.8. Enterprise SaaS with AI exposure.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>GEV</t>
+          <t>LSCC</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>02 Grid Equipment</t>
+          <t>06 AI Compute Silicon / Programmable logic</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>70.34999999999999</v>
+        <v>72.38</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -2195,16 +2223,16 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>LRCX</t>
+          <t>WDAY</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>10 Models, Software &amp; Applications / Enterprise SaaS</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>70.34999999999999</v>
+        <v>72.3</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -2226,16 +2254,16 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>ABBNY</t>
+          <t>RRC</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>70.15000000000001</v>
+        <v>72</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -2257,16 +2285,16 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>MPWR</t>
+          <t>EXE</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Power management silicon</t>
+          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>70.15000000000001</v>
+        <v>71.97</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
@@ -2288,16 +2316,16 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>VST</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
+          <t>01 Power Generation / Independent Power Producers (IPPs)</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>70</v>
+        <v>71.05</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
@@ -2314,29 +2342,25 @@
         </is>
       </c>
       <c r="H36" t="inlineStr"/>
-      <c r="J36" t="inlineStr">
-        <is>
-          <t>Added 2026-05-22 as substitute for CTRA (delisted). Pure score-driven pick: next-best ✓✓ at 75.62, same Layer 1 NG E&amp;P sub-category — preserves natural gas thesis concentration.</t>
-        </is>
-      </c>
+      <c r="J36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>CIEN</t>
+          <t>LRCX</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>69.84999999999999</v>
+        <v>70.95</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>✓✓</t>
         </is>
       </c>
       <c r="E37" t="n">
@@ -2354,7 +2378,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>PWR</t>
+          <t>ABBNY</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2363,11 +2387,11 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>69.65000000000001</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>✓✓</t>
         </is>
       </c>
       <c r="E38" t="n">
@@ -2385,20 +2409,20 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>ARM</t>
+          <t>AR</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
+          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>69.2</v>
+        <v>70.45</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>✓✓</t>
         </is>
       </c>
       <c r="E39" t="n">
@@ -2411,25 +2435,29 @@
         </is>
       </c>
       <c r="H39" t="inlineStr"/>
-      <c r="J39" t="inlineStr"/>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>Added 2026-05-22 as substitute for CTRA (delisted). Pure score-driven pick: next-best ✓✓ at 75.62, same Layer 1 NG E&amp;P sub-category — preserves natural gas thesis concentration.</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>TEL</t>
+          <t>CIEN</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
+          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>69.2</v>
+        <v>70.45</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>✓✓</t>
         </is>
       </c>
       <c r="E40" t="n">
@@ -2447,16 +2475,16 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>CEG</t>
+          <t>PWR</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>01 Power - IPP / Nuclear</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>69.09999999999999</v>
+        <v>69.95</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -2487,7 +2515,7 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>69.05</v>
+        <v>69.95</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
@@ -2509,16 +2537,16 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>FN</t>
+          <t>PATH</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
+          <t>10 Models, Software &amp; Applications / AI-powered automation</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>68.95</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
@@ -2549,7 +2577,7 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>68.8</v>
+        <v>69.84999999999999</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -2571,16 +2599,16 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>GLW</t>
+          <t>CEG</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
+          <t>01 Power - IPP / Nuclear</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>68.8</v>
+        <v>69.7</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
@@ -2602,16 +2630,16 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>ASML</t>
+          <t>FN</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>68.3</v>
+        <v>69.7</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -2633,16 +2661,16 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>KLAC</t>
+          <t>ARM</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>68.3</v>
+        <v>69.65000000000001</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -2664,16 +2692,16 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>AEIS</t>
+          <t>TEL</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
+          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>68.17</v>
+        <v>69.65000000000001</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -2695,16 +2723,16 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>AMAT</t>
+          <t>ADI</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>06 AI Compute Silicon / Analog &amp; mixed-signal (signal chain + power)</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>68.15000000000001</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
@@ -2726,16 +2754,16 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>TT</t>
+          <t>INTU</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>10 Models, Software &amp; Applications / Financial software</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>68.12</v>
+        <v>69.38</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
@@ -2757,16 +2785,16 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>TLN</t>
+          <t>ADBE</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>01 Power Generation / Independent Power Producers (IPPs)</t>
+          <t>10 Models, Software &amp; Applications / Creative &amp; design software</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>67.92</v>
+        <v>69.33</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
@@ -2788,16 +2816,16 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>BESIY</t>
+          <t>GLW</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>67.87</v>
+        <v>69.25</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
@@ -2819,16 +2847,16 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>HTHIY</t>
+          <t>ASML</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>67.84999999999999</v>
+        <v>69.05</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
@@ -2850,16 +2878,16 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>NOW</t>
+          <t>MPWR</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications</t>
+          <t>06 AI Compute Silicon / Power management silicon</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>67.8</v>
+        <v>69</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
@@ -2881,16 +2909,16 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>DDOG</t>
+          <t>AEIS</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI observability &amp; infrastructure software</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>67.7</v>
+        <v>68.92</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
@@ -2907,25 +2935,21 @@
         </is>
       </c>
       <c r="H55" t="inlineStr"/>
-      <c r="J55" t="inlineStr">
-        <is>
-          <t>Added 2026-05-25: score 75.4, Quality 100, PEG 0.7. Beats 4 existing portfolio names.</t>
-        </is>
-      </c>
+      <c r="J55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>CDNS</t>
+          <t>KLAC</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>67.40000000000001</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
@@ -2947,16 +2971,16 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>CSCO</t>
+          <t>NOW</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
+          <t>10 Models, Software &amp; Applications</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>67.40000000000001</v>
+        <v>68.84999999999999</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
@@ -2978,16 +3002,16 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>FORM</t>
+          <t>TLN</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
+          <t>01 Power Generation / Independent Power Producers (IPPs)</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>67.31999999999999</v>
+        <v>68.83</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
@@ -3009,16 +3033,16 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>DLR</t>
+          <t>BESIY</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>67.2</v>
+        <v>68.77</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
@@ -3040,16 +3064,16 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>SBGSY</t>
+          <t>AMAT</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>67.05</v>
+        <v>68.75</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
@@ -3071,7 +3095,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>JCI</t>
+          <t>TT</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -3080,7 +3104,7 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>66.8</v>
+        <v>68.58</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
@@ -3102,7 +3126,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>POWL</t>
+          <t>HTHIY</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -3111,7 +3135,7 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>66.75</v>
+        <v>68.3</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
@@ -3133,16 +3157,16 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>MTZ</t>
+          <t>DDOG</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>10 Models, Software &amp; Applications / AI observability &amp; infrastructure software</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>66.7</v>
+        <v>68.25</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
@@ -3159,21 +3183,25 @@
         </is>
       </c>
       <c r="H63" t="inlineStr"/>
-      <c r="J63" t="inlineStr"/>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>Added 2026-05-25: score 75.4, Quality 100, PEG 0.7. Beats 4 existing portfolio names.</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>NVT</t>
+          <t>DLR</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>66.55</v>
+        <v>67.95</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
@@ -3195,16 +3223,16 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>NEE</t>
+          <t>FORM</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>66.33</v>
+        <v>67.92</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
@@ -3226,16 +3254,16 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>CCJ</t>
+          <t>FTNT</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>01 Power Generation / Nuclear-specific</t>
+          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>66.12</v>
+        <v>67.88</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
@@ -3257,16 +3285,16 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>ONTO</t>
+          <t>CDNS</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>66.09999999999999</v>
+        <v>67.84999999999999</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
@@ -3288,16 +3316,16 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>TSEM</t>
+          <t>CSCO</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>05 Fabs &amp; Foundries</t>
+          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>66.09999999999999</v>
+        <v>67.84999999999999</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
@@ -3319,16 +3347,16 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>ENTG</t>
+          <t>SBGSY</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>66.05</v>
+        <v>67.5</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
@@ -3350,16 +3378,16 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>RMBS</t>
+          <t>POWL</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Memory (HBM is the bottleneck)</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>65.97</v>
+        <v>67.34999999999999</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
@@ -3381,7 +3409,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>AAON</t>
+          <t>JCI</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -3390,7 +3418,7 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>65.83</v>
+        <v>67.25</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
@@ -3412,16 +3440,16 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>GNRC</t>
+          <t>NVT</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>01 Power Generation / Distributed / on-site power</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>65.8</v>
+        <v>67.15000000000001</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
@@ -3443,16 +3471,16 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>MKSI</t>
+          <t>NEE</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>65.7</v>
+        <v>67.08</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
@@ -3474,16 +3502,16 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>HUBB</t>
+          <t>GEV</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>02 Grid Equipment</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>65.42</v>
+        <v>67</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
@@ -3505,16 +3533,16 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>MTZ</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>01 Power - Distributed</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>65.15000000000001</v>
+        <v>67</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
@@ -3536,16 +3564,16 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>PLAB</t>
+          <t>TSEM</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
+          <t>05 Fabs &amp; Foundries</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>65.15000000000001</v>
+        <v>66.7</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
@@ -3567,16 +3595,16 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>SNPS</t>
+          <t>ENTG</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>65.09999999999999</v>
+        <v>66.65000000000001</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
@@ -3598,16 +3626,16 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>FLEX</t>
+          <t>ONTO</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Contract manufacturing / ODMs</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>64.25</v>
+        <v>66.55</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
@@ -3629,16 +3657,16 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>ETN</t>
+          <t>TXN</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>06 AI Compute Silicon / Analog &amp; embedded (power management)</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>63.85</v>
+        <v>66.5</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
@@ -3660,16 +3688,16 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>MRVL</t>
+          <t>CCJ</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
+          <t>01 Power Generation / Nuclear-specific</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>63.73</v>
+        <v>66.42</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
@@ -3691,16 +3719,16 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>SNOW</t>
+          <t>RMBS</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications</t>
+          <t>06 AI Compute Silicon / Memory (HBM is the bottleneck)</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>63.4</v>
+        <v>66.42</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
@@ -3722,16 +3750,16 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>ORCL</t>
+          <t>GNRC</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
+          <t>01 Power Generation / Distributed / on-site power</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>63.35</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
@@ -3753,16 +3781,16 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>NXT</t>
+          <t>MKSI</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>01 Power Generation / Solar &amp; renewables equipment (behind-the-meter DC power)</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>63.17</v>
+        <v>66.3</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
@@ -3784,16 +3812,16 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>KLIC</t>
+          <t>AAON</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>63.08</v>
+        <v>66.27</v>
       </c>
       <c r="D84" t="inlineStr">
         <is>
@@ -3815,16 +3843,16 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>HPE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling</t>
+          <t>01 Power - Distributed</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>62.98</v>
+        <v>66.05</v>
       </c>
       <c r="D85" t="inlineStr">
         <is>
@@ -3846,16 +3874,16 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>CMI</t>
+          <t>HUBB</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>01 Power Generation / Distributed / on-site power</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>62.85</v>
+        <v>65.88</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
@@ -3877,16 +3905,16 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>IRM</t>
+          <t>PLAB</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>62.6</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="D87" t="inlineStr">
         <is>
@@ -3908,16 +3936,16 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>NBIS</t>
+          <t>SNPS</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Neoclouds (AI-native cloud providers)</t>
+          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>62.6</v>
+        <v>65.55</v>
       </c>
       <c r="D88" t="inlineStr">
         <is>
@@ -3934,25 +3962,21 @@
         </is>
       </c>
       <c r="H88" t="inlineStr"/>
-      <c r="J88" t="inlineStr">
-        <is>
-          <t>Removed 2026-05-25: dropped to ✓ (65.5) after reweight. Value 7.5 penalized by higher Value weight.</t>
-        </is>
-      </c>
+      <c r="J88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>SMCI</t>
+          <t>SNOW</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling</t>
+          <t>10 Models, Software &amp; Applications</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>62.45</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="D89" t="inlineStr">
         <is>
@@ -3974,16 +3998,16 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>CRWV</t>
+          <t>HIVE</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>09 Cloud - Neocloud</t>
+          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>62.23</v>
+        <v>65.22</v>
       </c>
       <c r="D90" t="inlineStr">
         <is>
@@ -4005,16 +4029,16 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>KN</t>
+          <t>FLEX</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>04 Semi Equip - Materials</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Contract manufacturing / ODMs</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>62.15</v>
+        <v>65</v>
       </c>
       <c r="D91" t="inlineStr">
         <is>
@@ -4036,16 +4060,16 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>LITE</t>
+          <t>NBIS</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
+          <t>09 Compute-as-a-Service / Neoclouds (AI-native cloud providers)</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>62.08</v>
+        <v>64.90000000000001</v>
       </c>
       <c r="D92" t="inlineStr">
         <is>
@@ -4062,21 +4086,25 @@
         </is>
       </c>
       <c r="H92" t="inlineStr"/>
-      <c r="J92" t="inlineStr"/>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>Removed 2026-05-25: dropped to ✓ (65.5) after reweight. Value 7.5 penalized by higher Value weight.</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>CRWD</t>
+          <t>MRVL</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
+          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>61.45</v>
+        <v>64.47</v>
       </c>
       <c r="D93" t="inlineStr">
         <is>
@@ -4098,16 +4126,16 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>BWXT</t>
+          <t>ETN</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>01 Power Generation / Nuclear-specific</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>61.12</v>
+        <v>64.3</v>
       </c>
       <c r="D94" t="inlineStr">
         <is>
@@ -4129,16 +4157,16 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>SMCI</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>61.05</v>
+        <v>64.25</v>
       </c>
       <c r="D95" t="inlineStr">
         <is>
@@ -4160,16 +4188,16 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>EQIX</t>
+          <t>ORCL</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>60.25</v>
+        <v>64.25</v>
       </c>
       <c r="D96" t="inlineStr">
         <is>
@@ -4191,16 +4219,16 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>HUT</t>
+          <t>HPE</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>60.25</v>
+        <v>63.73</v>
       </c>
       <c r="D97" t="inlineStr">
         <is>
@@ -4222,16 +4250,16 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>TTMI</t>
+          <t>KLIC</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / PCB / substrates</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>60.25</v>
+        <v>63.67</v>
       </c>
       <c r="D98" t="inlineStr">
         <is>
@@ -4253,16 +4281,16 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>COHR</t>
+          <t>NXT</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
+          <t>01 Power Generation / Solar &amp; renewables equipment (behind-the-meter DC power)</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>60.05</v>
+        <v>63.62</v>
       </c>
       <c r="D99" t="inlineStr">
         <is>
@@ -4284,16 +4312,16 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>DUK</t>
+          <t>AAPL</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>10 Models, Software &amp; Applications / Edge AI platforms</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>59.65</v>
+        <v>63.55</v>
       </c>
       <c r="D100" t="inlineStr">
         <is>
@@ -4315,16 +4343,16 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>GFS</t>
+          <t>IRM</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>05 Fabs &amp; Foundries</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>59.35</v>
+        <v>63.5</v>
       </c>
       <c r="D101" t="inlineStr">
         <is>
@@ -4346,16 +4374,16 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>AEP</t>
+          <t>HUT</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>58.92</v>
+        <v>63.45</v>
       </c>
       <c r="D102" t="inlineStr">
         <is>
@@ -4377,16 +4405,16 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>CARR</t>
+          <t>CMI</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>01 Power Generation / Distributed / on-site power</t>
         </is>
       </c>
       <c r="C103" t="n">
-        <v>58.02</v>
+        <v>63.3</v>
       </c>
       <c r="D103" t="inlineStr">
         <is>
@@ -4408,16 +4436,16 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>KN</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>04 Semi Equip - Materials</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>57.98</v>
+        <v>63.05</v>
       </c>
       <c r="D104" t="inlineStr">
         <is>
@@ -4439,16 +4467,16 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>PPL</t>
+          <t>SEI</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>01 Power Generation / Distributed / on-site power</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>57.92</v>
+        <v>62.9</v>
       </c>
       <c r="D105" t="inlineStr">
         <is>
@@ -4470,16 +4498,16 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>ATKR</t>
+          <t>LITE</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>57.55</v>
+        <v>62.68</v>
       </c>
       <c r="D106" t="inlineStr">
         <is>
@@ -4501,16 +4529,16 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>TEM</t>
+          <t>CRWV</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI-native vertical applications</t>
+          <t>09 Cloud - Neocloud</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>57.55</v>
+        <v>62.67</v>
       </c>
       <c r="D107" t="inlineStr">
         <is>
@@ -4532,16 +4560,16 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>ETR</t>
+          <t>P</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>56.9</v>
+        <v>61.65</v>
       </c>
       <c r="D108" t="inlineStr">
         <is>
@@ -4563,16 +4591,16 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>XEL</t>
+          <t>CRWD</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
         </is>
       </c>
       <c r="C109" t="n">
-        <v>56.6</v>
+        <v>61.65</v>
       </c>
       <c r="D109" t="inlineStr">
         <is>
@@ -4594,16 +4622,16 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>MDB</t>
+          <t>BWXT</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI data layer</t>
+          <t>01 Power Generation / Nuclear-specific</t>
         </is>
       </c>
       <c r="C110" t="n">
-        <v>55.8</v>
+        <v>61.58</v>
       </c>
       <c r="D110" t="inlineStr">
         <is>
@@ -4625,16 +4653,16 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>UCTT</t>
+          <t>TTMI</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
+          <t>04 Semiconductor Equipment &amp; Materials / PCB / substrates</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>55.27</v>
+        <v>61.45</v>
       </c>
       <c r="D111" t="inlineStr">
         <is>
@@ -4652,6 +4680,719 @@
       </c>
       <c r="H111" t="inlineStr"/>
       <c r="J111" t="inlineStr"/>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>EQIX</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+        </is>
+      </c>
+      <c r="C112" t="n">
+        <v>61</v>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E112" t="n">
+        <v>110</v>
+      </c>
+      <c r="F112" t="inlineStr"/>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr"/>
+      <c r="J112" t="inlineStr"/>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>COHR</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
+        </is>
+      </c>
+      <c r="C113" t="n">
+        <v>60.8</v>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E113" t="n">
+        <v>111</v>
+      </c>
+      <c r="F113" t="inlineStr"/>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr"/>
+      <c r="J113" t="inlineStr"/>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>NXPI</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>06 AI Compute Silicon / Analog &amp; embedded (auto/edge AI)</t>
+        </is>
+      </c>
+      <c r="C114" t="n">
+        <v>60.65</v>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E114" t="n">
+        <v>112</v>
+      </c>
+      <c r="F114" t="inlineStr"/>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr"/>
+      <c r="J114" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>DUK</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+        </is>
+      </c>
+      <c r="C115" t="n">
+        <v>60.1</v>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E115" t="n">
+        <v>113</v>
+      </c>
+      <c r="F115" t="inlineStr"/>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr"/>
+      <c r="J115" t="inlineStr"/>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>GFS</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>05 Fabs &amp; Foundries</t>
+        </is>
+      </c>
+      <c r="C116" t="n">
+        <v>59.95</v>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E116" t="n">
+        <v>114</v>
+      </c>
+      <c r="F116" t="inlineStr"/>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr"/>
+      <c r="J116" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>AEP</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+        </is>
+      </c>
+      <c r="C117" t="n">
+        <v>59.38</v>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E117" t="n">
+        <v>115</v>
+      </c>
+      <c r="F117" t="inlineStr"/>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr"/>
+      <c r="J117" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+        </is>
+      </c>
+      <c r="C118" t="n">
+        <v>58.73</v>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E118" t="n">
+        <v>116</v>
+      </c>
+      <c r="F118" t="inlineStr"/>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr"/>
+      <c r="J118" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>CARR</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+        </is>
+      </c>
+      <c r="C119" t="n">
+        <v>58.62</v>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E119" t="n">
+        <v>117</v>
+      </c>
+      <c r="F119" t="inlineStr"/>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr"/>
+      <c r="J119" t="inlineStr"/>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>WYFI</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>09 Compute-as-a-Service / Neoclouds (AI-native cloud providers)</t>
+        </is>
+      </c>
+      <c r="C120" t="n">
+        <v>58.5</v>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E120" t="n">
+        <v>118</v>
+      </c>
+      <c r="F120" t="inlineStr"/>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr"/>
+      <c r="J120" t="inlineStr"/>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>PPL</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+        </is>
+      </c>
+      <c r="C121" t="n">
+        <v>58.38</v>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E121" t="n">
+        <v>119</v>
+      </c>
+      <c r="F121" t="inlineStr"/>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr"/>
+      <c r="J121" t="inlineStr"/>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>ATKR</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>02 Grid &amp; Power Equipment</t>
+        </is>
+      </c>
+      <c r="C122" t="n">
+        <v>58.15</v>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E122" t="n">
+        <v>120</v>
+      </c>
+      <c r="F122" t="inlineStr"/>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr"/>
+      <c r="J122" t="inlineStr"/>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>TEM</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>10 Models, Software &amp; Applications / AI-native vertical applications</t>
+        </is>
+      </c>
+      <c r="C123" t="n">
+        <v>58</v>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E123" t="n">
+        <v>121</v>
+      </c>
+      <c r="F123" t="inlineStr"/>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr"/>
+      <c r="J123" t="inlineStr"/>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>06 AI Compute Silicon / Power management silicon (SiC/GaN)</t>
+        </is>
+      </c>
+      <c r="C124" t="n">
+        <v>57.77</v>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E124" t="n">
+        <v>122</v>
+      </c>
+      <c r="F124" t="inlineStr"/>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr"/>
+      <c r="J124" t="inlineStr"/>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>QCOM</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>06 AI Compute Silicon / Application processors &amp; connectivity (edge AI)</t>
+        </is>
+      </c>
+      <c r="C125" t="n">
+        <v>57.5</v>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E125" t="n">
+        <v>123</v>
+      </c>
+      <c r="F125" t="inlineStr"/>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr"/>
+      <c r="J125" t="inlineStr"/>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>APLD</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>09 Compute-as-a-Service / Neoclouds (AI-native cloud providers)</t>
+        </is>
+      </c>
+      <c r="C126" t="n">
+        <v>57.48</v>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E126" t="n">
+        <v>124</v>
+      </c>
+      <c r="F126" t="inlineStr"/>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr"/>
+      <c r="J126" t="inlineStr"/>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>MDB</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>10 Models, Software &amp; Applications / AI data layer</t>
+        </is>
+      </c>
+      <c r="C127" t="n">
+        <v>57.45</v>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E127" t="n">
+        <v>125</v>
+      </c>
+      <c r="F127" t="inlineStr"/>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr"/>
+      <c r="J127" t="inlineStr"/>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>ETR</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+        </is>
+      </c>
+      <c r="C128" t="n">
+        <v>57.35</v>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E128" t="n">
+        <v>126</v>
+      </c>
+      <c r="F128" t="inlineStr"/>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr"/>
+      <c r="J128" t="inlineStr"/>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>IREN</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
+        </is>
+      </c>
+      <c r="C129" t="n">
+        <v>57.25</v>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E129" t="n">
+        <v>127</v>
+      </c>
+      <c r="F129" t="inlineStr"/>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr"/>
+      <c r="J129" t="inlineStr"/>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>XEL</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+        </is>
+      </c>
+      <c r="C130" t="n">
+        <v>57.05</v>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E130" t="n">
+        <v>128</v>
+      </c>
+      <c r="F130" t="inlineStr"/>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr"/>
+      <c r="J130" t="inlineStr"/>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>UCTT</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
+        </is>
+      </c>
+      <c r="C131" t="n">
+        <v>55.88</v>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E131" t="n">
+        <v>129</v>
+      </c>
+      <c r="F131" t="inlineStr"/>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr"/>
+      <c r="J131" t="inlineStr"/>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>WULF</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
+        </is>
+      </c>
+      <c r="C132" t="n">
+        <v>55.77</v>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E132" t="n">
+        <v>130</v>
+      </c>
+      <c r="F132" t="inlineStr"/>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr"/>
+      <c r="J132" t="inlineStr"/>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>PSIX</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>01 Power Generation / Distributed / on-site power</t>
+        </is>
+      </c>
+      <c r="C133" t="n">
+        <v>55.6</v>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E133" t="n">
+        <v>131</v>
+      </c>
+      <c r="F133" t="inlineStr"/>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr"/>
+      <c r="J133" t="inlineStr"/>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>SO</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+        </is>
+      </c>
+      <c r="C134" t="n">
+        <v>55.33</v>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E134" t="n">
+        <v>132</v>
+      </c>
+      <c r="F134" t="inlineStr"/>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr"/>
+      <c r="J134" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -5181,7 +5922,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -5203,7 +5944,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Portfolio: $13,800 | Prices as of 2026-06-12</t>
+          <t>Portfolio: $13,800 | Prices as of 2026-06-17</t>
         </is>
       </c>
     </row>
@@ -5256,17 +5997,17 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>83.8</v>
+        <v>84.7</v>
       </c>
       <c r="C4" t="n">
-        <v>9.01</v>
+        <v>7.36</v>
       </c>
       <c r="D4">
         <f>C4/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E4" t="n">
-        <v>424.35</v>
+        <v>432.15</v>
       </c>
       <c r="F4">
         <f>IF(E4="","",ROUND(D4/E4,4))</f>
@@ -5289,17 +6030,17 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>83.3</v>
+        <v>84.09999999999999</v>
       </c>
       <c r="C5" t="n">
-        <v>8.800000000000001</v>
+        <v>7.14</v>
       </c>
       <c r="D5">
         <f>C5/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E5" t="n">
-        <v>205.16</v>
+        <v>204.65</v>
       </c>
       <c r="F5">
         <f>IF(E5="","",ROUND(D5/E5,4))</f>
@@ -5322,17 +6063,17 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>79.7</v>
+        <v>80.09999999999999</v>
       </c>
       <c r="C6" t="n">
-        <v>7.16</v>
+        <v>5.76</v>
       </c>
       <c r="D6">
         <f>C6/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E6" t="n">
-        <v>1999.61</v>
+        <v>1958.8</v>
       </c>
       <c r="F6">
         <f>IF(E6="","",ROUND(D6/E6,4))</f>
@@ -5355,17 +6096,17 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>78.90000000000001</v>
+        <v>80</v>
       </c>
       <c r="C7" t="n">
-        <v>6.83</v>
+        <v>5.71</v>
       </c>
       <c r="D7">
         <f>C7/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E7" t="n">
-        <v>996.5</v>
+        <v>1043.19</v>
       </c>
       <c r="F7">
         <f>IF(E7="","",ROUND(D7/E7,4))</f>
@@ -5388,17 +6129,17 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>78.5</v>
+        <v>79.40000000000001</v>
       </c>
       <c r="C8" t="n">
-        <v>6.65</v>
+        <v>5.51</v>
       </c>
       <c r="D8">
         <f>C8/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E8" t="n">
-        <v>566.55</v>
+        <v>567.58</v>
       </c>
       <c r="F8">
         <f>IF(E8="","",ROUND(D8/E8,4))</f>
@@ -5421,17 +6162,17 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>78.5</v>
+        <v>79.2</v>
       </c>
       <c r="C9" t="n">
-        <v>6.63</v>
+        <v>5.44</v>
       </c>
       <c r="D9">
         <f>C9/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E9" t="n">
-        <v>381.15</v>
+        <v>392.9</v>
       </c>
       <c r="F9">
         <f>IF(E9="","",ROUND(D9/E9,4))</f>
@@ -5454,17 +6195,17 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>78.3</v>
+        <v>78.90000000000001</v>
       </c>
       <c r="C10" t="n">
-        <v>6.56</v>
+        <v>5.34</v>
       </c>
       <c r="D10">
         <f>C10/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E10" t="n">
-        <v>253.99</v>
+        <v>249.33</v>
       </c>
       <c r="F10">
         <f>IF(E10="","",ROUND(D10/E10,4))</f>
@@ -5483,21 +6224,21 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ANET</t>
+          <t>APP</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>77.90000000000001</v>
+        <v>78.90000000000001</v>
       </c>
       <c r="C11" t="n">
-        <v>6.37</v>
+        <v>5.34</v>
       </c>
       <c r="D11">
         <f>C11/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E11" t="n">
-        <v>164.58</v>
+        <v>479.49</v>
       </c>
       <c r="F11">
         <f>IF(E11="","",ROUND(D11/E11,4))</f>
@@ -5516,21 +6257,21 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>ANET</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>76.8</v>
+        <v>78.5</v>
       </c>
       <c r="C12" t="n">
-        <v>5.87</v>
+        <v>5.19</v>
       </c>
       <c r="D12">
         <f>C12/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E12" t="n">
-        <v>388.41</v>
+        <v>164.93</v>
       </c>
       <c r="F12">
         <f>IF(E12="","",ROUND(D12/E12,4))</f>
@@ -5549,21 +6290,21 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ALAB</t>
+          <t>WDC</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>76.5</v>
+        <v>78</v>
       </c>
       <c r="C13" t="n">
-        <v>5.75</v>
+        <v>5.03</v>
       </c>
       <c r="D13">
         <f>C13/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E13" t="n">
-        <v>373.28</v>
+        <v>712.13</v>
       </c>
       <c r="F13">
         <f>IF(E13="","",ROUND(D13/E13,4))</f>
@@ -5582,21 +6323,21 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>FIX</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>76.40000000000001</v>
+        <v>77.2</v>
       </c>
       <c r="C14" t="n">
-        <v>5.69</v>
+        <v>4.75</v>
       </c>
       <c r="D14">
         <f>C14/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E14" t="n">
-        <v>1898.74</v>
+        <v>378.91</v>
       </c>
       <c r="F14">
         <f>IF(E14="","",ROUND(D14/E14,4))</f>
@@ -5615,21 +6356,21 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>ALAB</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>76.2</v>
+        <v>77.09999999999999</v>
       </c>
       <c r="C15" t="n">
-        <v>5.64</v>
+        <v>4.7</v>
       </c>
       <c r="D15">
         <f>C15/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E15" t="n">
-        <v>361.67</v>
+        <v>374.68</v>
       </c>
       <c r="F15">
         <f>IF(E15="","",ROUND(D15/E15,4))</f>
@@ -5648,21 +6389,21 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>EME</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>75.3</v>
+        <v>76.8</v>
       </c>
       <c r="C16" t="n">
-        <v>5.25</v>
+        <v>4.62</v>
       </c>
       <c r="D16">
         <f>C16/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E16" t="n">
-        <v>823.0700000000001</v>
+        <v>363.79</v>
       </c>
       <c r="F16">
         <f>IF(E16="","",ROUND(D16/E16,4))</f>
@@ -5681,21 +6422,21 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>PLTR</t>
+          <t>FIX</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>74.8</v>
+        <v>76.7</v>
       </c>
       <c r="C17" t="n">
-        <v>5.02</v>
+        <v>4.56</v>
       </c>
       <c r="D17">
         <f>C17/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E17" t="n">
-        <v>128.13</v>
+        <v>1931.77</v>
       </c>
       <c r="F17">
         <f>IF(E17="","",ROUND(D17/E17,4))</f>
@@ -5714,21 +6455,21 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>EQT</t>
+          <t>EME</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>73.8</v>
+        <v>75.5</v>
       </c>
       <c r="C18" t="n">
-        <v>4.58</v>
+        <v>4.16</v>
       </c>
       <c r="D18">
         <f>C18/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E18" t="n">
-        <v>51.88</v>
+        <v>827.5</v>
       </c>
       <c r="F18">
         <f>IF(E18="","",ROUND(D18/E18,4))</f>
@@ -5747,21 +6488,21 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>TER</t>
+          <t>ZS</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>73</v>
+        <v>75.5</v>
       </c>
       <c r="C19" t="n">
-        <v>4.2</v>
+        <v>4.15</v>
       </c>
       <c r="D19">
         <f>C19/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E19" t="n">
-        <v>403.95</v>
+        <v>124.38</v>
       </c>
       <c r="F19">
         <f>IF(E19="","",ROUND(D19/E19,4))</f>
@@ -5780,19 +6521,151 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
+          <t>PLTR</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>75.40000000000001</v>
+      </c>
+      <c r="C20" t="n">
+        <v>4.12</v>
+      </c>
+      <c r="D20">
+        <f>C20/100*'Sizing Rules'!$B$16</f>
+        <v/>
+      </c>
+      <c r="E20" t="n">
+        <v>130.63</v>
+      </c>
+      <c r="F20">
+        <f>IF(E20="","",ROUND(D20/E20,4))</f>
+        <v/>
+      </c>
+      <c r="G20">
+        <f>IF(E20="","",F20*E20)</f>
+        <v/>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>VRT</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>75</v>
+      </c>
+      <c r="C21" t="n">
+        <v>4</v>
+      </c>
+      <c r="D21">
+        <f>C21/100*'Sizing Rules'!$B$16</f>
+        <v/>
+      </c>
+      <c r="E21" t="n">
+        <v>317.58</v>
+      </c>
+      <c r="F21">
+        <f>IF(E21="","",ROUND(D21/E21,4))</f>
+        <v/>
+      </c>
+      <c r="G21">
+        <f>IF(E21="","",F21*E21)</f>
+        <v/>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>EQT</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>74.2</v>
+      </c>
+      <c r="C22" t="n">
+        <v>3.69</v>
+      </c>
+      <c r="D22">
+        <f>C22/100*'Sizing Rules'!$B$16</f>
+        <v/>
+      </c>
+      <c r="E22" t="n">
+        <v>51.13</v>
+      </c>
+      <c r="F22">
+        <f>IF(E22="","",ROUND(D22/E22,4))</f>
+        <v/>
+      </c>
+      <c r="G22">
+        <f>IF(E22="","",F22*E22)</f>
+        <v/>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>TER</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>73.5</v>
+      </c>
+      <c r="C23" t="n">
+        <v>3.44</v>
+      </c>
+      <c r="D23">
+        <f>C23/100*'Sizing Rules'!$B$16</f>
+        <v/>
+      </c>
+      <c r="E23" t="n">
+        <v>408.56</v>
+      </c>
+      <c r="F23">
+        <f>IF(E23="","",ROUND(D23/E23,4))</f>
+        <v/>
+      </c>
+      <c r="G23">
+        <f>IF(E23="","",F23*E23)</f>
+        <v/>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C20">
-        <f>SUM(C4:C19)</f>
-        <v/>
-      </c>
-      <c r="D20">
-        <f>SUM(D4:D19)</f>
-        <v/>
-      </c>
-      <c r="G20">
-        <f>SUM(G4:G19)</f>
+      <c r="C24">
+        <f>SUM(C4:C23)</f>
+        <v/>
+      </c>
+      <c r="D24">
+        <f>SUM(D4:D23)</f>
+        <v/>
+      </c>
+      <c r="G24">
+        <f>SUM(G4:G23)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
portfolio: tighten to 14-name 76-bar book (concentrate top names)
Raise entry score 74.5->76 (exit 73->74.5, 1.5pt hysteresis band) and resize:
+APP +WDC, -EME -PLTR -EQT -TER vs the prior book. Lifts NVDA 7.1%->9.3%,
TSM 7.3%->9.6%, top-5 share 31%->41% — higher weight to the top scorers per
Dom's concentration preference. Layer 6 (silicon) ~38%, layer caps off by design.
Mechanical pipeline output; allocation decision is Dom's (rule 5).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NWTt2N82FwnTLjQEKo3QnL
</commit_message>
<xml_diff>
--- a/00-master/portfolio.xlsx
+++ b/00-master/portfolio.xlsx
@@ -482,8 +482,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
@@ -496,7 +494,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
@@ -552,7 +549,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
@@ -620,7 +616,6 @@
         </is>
       </c>
     </row>
-    <row r="18"/>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
         <is>
@@ -656,7 +651,6 @@
         </is>
       </c>
     </row>
-    <row r="24"/>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
         <is>
@@ -669,7 +663,6 @@
         </is>
       </c>
     </row>
-    <row r="26"/>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
         <is>
@@ -678,7 +671,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-06-17 (refresh_targets.py — hysteresis pipeline)</t>
+          <t>2026-06-18 (refresh_targets.py — hysteresis pipeline)</t>
         </is>
       </c>
     </row>
@@ -1016,7 +1009,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>74.5</v>
+        <v>76</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -1031,11 +1024,11 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>73</v>
+        <v>74.5</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Holding EXITs when score &lt; this (2-run confirm, or immediate on --resize) (added 2026-06-09)</t>
+          <t>Holding EXITs when score &lt; this (2-run confirm, or immediate on --resize). 1.5pt dead-band below entry 76 (set 2026-06-18).</t>
         </is>
       </c>
     </row>
@@ -1070,7 +1063,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Target Portfolio (refreshed 2026-06-17, live Watchlist scores)</t>
+          <t>Target Portfolio (refreshed 2026-06-18, live Watchlist scores)</t>
         </is>
       </c>
     </row>
@@ -1158,11 +1151,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
       <c r="I3" t="n">
-        <v>7.36</v>
-      </c>
-      <c r="J3" t="inlineStr"/>
+        <v>9.630000000000001</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1196,11 +1187,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
       <c r="I4" t="n">
-        <v>7.14</v>
-      </c>
-      <c r="J4" t="inlineStr"/>
+        <v>9.34</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1234,9 +1223,8 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
       <c r="I5" t="n">
-        <v>5.76</v>
+        <v>7.53</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -1276,11 +1264,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr"/>
       <c r="I6" t="n">
-        <v>5.71</v>
-      </c>
-      <c r="J6" t="inlineStr"/>
+        <v>7.46</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1314,11 +1300,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr"/>
       <c r="I7" t="n">
-        <v>5.51</v>
-      </c>
-      <c r="J7" t="inlineStr"/>
+        <v>7.21</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1352,11 +1336,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr"/>
       <c r="I8" t="n">
-        <v>5.44</v>
-      </c>
-      <c r="J8" t="inlineStr"/>
+        <v>7.12</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1390,9 +1372,8 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr"/>
       <c r="I9" t="n">
-        <v>5.34</v>
+        <v>6.98</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
@@ -1424,7 +1405,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>ENTER (score 78.9)</t>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1432,11 +1413,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr"/>
       <c r="I10" t="n">
-        <v>5.34</v>
-      </c>
-      <c r="J10" t="inlineStr"/>
+        <v>6.98</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1470,11 +1449,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr"/>
       <c r="I11" t="n">
-        <v>5.19</v>
-      </c>
-      <c r="J11" t="inlineStr"/>
+        <v>6.79</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1500,7 +1477,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>ENTER (score 78.0)</t>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1508,11 +1485,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr"/>
       <c r="I12" t="n">
-        <v>5.03</v>
-      </c>
-      <c r="J12" t="inlineStr"/>
+        <v>6.57</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1546,11 +1521,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr"/>
       <c r="I13" t="n">
-        <v>4.75</v>
-      </c>
-      <c r="J13" t="inlineStr"/>
+        <v>6.21</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1584,11 +1557,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr"/>
       <c r="I14" t="n">
-        <v>4.7</v>
-      </c>
-      <c r="J14" t="inlineStr"/>
+        <v>6.15</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1622,11 +1593,9 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr"/>
       <c r="I15" t="n">
-        <v>4.62</v>
-      </c>
-      <c r="J15" t="inlineStr"/>
+        <v>6.04</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1660,9 +1629,8 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr"/>
       <c r="I16" t="n">
-        <v>4.56</v>
+        <v>5.96</v>
       </c>
       <c r="J16" t="inlineStr">
         <is>
@@ -1694,17 +1662,13 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>HOLD</t>
+          <t>EXIT (resize, score 75.5 &lt; 76.0)</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="n">
-        <v>4.16</v>
+          <t>N</t>
+        </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
@@ -1736,19 +1700,14 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>ENTER (score 75.5)</t>
+          <t>EXIT (resize, score 75.5 &lt; 76.0)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="n">
-        <v>4.15</v>
-      </c>
-      <c r="J18" t="inlineStr"/>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1774,19 +1733,14 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>HOLD</t>
+          <t>EXIT (resize, score 75.4 &lt; 76.0)</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="n">
-        <v>4.12</v>
-      </c>
-      <c r="J19" t="inlineStr"/>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1812,19 +1766,14 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>ENTER (score 75.0)</t>
+          <t>EXIT (resize, score 75.0 &lt; 76.0)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="n">
-        <v>4</v>
-      </c>
-      <c r="J20" t="inlineStr"/>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1848,13 +1797,11 @@
       <c r="E21" t="n">
         <v>19</v>
       </c>
-      <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr"/>
       <c r="J21" t="inlineStr">
         <is>
           <t>Removed 2026-05-25: score 74.1 fell below natural 17-name cutoff (ARM 74.2). First name out.</t>
@@ -1885,19 +1832,14 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>HOLD</t>
+          <t>EXIT (resize, score 74.2 &lt; 76.0)</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="n">
-        <v>3.69</v>
-      </c>
-      <c r="J22" t="inlineStr"/>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1923,19 +1865,14 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>HOLD</t>
+          <t>EXIT (resize, score 73.5 &lt; 76.0)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="n">
-        <v>3.44</v>
-      </c>
-      <c r="J23" t="inlineStr"/>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1959,14 +1896,11 @@
       <c r="E24" t="n">
         <v>22</v>
       </c>
-      <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1990,14 +1924,11 @@
       <c r="E25" t="n">
         <v>23</v>
       </c>
-      <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr"/>
-      <c r="J25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2021,14 +1952,11 @@
       <c r="E26" t="n">
         <v>24</v>
       </c>
-      <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2052,14 +1980,11 @@
       <c r="E27" t="n">
         <v>25</v>
       </c>
-      <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2083,14 +2008,11 @@
       <c r="E28" t="n">
         <v>26</v>
       </c>
-      <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2114,14 +2036,11 @@
       <c r="E29" t="n">
         <v>27</v>
       </c>
-      <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2145,14 +2064,11 @@
       <c r="E30" t="n">
         <v>28</v>
       </c>
-      <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2176,13 +2092,11 @@
       <c r="E31" t="n">
         <v>29</v>
       </c>
-      <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr"/>
       <c r="J31" t="inlineStr">
         <is>
           <t>Added 2026-05-25: score 74.8, Quality 97, PEG 0.8. Enterprise SaaS with AI exposure.</t>
@@ -2211,14 +2125,11 @@
       <c r="E32" t="n">
         <v>30</v>
       </c>
-      <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr"/>
-      <c r="J32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2242,14 +2153,11 @@
       <c r="E33" t="n">
         <v>31</v>
       </c>
-      <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr"/>
-      <c r="J33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2273,14 +2181,11 @@
       <c r="E34" t="n">
         <v>32</v>
       </c>
-      <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr"/>
-      <c r="J34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2304,14 +2209,11 @@
       <c r="E35" t="n">
         <v>33</v>
       </c>
-      <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr"/>
-      <c r="J35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2335,14 +2237,11 @@
       <c r="E36" t="n">
         <v>34</v>
       </c>
-      <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr"/>
-      <c r="J36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2366,14 +2265,11 @@
       <c r="E37" t="n">
         <v>35</v>
       </c>
-      <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr"/>
-      <c r="J37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2397,14 +2293,11 @@
       <c r="E38" t="n">
         <v>36</v>
       </c>
-      <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr"/>
-      <c r="J38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2428,13 +2321,11 @@
       <c r="E39" t="n">
         <v>37</v>
       </c>
-      <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr"/>
       <c r="J39" t="inlineStr">
         <is>
           <t>Added 2026-05-22 as substitute for CTRA (delisted). Pure score-driven pick: next-best ✓✓ at 75.62, same Layer 1 NG E&amp;P sub-category — preserves natural gas thesis concentration.</t>
@@ -2463,14 +2354,11 @@
       <c r="E40" t="n">
         <v>38</v>
       </c>
-      <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr"/>
-      <c r="J40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2494,14 +2382,11 @@
       <c r="E41" t="n">
         <v>39</v>
       </c>
-      <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr"/>
-      <c r="J41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2525,14 +2410,11 @@
       <c r="E42" t="n">
         <v>40</v>
       </c>
-      <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr"/>
-      <c r="J42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2556,14 +2438,11 @@
       <c r="E43" t="n">
         <v>41</v>
       </c>
-      <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr"/>
-      <c r="J43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2587,14 +2466,11 @@
       <c r="E44" t="n">
         <v>42</v>
       </c>
-      <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr"/>
-      <c r="J44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2618,14 +2494,11 @@
       <c r="E45" t="n">
         <v>43</v>
       </c>
-      <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr"/>
-      <c r="J45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2649,14 +2522,11 @@
       <c r="E46" t="n">
         <v>44</v>
       </c>
-      <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H46" t="inlineStr"/>
-      <c r="J46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2680,14 +2550,11 @@
       <c r="E47" t="n">
         <v>45</v>
       </c>
-      <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H47" t="inlineStr"/>
-      <c r="J47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2711,14 +2578,11 @@
       <c r="E48" t="n">
         <v>46</v>
       </c>
-      <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H48" t="inlineStr"/>
-      <c r="J48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2742,14 +2606,11 @@
       <c r="E49" t="n">
         <v>47</v>
       </c>
-      <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H49" t="inlineStr"/>
-      <c r="J49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2773,14 +2634,11 @@
       <c r="E50" t="n">
         <v>48</v>
       </c>
-      <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H50" t="inlineStr"/>
-      <c r="J50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2804,14 +2662,11 @@
       <c r="E51" t="n">
         <v>49</v>
       </c>
-      <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H51" t="inlineStr"/>
-      <c r="J51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2835,14 +2690,11 @@
       <c r="E52" t="n">
         <v>50</v>
       </c>
-      <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H52" t="inlineStr"/>
-      <c r="J52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2866,14 +2718,11 @@
       <c r="E53" t="n">
         <v>51</v>
       </c>
-      <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H53" t="inlineStr"/>
-      <c r="J53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2897,14 +2746,11 @@
       <c r="E54" t="n">
         <v>52</v>
       </c>
-      <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H54" t="inlineStr"/>
-      <c r="J54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2928,14 +2774,11 @@
       <c r="E55" t="n">
         <v>53</v>
       </c>
-      <c r="F55" t="inlineStr"/>
       <c r="G55" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H55" t="inlineStr"/>
-      <c r="J55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -2959,14 +2802,11 @@
       <c r="E56" t="n">
         <v>54</v>
       </c>
-      <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H56" t="inlineStr"/>
-      <c r="J56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -2990,14 +2830,11 @@
       <c r="E57" t="n">
         <v>55</v>
       </c>
-      <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H57" t="inlineStr"/>
-      <c r="J57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -3021,14 +2858,11 @@
       <c r="E58" t="n">
         <v>56</v>
       </c>
-      <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H58" t="inlineStr"/>
-      <c r="J58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -3052,14 +2886,11 @@
       <c r="E59" t="n">
         <v>57</v>
       </c>
-      <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H59" t="inlineStr"/>
-      <c r="J59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -3083,14 +2914,11 @@
       <c r="E60" t="n">
         <v>58</v>
       </c>
-      <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H60" t="inlineStr"/>
-      <c r="J60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -3114,14 +2942,11 @@
       <c r="E61" t="n">
         <v>59</v>
       </c>
-      <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H61" t="inlineStr"/>
-      <c r="J61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -3145,14 +2970,11 @@
       <c r="E62" t="n">
         <v>60</v>
       </c>
-      <c r="F62" t="inlineStr"/>
       <c r="G62" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H62" t="inlineStr"/>
-      <c r="J62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -3176,13 +2998,11 @@
       <c r="E63" t="n">
         <v>61</v>
       </c>
-      <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H63" t="inlineStr"/>
       <c r="J63" t="inlineStr">
         <is>
           <t>Added 2026-05-25: score 75.4, Quality 100, PEG 0.7. Beats 4 existing portfolio names.</t>
@@ -3211,14 +3031,11 @@
       <c r="E64" t="n">
         <v>62</v>
       </c>
-      <c r="F64" t="inlineStr"/>
       <c r="G64" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H64" t="inlineStr"/>
-      <c r="J64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -3242,14 +3059,11 @@
       <c r="E65" t="n">
         <v>63</v>
       </c>
-      <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H65" t="inlineStr"/>
-      <c r="J65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -3273,14 +3087,11 @@
       <c r="E66" t="n">
         <v>64</v>
       </c>
-      <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H66" t="inlineStr"/>
-      <c r="J66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -3304,14 +3115,11 @@
       <c r="E67" t="n">
         <v>65</v>
       </c>
-      <c r="F67" t="inlineStr"/>
       <c r="G67" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H67" t="inlineStr"/>
-      <c r="J67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -3335,14 +3143,11 @@
       <c r="E68" t="n">
         <v>66</v>
       </c>
-      <c r="F68" t="inlineStr"/>
       <c r="G68" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H68" t="inlineStr"/>
-      <c r="J68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -3366,14 +3171,11 @@
       <c r="E69" t="n">
         <v>67</v>
       </c>
-      <c r="F69" t="inlineStr"/>
       <c r="G69" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H69" t="inlineStr"/>
-      <c r="J69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -3397,14 +3199,11 @@
       <c r="E70" t="n">
         <v>68</v>
       </c>
-      <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H70" t="inlineStr"/>
-      <c r="J70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -3428,14 +3227,11 @@
       <c r="E71" t="n">
         <v>69</v>
       </c>
-      <c r="F71" t="inlineStr"/>
       <c r="G71" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H71" t="inlineStr"/>
-      <c r="J71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -3459,14 +3255,11 @@
       <c r="E72" t="n">
         <v>70</v>
       </c>
-      <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H72" t="inlineStr"/>
-      <c r="J72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -3490,14 +3283,11 @@
       <c r="E73" t="n">
         <v>71</v>
       </c>
-      <c r="F73" t="inlineStr"/>
       <c r="G73" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H73" t="inlineStr"/>
-      <c r="J73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -3521,14 +3311,11 @@
       <c r="E74" t="n">
         <v>72</v>
       </c>
-      <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H74" t="inlineStr"/>
-      <c r="J74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -3552,14 +3339,11 @@
       <c r="E75" t="n">
         <v>73</v>
       </c>
-      <c r="F75" t="inlineStr"/>
       <c r="G75" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H75" t="inlineStr"/>
-      <c r="J75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -3583,14 +3367,11 @@
       <c r="E76" t="n">
         <v>74</v>
       </c>
-      <c r="F76" t="inlineStr"/>
       <c r="G76" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H76" t="inlineStr"/>
-      <c r="J76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -3614,14 +3395,11 @@
       <c r="E77" t="n">
         <v>75</v>
       </c>
-      <c r="F77" t="inlineStr"/>
       <c r="G77" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H77" t="inlineStr"/>
-      <c r="J77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -3645,14 +3423,11 @@
       <c r="E78" t="n">
         <v>76</v>
       </c>
-      <c r="F78" t="inlineStr"/>
       <c r="G78" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H78" t="inlineStr"/>
-      <c r="J78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -3676,14 +3451,11 @@
       <c r="E79" t="n">
         <v>77</v>
       </c>
-      <c r="F79" t="inlineStr"/>
       <c r="G79" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H79" t="inlineStr"/>
-      <c r="J79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -3707,14 +3479,11 @@
       <c r="E80" t="n">
         <v>78</v>
       </c>
-      <c r="F80" t="inlineStr"/>
       <c r="G80" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H80" t="inlineStr"/>
-      <c r="J80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -3738,14 +3507,11 @@
       <c r="E81" t="n">
         <v>79</v>
       </c>
-      <c r="F81" t="inlineStr"/>
       <c r="G81" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H81" t="inlineStr"/>
-      <c r="J81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -3769,14 +3535,11 @@
       <c r="E82" t="n">
         <v>80</v>
       </c>
-      <c r="F82" t="inlineStr"/>
       <c r="G82" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H82" t="inlineStr"/>
-      <c r="J82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -3800,14 +3563,11 @@
       <c r="E83" t="n">
         <v>81</v>
       </c>
-      <c r="F83" t="inlineStr"/>
       <c r="G83" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H83" t="inlineStr"/>
-      <c r="J83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -3831,14 +3591,11 @@
       <c r="E84" t="n">
         <v>82</v>
       </c>
-      <c r="F84" t="inlineStr"/>
       <c r="G84" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H84" t="inlineStr"/>
-      <c r="J84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -3862,14 +3619,11 @@
       <c r="E85" t="n">
         <v>83</v>
       </c>
-      <c r="F85" t="inlineStr"/>
       <c r="G85" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H85" t="inlineStr"/>
-      <c r="J85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -3893,14 +3647,11 @@
       <c r="E86" t="n">
         <v>84</v>
       </c>
-      <c r="F86" t="inlineStr"/>
       <c r="G86" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H86" t="inlineStr"/>
-      <c r="J86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -3924,14 +3675,11 @@
       <c r="E87" t="n">
         <v>85</v>
       </c>
-      <c r="F87" t="inlineStr"/>
       <c r="G87" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H87" t="inlineStr"/>
-      <c r="J87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -3955,14 +3703,11 @@
       <c r="E88" t="n">
         <v>86</v>
       </c>
-      <c r="F88" t="inlineStr"/>
       <c r="G88" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H88" t="inlineStr"/>
-      <c r="J88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -3986,14 +3731,11 @@
       <c r="E89" t="n">
         <v>87</v>
       </c>
-      <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H89" t="inlineStr"/>
-      <c r="J89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -4017,14 +3759,11 @@
       <c r="E90" t="n">
         <v>88</v>
       </c>
-      <c r="F90" t="inlineStr"/>
       <c r="G90" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H90" t="inlineStr"/>
-      <c r="J90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -4048,14 +3787,11 @@
       <c r="E91" t="n">
         <v>89</v>
       </c>
-      <c r="F91" t="inlineStr"/>
       <c r="G91" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H91" t="inlineStr"/>
-      <c r="J91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -4079,13 +3815,11 @@
       <c r="E92" t="n">
         <v>90</v>
       </c>
-      <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H92" t="inlineStr"/>
       <c r="J92" t="inlineStr">
         <is>
           <t>Removed 2026-05-25: dropped to ✓ (65.5) after reweight. Value 7.5 penalized by higher Value weight.</t>
@@ -4114,14 +3848,11 @@
       <c r="E93" t="n">
         <v>91</v>
       </c>
-      <c r="F93" t="inlineStr"/>
       <c r="G93" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H93" t="inlineStr"/>
-      <c r="J93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -4145,14 +3876,11 @@
       <c r="E94" t="n">
         <v>92</v>
       </c>
-      <c r="F94" t="inlineStr"/>
       <c r="G94" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H94" t="inlineStr"/>
-      <c r="J94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -4176,14 +3904,11 @@
       <c r="E95" t="n">
         <v>93</v>
       </c>
-      <c r="F95" t="inlineStr"/>
       <c r="G95" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H95" t="inlineStr"/>
-      <c r="J95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -4207,14 +3932,11 @@
       <c r="E96" t="n">
         <v>94</v>
       </c>
-      <c r="F96" t="inlineStr"/>
       <c r="G96" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H96" t="inlineStr"/>
-      <c r="J96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -4238,14 +3960,11 @@
       <c r="E97" t="n">
         <v>95</v>
       </c>
-      <c r="F97" t="inlineStr"/>
       <c r="G97" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H97" t="inlineStr"/>
-      <c r="J97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -4269,14 +3988,11 @@
       <c r="E98" t="n">
         <v>96</v>
       </c>
-      <c r="F98" t="inlineStr"/>
       <c r="G98" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H98" t="inlineStr"/>
-      <c r="J98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -4300,14 +4016,11 @@
       <c r="E99" t="n">
         <v>97</v>
       </c>
-      <c r="F99" t="inlineStr"/>
       <c r="G99" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H99" t="inlineStr"/>
-      <c r="J99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -4331,14 +4044,11 @@
       <c r="E100" t="n">
         <v>98</v>
       </c>
-      <c r="F100" t="inlineStr"/>
       <c r="G100" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H100" t="inlineStr"/>
-      <c r="J100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -4362,14 +4072,11 @@
       <c r="E101" t="n">
         <v>99</v>
       </c>
-      <c r="F101" t="inlineStr"/>
       <c r="G101" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H101" t="inlineStr"/>
-      <c r="J101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -4393,14 +4100,11 @@
       <c r="E102" t="n">
         <v>100</v>
       </c>
-      <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H102" t="inlineStr"/>
-      <c r="J102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -4424,14 +4128,11 @@
       <c r="E103" t="n">
         <v>101</v>
       </c>
-      <c r="F103" t="inlineStr"/>
       <c r="G103" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H103" t="inlineStr"/>
-      <c r="J103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -4455,14 +4156,11 @@
       <c r="E104" t="n">
         <v>102</v>
       </c>
-      <c r="F104" t="inlineStr"/>
       <c r="G104" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H104" t="inlineStr"/>
-      <c r="J104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -4486,14 +4184,11 @@
       <c r="E105" t="n">
         <v>103</v>
       </c>
-      <c r="F105" t="inlineStr"/>
       <c r="G105" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H105" t="inlineStr"/>
-      <c r="J105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -4517,14 +4212,11 @@
       <c r="E106" t="n">
         <v>104</v>
       </c>
-      <c r="F106" t="inlineStr"/>
       <c r="G106" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H106" t="inlineStr"/>
-      <c r="J106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -4548,14 +4240,11 @@
       <c r="E107" t="n">
         <v>105</v>
       </c>
-      <c r="F107" t="inlineStr"/>
       <c r="G107" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H107" t="inlineStr"/>
-      <c r="J107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -4579,14 +4268,11 @@
       <c r="E108" t="n">
         <v>106</v>
       </c>
-      <c r="F108" t="inlineStr"/>
       <c r="G108" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H108" t="inlineStr"/>
-      <c r="J108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -4610,14 +4296,11 @@
       <c r="E109" t="n">
         <v>107</v>
       </c>
-      <c r="F109" t="inlineStr"/>
       <c r="G109" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H109" t="inlineStr"/>
-      <c r="J109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -4641,14 +4324,11 @@
       <c r="E110" t="n">
         <v>108</v>
       </c>
-      <c r="F110" t="inlineStr"/>
       <c r="G110" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H110" t="inlineStr"/>
-      <c r="J110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -4672,14 +4352,11 @@
       <c r="E111" t="n">
         <v>109</v>
       </c>
-      <c r="F111" t="inlineStr"/>
       <c r="G111" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H111" t="inlineStr"/>
-      <c r="J111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -4703,14 +4380,11 @@
       <c r="E112" t="n">
         <v>110</v>
       </c>
-      <c r="F112" t="inlineStr"/>
       <c r="G112" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H112" t="inlineStr"/>
-      <c r="J112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -4734,14 +4408,11 @@
       <c r="E113" t="n">
         <v>111</v>
       </c>
-      <c r="F113" t="inlineStr"/>
       <c r="G113" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H113" t="inlineStr"/>
-      <c r="J113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -4765,14 +4436,11 @@
       <c r="E114" t="n">
         <v>112</v>
       </c>
-      <c r="F114" t="inlineStr"/>
       <c r="G114" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H114" t="inlineStr"/>
-      <c r="J114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -4796,14 +4464,11 @@
       <c r="E115" t="n">
         <v>113</v>
       </c>
-      <c r="F115" t="inlineStr"/>
       <c r="G115" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H115" t="inlineStr"/>
-      <c r="J115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -4827,14 +4492,11 @@
       <c r="E116" t="n">
         <v>114</v>
       </c>
-      <c r="F116" t="inlineStr"/>
       <c r="G116" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H116" t="inlineStr"/>
-      <c r="J116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -4858,14 +4520,11 @@
       <c r="E117" t="n">
         <v>115</v>
       </c>
-      <c r="F117" t="inlineStr"/>
       <c r="G117" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H117" t="inlineStr"/>
-      <c r="J117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -4889,14 +4548,11 @@
       <c r="E118" t="n">
         <v>116</v>
       </c>
-      <c r="F118" t="inlineStr"/>
       <c r="G118" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H118" t="inlineStr"/>
-      <c r="J118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -4920,14 +4576,11 @@
       <c r="E119" t="n">
         <v>117</v>
       </c>
-      <c r="F119" t="inlineStr"/>
       <c r="G119" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H119" t="inlineStr"/>
-      <c r="J119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -4951,14 +4604,11 @@
       <c r="E120" t="n">
         <v>118</v>
       </c>
-      <c r="F120" t="inlineStr"/>
       <c r="G120" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H120" t="inlineStr"/>
-      <c r="J120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -4982,14 +4632,11 @@
       <c r="E121" t="n">
         <v>119</v>
       </c>
-      <c r="F121" t="inlineStr"/>
       <c r="G121" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H121" t="inlineStr"/>
-      <c r="J121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -5013,14 +4660,11 @@
       <c r="E122" t="n">
         <v>120</v>
       </c>
-      <c r="F122" t="inlineStr"/>
       <c r="G122" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H122" t="inlineStr"/>
-      <c r="J122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -5044,14 +4688,11 @@
       <c r="E123" t="n">
         <v>121</v>
       </c>
-      <c r="F123" t="inlineStr"/>
       <c r="G123" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H123" t="inlineStr"/>
-      <c r="J123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -5075,14 +4716,11 @@
       <c r="E124" t="n">
         <v>122</v>
       </c>
-      <c r="F124" t="inlineStr"/>
       <c r="G124" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H124" t="inlineStr"/>
-      <c r="J124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -5106,14 +4744,11 @@
       <c r="E125" t="n">
         <v>123</v>
       </c>
-      <c r="F125" t="inlineStr"/>
       <c r="G125" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H125" t="inlineStr"/>
-      <c r="J125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -5137,14 +4772,11 @@
       <c r="E126" t="n">
         <v>124</v>
       </c>
-      <c r="F126" t="inlineStr"/>
       <c r="G126" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H126" t="inlineStr"/>
-      <c r="J126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -5168,14 +4800,11 @@
       <c r="E127" t="n">
         <v>125</v>
       </c>
-      <c r="F127" t="inlineStr"/>
       <c r="G127" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H127" t="inlineStr"/>
-      <c r="J127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -5199,14 +4828,11 @@
       <c r="E128" t="n">
         <v>126</v>
       </c>
-      <c r="F128" t="inlineStr"/>
       <c r="G128" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H128" t="inlineStr"/>
-      <c r="J128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -5230,14 +4856,11 @@
       <c r="E129" t="n">
         <v>127</v>
       </c>
-      <c r="F129" t="inlineStr"/>
       <c r="G129" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H129" t="inlineStr"/>
-      <c r="J129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -5261,14 +4884,11 @@
       <c r="E130" t="n">
         <v>128</v>
       </c>
-      <c r="F130" t="inlineStr"/>
       <c r="G130" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H130" t="inlineStr"/>
-      <c r="J130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -5292,14 +4912,11 @@
       <c r="E131" t="n">
         <v>129</v>
       </c>
-      <c r="F131" t="inlineStr"/>
       <c r="G131" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H131" t="inlineStr"/>
-      <c r="J131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -5323,14 +4940,11 @@
       <c r="E132" t="n">
         <v>130</v>
       </c>
-      <c r="F132" t="inlineStr"/>
       <c r="G132" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H132" t="inlineStr"/>
-      <c r="J132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -5354,14 +4968,11 @@
       <c r="E133" t="n">
         <v>131</v>
       </c>
-      <c r="F133" t="inlineStr"/>
       <c r="G133" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H133" t="inlineStr"/>
-      <c r="J133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -5385,14 +4996,11 @@
       <c r="E134" t="n">
         <v>132</v>
       </c>
-      <c r="F134" t="inlineStr"/>
       <c r="G134" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H134" t="inlineStr"/>
-      <c r="J134" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -5922,7 +5530,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -5944,7 +5552,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Portfolio: $13,800 | Prices as of 2026-06-17</t>
+          <t>Portfolio: $13,800 | Prices as of 2026-06-18</t>
         </is>
       </c>
     </row>
@@ -6000,14 +5608,14 @@
         <v>84.7</v>
       </c>
       <c r="C4" t="n">
-        <v>7.36</v>
+        <v>9.630000000000001</v>
       </c>
       <c r="D4">
         <f>C4/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E4" t="n">
-        <v>432.15</v>
+        <v>462.12</v>
       </c>
       <c r="F4">
         <f>IF(E4="","",ROUND(D4/E4,4))</f>
@@ -6033,14 +5641,14 @@
         <v>84.09999999999999</v>
       </c>
       <c r="C5" t="n">
-        <v>7.14</v>
+        <v>9.34</v>
       </c>
       <c r="D5">
         <f>C5/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E5" t="n">
-        <v>204.65</v>
+        <v>210.69</v>
       </c>
       <c r="F5">
         <f>IF(E5="","",ROUND(D5/E5,4))</f>
@@ -6066,14 +5674,14 @@
         <v>80.09999999999999</v>
       </c>
       <c r="C6" t="n">
-        <v>5.76</v>
+        <v>7.53</v>
       </c>
       <c r="D6">
         <f>C6/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E6" t="n">
-        <v>1958.8</v>
+        <v>2184.75</v>
       </c>
       <c r="F6">
         <f>IF(E6="","",ROUND(D6/E6,4))</f>
@@ -6099,14 +5707,14 @@
         <v>80</v>
       </c>
       <c r="C7" t="n">
-        <v>5.71</v>
+        <v>7.46</v>
       </c>
       <c r="D7">
         <f>C7/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E7" t="n">
-        <v>1043.19</v>
+        <v>1133.99</v>
       </c>
       <c r="F7">
         <f>IF(E7="","",ROUND(D7/E7,4))</f>
@@ -6132,14 +5740,14 @@
         <v>79.40000000000001</v>
       </c>
       <c r="C8" t="n">
-        <v>5.51</v>
+        <v>7.21</v>
       </c>
       <c r="D8">
         <f>C8/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E8" t="n">
-        <v>567.58</v>
+        <v>577.22</v>
       </c>
       <c r="F8">
         <f>IF(E8="","",ROUND(D8/E8,4))</f>
@@ -6165,14 +5773,14 @@
         <v>79.2</v>
       </c>
       <c r="C9" t="n">
-        <v>5.44</v>
+        <v>7.12</v>
       </c>
       <c r="D9">
         <f>C9/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E9" t="n">
-        <v>392.9</v>
+        <v>411.35</v>
       </c>
       <c r="F9">
         <f>IF(E9="","",ROUND(D9/E9,4))</f>
@@ -6191,21 +5799,21 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CRDO</t>
+          <t>APP</t>
         </is>
       </c>
       <c r="B10" t="n">
         <v>78.90000000000001</v>
       </c>
       <c r="C10" t="n">
-        <v>5.34</v>
+        <v>6.98</v>
       </c>
       <c r="D10">
         <f>C10/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E10" t="n">
-        <v>249.33</v>
+        <v>469.71</v>
       </c>
       <c r="F10">
         <f>IF(E10="","",ROUND(D10/E10,4))</f>
@@ -6224,21 +5832,21 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>APP</t>
+          <t>CRDO</t>
         </is>
       </c>
       <c r="B11" t="n">
         <v>78.90000000000001</v>
       </c>
       <c r="C11" t="n">
-        <v>5.34</v>
+        <v>6.98</v>
       </c>
       <c r="D11">
         <f>C11/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E11" t="n">
-        <v>479.49</v>
+        <v>271.83</v>
       </c>
       <c r="F11">
         <f>IF(E11="","",ROUND(D11/E11,4))</f>
@@ -6264,14 +5872,14 @@
         <v>78.5</v>
       </c>
       <c r="C12" t="n">
-        <v>5.19</v>
+        <v>6.79</v>
       </c>
       <c r="D12">
         <f>C12/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E12" t="n">
-        <v>164.93</v>
+        <v>169.67</v>
       </c>
       <c r="F12">
         <f>IF(E12="","",ROUND(D12/E12,4))</f>
@@ -6297,14 +5905,14 @@
         <v>78</v>
       </c>
       <c r="C13" t="n">
-        <v>5.03</v>
+        <v>6.57</v>
       </c>
       <c r="D13">
         <f>C13/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E13" t="n">
-        <v>712.13</v>
+        <v>746.23</v>
       </c>
       <c r="F13">
         <f>IF(E13="","",ROUND(D13/E13,4))</f>
@@ -6330,14 +5938,14 @@
         <v>77.2</v>
       </c>
       <c r="C14" t="n">
-        <v>4.75</v>
+        <v>6.21</v>
       </c>
       <c r="D14">
         <f>C14/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E14" t="n">
-        <v>378.91</v>
+        <v>379.4</v>
       </c>
       <c r="F14">
         <f>IF(E14="","",ROUND(D14/E14,4))</f>
@@ -6363,14 +5971,14 @@
         <v>77.09999999999999</v>
       </c>
       <c r="C15" t="n">
-        <v>4.7</v>
+        <v>6.15</v>
       </c>
       <c r="D15">
         <f>C15/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E15" t="n">
-        <v>374.68</v>
+        <v>417.07</v>
       </c>
       <c r="F15">
         <f>IF(E15="","",ROUND(D15/E15,4))</f>
@@ -6396,14 +6004,14 @@
         <v>76.8</v>
       </c>
       <c r="C16" t="n">
-        <v>4.62</v>
+        <v>6.04</v>
       </c>
       <c r="D16">
         <f>C16/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E16" t="n">
-        <v>363.79</v>
+        <v>368.03</v>
       </c>
       <c r="F16">
         <f>IF(E16="","",ROUND(D16/E16,4))</f>
@@ -6429,14 +6037,14 @@
         <v>76.7</v>
       </c>
       <c r="C17" t="n">
-        <v>4.56</v>
+        <v>5.96</v>
       </c>
       <c r="D17">
         <f>C17/100*'Sizing Rules'!$B$16</f>
         <v/>
       </c>
       <c r="E17" t="n">
-        <v>1931.77</v>
+        <v>1967.41</v>
       </c>
       <c r="F17">
         <f>IF(E17="","",ROUND(D17/E17,4))</f>
@@ -6455,217 +6063,19 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>EME</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>75.5</v>
-      </c>
-      <c r="C18" t="n">
-        <v>4.16</v>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="C18">
+        <f>SUM(C4:C17)</f>
+        <v/>
       </c>
       <c r="D18">
-        <f>C18/100*'Sizing Rules'!$B$16</f>
-        <v/>
-      </c>
-      <c r="E18" t="n">
-        <v>827.5</v>
-      </c>
-      <c r="F18">
-        <f>IF(E18="","",ROUND(D18/E18,4))</f>
+        <f>SUM(D4:D17)</f>
         <v/>
       </c>
       <c r="G18">
-        <f>IF(E18="","",F18*E18)</f>
-        <v/>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>ZS</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>75.5</v>
-      </c>
-      <c r="C19" t="n">
-        <v>4.15</v>
-      </c>
-      <c r="D19">
-        <f>C19/100*'Sizing Rules'!$B$16</f>
-        <v/>
-      </c>
-      <c r="E19" t="n">
-        <v>124.38</v>
-      </c>
-      <c r="F19">
-        <f>IF(E19="","",ROUND(D19/E19,4))</f>
-        <v/>
-      </c>
-      <c r="G19">
-        <f>IF(E19="","",F19*E19)</f>
-        <v/>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>PLTR</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>75.40000000000001</v>
-      </c>
-      <c r="C20" t="n">
-        <v>4.12</v>
-      </c>
-      <c r="D20">
-        <f>C20/100*'Sizing Rules'!$B$16</f>
-        <v/>
-      </c>
-      <c r="E20" t="n">
-        <v>130.63</v>
-      </c>
-      <c r="F20">
-        <f>IF(E20="","",ROUND(D20/E20,4))</f>
-        <v/>
-      </c>
-      <c r="G20">
-        <f>IF(E20="","",F20*E20)</f>
-        <v/>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>VRT</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>75</v>
-      </c>
-      <c r="C21" t="n">
-        <v>4</v>
-      </c>
-      <c r="D21">
-        <f>C21/100*'Sizing Rules'!$B$16</f>
-        <v/>
-      </c>
-      <c r="E21" t="n">
-        <v>317.58</v>
-      </c>
-      <c r="F21">
-        <f>IF(E21="","",ROUND(D21/E21,4))</f>
-        <v/>
-      </c>
-      <c r="G21">
-        <f>IF(E21="","",F21*E21)</f>
-        <v/>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>EQT</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>74.2</v>
-      </c>
-      <c r="C22" t="n">
-        <v>3.69</v>
-      </c>
-      <c r="D22">
-        <f>C22/100*'Sizing Rules'!$B$16</f>
-        <v/>
-      </c>
-      <c r="E22" t="n">
-        <v>51.13</v>
-      </c>
-      <c r="F22">
-        <f>IF(E22="","",ROUND(D22/E22,4))</f>
-        <v/>
-      </c>
-      <c r="G22">
-        <f>IF(E22="","",F22*E22)</f>
-        <v/>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>TER</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>73.5</v>
-      </c>
-      <c r="C23" t="n">
-        <v>3.44</v>
-      </c>
-      <c r="D23">
-        <f>C23/100*'Sizing Rules'!$B$16</f>
-        <v/>
-      </c>
-      <c r="E23" t="n">
-        <v>408.56</v>
-      </c>
-      <c r="F23">
-        <f>IF(E23="","",ROUND(D23/E23,4))</f>
-        <v/>
-      </c>
-      <c r="G23">
-        <f>IF(E23="","",F23*E23)</f>
-        <v/>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="C24">
-        <f>SUM(C4:C23)</f>
-        <v/>
-      </c>
-      <c r="D24">
-        <f>SUM(D4:D23)</f>
-        <v/>
-      </c>
-      <c r="G24">
-        <f>SUM(G4:G23)</f>
+        <f>SUM(G4:G17)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(data): refresh Targets sheet scores from 2026-06-24 Watchlist
Re-pulled TOTAL/Tier for all 132 ranked names from the refreshed
Watchlist, re-sorted by score, renumbered Rank. Status (HOLD, 14) and
Include? preserved exactly — no position changes (asserted before save).

Movers among holdings: TSM ->87.9 (✓✓✓, #1); WDC ->71.62 fell to rank
32. Field movers: PLAB/AR/HTHIY up, UMC/UCTT down.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/00-master/portfolio.xlsx
+++ b/00-master/portfolio.xlsx
@@ -1058,7 +1058,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Target Portfolio (refreshed 2026-06-19, live Watchlist scores)</t>
+          <t>Target Portfolio (refreshed 2026-06-24, live Watchlist scores)</t>
         </is>
       </c>
     </row>
@@ -1126,11 +1126,11 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>84.7</v>
+        <v>87.90000000000001</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>✓✓</t>
+          <t>✓✓✓</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -1271,16 +1271,16 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>MU</t>
+          <t>META</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>06 Silicon - Memory</t>
+          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>79.95</v>
+        <v>79.5</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -1307,16 +1307,16 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>AVGO</t>
+          <t>MU</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
+          <t>06 Silicon - Memory</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>79.2</v>
+        <v>79.34999999999999</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -1343,16 +1343,16 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>META</t>
+          <t>AVGO</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
+          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>78.90000000000001</v>
+        <v>79.2</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -1379,16 +1379,16 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>APP</t>
+          <t>ANET</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI advertising</t>
+          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>78.90000000000001</v>
+        <v>78.48</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -1415,16 +1415,16 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ANET</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
+          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>78.48</v>
+        <v>78.40000000000001</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -1451,16 +1451,16 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>WDC</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
+          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>78</v>
+        <v>78.03</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -1487,16 +1487,16 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>ALAB</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
+          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>77.2</v>
+        <v>77.08</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -1523,16 +1523,16 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ALAB</t>
+          <t>APP</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
+          <t>10 Models, Software &amp; Applications / AI advertising</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>77.08</v>
+        <v>76.90000000000001</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -1559,16 +1559,16 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>FIX</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>76.83</v>
+        <v>76.65000000000001</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -1595,16 +1595,16 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>FIX</t>
+          <t>PLTR</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>10 Models, Software &amp; Applications</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>76.65000000000001</v>
+        <v>76.40000000000001</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -1614,14 +1614,9 @@
       <c r="E16" t="n">
         <v>14</v>
       </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>HOLD</t>
-        </is>
-      </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="I16" t="n">
@@ -1636,16 +1631,16 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>EME</t>
+          <t>ZS</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>75.5</v>
+        <v>75.47</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -1669,16 +1664,16 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ZS</t>
+          <t>VRT</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
+          <t>03 DC Infrastructure</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>75.47</v>
+        <v>75.3</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -1697,16 +1692,16 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>PLTR</t>
+          <t>EME</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>75.40000000000001</v>
+        <v>74.75</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -1725,16 +1720,16 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>VRT</t>
+          <t>WDAY</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>03 DC Infrastructure</t>
+          <t>10 Models, Software &amp; Applications / Enterprise SaaS</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>75.05</v>
+        <v>74.7</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -1753,16 +1748,16 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>EQT</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / GPUs / merchant accelerators</t>
+          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>74.58</v>
+        <v>74.65000000000001</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -1786,16 +1781,16 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>EQT</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
+          <t>06 AI Compute Silicon / GPUs / merchant accelerators</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>74.15000000000001</v>
+        <v>74.58</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -1814,16 +1809,16 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>TER</t>
+          <t>ADSK</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>10 Models, Software &amp; Applications / Design &amp; engineering software</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>73.45</v>
+        <v>74.25</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -1842,16 +1837,16 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>KEYS</t>
+          <t>AR</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
+          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>73.22</v>
+        <v>74.08</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -1870,16 +1865,16 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>ADSK</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / Design &amp; engineering software</t>
+          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>73.15000000000001</v>
+        <v>73.3</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -1898,16 +1893,16 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>STX</t>
+          <t>KEYS</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>72.75</v>
+        <v>73.22</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -1926,16 +1921,16 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>APH</t>
+          <t>TER</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>72.72</v>
+        <v>73.05</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -1954,16 +1949,16 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
+          <t>10 Models, Software &amp; Applications</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>72.7</v>
+        <v>72.8</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -1982,16 +1977,16 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>DELL</t>
+          <t>STX</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>72.67</v>
+        <v>72.75</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -2010,16 +2005,16 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>PANW</t>
+          <t>RRC</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
+          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>72.65000000000001</v>
+        <v>72.75</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
@@ -2038,16 +2033,16 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>PANW</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications</t>
+          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>72.40000000000001</v>
+        <v>72.65000000000001</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -2071,16 +2066,16 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>LSCC</t>
+          <t>HTHIY</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Programmable logic</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>72.38</v>
+        <v>72.05</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -2099,16 +2094,16 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>WDAY</t>
+          <t>LSCC</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / Enterprise SaaS</t>
+          <t>06 AI Compute Silicon / Programmable logic</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>72.3</v>
+        <v>71.98</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -2127,16 +2122,16 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>RRC</t>
+          <t>WDC</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>72</v>
+        <v>71.62</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -2146,25 +2141,30 @@
       <c r="E34" t="n">
         <v>32</v>
       </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>EXE</t>
+          <t>DELL</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>71.97</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
@@ -2183,16 +2183,16 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>VST</t>
+          <t>PLAB</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>01 Power Generation / Independent Power Producers (IPPs)</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>71.05</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
@@ -2211,16 +2211,16 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>LRCX</t>
+          <t>CIEN</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>70.95</v>
+        <v>71.45</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
@@ -2239,16 +2239,16 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>ABBNY</t>
+          <t>EXE</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>70.59999999999999</v>
+        <v>71.22</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -2267,16 +2267,16 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>ARM</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
+          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>70.45</v>
+        <v>71.15000000000001</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -2300,16 +2300,16 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>CIEN</t>
+          <t>VST</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
+          <t>01 Power Generation / Independent Power Producers (IPPs)</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>70.45</v>
+        <v>71.05</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -2328,16 +2328,16 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>MOD</t>
+          <t>DDOG</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>10 Models, Software &amp; Applications / AI observability &amp; infrastructure software</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>70.09999999999999</v>
+        <v>71</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -2356,20 +2356,20 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>PWR</t>
+          <t>APH</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>69.95</v>
+        <v>70.92</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>✓✓</t>
         </is>
       </c>
       <c r="E42" t="n">
@@ -2384,20 +2384,20 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>UMC</t>
+          <t>FN</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>05 Fabs &amp; Foundries</t>
+          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>69.95</v>
+        <v>70.09999999999999</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>✓✓</t>
         </is>
       </c>
       <c r="E43" t="n">
@@ -2412,16 +2412,16 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>PATH</t>
+          <t>PWR</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI-powered automation</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>69.90000000000001</v>
+        <v>69.95</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -2440,16 +2440,16 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>CEG</t>
+          <t>ASML</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>01 Power - IPP / Nuclear</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>69.7</v>
+        <v>69.95</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
@@ -2468,16 +2468,16 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>FN</t>
+          <t>PATH</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
+          <t>10 Models, Software &amp; Applications / AI-powered automation</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>69.7</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -2496,16 +2496,16 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>ARM</t>
+          <t>MOD</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>69.65000000000001</v>
+        <v>69.7</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -2524,16 +2524,16 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>TEL</t>
+          <t>LRCX</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>69.65000000000001</v>
+        <v>69.45</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -2552,16 +2552,16 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>ADI</t>
+          <t>NOW</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Analog &amp; mixed-signal (signal chain + power)</t>
+          <t>10 Models, Software &amp; Applications</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>69.40000000000001</v>
+        <v>69.45</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
@@ -2580,16 +2580,16 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>INTU</t>
+          <t>ADI</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / Financial software</t>
+          <t>06 AI Compute Silicon / Analog &amp; mixed-signal (signal chain + power)</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>69.38</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
@@ -2608,16 +2608,16 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>ADBE</t>
+          <t>MPWR</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / Creative &amp; design software</t>
+          <t>06 AI Compute Silicon / Power management silicon</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>69.33</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
@@ -2664,16 +2664,16 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>ASML</t>
+          <t>ABBNY</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>69.05</v>
+        <v>69</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
@@ -2692,16 +2692,16 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>MPWR</t>
+          <t>CCJ</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Power management silicon</t>
+          <t>01 Power Generation / Nuclear-specific</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>69</v>
+        <v>68.92</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
@@ -2720,16 +2720,16 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>AEIS</t>
+          <t>INTU</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
+          <t>10 Models, Software &amp; Applications / Financial software</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>68.92</v>
+        <v>68.63</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
@@ -2757,7 +2757,7 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>68.90000000000001</v>
+        <v>68.5</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
@@ -2776,16 +2776,16 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>NOW</t>
+          <t>CDNS</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications</t>
+          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>68.84999999999999</v>
+        <v>68.45</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
@@ -2804,16 +2804,16 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>TLN</t>
+          <t>FTNT</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>01 Power Generation / Independent Power Producers (IPPs)</t>
+          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>68.83</v>
+        <v>68.25</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
@@ -2832,16 +2832,16 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>BESIY</t>
+          <t>NVT</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>68.77</v>
+        <v>68.15000000000001</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
@@ -2860,16 +2860,16 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>AMAT</t>
+          <t>TLN</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>01 Power Generation / Independent Power Producers (IPPs)</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>68.75</v>
+        <v>68.08</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
@@ -2888,16 +2888,16 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>TT</t>
+          <t>CSCO</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>68.58</v>
+        <v>68</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
@@ -2916,16 +2916,16 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>HTHIY</t>
+          <t>FORM</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>68.3</v>
+        <v>67.92</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
@@ -2944,16 +2944,16 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>DDOG</t>
+          <t>TT</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI observability &amp; infrastructure software</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>68.25</v>
+        <v>67.83</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
@@ -2986,7 +2986,7 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>67.95</v>
+        <v>67.8</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
@@ -3005,16 +3005,16 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>FORM</t>
+          <t>AEIS</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>67.92</v>
+        <v>67.72</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
@@ -3033,16 +3033,16 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>FTNT</t>
+          <t>NEE</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>67.88</v>
+        <v>67.67</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
@@ -3061,16 +3061,16 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>CDNS</t>
+          <t>POWL</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>67.84999999999999</v>
+        <v>67.34999999999999</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
@@ -3089,16 +3089,16 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>CSCO</t>
+          <t>AAON</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>67.84999999999999</v>
+        <v>67.25</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
@@ -3117,16 +3117,16 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>SBGSY</t>
+          <t>TXN</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>06 AI Compute Silicon / Analog &amp; embedded (power management)</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>67.5</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
@@ -3145,16 +3145,16 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>NVT</t>
+          <t>AMAT</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>67.40000000000001</v>
+        <v>67.05</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
@@ -3173,7 +3173,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>POWL</t>
+          <t>MTZ</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -3182,7 +3182,7 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>67.34999999999999</v>
+        <v>67</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
@@ -3201,16 +3201,16 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>JCI</t>
+          <t>RMBS</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>06 AI Compute Silicon / Memory (HBM is the bottleneck)</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>67.25</v>
+        <v>66.92</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
@@ -3229,16 +3229,16 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>NEE</t>
+          <t>ONTO</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>67.08</v>
+        <v>66.72</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
@@ -3257,16 +3257,16 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>GEV</t>
+          <t>JCI</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>02 Grid Equipment</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>67</v>
+        <v>66.5</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
@@ -3285,16 +3285,16 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>MTZ</t>
+          <t>HPE</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>67</v>
+        <v>66.47</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
@@ -3313,16 +3313,16 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>TSEM</t>
+          <t>MKSI</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>05 Fabs &amp; Foundries</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>66.7</v>
+        <v>66.45</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
@@ -3341,16 +3341,16 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>ENTG</t>
+          <t>ADBE</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
+          <t>10 Models, Software &amp; Applications / Creative &amp; design software</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>66.65000000000001</v>
+        <v>66.33</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
@@ -3369,16 +3369,16 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>ONTO</t>
+          <t>CEG</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>01 Power - IPP / Nuclear</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>66.55</v>
+        <v>66.28</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
@@ -3397,16 +3397,16 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>TXN</t>
+          <t>BESIY</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Analog &amp; embedded (power management)</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>66.5</v>
+        <v>66.09999999999999</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
@@ -3425,16 +3425,16 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>HPE</t>
+          <t>TSEM</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling</t>
+          <t>05 Fabs &amp; Foundries</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>66.47</v>
+        <v>66.09999999999999</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
@@ -3453,16 +3453,16 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>CCJ</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>01 Power Generation / Nuclear-specific</t>
+          <t>01 Power - Distributed</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>66.42</v>
+        <v>66.05</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
@@ -3481,16 +3481,16 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>RMBS</t>
+          <t>SBGSY</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Memory (HBM is the bottleneck)</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>66.42</v>
+        <v>66</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
@@ -3509,16 +3509,16 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>GNRC</t>
+          <t>SNPS</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>01 Power Generation / Distributed / on-site power</t>
+          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>66.40000000000001</v>
+        <v>65.55</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
@@ -3537,16 +3537,16 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>MKSI</t>
+          <t>TEL</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
+          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>66.3</v>
+        <v>65.53</v>
       </c>
       <c r="D84" t="inlineStr">
         <is>
@@ -3565,16 +3565,16 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>AAON</t>
+          <t>GEV</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>02 Grid Equipment</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>66.27</v>
+        <v>65.5</v>
       </c>
       <c r="D85" t="inlineStr">
         <is>
@@ -3593,16 +3593,16 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>ENTG</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>01 Power - Distributed</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>66.05</v>
+        <v>65.45</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
@@ -3621,16 +3621,16 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>HUBB</t>
+          <t>UMC</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>05 Fabs &amp; Foundries</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>65.88</v>
+        <v>65.34999999999999</v>
       </c>
       <c r="D87" t="inlineStr">
         <is>
@@ -3649,16 +3649,16 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>PLAB</t>
+          <t>ORCL</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
+          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>65.59999999999999</v>
+        <v>65.3</v>
       </c>
       <c r="D88" t="inlineStr">
         <is>
@@ -3677,16 +3677,16 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>SNPS</t>
+          <t>GNRC</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
+          <t>01 Power Generation / Distributed / on-site power</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>65.55</v>
+        <v>65.2</v>
       </c>
       <c r="D89" t="inlineStr">
         <is>
@@ -3705,16 +3705,16 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>SNOW</t>
+          <t>NXT</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications</t>
+          <t>01 Power Generation / Solar &amp; renewables equipment (behind-the-meter DC power)</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>65.40000000000001</v>
+        <v>65.12</v>
       </c>
       <c r="D90" t="inlineStr">
         <is>
@@ -3733,16 +3733,16 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>HIVE</t>
+          <t>HUBB</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>65.22</v>
+        <v>64.67</v>
       </c>
       <c r="D91" t="inlineStr">
         <is>
@@ -3761,16 +3761,16 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>FLEX</t>
+          <t>MRVL</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Contract manufacturing / ODMs</t>
+          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>65</v>
+        <v>64.47</v>
       </c>
       <c r="D92" t="inlineStr">
         <is>
@@ -3789,16 +3789,16 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>NBIS</t>
+          <t>ETN</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Neoclouds (AI-native cloud providers)</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>64.90000000000001</v>
+        <v>64.3</v>
       </c>
       <c r="D93" t="inlineStr">
         <is>
@@ -3822,16 +3822,16 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>MRVL</t>
+          <t>SMCI</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>64.47</v>
+        <v>64.25</v>
       </c>
       <c r="D94" t="inlineStr">
         <is>
@@ -3850,16 +3850,16 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>ETN</t>
+          <t>LITE</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>64.3</v>
+        <v>64.17</v>
       </c>
       <c r="D95" t="inlineStr">
         <is>
@@ -3878,16 +3878,16 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>SMCI</t>
+          <t>HIVE</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling</t>
+          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>64.25</v>
+        <v>64.05</v>
       </c>
       <c r="D96" t="inlineStr">
         <is>
@@ -3906,16 +3906,16 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>ORCL</t>
+          <t>IRM</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>64.25</v>
+        <v>63.75</v>
       </c>
       <c r="D97" t="inlineStr">
         <is>
@@ -3934,16 +3934,16 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>IRM</t>
+          <t>SNOW</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>10 Models, Software &amp; Applications</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>63.75</v>
+        <v>63.57</v>
       </c>
       <c r="D98" t="inlineStr">
         <is>
@@ -3962,16 +3962,16 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>KLIC</t>
+          <t>CMI</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>01 Power Generation / Distributed / on-site power</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>63.67</v>
+        <v>63.3</v>
       </c>
       <c r="D99" t="inlineStr">
         <is>
@@ -3990,16 +3990,16 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>NXT</t>
+          <t>KLIC</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>01 Power Generation / Solar &amp; renewables equipment (behind-the-meter DC power)</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>63.62</v>
+        <v>63.17</v>
       </c>
       <c r="D100" t="inlineStr">
         <is>
@@ -4018,16 +4018,16 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>AAPL</t>
+          <t>FLEX</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / Edge AI platforms</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Contract manufacturing / ODMs</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>63.55</v>
+        <v>63.05</v>
       </c>
       <c r="D101" t="inlineStr">
         <is>
@@ -4046,16 +4046,16 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>HUT</t>
+          <t>KN</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
+          <t>04 Semi Equip - Materials</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>63.45</v>
+        <v>62.7</v>
       </c>
       <c r="D102" t="inlineStr">
         <is>
@@ -4074,16 +4074,16 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>CMI</t>
+          <t>CRWV</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>01 Power Generation / Distributed / on-site power</t>
+          <t>09 Cloud - Neocloud</t>
         </is>
       </c>
       <c r="C103" t="n">
-        <v>63.3</v>
+        <v>62.67</v>
       </c>
       <c r="D103" t="inlineStr">
         <is>
@@ -4102,16 +4102,16 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>KN</t>
+          <t>SEI</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>04 Semi Equip - Materials</t>
+          <t>01 Power Generation / Distributed / on-site power</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>63.05</v>
+        <v>62.55</v>
       </c>
       <c r="D104" t="inlineStr">
         <is>
@@ -4130,16 +4130,16 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>SEI</t>
+          <t>AAPL</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>01 Power Generation / Distributed / on-site power</t>
+          <t>10 Models, Software &amp; Applications / Edge AI platforms</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>62.9</v>
+        <v>62.2</v>
       </c>
       <c r="D105" t="inlineStr">
         <is>
@@ -4158,16 +4158,16 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>LITE</t>
+          <t>NBIS</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
+          <t>09 Compute-as-a-Service / Neoclouds (AI-native cloud providers)</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>62.68</v>
+        <v>61.82</v>
       </c>
       <c r="D106" t="inlineStr">
         <is>
@@ -4186,16 +4186,16 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>CRWV</t>
+          <t>P</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>09 Cloud - Neocloud</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>62.67</v>
+        <v>61.65</v>
       </c>
       <c r="D107" t="inlineStr">
         <is>
@@ -4214,12 +4214,12 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>CRWD</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
+          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -4242,16 +4242,16 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>CRWD</t>
+          <t>BWXT</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
+          <t>01 Power Generation / Nuclear-specific</t>
         </is>
       </c>
       <c r="C109" t="n">
-        <v>61.65</v>
+        <v>61.58</v>
       </c>
       <c r="D109" t="inlineStr">
         <is>
@@ -4270,16 +4270,16 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>BWXT</t>
+          <t>COHR</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>01 Power Generation / Nuclear-specific</t>
+          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
         </is>
       </c>
       <c r="C110" t="n">
-        <v>61.58</v>
+        <v>61.55</v>
       </c>
       <c r="D110" t="inlineStr">
         <is>
@@ -4298,16 +4298,16 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>TTMI</t>
+          <t>NXPI</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / PCB / substrates</t>
+          <t>06 AI Compute Silicon / Analog &amp; embedded (auto/edge AI)</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>61.45</v>
+        <v>61.4</v>
       </c>
       <c r="D111" t="inlineStr">
         <is>
@@ -4326,16 +4326,16 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>EQIX</t>
+          <t>MDB</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>10 Models, Software &amp; Applications / AI data layer</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>61</v>
+        <v>61.32</v>
       </c>
       <c r="D112" t="inlineStr">
         <is>
@@ -4354,16 +4354,16 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>COHR</t>
+          <t>HUT</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
+          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
         </is>
       </c>
       <c r="C113" t="n">
-        <v>60.8</v>
+        <v>61.2</v>
       </c>
       <c r="D113" t="inlineStr">
         <is>
@@ -4382,16 +4382,16 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>NXPI</t>
+          <t>ATKR</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Analog &amp; embedded (auto/edge AI)</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>60.65</v>
+        <v>61.15</v>
       </c>
       <c r="D114" t="inlineStr">
         <is>
@@ -4410,16 +4410,16 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>DUK</t>
+          <t>EQIX</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>60.1</v>
+        <v>61</v>
       </c>
       <c r="D115" t="inlineStr">
         <is>
@@ -4447,7 +4447,7 @@
         </is>
       </c>
       <c r="C116" t="n">
-        <v>59.95</v>
+        <v>60.7</v>
       </c>
       <c r="D116" t="inlineStr">
         <is>
@@ -4466,16 +4466,16 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>AEP</t>
+          <t>TTMI</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>04 Semiconductor Equipment &amp; Materials / PCB / substrates</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>59.38</v>
+        <v>60.45</v>
       </c>
       <c r="D117" t="inlineStr">
         <is>
@@ -4494,16 +4494,16 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>CARR</t>
+          <t>DUK</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>59</v>
+        <v>60.1</v>
       </c>
       <c r="D118" t="inlineStr">
         <is>
@@ -4531,7 +4531,7 @@
         </is>
       </c>
       <c r="C119" t="n">
-        <v>58.73</v>
+        <v>59.1</v>
       </c>
       <c r="D119" t="inlineStr">
         <is>
@@ -4550,16 +4550,16 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>WYFI</t>
+          <t>CARR</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Neoclouds (AI-native cloud providers)</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>58.5</v>
+        <v>59</v>
       </c>
       <c r="D120" t="inlineStr">
         <is>
@@ -4578,16 +4578,16 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>PPL</t>
+          <t>QCOM</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>06 AI Compute Silicon / Application processors &amp; connectivity (edge AI)</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>58.38</v>
+        <v>59</v>
       </c>
       <c r="D121" t="inlineStr">
         <is>
@@ -4606,16 +4606,16 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>ATKR</t>
+          <t>AEP</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>58.15</v>
+        <v>58.77</v>
       </c>
       <c r="D122" t="inlineStr">
         <is>
@@ -4634,16 +4634,16 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>TEM</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI-native vertical applications</t>
+          <t>06 AI Compute Silicon / Power management silicon (SiC/GaN)</t>
         </is>
       </c>
       <c r="C123" t="n">
-        <v>58</v>
+        <v>58.52</v>
       </c>
       <c r="D123" t="inlineStr">
         <is>
@@ -4662,16 +4662,16 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PPL</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Power management silicon (SiC/GaN)</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C124" t="n">
-        <v>57.77</v>
+        <v>58.38</v>
       </c>
       <c r="D124" t="inlineStr">
         <is>
@@ -4690,16 +4690,16 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>QCOM</t>
+          <t>TEM</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Application processors &amp; connectivity (edge AI)</t>
+          <t>10 Models, Software &amp; Applications / AI-native vertical applications</t>
         </is>
       </c>
       <c r="C125" t="n">
-        <v>57.5</v>
+        <v>58</v>
       </c>
       <c r="D125" t="inlineStr">
         <is>
@@ -4718,16 +4718,16 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>APLD</t>
+          <t>IREN</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Neoclouds (AI-native cloud providers)</t>
+          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
         </is>
       </c>
       <c r="C126" t="n">
-        <v>57.48</v>
+        <v>57.12</v>
       </c>
       <c r="D126" t="inlineStr">
         <is>
@@ -4746,16 +4746,16 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>MDB</t>
+          <t>XEL</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI data layer</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C127" t="n">
-        <v>57.45</v>
+        <v>57.05</v>
       </c>
       <c r="D127" t="inlineStr">
         <is>
@@ -4774,16 +4774,16 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>ETR</t>
+          <t>WYFI</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>09 Compute-as-a-Service / Neoclouds (AI-native cloud providers)</t>
         </is>
       </c>
       <c r="C128" t="n">
-        <v>57.35</v>
+        <v>56.88</v>
       </c>
       <c r="D128" t="inlineStr">
         <is>
@@ -4802,16 +4802,16 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>IREN</t>
+          <t>PSIX</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
+          <t>01 Power Generation / Distributed / on-site power</t>
         </is>
       </c>
       <c r="C129" t="n">
-        <v>57.25</v>
+        <v>56.35</v>
       </c>
       <c r="D129" t="inlineStr">
         <is>
@@ -4830,7 +4830,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>XEL</t>
+          <t>ETR</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -4839,7 +4839,7 @@
         </is>
       </c>
       <c r="C130" t="n">
-        <v>57.05</v>
+        <v>56.15</v>
       </c>
       <c r="D130" t="inlineStr">
         <is>
@@ -4858,16 +4858,16 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>UCTT</t>
+          <t>SO</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C131" t="n">
-        <v>55.88</v>
+        <v>55.33</v>
       </c>
       <c r="D131" t="inlineStr">
         <is>
@@ -4886,20 +4886,20 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>WULF</t>
+          <t>APLD</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
+          <t>09 Compute-as-a-Service / Neoclouds (AI-native cloud providers)</t>
         </is>
       </c>
       <c r="C132" t="n">
-        <v>55.77</v>
+        <v>54.73</v>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>?</t>
         </is>
       </c>
       <c r="E132" t="n">
@@ -4914,20 +4914,20 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>PSIX</t>
+          <t>WULF</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>01 Power Generation / Distributed / on-site power</t>
+          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
         </is>
       </c>
       <c r="C133" t="n">
-        <v>55.6</v>
+        <v>52.94</v>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>?</t>
         </is>
       </c>
       <c r="E133" t="n">
@@ -4942,20 +4942,20 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>SO</t>
+          <t>UCTT</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
         </is>
       </c>
       <c r="C134" t="n">
-        <v>55.33</v>
+        <v>51.62</v>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>?</t>
         </is>
       </c>
       <c r="E134" t="n">

</xml_diff>

<commit_message>
fix(data): realign Targets cols 8-10 after re-sort (Override/Target%/Notes)
The 2026-06-24 Targets re-sort (6d78941) only carried cols 1-7, leaving
Override/Target %/Notes pinned to old row positions — misaligning
position sizing (e.g. WDC's 6.56% Target stranded). Redone carrying all
10 columns per ticker, asserted before save: HOLD set unchanged (14),
Target%-row set unchanged, every HOLD has a Target%. export_site_data
now runs clean.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/00-master/portfolio.xlsx
+++ b/00-master/portfolio.xlsx
@@ -1058,7 +1058,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Target Portfolio (refreshed 2026-06-19, live Watchlist scores)</t>
+          <t>Target Portfolio (refreshed 2026-06-24, live Watchlist scores)</t>
         </is>
       </c>
     </row>
@@ -1126,11 +1126,11 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>84.7</v>
+        <v>87.90000000000001</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>✓✓</t>
+          <t>✓✓✓</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -1271,16 +1271,16 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>MU</t>
+          <t>META</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>06 Silicon - Memory</t>
+          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>79.95</v>
+        <v>79.5</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -1301,22 +1301,22 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>7.44</v>
+        <v>6.97</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>AVGO</t>
+          <t>MU</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
+          <t>06 Silicon - Memory</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>79.2</v>
+        <v>79.34999999999999</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -1337,22 +1337,22 @@
         </is>
       </c>
       <c r="I8" t="n">
-        <v>7.1</v>
+        <v>7.44</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>META</t>
+          <t>AVGO</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
+          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>78.90000000000001</v>
+        <v>79.2</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -1373,22 +1373,22 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>6.97</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>APP</t>
+          <t>ANET</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI advertising</t>
+          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>78.90000000000001</v>
+        <v>78.48</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -1409,22 +1409,22 @@
         </is>
       </c>
       <c r="I10" t="n">
-        <v>6.97</v>
+        <v>6.77</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ANET</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
+          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>78.48</v>
+        <v>78.40000000000001</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -1445,22 +1445,22 @@
         </is>
       </c>
       <c r="I11" t="n">
-        <v>6.77</v>
+        <v>6.19</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>WDC</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
+          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>78</v>
+        <v>78.03</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -1481,22 +1481,22 @@
         </is>
       </c>
       <c r="I12" t="n">
-        <v>6.56</v>
+        <v>6.02</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>ALAB</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
+          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>77.2</v>
+        <v>77.08</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -1517,22 +1517,22 @@
         </is>
       </c>
       <c r="I13" t="n">
-        <v>6.19</v>
+        <v>6.14</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ALAB</t>
+          <t>APP</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
+          <t>10 Models, Software &amp; Applications / AI advertising</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>77.08</v>
+        <v>76.90000000000001</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -1553,22 +1553,22 @@
         </is>
       </c>
       <c r="I14" t="n">
-        <v>6.14</v>
+        <v>6.97</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>FIX</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>76.83</v>
+        <v>76.65000000000001</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -1589,22 +1589,27 @@
         </is>
       </c>
       <c r="I15" t="n">
-        <v>6.02</v>
+        <v>5.94</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Manually excluded 2026-05-18: $1,854 share price prevents reasonable position sizing below ~$50k portfolio. Conscious framework override. | Override removed 2026-06-09: fractional shares adopted, share-price constraint obsolete (Dom decision).</t>
+        </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>FIX</t>
+          <t>PLTR</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>10 Models, Software &amp; Applications</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>76.65000000000001</v>
+        <v>76.40000000000001</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -1614,38 +1619,25 @@
       <c r="E16" t="n">
         <v>14</v>
       </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>HOLD</t>
-        </is>
-      </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I16" t="n">
-        <v>5.94</v>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>Manually excluded 2026-05-18: $1,854 share price prevents reasonable position sizing below ~$50k portfolio. Conscious framework override. | Override removed 2026-06-09: fractional shares adopted, share-price constraint obsolete (Dom decision).</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>EME</t>
+          <t>ZS</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>75.5</v>
+        <v>75.47</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -1660,25 +1652,20 @@
           <t>N</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>Added 2026-05-25: score 75.2, DC construction, strong momentum (86.7).</t>
-        </is>
-      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ZS</t>
+          <t>VRT</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
+          <t>03 DC Infrastructure</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>75.47</v>
+        <v>75.3</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -1697,16 +1684,16 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>PLTR</t>
+          <t>EME</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>75.40000000000001</v>
+        <v>74.75</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -1721,20 +1708,25 @@
           <t>N</t>
         </is>
       </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Added 2026-05-25: score 75.2, DC construction, strong momentum (86.7).</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>VRT</t>
+          <t>WDAY</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>03 DC Infrastructure</t>
+          <t>10 Models, Software &amp; Applications / Enterprise SaaS</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>75.05</v>
+        <v>74.7</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -1753,16 +1745,16 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>EQT</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / GPUs / merchant accelerators</t>
+          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>74.58</v>
+        <v>74.65000000000001</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -1777,25 +1769,20 @@
           <t>N</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>Removed 2026-05-25: score 74.1 fell below natural 17-name cutoff (ARM 74.2). First name out.</t>
-        </is>
-      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>EQT</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
+          <t>06 AI Compute Silicon / GPUs / merchant accelerators</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>74.15000000000001</v>
+        <v>74.58</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -1810,20 +1797,25 @@
           <t>N</t>
         </is>
       </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Removed 2026-05-25: score 74.1 fell below natural 17-name cutoff (ARM 74.2). First name out.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>TER</t>
+          <t>ADSK</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>10 Models, Software &amp; Applications / Design &amp; engineering software</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>73.45</v>
+        <v>74.25</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -1842,16 +1834,16 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>KEYS</t>
+          <t>AR</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
+          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>73.22</v>
+        <v>74.08</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -1866,20 +1858,25 @@
           <t>N</t>
         </is>
       </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Added 2026-05-22 as substitute for CTRA (delisted). Pure score-driven pick: next-best ✓✓ at 75.62, same Layer 1 NG E&amp;P sub-category — preserves natural gas thesis concentration.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>ADSK</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / Design &amp; engineering software</t>
+          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>73.15000000000001</v>
+        <v>73.3</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -1898,16 +1895,16 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>STX</t>
+          <t>KEYS</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>72.75</v>
+        <v>73.22</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -1926,16 +1923,16 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>APH</t>
+          <t>TER</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>72.72</v>
+        <v>73.05</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -1954,16 +1951,16 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
+          <t>10 Models, Software &amp; Applications</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>72.7</v>
+        <v>72.8</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -1978,20 +1975,25 @@
           <t>N</t>
         </is>
       </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>Added 2026-05-25: score 74.8, Quality 97, PEG 0.8. Enterprise SaaS with AI exposure.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>DELL</t>
+          <t>STX</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>72.67</v>
+        <v>72.75</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -2010,16 +2012,16 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>PANW</t>
+          <t>RRC</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
+          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>72.65000000000001</v>
+        <v>72.75</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
@@ -2038,16 +2040,16 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>PANW</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications</t>
+          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>72.40000000000001</v>
+        <v>72.65000000000001</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -2062,25 +2064,20 @@
           <t>N</t>
         </is>
       </c>
-      <c r="J31" t="inlineStr">
-        <is>
-          <t>Added 2026-05-25: score 74.8, Quality 97, PEG 0.8. Enterprise SaaS with AI exposure.</t>
-        </is>
-      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>LSCC</t>
+          <t>HTHIY</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Programmable logic</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>72.38</v>
+        <v>72.05</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -2099,16 +2096,16 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>WDAY</t>
+          <t>LSCC</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / Enterprise SaaS</t>
+          <t>06 AI Compute Silicon / Programmable logic</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>72.3</v>
+        <v>71.98</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -2127,16 +2124,16 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>RRC</t>
+          <t>WDC</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>72</v>
+        <v>71.62</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -2146,25 +2143,33 @@
       <c r="E34" t="n">
         <v>32</v>
       </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
+        <v>6.56</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>EXE</t>
+          <t>DELL</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>71.97</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
@@ -2183,16 +2188,16 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>VST</t>
+          <t>PLAB</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>01 Power Generation / Independent Power Producers (IPPs)</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>71.05</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
@@ -2211,16 +2216,16 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>LRCX</t>
+          <t>CIEN</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>70.95</v>
+        <v>71.45</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
@@ -2239,16 +2244,16 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>ABBNY</t>
+          <t>EXE</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>70.59999999999999</v>
+        <v>71.22</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -2267,16 +2272,16 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>ARM</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
+          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>70.45</v>
+        <v>71.15000000000001</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -2291,25 +2296,20 @@
           <t>N</t>
         </is>
       </c>
-      <c r="J39" t="inlineStr">
-        <is>
-          <t>Added 2026-05-22 as substitute for CTRA (delisted). Pure score-driven pick: next-best ✓✓ at 75.62, same Layer 1 NG E&amp;P sub-category — preserves natural gas thesis concentration.</t>
-        </is>
-      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>CIEN</t>
+          <t>VST</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
+          <t>01 Power Generation / Independent Power Producers (IPPs)</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>70.45</v>
+        <v>71.05</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -2328,16 +2328,16 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>MOD</t>
+          <t>DDOG</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>10 Models, Software &amp; Applications / AI observability &amp; infrastructure software</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>70.09999999999999</v>
+        <v>71</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -2352,24 +2352,29 @@
           <t>N</t>
         </is>
       </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Added 2026-05-25: score 75.4, Quality 100, PEG 0.7. Beats 4 existing portfolio names.</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>PWR</t>
+          <t>APH</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>69.95</v>
+        <v>70.92</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>✓✓</t>
         </is>
       </c>
       <c r="E42" t="n">
@@ -2384,20 +2389,20 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>UMC</t>
+          <t>FN</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>05 Fabs &amp; Foundries</t>
+          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>69.95</v>
+        <v>70.09999999999999</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>✓✓</t>
         </is>
       </c>
       <c r="E43" t="n">
@@ -2412,16 +2417,16 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>PATH</t>
+          <t>PWR</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI-powered automation</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>69.90000000000001</v>
+        <v>69.95</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -2440,16 +2445,16 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>CEG</t>
+          <t>ASML</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>01 Power - IPP / Nuclear</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>69.7</v>
+        <v>69.95</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
@@ -2468,16 +2473,16 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>FN</t>
+          <t>PATH</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
+          <t>10 Models, Software &amp; Applications / AI-powered automation</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>69.7</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -2496,16 +2501,16 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>ARM</t>
+          <t>MOD</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>69.65000000000001</v>
+        <v>69.7</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -2524,16 +2529,16 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>TEL</t>
+          <t>LRCX</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>69.65000000000001</v>
+        <v>69.45</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -2552,16 +2557,16 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>ADI</t>
+          <t>NOW</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Analog &amp; mixed-signal (signal chain + power)</t>
+          <t>10 Models, Software &amp; Applications</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>69.40000000000001</v>
+        <v>69.45</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
@@ -2580,16 +2585,16 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>INTU</t>
+          <t>ADI</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / Financial software</t>
+          <t>06 AI Compute Silicon / Analog &amp; mixed-signal (signal chain + power)</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>69.38</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
@@ -2608,16 +2613,16 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>ADBE</t>
+          <t>MPWR</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / Creative &amp; design software</t>
+          <t>06 AI Compute Silicon / Power management silicon</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>69.33</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
@@ -2664,16 +2669,16 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>ASML</t>
+          <t>ABBNY</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>69.05</v>
+        <v>69</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
@@ -2692,16 +2697,16 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>MPWR</t>
+          <t>CCJ</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Power management silicon</t>
+          <t>01 Power Generation / Nuclear-specific</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>69</v>
+        <v>68.92</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
@@ -2720,16 +2725,16 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>AEIS</t>
+          <t>INTU</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
+          <t>10 Models, Software &amp; Applications / Financial software</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>68.92</v>
+        <v>68.63</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
@@ -2757,7 +2762,7 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>68.90000000000001</v>
+        <v>68.5</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
@@ -2776,16 +2781,16 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>NOW</t>
+          <t>CDNS</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications</t>
+          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>68.84999999999999</v>
+        <v>68.45</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
@@ -2804,16 +2809,16 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>TLN</t>
+          <t>FTNT</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>01 Power Generation / Independent Power Producers (IPPs)</t>
+          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>68.83</v>
+        <v>68.25</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
@@ -2832,16 +2837,16 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>BESIY</t>
+          <t>NVT</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>68.77</v>
+        <v>68.15000000000001</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
@@ -2860,16 +2865,16 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>AMAT</t>
+          <t>TLN</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>01 Power Generation / Independent Power Producers (IPPs)</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>68.75</v>
+        <v>68.08</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
@@ -2888,16 +2893,16 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>TT</t>
+          <t>CSCO</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>68.58</v>
+        <v>68</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
@@ -2916,16 +2921,16 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>HTHIY</t>
+          <t>FORM</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>68.3</v>
+        <v>67.92</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
@@ -2944,16 +2949,16 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>DDOG</t>
+          <t>TT</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI observability &amp; infrastructure software</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>68.25</v>
+        <v>67.83</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
@@ -2968,11 +2973,6 @@
           <t>N</t>
         </is>
       </c>
-      <c r="J63" t="inlineStr">
-        <is>
-          <t>Added 2026-05-25: score 75.4, Quality 100, PEG 0.7. Beats 4 existing portfolio names.</t>
-        </is>
-      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -2986,7 +2986,7 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>67.95</v>
+        <v>67.8</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
@@ -3005,16 +3005,16 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>FORM</t>
+          <t>AEIS</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>67.92</v>
+        <v>67.72</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
@@ -3033,16 +3033,16 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>FTNT</t>
+          <t>NEE</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>67.88</v>
+        <v>67.67</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
@@ -3061,16 +3061,16 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>CDNS</t>
+          <t>POWL</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>67.84999999999999</v>
+        <v>67.34999999999999</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
@@ -3089,16 +3089,16 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>CSCO</t>
+          <t>AAON</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>67.84999999999999</v>
+        <v>67.25</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
@@ -3117,16 +3117,16 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>SBGSY</t>
+          <t>TXN</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>06 AI Compute Silicon / Analog &amp; embedded (power management)</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>67.5</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
@@ -3145,16 +3145,16 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>NVT</t>
+          <t>AMAT</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>67.40000000000001</v>
+        <v>67.05</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
@@ -3173,7 +3173,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>POWL</t>
+          <t>MTZ</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -3182,7 +3182,7 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>67.34999999999999</v>
+        <v>67</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
@@ -3201,16 +3201,16 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>JCI</t>
+          <t>RMBS</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>06 AI Compute Silicon / Memory (HBM is the bottleneck)</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>67.25</v>
+        <v>66.92</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
@@ -3229,16 +3229,16 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>NEE</t>
+          <t>ONTO</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>67.08</v>
+        <v>66.72</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
@@ -3257,16 +3257,16 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>GEV</t>
+          <t>JCI</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>02 Grid Equipment</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>67</v>
+        <v>66.5</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
@@ -3285,16 +3285,16 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>MTZ</t>
+          <t>HPE</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>67</v>
+        <v>66.47</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
@@ -3313,16 +3313,16 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>TSEM</t>
+          <t>MKSI</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>05 Fabs &amp; Foundries</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>66.7</v>
+        <v>66.45</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
@@ -3341,16 +3341,16 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>ENTG</t>
+          <t>ADBE</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
+          <t>10 Models, Software &amp; Applications / Creative &amp; design software</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>66.65000000000001</v>
+        <v>66.33</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
@@ -3369,16 +3369,16 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>ONTO</t>
+          <t>CEG</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>01 Power - IPP / Nuclear</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>66.55</v>
+        <v>66.28</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
@@ -3397,16 +3397,16 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>TXN</t>
+          <t>BESIY</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Analog &amp; embedded (power management)</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>66.5</v>
+        <v>66.09999999999999</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
@@ -3425,16 +3425,16 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>HPE</t>
+          <t>TSEM</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling</t>
+          <t>05 Fabs &amp; Foundries</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>66.47</v>
+        <v>66.09999999999999</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
@@ -3453,16 +3453,16 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>CCJ</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>01 Power Generation / Nuclear-specific</t>
+          <t>01 Power - Distributed</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>66.42</v>
+        <v>66.05</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
@@ -3481,16 +3481,16 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>RMBS</t>
+          <t>SBGSY</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Memory (HBM is the bottleneck)</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>66.42</v>
+        <v>66</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
@@ -3509,16 +3509,16 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>GNRC</t>
+          <t>SNPS</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>01 Power Generation / Distributed / on-site power</t>
+          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>66.40000000000001</v>
+        <v>65.55</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
@@ -3537,16 +3537,16 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>MKSI</t>
+          <t>TEL</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
+          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>66.3</v>
+        <v>65.53</v>
       </c>
       <c r="D84" t="inlineStr">
         <is>
@@ -3565,16 +3565,16 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>AAON</t>
+          <t>GEV</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>02 Grid Equipment</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>66.27</v>
+        <v>65.5</v>
       </c>
       <c r="D85" t="inlineStr">
         <is>
@@ -3593,16 +3593,16 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>ENTG</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>01 Power - Distributed</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>66.05</v>
+        <v>65.45</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
@@ -3621,16 +3621,16 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>HUBB</t>
+          <t>UMC</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>05 Fabs &amp; Foundries</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>65.88</v>
+        <v>65.34999999999999</v>
       </c>
       <c r="D87" t="inlineStr">
         <is>
@@ -3649,16 +3649,16 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>PLAB</t>
+          <t>ORCL</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
+          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>65.59999999999999</v>
+        <v>65.3</v>
       </c>
       <c r="D88" t="inlineStr">
         <is>
@@ -3677,16 +3677,16 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>SNPS</t>
+          <t>GNRC</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
+          <t>01 Power Generation / Distributed / on-site power</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>65.55</v>
+        <v>65.2</v>
       </c>
       <c r="D89" t="inlineStr">
         <is>
@@ -3705,16 +3705,16 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>SNOW</t>
+          <t>NXT</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications</t>
+          <t>01 Power Generation / Solar &amp; renewables equipment (behind-the-meter DC power)</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>65.40000000000001</v>
+        <v>65.12</v>
       </c>
       <c r="D90" t="inlineStr">
         <is>
@@ -3733,16 +3733,16 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>HIVE</t>
+          <t>HUBB</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>65.22</v>
+        <v>64.67</v>
       </c>
       <c r="D91" t="inlineStr">
         <is>
@@ -3761,16 +3761,16 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>FLEX</t>
+          <t>MRVL</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Contract manufacturing / ODMs</t>
+          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>65</v>
+        <v>64.47</v>
       </c>
       <c r="D92" t="inlineStr">
         <is>
@@ -3789,16 +3789,16 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>NBIS</t>
+          <t>ETN</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Neoclouds (AI-native cloud providers)</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>64.90000000000001</v>
+        <v>64.3</v>
       </c>
       <c r="D93" t="inlineStr">
         <is>
@@ -3813,25 +3813,20 @@
           <t>N</t>
         </is>
       </c>
-      <c r="J93" t="inlineStr">
-        <is>
-          <t>Removed 2026-05-25: dropped to ✓ (65.5) after reweight. Value 7.5 penalized by higher Value weight.</t>
-        </is>
-      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>MRVL</t>
+          <t>SMCI</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>64.47</v>
+        <v>64.25</v>
       </c>
       <c r="D94" t="inlineStr">
         <is>
@@ -3850,16 +3845,16 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>ETN</t>
+          <t>LITE</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>64.3</v>
+        <v>64.17</v>
       </c>
       <c r="D95" t="inlineStr">
         <is>
@@ -3878,16 +3873,16 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>SMCI</t>
+          <t>HIVE</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling</t>
+          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>64.25</v>
+        <v>64.05</v>
       </c>
       <c r="D96" t="inlineStr">
         <is>
@@ -3906,16 +3901,16 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>ORCL</t>
+          <t>IRM</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>64.25</v>
+        <v>63.75</v>
       </c>
       <c r="D97" t="inlineStr">
         <is>
@@ -3934,16 +3929,16 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>IRM</t>
+          <t>SNOW</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>10 Models, Software &amp; Applications</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>63.75</v>
+        <v>63.57</v>
       </c>
       <c r="D98" t="inlineStr">
         <is>
@@ -3962,16 +3957,16 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>KLIC</t>
+          <t>CMI</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>01 Power Generation / Distributed / on-site power</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>63.67</v>
+        <v>63.3</v>
       </c>
       <c r="D99" t="inlineStr">
         <is>
@@ -3990,16 +3985,16 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>NXT</t>
+          <t>KLIC</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>01 Power Generation / Solar &amp; renewables equipment (behind-the-meter DC power)</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>63.62</v>
+        <v>63.17</v>
       </c>
       <c r="D100" t="inlineStr">
         <is>
@@ -4018,16 +4013,16 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>AAPL</t>
+          <t>FLEX</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / Edge AI platforms</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Contract manufacturing / ODMs</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>63.55</v>
+        <v>63.05</v>
       </c>
       <c r="D101" t="inlineStr">
         <is>
@@ -4046,16 +4041,16 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>HUT</t>
+          <t>KN</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
+          <t>04 Semi Equip - Materials</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>63.45</v>
+        <v>62.7</v>
       </c>
       <c r="D102" t="inlineStr">
         <is>
@@ -4074,16 +4069,16 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>CMI</t>
+          <t>CRWV</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>01 Power Generation / Distributed / on-site power</t>
+          <t>09 Cloud - Neocloud</t>
         </is>
       </c>
       <c r="C103" t="n">
-        <v>63.3</v>
+        <v>62.67</v>
       </c>
       <c r="D103" t="inlineStr">
         <is>
@@ -4102,16 +4097,16 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>KN</t>
+          <t>SEI</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>04 Semi Equip - Materials</t>
+          <t>01 Power Generation / Distributed / on-site power</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>63.05</v>
+        <v>62.55</v>
       </c>
       <c r="D104" t="inlineStr">
         <is>
@@ -4130,16 +4125,16 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>SEI</t>
+          <t>AAPL</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>01 Power Generation / Distributed / on-site power</t>
+          <t>10 Models, Software &amp; Applications / Edge AI platforms</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>62.9</v>
+        <v>62.2</v>
       </c>
       <c r="D105" t="inlineStr">
         <is>
@@ -4158,16 +4153,16 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>LITE</t>
+          <t>NBIS</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
+          <t>09 Compute-as-a-Service / Neoclouds (AI-native cloud providers)</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>62.68</v>
+        <v>61.82</v>
       </c>
       <c r="D106" t="inlineStr">
         <is>
@@ -4182,20 +4177,25 @@
           <t>N</t>
         </is>
       </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>Removed 2026-05-25: dropped to ✓ (65.5) after reweight. Value 7.5 penalized by higher Value weight.</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>CRWV</t>
+          <t>P</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>09 Cloud - Neocloud</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>62.67</v>
+        <v>61.65</v>
       </c>
       <c r="D107" t="inlineStr">
         <is>
@@ -4214,12 +4214,12 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>CRWD</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
+          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -4242,16 +4242,16 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>CRWD</t>
+          <t>BWXT</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
+          <t>01 Power Generation / Nuclear-specific</t>
         </is>
       </c>
       <c r="C109" t="n">
-        <v>61.65</v>
+        <v>61.58</v>
       </c>
       <c r="D109" t="inlineStr">
         <is>
@@ -4270,16 +4270,16 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>BWXT</t>
+          <t>COHR</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>01 Power Generation / Nuclear-specific</t>
+          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
         </is>
       </c>
       <c r="C110" t="n">
-        <v>61.58</v>
+        <v>61.55</v>
       </c>
       <c r="D110" t="inlineStr">
         <is>
@@ -4298,16 +4298,16 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>TTMI</t>
+          <t>NXPI</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / PCB / substrates</t>
+          <t>06 AI Compute Silicon / Analog &amp; embedded (auto/edge AI)</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>61.45</v>
+        <v>61.4</v>
       </c>
       <c r="D111" t="inlineStr">
         <is>
@@ -4326,16 +4326,16 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>EQIX</t>
+          <t>MDB</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>10 Models, Software &amp; Applications / AI data layer</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>61</v>
+        <v>61.32</v>
       </c>
       <c r="D112" t="inlineStr">
         <is>
@@ -4354,16 +4354,16 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>COHR</t>
+          <t>HUT</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
+          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
         </is>
       </c>
       <c r="C113" t="n">
-        <v>60.8</v>
+        <v>61.2</v>
       </c>
       <c r="D113" t="inlineStr">
         <is>
@@ -4382,16 +4382,16 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>NXPI</t>
+          <t>ATKR</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Analog &amp; embedded (auto/edge AI)</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>60.65</v>
+        <v>61.15</v>
       </c>
       <c r="D114" t="inlineStr">
         <is>
@@ -4410,16 +4410,16 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>DUK</t>
+          <t>EQIX</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>60.1</v>
+        <v>61</v>
       </c>
       <c r="D115" t="inlineStr">
         <is>
@@ -4447,7 +4447,7 @@
         </is>
       </c>
       <c r="C116" t="n">
-        <v>59.95</v>
+        <v>60.7</v>
       </c>
       <c r="D116" t="inlineStr">
         <is>
@@ -4466,16 +4466,16 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>AEP</t>
+          <t>TTMI</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>04 Semiconductor Equipment &amp; Materials / PCB / substrates</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>59.38</v>
+        <v>60.45</v>
       </c>
       <c r="D117" t="inlineStr">
         <is>
@@ -4494,16 +4494,16 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>CARR</t>
+          <t>DUK</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>59</v>
+        <v>60.1</v>
       </c>
       <c r="D118" t="inlineStr">
         <is>
@@ -4531,7 +4531,7 @@
         </is>
       </c>
       <c r="C119" t="n">
-        <v>58.73</v>
+        <v>59.1</v>
       </c>
       <c r="D119" t="inlineStr">
         <is>
@@ -4550,16 +4550,16 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>WYFI</t>
+          <t>CARR</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Neoclouds (AI-native cloud providers)</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>58.5</v>
+        <v>59</v>
       </c>
       <c r="D120" t="inlineStr">
         <is>
@@ -4578,16 +4578,16 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>PPL</t>
+          <t>QCOM</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>06 AI Compute Silicon / Application processors &amp; connectivity (edge AI)</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>58.38</v>
+        <v>59</v>
       </c>
       <c r="D121" t="inlineStr">
         <is>
@@ -4606,16 +4606,16 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>ATKR</t>
+          <t>AEP</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>58.15</v>
+        <v>58.77</v>
       </c>
       <c r="D122" t="inlineStr">
         <is>
@@ -4634,16 +4634,16 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>TEM</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI-native vertical applications</t>
+          <t>06 AI Compute Silicon / Power management silicon (SiC/GaN)</t>
         </is>
       </c>
       <c r="C123" t="n">
-        <v>58</v>
+        <v>58.52</v>
       </c>
       <c r="D123" t="inlineStr">
         <is>
@@ -4662,16 +4662,16 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>PPL</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Power management silicon (SiC/GaN)</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C124" t="n">
-        <v>57.77</v>
+        <v>58.38</v>
       </c>
       <c r="D124" t="inlineStr">
         <is>
@@ -4690,16 +4690,16 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>QCOM</t>
+          <t>TEM</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Application processors &amp; connectivity (edge AI)</t>
+          <t>10 Models, Software &amp; Applications / AI-native vertical applications</t>
         </is>
       </c>
       <c r="C125" t="n">
-        <v>57.5</v>
+        <v>58</v>
       </c>
       <c r="D125" t="inlineStr">
         <is>
@@ -4718,16 +4718,16 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>APLD</t>
+          <t>IREN</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Neoclouds (AI-native cloud providers)</t>
+          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
         </is>
       </c>
       <c r="C126" t="n">
-        <v>57.48</v>
+        <v>57.12</v>
       </c>
       <c r="D126" t="inlineStr">
         <is>
@@ -4746,16 +4746,16 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>MDB</t>
+          <t>XEL</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI data layer</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C127" t="n">
-        <v>57.45</v>
+        <v>57.05</v>
       </c>
       <c r="D127" t="inlineStr">
         <is>
@@ -4774,16 +4774,16 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>ETR</t>
+          <t>WYFI</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>09 Compute-as-a-Service / Neoclouds (AI-native cloud providers)</t>
         </is>
       </c>
       <c r="C128" t="n">
-        <v>57.35</v>
+        <v>56.88</v>
       </c>
       <c r="D128" t="inlineStr">
         <is>
@@ -4802,16 +4802,16 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>IREN</t>
+          <t>PSIX</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
+          <t>01 Power Generation / Distributed / on-site power</t>
         </is>
       </c>
       <c r="C129" t="n">
-        <v>57.25</v>
+        <v>56.35</v>
       </c>
       <c r="D129" t="inlineStr">
         <is>
@@ -4830,7 +4830,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>XEL</t>
+          <t>ETR</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -4839,7 +4839,7 @@
         </is>
       </c>
       <c r="C130" t="n">
-        <v>57.05</v>
+        <v>56.15</v>
       </c>
       <c r="D130" t="inlineStr">
         <is>
@@ -4858,16 +4858,16 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>UCTT</t>
+          <t>SO</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C131" t="n">
-        <v>55.88</v>
+        <v>55.33</v>
       </c>
       <c r="D131" t="inlineStr">
         <is>
@@ -4886,20 +4886,20 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>WULF</t>
+          <t>APLD</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
+          <t>09 Compute-as-a-Service / Neoclouds (AI-native cloud providers)</t>
         </is>
       </c>
       <c r="C132" t="n">
-        <v>55.77</v>
+        <v>54.73</v>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>?</t>
         </is>
       </c>
       <c r="E132" t="n">
@@ -4914,20 +4914,20 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>PSIX</t>
+          <t>WULF</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>01 Power Generation / Distributed / on-site power</t>
+          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
         </is>
       </c>
       <c r="C133" t="n">
-        <v>55.6</v>
+        <v>52.94</v>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>?</t>
         </is>
       </c>
       <c r="E133" t="n">
@@ -4942,20 +4942,20 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>SO</t>
+          <t>UCTT</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
         </is>
       </c>
       <c r="C134" t="n">
-        <v>55.33</v>
+        <v>51.62</v>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>?</t>
         </is>
       </c>
       <c r="E134" t="n">

</xml_diff>

<commit_message>
fix(deploy): lazy yfinance imports so site-deploy pytest passes
The deploy gate runs `pytest tests` with only openpyxl+pytest (no
yfinance, by design). test_refresh_objective_inputs imported the skill
module, which imported batch_score -> yfinance at load -> collection
error -> deploy failed. Made yfinance/batch_score/momentum imports lazy
(inside the real fetchers); mw_staleness_flag now uses a local
_is_layer9_capacity/_CAPACITY_JSON instead of importing batch_score.
Adds test_module_imports_without_yfinance (subprocess, yfinance blocked).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/00-master/portfolio.xlsx
+++ b/00-master/portfolio.xlsx
@@ -1058,7 +1058,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Target Portfolio (refreshed 2026-06-24, live Watchlist scores)</t>
+          <t>Target Portfolio (refreshed 2026-06-19, live Watchlist scores)</t>
         </is>
       </c>
     </row>
@@ -1126,11 +1126,11 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>87.90000000000001</v>
+        <v>84.7</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>✓✓✓</t>
+          <t>✓✓</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -1271,16 +1271,16 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>META</t>
+          <t>MU</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
+          <t>06 Silicon - Memory</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>79.5</v>
+        <v>79.95</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -1307,16 +1307,16 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>MU</t>
+          <t>AVGO</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>06 Silicon - Memory</t>
+          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>79.34999999999999</v>
+        <v>79.2</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -1343,16 +1343,16 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>AVGO</t>
+          <t>META</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
+          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>79.2</v>
+        <v>78.90000000000001</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -1379,16 +1379,16 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ANET</t>
+          <t>APP</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
+          <t>10 Models, Software &amp; Applications / AI advertising</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>78.48</v>
+        <v>78.90000000000001</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -1415,16 +1415,16 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>ANET</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
+          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>78.40000000000001</v>
+        <v>78.48</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -1451,16 +1451,16 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>WDC</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>78.03</v>
+        <v>78</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -1487,16 +1487,16 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ALAB</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
+          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>77.08</v>
+        <v>77.2</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -1523,16 +1523,16 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>APP</t>
+          <t>ALAB</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI advertising</t>
+          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>76.90000000000001</v>
+        <v>77.08</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -1559,16 +1559,16 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>FIX</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>76.65000000000001</v>
+        <v>76.83</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -1595,16 +1595,16 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>PLTR</t>
+          <t>FIX</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>76.40000000000001</v>
+        <v>76.65000000000001</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -1614,9 +1614,14 @@
       <c r="E16" t="n">
         <v>14</v>
       </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="I16" t="n">
@@ -1631,16 +1636,16 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ZS</t>
+          <t>EME</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>75.47</v>
+        <v>75.5</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -1664,16 +1669,16 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>VRT</t>
+          <t>ZS</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>03 DC Infrastructure</t>
+          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>75.3</v>
+        <v>75.47</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -1692,16 +1697,16 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>EME</t>
+          <t>PLTR</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>10 Models, Software &amp; Applications</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>74.75</v>
+        <v>75.40000000000001</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -1720,16 +1725,16 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>WDAY</t>
+          <t>VRT</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / Enterprise SaaS</t>
+          <t>03 DC Infrastructure</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>74.7</v>
+        <v>75.05</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -1748,16 +1753,16 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>EQT</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
+          <t>06 AI Compute Silicon / GPUs / merchant accelerators</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>74.65000000000001</v>
+        <v>74.58</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -1781,16 +1786,16 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>EQT</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / GPUs / merchant accelerators</t>
+          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>74.58</v>
+        <v>74.15000000000001</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -1809,16 +1814,16 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>ADSK</t>
+          <t>TER</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / Design &amp; engineering software</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>74.25</v>
+        <v>73.45</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -1837,16 +1842,16 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>KEYS</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>74.08</v>
+        <v>73.22</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -1865,16 +1870,16 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>ADSK</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
+          <t>10 Models, Software &amp; Applications / Design &amp; engineering software</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>73.3</v>
+        <v>73.15000000000001</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -1893,16 +1898,16 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>KEYS</t>
+          <t>STX</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>73.22</v>
+        <v>72.75</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -1921,16 +1926,16 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>TER</t>
+          <t>APH</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>73.05</v>
+        <v>72.72</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -1949,16 +1954,16 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications</t>
+          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>72.8</v>
+        <v>72.7</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -1977,16 +1982,16 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>STX</t>
+          <t>DELL</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>72.75</v>
+        <v>72.67</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -2005,16 +2010,16 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>RRC</t>
+          <t>PANW</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
+          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>72.75</v>
+        <v>72.65000000000001</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
@@ -2033,16 +2038,16 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>PANW</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
+          <t>10 Models, Software &amp; Applications</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>72.65000000000001</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -2066,16 +2071,16 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>HTHIY</t>
+          <t>LSCC</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>06 AI Compute Silicon / Programmable logic</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>72.05</v>
+        <v>72.38</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -2094,16 +2099,16 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>LSCC</t>
+          <t>WDAY</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Programmable logic</t>
+          <t>10 Models, Software &amp; Applications / Enterprise SaaS</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>71.98</v>
+        <v>72.3</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -2122,16 +2127,16 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>WDC</t>
+          <t>RRC</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
+          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>71.62</v>
+        <v>72</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -2141,30 +2146,25 @@
       <c r="E34" t="n">
         <v>32</v>
       </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>HOLD</t>
-        </is>
-      </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>DELL</t>
+          <t>EXE</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling</t>
+          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>71.59999999999999</v>
+        <v>71.97</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
@@ -2183,16 +2183,16 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>PLAB</t>
+          <t>VST</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
+          <t>01 Power Generation / Independent Power Producers (IPPs)</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>71.59999999999999</v>
+        <v>71.05</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
@@ -2211,16 +2211,16 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>CIEN</t>
+          <t>LRCX</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>71.45</v>
+        <v>70.95</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
@@ -2239,16 +2239,16 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>EXE</t>
+          <t>ABBNY</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>71.22</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -2267,16 +2267,16 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>ARM</t>
+          <t>AR</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
+          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>71.15000000000001</v>
+        <v>70.45</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -2300,16 +2300,16 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>VST</t>
+          <t>CIEN</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>01 Power Generation / Independent Power Producers (IPPs)</t>
+          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>71.05</v>
+        <v>70.45</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -2328,16 +2328,16 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>DDOG</t>
+          <t>MOD</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI observability &amp; infrastructure software</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>71</v>
+        <v>70.09999999999999</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -2356,20 +2356,20 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>APH</t>
+          <t>PWR</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>70.92</v>
+        <v>69.95</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>✓✓</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="E42" t="n">
@@ -2384,20 +2384,20 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>FN</t>
+          <t>UMC</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
+          <t>05 Fabs &amp; Foundries</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>70.09999999999999</v>
+        <v>69.95</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>✓✓</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="E43" t="n">
@@ -2412,16 +2412,16 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>PWR</t>
+          <t>PATH</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>10 Models, Software &amp; Applications / AI-powered automation</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>69.95</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -2440,16 +2440,16 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>ASML</t>
+          <t>CEG</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>01 Power - IPP / Nuclear</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>69.95</v>
+        <v>69.7</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
@@ -2468,16 +2468,16 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>PATH</t>
+          <t>FN</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI-powered automation</t>
+          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>69.90000000000001</v>
+        <v>69.7</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -2496,16 +2496,16 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>MOD</t>
+          <t>ARM</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>69.7</v>
+        <v>69.65000000000001</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -2524,16 +2524,16 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>LRCX</t>
+          <t>TEL</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>69.45</v>
+        <v>69.65000000000001</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -2552,16 +2552,16 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>NOW</t>
+          <t>ADI</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications</t>
+          <t>06 AI Compute Silicon / Analog &amp; mixed-signal (signal chain + power)</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>69.45</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
@@ -2580,16 +2580,16 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>ADI</t>
+          <t>INTU</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Analog &amp; mixed-signal (signal chain + power)</t>
+          <t>10 Models, Software &amp; Applications / Financial software</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>69.40000000000001</v>
+        <v>69.38</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
@@ -2608,16 +2608,16 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>MPWR</t>
+          <t>ADBE</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Power management silicon</t>
+          <t>10 Models, Software &amp; Applications / Creative &amp; design software</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>69.40000000000001</v>
+        <v>69.33</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
@@ -2664,16 +2664,16 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>ABBNY</t>
+          <t>ASML</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>69</v>
+        <v>69.05</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
@@ -2692,16 +2692,16 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>CCJ</t>
+          <t>MPWR</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>01 Power Generation / Nuclear-specific</t>
+          <t>06 AI Compute Silicon / Power management silicon</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>68.92</v>
+        <v>69</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
@@ -2720,16 +2720,16 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>INTU</t>
+          <t>AEIS</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / Financial software</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>68.63</v>
+        <v>68.92</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
@@ -2757,7 +2757,7 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>68.5</v>
+        <v>68.90000000000001</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
@@ -2776,16 +2776,16 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>CDNS</t>
+          <t>NOW</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
+          <t>10 Models, Software &amp; Applications</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>68.45</v>
+        <v>68.84999999999999</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
@@ -2804,16 +2804,16 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>FTNT</t>
+          <t>TLN</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
+          <t>01 Power Generation / Independent Power Producers (IPPs)</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>68.25</v>
+        <v>68.83</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
@@ -2832,16 +2832,16 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>NVT</t>
+          <t>BESIY</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>68.15000000000001</v>
+        <v>68.77</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
@@ -2860,16 +2860,16 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>TLN</t>
+          <t>AMAT</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>01 Power Generation / Independent Power Producers (IPPs)</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>68.08</v>
+        <v>68.75</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
@@ -2888,16 +2888,16 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>CSCO</t>
+          <t>TT</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>68</v>
+        <v>68.58</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
@@ -2916,16 +2916,16 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>FORM</t>
+          <t>HTHIY</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>67.92</v>
+        <v>68.3</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
@@ -2944,16 +2944,16 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>TT</t>
+          <t>DDOG</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>10 Models, Software &amp; Applications / AI observability &amp; infrastructure software</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>67.83</v>
+        <v>68.25</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
@@ -2986,7 +2986,7 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>67.8</v>
+        <v>67.95</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
@@ -3005,16 +3005,16 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>AEIS</t>
+          <t>FORM</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>67.72</v>
+        <v>67.92</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
@@ -3033,16 +3033,16 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>NEE</t>
+          <t>FTNT</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>67.67</v>
+        <v>67.88</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
@@ -3061,16 +3061,16 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>POWL</t>
+          <t>CDNS</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>67.34999999999999</v>
+        <v>67.84999999999999</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
@@ -3089,16 +3089,16 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>AAON</t>
+          <t>CSCO</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>67.25</v>
+        <v>67.84999999999999</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
@@ -3117,16 +3117,16 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>TXN</t>
+          <t>SBGSY</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Analog &amp; embedded (power management)</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>67.09999999999999</v>
+        <v>67.5</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
@@ -3145,16 +3145,16 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>AMAT</t>
+          <t>NVT</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>67.05</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
@@ -3173,7 +3173,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>MTZ</t>
+          <t>POWL</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -3182,7 +3182,7 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>67</v>
+        <v>67.34999999999999</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
@@ -3201,16 +3201,16 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>RMBS</t>
+          <t>JCI</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Memory (HBM is the bottleneck)</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>66.92</v>
+        <v>67.25</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
@@ -3229,16 +3229,16 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>ONTO</t>
+          <t>NEE</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>66.72</v>
+        <v>67.08</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
@@ -3257,16 +3257,16 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>JCI</t>
+          <t>GEV</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>02 Grid Equipment</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>66.5</v>
+        <v>67</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
@@ -3285,16 +3285,16 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>HPE</t>
+          <t>MTZ</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>66.47</v>
+        <v>67</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
@@ -3313,16 +3313,16 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>MKSI</t>
+          <t>TSEM</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
+          <t>05 Fabs &amp; Foundries</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>66.45</v>
+        <v>66.7</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
@@ -3341,16 +3341,16 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>ADBE</t>
+          <t>ENTG</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / Creative &amp; design software</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>66.33</v>
+        <v>66.65000000000001</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
@@ -3369,16 +3369,16 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>CEG</t>
+          <t>ONTO</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>01 Power - IPP / Nuclear</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>66.28</v>
+        <v>66.55</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
@@ -3397,16 +3397,16 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>BESIY</t>
+          <t>TXN</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>06 AI Compute Silicon / Analog &amp; embedded (power management)</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>66.09999999999999</v>
+        <v>66.5</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
@@ -3425,16 +3425,16 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>TSEM</t>
+          <t>HPE</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>05 Fabs &amp; Foundries</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>66.09999999999999</v>
+        <v>66.47</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
@@ -3453,16 +3453,16 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>CCJ</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>01 Power - Distributed</t>
+          <t>01 Power Generation / Nuclear-specific</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>66.05</v>
+        <v>66.42</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
@@ -3481,16 +3481,16 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>SBGSY</t>
+          <t>RMBS</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>06 AI Compute Silicon / Memory (HBM is the bottleneck)</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>66</v>
+        <v>66.42</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
@@ -3509,16 +3509,16 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>SNPS</t>
+          <t>GNRC</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
+          <t>01 Power Generation / Distributed / on-site power</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>65.55</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
@@ -3537,16 +3537,16 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>TEL</t>
+          <t>MKSI</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>65.53</v>
+        <v>66.3</v>
       </c>
       <c r="D84" t="inlineStr">
         <is>
@@ -3565,16 +3565,16 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>GEV</t>
+          <t>AAON</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>02 Grid Equipment</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>65.5</v>
+        <v>66.27</v>
       </c>
       <c r="D85" t="inlineStr">
         <is>
@@ -3593,16 +3593,16 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>ENTG</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
+          <t>01 Power - Distributed</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>65.45</v>
+        <v>66.05</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
@@ -3621,16 +3621,16 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>UMC</t>
+          <t>HUBB</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>05 Fabs &amp; Foundries</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>65.34999999999999</v>
+        <v>65.88</v>
       </c>
       <c r="D87" t="inlineStr">
         <is>
@@ -3649,16 +3649,16 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>ORCL</t>
+          <t>PLAB</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>65.3</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="D88" t="inlineStr">
         <is>
@@ -3677,16 +3677,16 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>GNRC</t>
+          <t>SNPS</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>01 Power Generation / Distributed / on-site power</t>
+          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>65.2</v>
+        <v>65.55</v>
       </c>
       <c r="D89" t="inlineStr">
         <is>
@@ -3705,16 +3705,16 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>NXT</t>
+          <t>SNOW</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>01 Power Generation / Solar &amp; renewables equipment (behind-the-meter DC power)</t>
+          <t>10 Models, Software &amp; Applications</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>65.12</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="D90" t="inlineStr">
         <is>
@@ -3733,16 +3733,16 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>HUBB</t>
+          <t>HIVE</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>64.67</v>
+        <v>65.22</v>
       </c>
       <c r="D91" t="inlineStr">
         <is>
@@ -3761,16 +3761,16 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>MRVL</t>
+          <t>FLEX</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Contract manufacturing / ODMs</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>64.47</v>
+        <v>65</v>
       </c>
       <c r="D92" t="inlineStr">
         <is>
@@ -3789,16 +3789,16 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>ETN</t>
+          <t>NBIS</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>09 Compute-as-a-Service / Neoclouds (AI-native cloud providers)</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>64.3</v>
+        <v>64.90000000000001</v>
       </c>
       <c r="D93" t="inlineStr">
         <is>
@@ -3822,16 +3822,16 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>SMCI</t>
+          <t>MRVL</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling</t>
+          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>64.25</v>
+        <v>64.47</v>
       </c>
       <c r="D94" t="inlineStr">
         <is>
@@ -3850,16 +3850,16 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>LITE</t>
+          <t>ETN</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>64.17</v>
+        <v>64.3</v>
       </c>
       <c r="D95" t="inlineStr">
         <is>
@@ -3878,16 +3878,16 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>HIVE</t>
+          <t>SMCI</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>64.05</v>
+        <v>64.25</v>
       </c>
       <c r="D96" t="inlineStr">
         <is>
@@ -3906,16 +3906,16 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>IRM</t>
+          <t>ORCL</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>63.75</v>
+        <v>64.25</v>
       </c>
       <c r="D97" t="inlineStr">
         <is>
@@ -3934,16 +3934,16 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>SNOW</t>
+          <t>IRM</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>63.57</v>
+        <v>63.75</v>
       </c>
       <c r="D98" t="inlineStr">
         <is>
@@ -3962,16 +3962,16 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>CMI</t>
+          <t>KLIC</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>01 Power Generation / Distributed / on-site power</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>63.3</v>
+        <v>63.67</v>
       </c>
       <c r="D99" t="inlineStr">
         <is>
@@ -3990,16 +3990,16 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>KLIC</t>
+          <t>NXT</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>01 Power Generation / Solar &amp; renewables equipment (behind-the-meter DC power)</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>63.17</v>
+        <v>63.62</v>
       </c>
       <c r="D100" t="inlineStr">
         <is>
@@ -4018,16 +4018,16 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>FLEX</t>
+          <t>AAPL</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Contract manufacturing / ODMs</t>
+          <t>10 Models, Software &amp; Applications / Edge AI platforms</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>63.05</v>
+        <v>63.55</v>
       </c>
       <c r="D101" t="inlineStr">
         <is>
@@ -4046,16 +4046,16 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>KN</t>
+          <t>HUT</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>04 Semi Equip - Materials</t>
+          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>62.7</v>
+        <v>63.45</v>
       </c>
       <c r="D102" t="inlineStr">
         <is>
@@ -4074,16 +4074,16 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>CRWV</t>
+          <t>CMI</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>09 Cloud - Neocloud</t>
+          <t>01 Power Generation / Distributed / on-site power</t>
         </is>
       </c>
       <c r="C103" t="n">
-        <v>62.67</v>
+        <v>63.3</v>
       </c>
       <c r="D103" t="inlineStr">
         <is>
@@ -4102,16 +4102,16 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>SEI</t>
+          <t>KN</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>01 Power Generation / Distributed / on-site power</t>
+          <t>04 Semi Equip - Materials</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>62.55</v>
+        <v>63.05</v>
       </c>
       <c r="D104" t="inlineStr">
         <is>
@@ -4130,16 +4130,16 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>AAPL</t>
+          <t>SEI</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / Edge AI platforms</t>
+          <t>01 Power Generation / Distributed / on-site power</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>62.2</v>
+        <v>62.9</v>
       </c>
       <c r="D105" t="inlineStr">
         <is>
@@ -4158,16 +4158,16 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>NBIS</t>
+          <t>LITE</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Neoclouds (AI-native cloud providers)</t>
+          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>61.82</v>
+        <v>62.68</v>
       </c>
       <c r="D106" t="inlineStr">
         <is>
@@ -4186,16 +4186,16 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>CRWV</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
+          <t>09 Cloud - Neocloud</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>61.65</v>
+        <v>62.67</v>
       </c>
       <c r="D107" t="inlineStr">
         <is>
@@ -4214,12 +4214,12 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>CRWD</t>
+          <t>P</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -4242,16 +4242,16 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>BWXT</t>
+          <t>CRWD</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>01 Power Generation / Nuclear-specific</t>
+          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
         </is>
       </c>
       <c r="C109" t="n">
-        <v>61.58</v>
+        <v>61.65</v>
       </c>
       <c r="D109" t="inlineStr">
         <is>
@@ -4270,16 +4270,16 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>COHR</t>
+          <t>BWXT</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
+          <t>01 Power Generation / Nuclear-specific</t>
         </is>
       </c>
       <c r="C110" t="n">
-        <v>61.55</v>
+        <v>61.58</v>
       </c>
       <c r="D110" t="inlineStr">
         <is>
@@ -4298,16 +4298,16 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>NXPI</t>
+          <t>TTMI</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Analog &amp; embedded (auto/edge AI)</t>
+          <t>04 Semiconductor Equipment &amp; Materials / PCB / substrates</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>61.4</v>
+        <v>61.45</v>
       </c>
       <c r="D111" t="inlineStr">
         <is>
@@ -4326,16 +4326,16 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>MDB</t>
+          <t>EQIX</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI data layer</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>61.32</v>
+        <v>61</v>
       </c>
       <c r="D112" t="inlineStr">
         <is>
@@ -4354,16 +4354,16 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>HUT</t>
+          <t>COHR</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
+          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
         </is>
       </c>
       <c r="C113" t="n">
-        <v>61.2</v>
+        <v>60.8</v>
       </c>
       <c r="D113" t="inlineStr">
         <is>
@@ -4382,16 +4382,16 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>ATKR</t>
+          <t>NXPI</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>06 AI Compute Silicon / Analog &amp; embedded (auto/edge AI)</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>61.15</v>
+        <v>60.65</v>
       </c>
       <c r="D114" t="inlineStr">
         <is>
@@ -4410,16 +4410,16 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>EQIX</t>
+          <t>DUK</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>61</v>
+        <v>60.1</v>
       </c>
       <c r="D115" t="inlineStr">
         <is>
@@ -4447,7 +4447,7 @@
         </is>
       </c>
       <c r="C116" t="n">
-        <v>60.7</v>
+        <v>59.95</v>
       </c>
       <c r="D116" t="inlineStr">
         <is>
@@ -4466,16 +4466,16 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>TTMI</t>
+          <t>AEP</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / PCB / substrates</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>60.45</v>
+        <v>59.38</v>
       </c>
       <c r="D117" t="inlineStr">
         <is>
@@ -4494,16 +4494,16 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>DUK</t>
+          <t>CARR</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>60.1</v>
+        <v>59</v>
       </c>
       <c r="D118" t="inlineStr">
         <is>
@@ -4531,7 +4531,7 @@
         </is>
       </c>
       <c r="C119" t="n">
-        <v>59.1</v>
+        <v>58.73</v>
       </c>
       <c r="D119" t="inlineStr">
         <is>
@@ -4550,16 +4550,16 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>CARR</t>
+          <t>WYFI</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>09 Compute-as-a-Service / Neoclouds (AI-native cloud providers)</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>59</v>
+        <v>58.5</v>
       </c>
       <c r="D120" t="inlineStr">
         <is>
@@ -4578,16 +4578,16 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>QCOM</t>
+          <t>PPL</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Application processors &amp; connectivity (edge AI)</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>59</v>
+        <v>58.38</v>
       </c>
       <c r="D121" t="inlineStr">
         <is>
@@ -4606,16 +4606,16 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>AEP</t>
+          <t>ATKR</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>58.77</v>
+        <v>58.15</v>
       </c>
       <c r="D122" t="inlineStr">
         <is>
@@ -4634,16 +4634,16 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>TEM</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Power management silicon (SiC/GaN)</t>
+          <t>10 Models, Software &amp; Applications / AI-native vertical applications</t>
         </is>
       </c>
       <c r="C123" t="n">
-        <v>58.52</v>
+        <v>58</v>
       </c>
       <c r="D123" t="inlineStr">
         <is>
@@ -4662,16 +4662,16 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>PPL</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>06 AI Compute Silicon / Power management silicon (SiC/GaN)</t>
         </is>
       </c>
       <c r="C124" t="n">
-        <v>58.38</v>
+        <v>57.77</v>
       </c>
       <c r="D124" t="inlineStr">
         <is>
@@ -4690,16 +4690,16 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>TEM</t>
+          <t>QCOM</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI-native vertical applications</t>
+          <t>06 AI Compute Silicon / Application processors &amp; connectivity (edge AI)</t>
         </is>
       </c>
       <c r="C125" t="n">
-        <v>58</v>
+        <v>57.5</v>
       </c>
       <c r="D125" t="inlineStr">
         <is>
@@ -4718,16 +4718,16 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>IREN</t>
+          <t>APLD</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
+          <t>09 Compute-as-a-Service / Neoclouds (AI-native cloud providers)</t>
         </is>
       </c>
       <c r="C126" t="n">
-        <v>57.12</v>
+        <v>57.48</v>
       </c>
       <c r="D126" t="inlineStr">
         <is>
@@ -4746,16 +4746,16 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>XEL</t>
+          <t>MDB</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>10 Models, Software &amp; Applications / AI data layer</t>
         </is>
       </c>
       <c r="C127" t="n">
-        <v>57.05</v>
+        <v>57.45</v>
       </c>
       <c r="D127" t="inlineStr">
         <is>
@@ -4774,16 +4774,16 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>WYFI</t>
+          <t>ETR</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Neoclouds (AI-native cloud providers)</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C128" t="n">
-        <v>56.88</v>
+        <v>57.35</v>
       </c>
       <c r="D128" t="inlineStr">
         <is>
@@ -4802,16 +4802,16 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>PSIX</t>
+          <t>IREN</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>01 Power Generation / Distributed / on-site power</t>
+          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
         </is>
       </c>
       <c r="C129" t="n">
-        <v>56.35</v>
+        <v>57.25</v>
       </c>
       <c r="D129" t="inlineStr">
         <is>
@@ -4830,7 +4830,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>ETR</t>
+          <t>XEL</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -4839,7 +4839,7 @@
         </is>
       </c>
       <c r="C130" t="n">
-        <v>56.15</v>
+        <v>57.05</v>
       </c>
       <c r="D130" t="inlineStr">
         <is>
@@ -4858,16 +4858,16 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>SO</t>
+          <t>UCTT</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
         </is>
       </c>
       <c r="C131" t="n">
-        <v>55.33</v>
+        <v>55.88</v>
       </c>
       <c r="D131" t="inlineStr">
         <is>
@@ -4886,20 +4886,20 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>APLD</t>
+          <t>WULF</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Neoclouds (AI-native cloud providers)</t>
+          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
         </is>
       </c>
       <c r="C132" t="n">
-        <v>54.73</v>
+        <v>55.77</v>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="E132" t="n">
@@ -4914,20 +4914,20 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>WULF</t>
+          <t>PSIX</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
+          <t>01 Power Generation / Distributed / on-site power</t>
         </is>
       </c>
       <c r="C133" t="n">
-        <v>52.94</v>
+        <v>55.6</v>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="E133" t="n">
@@ -4942,20 +4942,20 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>UCTT</t>
+          <t>SO</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C134" t="n">
-        <v>51.62</v>
+        <v>55.33</v>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="E134" t="n">

</xml_diff>

<commit_message>
Weekly scan 2026-06-26: MU Q3 earnings ✓✓→✓✓✓, RDDT gate cleared, WDC EXIT confirmed
MU: score 79.35→86.40 (✓✓✓) on Q3 FY26 beat ($41.5B rev, 84.9% GM, 16 take-or-pay SCAs). RDDT thesis written, gate cleared (79.4, first-in-line for WDC slot). WDC EXIT confirmed (71.6, no SNDK data distortion). PLTR documented as 2nd-in-line at 76.4.
</commit_message>
<xml_diff>
--- a/00-master/portfolio.xlsx
+++ b/00-master/portfolio.xlsx
@@ -1041,7 +1041,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J134"/>
+  <dimension ref="A1:K134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1058,7 +1058,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Target Portfolio (refreshed 2026-06-24, live Watchlist scores)</t>
+          <t>Target Portfolio (refreshed 2026-06-26, live Watchlist scores)</t>
         </is>
       </c>
     </row>
@@ -1316,11 +1316,11 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>79.34999999999999</v>
+        <v>86.40000000000001</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>✓✓</t>
+          <t>✓✓✓</t>
         </is>
       </c>
       <c r="E8" t="n">

</xml_diff>

<commit_message>
data: corrective rebalance — MU/TSM to ✓✓✓ top weights (10.3%), +RDDT +PLTR -WDC
Forced --resize re-weight on the live workbook fixes the MU inversion (✓✓✓
86.4 was 7.4%, below NVDA ✓✓ at 9.3%); MU/TSM now lead at 10.32%, weights
monotonic in score. Reconciles drift since 2026-06-18: WDC (71.6 < exit) exits,
RDDT (79.4) + PLTR (76.4) enter (Dom-approved full rebalance). New 2026-06-29
model event stores tiers as the crossing baseline; series rebuilt to as_of
2026-06-29. Adds the score-monotonicity data gate.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/00-master/portfolio.xlsx
+++ b/00-master/portfolio.xlsx
@@ -480,6 +480,8 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
@@ -492,6 +494,7 @@
         </is>
       </c>
     </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
@@ -547,6 +550,7 @@
         </is>
       </c>
     </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
@@ -614,6 +618,7 @@
         </is>
       </c>
     </row>
+    <row r="18"/>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
         <is>
@@ -649,6 +654,7 @@
         </is>
       </c>
     </row>
+    <row r="24"/>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
         <is>
@@ -661,6 +667,7 @@
         </is>
       </c>
     </row>
+    <row r="26"/>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
         <is>
@@ -669,7 +676,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-06-19 (refresh_targets.py — hysteresis pipeline)</t>
+          <t>2026-06-29 (refresh_targets.py — hysteresis pipeline)</t>
         </is>
       </c>
     </row>
@@ -701,6 +708,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
         <is>
@@ -763,6 +771,7 @@
         </is>
       </c>
     </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
@@ -892,6 +901,7 @@
         <v>40</v>
       </c>
     </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
@@ -1041,7 +1051,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K134"/>
+  <dimension ref="A1:J138"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1058,7 +1068,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Target Portfolio (refreshed 2026-06-26, live Watchlist scores)</t>
+          <t>Target Portfolio (refreshed 2026-06-29, live Watchlist scores)</t>
         </is>
       </c>
     </row>
@@ -1146,27 +1156,29 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="H3" t="inlineStr"/>
       <c r="I3" t="n">
-        <v>9.6</v>
-      </c>
+        <v>10.32</v>
+      </c>
+      <c r="J3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>NVDA</t>
+          <t>MU</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / GPUs / merchant accelerators</t>
+          <t>06 Silicon - Memory</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>84.08</v>
+        <v>86.40000000000001</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>✓✓</t>
+          <t>✓✓✓</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -1182,23 +1194,25 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="H4" t="inlineStr"/>
       <c r="I4" t="n">
-        <v>9.32</v>
-      </c>
+        <v>10.32</v>
+      </c>
+      <c r="J4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SNDK</t>
+          <t>NVDA</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Memory (HBM is the bottleneck)</t>
+          <t>06 AI Compute Silicon / GPUs / merchant accelerators</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>80.09999999999999</v>
+        <v>84.08</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -1218,28 +1232,25 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="H5" t="inlineStr"/>
       <c r="I5" t="n">
-        <v>7.51</v>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>Manually excluded 2026-05-18: $1,333 share price prevents capital-efficient sizing below ~$25k. Conscious framework override (target ~$10k portfolio). | Override removed 2026-06-09: fractional shares adopted, share-price constraint obsolete (Dom decision).</t>
-        </is>
-      </c>
+        <v>8.23</v>
+      </c>
+      <c r="J5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CRDO</t>
+          <t>SNDK</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Connectivity ASICs</t>
+          <t>06 AI Compute Silicon / Memory (HBM is the bottleneck)</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>80</v>
+        <v>80.09999999999999</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -1259,28 +1270,29 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="H6" t="inlineStr"/>
       <c r="I6" t="n">
-        <v>7.47</v>
+        <v>6.63</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Added 2026-05-25: score 78.4, ranked #4 in reweighted watchlist. Optical connectivity pure-play.</t>
+          <t>Manually excluded 2026-05-18: $1,333 share price prevents capital-efficient sizing below ~$25k. Conscious framework override (target ~$10k portfolio). | Override removed 2026-06-09: fractional shares adopted, share-price constraint obsolete (Dom decision).</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>META</t>
+          <t>CRDO</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
+          <t>07 Optical, Networking &amp; Interconnect / Connectivity ASICs</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>79.5</v>
+        <v>80</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -1300,27 +1312,33 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="H7" t="inlineStr"/>
       <c r="I7" t="n">
-        <v>6.97</v>
+        <v>6.59</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Added 2026-05-25: score 78.4, ranked #4 in reweighted watchlist. Optical connectivity pure-play.</t>
+        </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>MU</t>
+          <t>META</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>06 Silicon - Memory</t>
+          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>86.40000000000001</v>
+        <v>79.5</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>✓✓✓</t>
+          <t>✓✓</t>
         </is>
       </c>
       <c r="E8" t="n">
@@ -1336,23 +1354,25 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="H8" t="inlineStr"/>
       <c r="I8" t="n">
-        <v>7.44</v>
-      </c>
+        <v>6.39</v>
+      </c>
+      <c r="J8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>AVGO</t>
+          <t>RDDT</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
+          <t>10 Models, Software &amp; Applications / AI advertising</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>79.2</v>
+        <v>79.40000000000001</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -1364,7 +1384,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>HOLD</t>
+          <t>ENTER (score 79.4)</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1372,23 +1392,25 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="H9" t="inlineStr"/>
       <c r="I9" t="n">
-        <v>7.1</v>
-      </c>
+        <v>6.35</v>
+      </c>
+      <c r="J9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ANET</t>
+          <t>AVGO</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
+          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>78.48</v>
+        <v>79.2</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -1408,23 +1430,25 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="H10" t="inlineStr"/>
       <c r="I10" t="n">
-        <v>6.77</v>
-      </c>
+        <v>6.27</v>
+      </c>
+      <c r="J10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>ANET</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
+          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>78.40000000000001</v>
+        <v>78.48</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -1444,14 +1468,16 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="H11" t="inlineStr"/>
       <c r="I11" t="n">
-        <v>6.19</v>
-      </c>
+        <v>5.98</v>
+      </c>
+      <c r="J11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1460,7 +1486,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>78.03</v>
+        <v>78.40000000000001</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -1480,23 +1506,25 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="H12" t="inlineStr"/>
       <c r="I12" t="n">
-        <v>6.02</v>
-      </c>
+        <v>5.95</v>
+      </c>
+      <c r="J12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ALAB</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
+          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>77.08</v>
+        <v>78.03</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -1516,23 +1544,25 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="H13" t="inlineStr"/>
       <c r="I13" t="n">
-        <v>6.14</v>
-      </c>
+        <v>5.8</v>
+      </c>
+      <c r="J13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>APP</t>
+          <t>ALAB</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI advertising</t>
+          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>76.90000000000001</v>
+        <v>77.08</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -1552,23 +1582,25 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="H14" t="inlineStr"/>
       <c r="I14" t="n">
-        <v>6.97</v>
-      </c>
+        <v>5.42</v>
+      </c>
+      <c r="J14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>FIX</t>
+          <t>APP</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>10 Models, Software &amp; Applications / AI advertising</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>76.65000000000001</v>
+        <v>76.90000000000001</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -1588,28 +1620,25 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="H15" t="inlineStr"/>
       <c r="I15" t="n">
-        <v>5.94</v>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>Manually excluded 2026-05-18: $1,854 share price prevents reasonable position sizing below ~$50k portfolio. Conscious framework override. | Override removed 2026-06-09: fractional shares adopted, share-price constraint obsolete (Dom decision).</t>
-        </is>
-      </c>
+        <v>5.35</v>
+      </c>
+      <c r="J15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>PLTR</t>
+          <t>FIX</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>76.40000000000001</v>
+        <v>76.65000000000001</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -1619,25 +1648,39 @@
       <c r="E16" t="n">
         <v>14</v>
       </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Manually excluded 2026-05-18: $1,854 share price prevents reasonable position sizing below ~$50k portfolio. Conscious framework override. | Override removed 2026-06-09: fractional shares adopted, share-price constraint obsolete (Dom decision).</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ZS</t>
+          <t>PLTR</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
+          <t>10 Models, Software &amp; Applications</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>75.47</v>
+        <v>76.40000000000001</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -1647,25 +1690,35 @@
       <c r="E17" t="n">
         <v>15</v>
       </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>ENTER (score 76.4)</t>
+        </is>
+      </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="n">
+        <v>5.15</v>
+      </c>
+      <c r="J17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>VRT</t>
+          <t>ZS</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>03 DC Infrastructure</t>
+          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>75.3</v>
+        <v>75.47</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -1675,25 +1728,28 @@
       <c r="E18" t="n">
         <v>16</v>
       </c>
+      <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>EME</t>
+          <t>VRT</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>03 DC Infrastructure</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>74.75</v>
+        <v>75.3</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -1703,30 +1759,28 @@
       <c r="E19" t="n">
         <v>17</v>
       </c>
+      <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>Added 2026-05-25: score 75.2, DC construction, strong momentum (86.7).</t>
-        </is>
-      </c>
+      <c r="H19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>WDAY</t>
+          <t>EME</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / Enterprise SaaS</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>74.7</v>
+        <v>74.75</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -1736,25 +1790,32 @@
       <c r="E20" t="n">
         <v>18</v>
       </c>
+      <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
           <t>N</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr"/>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Added 2026-05-25: score 75.2, DC construction, strong momentum (86.7).</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>EQT</t>
+          <t>WDAY</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
+          <t>10 Models, Software &amp; Applications / Enterprise SaaS</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>74.65000000000001</v>
+        <v>74.7</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -1764,25 +1825,28 @@
       <c r="E21" t="n">
         <v>19</v>
       </c>
+      <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>EQT</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / GPUs / merchant accelerators</t>
+          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>74.58</v>
+        <v>74.65000000000001</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -1792,30 +1856,28 @@
       <c r="E22" t="n">
         <v>20</v>
       </c>
+      <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>Removed 2026-05-25: score 74.1 fell below natural 17-name cutoff (ARM 74.2). First name out.</t>
-        </is>
-      </c>
+      <c r="H22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>ADSK</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / Design &amp; engineering software</t>
+          <t>06 AI Compute Silicon / GPUs / merchant accelerators</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>74.25</v>
+        <v>74.58</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -1825,25 +1887,32 @@
       <c r="E23" t="n">
         <v>21</v>
       </c>
+      <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
           <t>N</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr"/>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Removed 2026-05-25: score 74.1 fell below natural 17-name cutoff (ARM 74.2). First name out.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>ADSK</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
+          <t>10 Models, Software &amp; Applications / Design &amp; engineering software</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>74.08</v>
+        <v>74.25</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -1853,30 +1922,28 @@
       <c r="E24" t="n">
         <v>22</v>
       </c>
+      <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>Added 2026-05-22 as substitute for CTRA (delisted). Pure score-driven pick: next-best ✓✓ at 75.62, same Layer 1 NG E&amp;P sub-category — preserves natural gas thesis concentration.</t>
-        </is>
-      </c>
+      <c r="H24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>AR</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
+          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>73.3</v>
+        <v>74.08</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -1886,25 +1953,32 @@
       <c r="E25" t="n">
         <v>23</v>
       </c>
+      <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
           <t>N</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr"/>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Added 2026-05-22 as substitute for CTRA (delisted). Pure score-driven pick: next-best ✓✓ at 75.62, same Layer 1 NG E&amp;P sub-category — preserves natural gas thesis concentration.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>KEYS</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
+          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>73.22</v>
+        <v>73.3</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -1914,25 +1988,28 @@
       <c r="E26" t="n">
         <v>24</v>
       </c>
+      <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H26" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>TER</t>
+          <t>KEYS</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>73.05</v>
+        <v>73.22</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -1942,25 +2019,28 @@
       <c r="E27" t="n">
         <v>25</v>
       </c>
+      <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>TER</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>72.8</v>
+        <v>73.05</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -1970,30 +2050,28 @@
       <c r="E28" t="n">
         <v>26</v>
       </c>
+      <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr">
-        <is>
-          <t>Added 2026-05-25: score 74.8, Quality 97, PEG 0.8. Enterprise SaaS with AI exposure.</t>
-        </is>
-      </c>
+      <c r="H28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>STX</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
+          <t>10 Models, Software &amp; Applications</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>72.75</v>
+        <v>72.8</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -2003,9 +2081,16 @@
       <c r="E29" t="n">
         <v>27</v>
       </c>
+      <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr">
         <is>
           <t>N</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr"/>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>Added 2026-05-25: score 74.8, Quality 97, PEG 0.8. Enterprise SaaS with AI exposure.</t>
         </is>
       </c>
     </row>
@@ -2031,25 +2116,28 @@
       <c r="E30" t="n">
         <v>28</v>
       </c>
+      <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>PANW</t>
+          <t>STX</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>72.65000000000001</v>
+        <v>72.75</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -2059,25 +2147,28 @@
       <c r="E31" t="n">
         <v>29</v>
       </c>
+      <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H31" t="inlineStr"/>
+      <c r="J31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>HTHIY</t>
+          <t>PANW</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>72.05</v>
+        <v>72.65000000000001</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -2087,25 +2178,28 @@
       <c r="E32" t="n">
         <v>30</v>
       </c>
+      <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H32" t="inlineStr"/>
+      <c r="J32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>LSCC</t>
+          <t>HTHIY</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Programmable logic</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>71.98</v>
+        <v>72.05</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -2115,25 +2209,28 @@
       <c r="E33" t="n">
         <v>31</v>
       </c>
+      <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H33" t="inlineStr"/>
+      <c r="J33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>WDC</t>
+          <t>LSCC</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
+          <t>06 AI Compute Silicon / Programmable logic</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>71.62</v>
+        <v>71.98</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -2143,33 +2240,28 @@
       <c r="E34" t="n">
         <v>32</v>
       </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>HOLD</t>
-        </is>
-      </c>
+      <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I34" t="n">
-        <v>6.56</v>
-      </c>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr"/>
+      <c r="J34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>DELL</t>
+          <t>WDC</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>71.59999999999999</v>
+        <v>71.62</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
@@ -2179,11 +2271,18 @@
       <c r="E35" t="n">
         <v>33</v>
       </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>EXIT (resize, score 71.6 &lt; 74.5)</t>
+        </is>
+      </c>
       <c r="G35" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H35" t="inlineStr"/>
+      <c r="J35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2207,25 +2306,28 @@
       <c r="E36" t="n">
         <v>34</v>
       </c>
+      <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H36" t="inlineStr"/>
+      <c r="J36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>CIEN</t>
+          <t>DELL</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>71.45</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
@@ -2235,25 +2337,28 @@
       <c r="E37" t="n">
         <v>35</v>
       </c>
+      <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H37" t="inlineStr"/>
+      <c r="J37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>EXE</t>
+          <t>CIEN</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
+          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>71.22</v>
+        <v>71.45</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -2263,25 +2368,28 @@
       <c r="E38" t="n">
         <v>36</v>
       </c>
+      <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H38" t="inlineStr"/>
+      <c r="J38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>ARM</t>
+          <t>EXE</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
+          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>71.15000000000001</v>
+        <v>71.22</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -2291,25 +2399,28 @@
       <c r="E39" t="n">
         <v>37</v>
       </c>
+      <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H39" t="inlineStr"/>
+      <c r="J39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>VST</t>
+          <t>ARM</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>01 Power Generation / Independent Power Producers (IPPs)</t>
+          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>71.05</v>
+        <v>71.15000000000001</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -2319,25 +2430,28 @@
       <c r="E40" t="n">
         <v>38</v>
       </c>
+      <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H40" t="inlineStr"/>
+      <c r="J40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>DDOG</t>
+          <t>VST</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI observability &amp; infrastructure software</t>
+          <t>01 Power Generation / Independent Power Producers (IPPs)</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>71</v>
+        <v>71.05</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -2347,30 +2461,28 @@
       <c r="E41" t="n">
         <v>39</v>
       </c>
+      <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="J41" t="inlineStr">
-        <is>
-          <t>Added 2026-05-25: score 75.4, Quality 100, PEG 0.7. Beats 4 existing portfolio names.</t>
-        </is>
-      </c>
+      <c r="H41" t="inlineStr"/>
+      <c r="J41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>APH</t>
+          <t>DDOG</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
+          <t>10 Models, Software &amp; Applications / AI observability &amp; infrastructure software</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>70.92</v>
+        <v>71</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
@@ -2380,25 +2492,32 @@
       <c r="E42" t="n">
         <v>40</v>
       </c>
+      <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr">
         <is>
           <t>N</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr"/>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>Added 2026-05-25: score 75.4, Quality 100, PEG 0.7. Beats 4 existing portfolio names.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>FN</t>
+          <t>APH</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
+          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>70.09999999999999</v>
+        <v>70.92</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
@@ -2408,49 +2527,55 @@
       <c r="E43" t="n">
         <v>41</v>
       </c>
+      <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H43" t="inlineStr"/>
+      <c r="J43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>PWR</t>
+          <t>FN</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>69.95</v>
+        <v>70.09999999999999</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>✓✓</t>
         </is>
       </c>
       <c r="E44" t="n">
         <v>42</v>
       </c>
+      <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H44" t="inlineStr"/>
+      <c r="J44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>ASML</t>
+          <t>PWR</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -2464,25 +2589,28 @@
       <c r="E45" t="n">
         <v>43</v>
       </c>
+      <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H45" t="inlineStr"/>
+      <c r="J45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>PATH</t>
+          <t>ASML</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI-powered automation</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>69.90000000000001</v>
+        <v>69.95</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -2492,25 +2620,28 @@
       <c r="E46" t="n">
         <v>44</v>
       </c>
+      <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H46" t="inlineStr"/>
+      <c r="J46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>MOD</t>
+          <t>PATH</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>10 Models, Software &amp; Applications / AI-powered automation</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>69.7</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -2520,25 +2651,28 @@
       <c r="E47" t="n">
         <v>45</v>
       </c>
+      <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H47" t="inlineStr"/>
+      <c r="J47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>LRCX</t>
+          <t>MOD</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>69.45</v>
+        <v>69.7</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -2548,21 +2682,24 @@
       <c r="E48" t="n">
         <v>46</v>
       </c>
+      <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H48" t="inlineStr"/>
+      <c r="J48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>NOW</t>
+          <t>LRCX</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -2576,25 +2713,28 @@
       <c r="E49" t="n">
         <v>47</v>
       </c>
+      <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H49" t="inlineStr"/>
+      <c r="J49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>ADI</t>
+          <t>NOW</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Analog &amp; mixed-signal (signal chain + power)</t>
+          <t>10 Models, Software &amp; Applications</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>69.40000000000001</v>
+        <v>69.45</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
@@ -2604,11 +2744,14 @@
       <c r="E50" t="n">
         <v>48</v>
       </c>
+      <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H50" t="inlineStr"/>
+      <c r="J50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2632,25 +2775,28 @@
       <c r="E51" t="n">
         <v>49</v>
       </c>
+      <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H51" t="inlineStr"/>
+      <c r="J51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>GLW</t>
+          <t>ADI</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
+          <t>06 AI Compute Silicon / Analog &amp; mixed-signal (signal chain + power)</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>69.25</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
@@ -2660,25 +2806,28 @@
       <c r="E52" t="n">
         <v>50</v>
       </c>
+      <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H52" t="inlineStr"/>
+      <c r="J52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>ABBNY</t>
+          <t>GLW</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>69</v>
+        <v>69.25</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
@@ -2688,25 +2837,28 @@
       <c r="E53" t="n">
         <v>51</v>
       </c>
+      <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H53" t="inlineStr"/>
+      <c r="J53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>CCJ</t>
+          <t>ABBNY</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>01 Power Generation / Nuclear-specific</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>68.92</v>
+        <v>69</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
@@ -2716,25 +2868,28 @@
       <c r="E54" t="n">
         <v>52</v>
       </c>
+      <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H54" t="inlineStr"/>
+      <c r="J54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>INTU</t>
+          <t>CCJ</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / Financial software</t>
+          <t>01 Power Generation / Nuclear-specific</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>68.63</v>
+        <v>68.92</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
@@ -2744,25 +2899,28 @@
       <c r="E55" t="n">
         <v>53</v>
       </c>
+      <c r="F55" t="inlineStr"/>
       <c r="G55" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H55" t="inlineStr"/>
+      <c r="J55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>KLAC</t>
+          <t>INTU</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>10 Models, Software &amp; Applications / Financial software</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>68.5</v>
+        <v>68.63</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
@@ -2772,25 +2930,28 @@
       <c r="E56" t="n">
         <v>54</v>
       </c>
+      <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H56" t="inlineStr"/>
+      <c r="J56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>CDNS</t>
+          <t>KLAC</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>68.45</v>
+        <v>68.5</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
@@ -2800,25 +2961,28 @@
       <c r="E57" t="n">
         <v>55</v>
       </c>
+      <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H57" t="inlineStr"/>
+      <c r="J57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>FTNT</t>
+          <t>CDNS</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
+          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>68.25</v>
+        <v>68.45</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
@@ -2828,25 +2992,28 @@
       <c r="E58" t="n">
         <v>56</v>
       </c>
+      <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H58" t="inlineStr"/>
+      <c r="J58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>NVT</t>
+          <t>FTNT</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>68.15000000000001</v>
+        <v>68.25</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
@@ -2856,25 +3023,28 @@
       <c r="E59" t="n">
         <v>57</v>
       </c>
+      <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H59" t="inlineStr"/>
+      <c r="J59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>TLN</t>
+          <t>NVT</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>01 Power Generation / Independent Power Producers (IPPs)</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>68.08</v>
+        <v>68.15000000000001</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
@@ -2884,25 +3054,28 @@
       <c r="E60" t="n">
         <v>58</v>
       </c>
+      <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H60" t="inlineStr"/>
+      <c r="J60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>CSCO</t>
+          <t>TLN</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
+          <t>01 Power Generation / Independent Power Producers (IPPs)</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>68</v>
+        <v>68.08</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
@@ -2912,25 +3085,28 @@
       <c r="E61" t="n">
         <v>59</v>
       </c>
+      <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H61" t="inlineStr"/>
+      <c r="J61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>FORM</t>
+          <t>CSCO</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
+          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>67.92</v>
+        <v>68</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
@@ -2940,25 +3116,28 @@
       <c r="E62" t="n">
         <v>60</v>
       </c>
+      <c r="F62" t="inlineStr"/>
       <c r="G62" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H62" t="inlineStr"/>
+      <c r="J62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>TT</t>
+          <t>FORM</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>67.83</v>
+        <v>67.92</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
@@ -2968,16 +3147,19 @@
       <c r="E63" t="n">
         <v>61</v>
       </c>
+      <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H63" t="inlineStr"/>
+      <c r="J63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>DLR</t>
+          <t>TT</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -2986,7 +3168,7 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>67.8</v>
+        <v>67.83</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
@@ -2996,25 +3178,28 @@
       <c r="E64" t="n">
         <v>62</v>
       </c>
+      <c r="F64" t="inlineStr"/>
       <c r="G64" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H64" t="inlineStr"/>
+      <c r="J64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>AEIS</t>
+          <t>DLR</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>67.72</v>
+        <v>67.8</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
@@ -3024,25 +3209,28 @@
       <c r="E65" t="n">
         <v>63</v>
       </c>
+      <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H65" t="inlineStr"/>
+      <c r="J65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>NEE</t>
+          <t>AEIS</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>67.67</v>
+        <v>67.72</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
@@ -3052,25 +3240,28 @@
       <c r="E66" t="n">
         <v>64</v>
       </c>
+      <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H66" t="inlineStr"/>
+      <c r="J66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>POWL</t>
+          <t>NEE</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>67.34999999999999</v>
+        <v>67.67</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
@@ -3080,25 +3271,28 @@
       <c r="E67" t="n">
         <v>65</v>
       </c>
+      <c r="F67" t="inlineStr"/>
       <c r="G67" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H67" t="inlineStr"/>
+      <c r="J67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>AAON</t>
+          <t>POWL</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>67.25</v>
+        <v>67.34999999999999</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
@@ -3108,25 +3302,28 @@
       <c r="E68" t="n">
         <v>66</v>
       </c>
+      <c r="F68" t="inlineStr"/>
       <c r="G68" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H68" t="inlineStr"/>
+      <c r="J68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>TXN</t>
+          <t>AAON</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Analog &amp; embedded (power management)</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>67.09999999999999</v>
+        <v>67.25</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
@@ -3136,25 +3333,28 @@
       <c r="E69" t="n">
         <v>67</v>
       </c>
+      <c r="F69" t="inlineStr"/>
       <c r="G69" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H69" t="inlineStr"/>
+      <c r="J69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>AMAT</t>
+          <t>TXN</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>06 AI Compute Silicon / Analog &amp; embedded (power management)</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>67.05</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
@@ -3164,25 +3364,28 @@
       <c r="E70" t="n">
         <v>68</v>
       </c>
+      <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H70" t="inlineStr"/>
+      <c r="J70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>MTZ</t>
+          <t>AMAT</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>67</v>
+        <v>67.05</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
@@ -3192,25 +3395,28 @@
       <c r="E71" t="n">
         <v>69</v>
       </c>
+      <c r="F71" t="inlineStr"/>
       <c r="G71" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H71" t="inlineStr"/>
+      <c r="J71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>RMBS</t>
+          <t>MTZ</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Memory (HBM is the bottleneck)</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>66.92</v>
+        <v>67</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
@@ -3220,25 +3426,28 @@
       <c r="E72" t="n">
         <v>70</v>
       </c>
+      <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H72" t="inlineStr"/>
+      <c r="J72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>ONTO</t>
+          <t>RMBS</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>06 AI Compute Silicon / Memory (HBM is the bottleneck)</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>66.72</v>
+        <v>66.92</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
@@ -3248,25 +3457,28 @@
       <c r="E73" t="n">
         <v>71</v>
       </c>
+      <c r="F73" t="inlineStr"/>
       <c r="G73" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H73" t="inlineStr"/>
+      <c r="J73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>JCI</t>
+          <t>ONTO</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>66.5</v>
+        <v>66.72</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
@@ -3276,25 +3488,28 @@
       <c r="E74" t="n">
         <v>72</v>
       </c>
+      <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H74" t="inlineStr"/>
+      <c r="J74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>HPE</t>
+          <t>JCI</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>66.47</v>
+        <v>66.5</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
@@ -3304,25 +3519,28 @@
       <c r="E75" t="n">
         <v>73</v>
       </c>
+      <c r="F75" t="inlineStr"/>
       <c r="G75" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H75" t="inlineStr"/>
+      <c r="J75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>MKSI</t>
+          <t>HPE</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>66.45</v>
+        <v>66.47</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
@@ -3332,25 +3550,28 @@
       <c r="E76" t="n">
         <v>74</v>
       </c>
+      <c r="F76" t="inlineStr"/>
       <c r="G76" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H76" t="inlineStr"/>
+      <c r="J76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>ADBE</t>
+          <t>MKSI</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / Creative &amp; design software</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>66.33</v>
+        <v>66.45</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
@@ -3360,25 +3581,28 @@
       <c r="E77" t="n">
         <v>75</v>
       </c>
+      <c r="F77" t="inlineStr"/>
       <c r="G77" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H77" t="inlineStr"/>
+      <c r="J77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>CEG</t>
+          <t>ADBE</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>01 Power - IPP / Nuclear</t>
+          <t>10 Models, Software &amp; Applications / Creative &amp; design software</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>66.28</v>
+        <v>66.33</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
@@ -3388,25 +3612,28 @@
       <c r="E78" t="n">
         <v>76</v>
       </c>
+      <c r="F78" t="inlineStr"/>
       <c r="G78" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H78" t="inlineStr"/>
+      <c r="J78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>BESIY</t>
+          <t>CEG</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>01 Power - IPP / Nuclear</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>66.09999999999999</v>
+        <v>66.28</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
@@ -3416,11 +3643,14 @@
       <c r="E79" t="n">
         <v>77</v>
       </c>
+      <c r="F79" t="inlineStr"/>
       <c r="G79" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H79" t="inlineStr"/>
+      <c r="J79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -3444,25 +3674,28 @@
       <c r="E80" t="n">
         <v>78</v>
       </c>
+      <c r="F80" t="inlineStr"/>
       <c r="G80" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H80" t="inlineStr"/>
+      <c r="J80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>BESIY</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>01 Power - Distributed</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>66.05</v>
+        <v>66.09999999999999</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
@@ -3472,25 +3705,28 @@
       <c r="E81" t="n">
         <v>79</v>
       </c>
+      <c r="F81" t="inlineStr"/>
       <c r="G81" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H81" t="inlineStr"/>
+      <c r="J81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>SBGSY</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>01 Power - Distributed</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>66</v>
+        <v>66.05</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
@@ -3500,25 +3736,28 @@
       <c r="E82" t="n">
         <v>80</v>
       </c>
+      <c r="F82" t="inlineStr"/>
       <c r="G82" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H82" t="inlineStr"/>
+      <c r="J82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>SNPS</t>
+          <t>SBGSY</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>65.55</v>
+        <v>66</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
@@ -3528,25 +3767,28 @@
       <c r="E83" t="n">
         <v>81</v>
       </c>
+      <c r="F83" t="inlineStr"/>
       <c r="G83" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H83" t="inlineStr"/>
+      <c r="J83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>TEL</t>
+          <t>SNPS</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
+          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>65.53</v>
+        <v>65.55</v>
       </c>
       <c r="D84" t="inlineStr">
         <is>
@@ -3556,25 +3798,28 @@
       <c r="E84" t="n">
         <v>82</v>
       </c>
+      <c r="F84" t="inlineStr"/>
       <c r="G84" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H84" t="inlineStr"/>
+      <c r="J84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>GEV</t>
+          <t>TEL</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>02 Grid Equipment</t>
+          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>65.5</v>
+        <v>65.53</v>
       </c>
       <c r="D85" t="inlineStr">
         <is>
@@ -3584,25 +3829,28 @@
       <c r="E85" t="n">
         <v>83</v>
       </c>
+      <c r="F85" t="inlineStr"/>
       <c r="G85" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H85" t="inlineStr"/>
+      <c r="J85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>ENTG</t>
+          <t>GEV</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
+          <t>02 Grid Equipment</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>65.45</v>
+        <v>65.5</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
@@ -3612,25 +3860,28 @@
       <c r="E86" t="n">
         <v>84</v>
       </c>
+      <c r="F86" t="inlineStr"/>
       <c r="G86" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H86" t="inlineStr"/>
+      <c r="J86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>UMC</t>
+          <t>ENTG</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>05 Fabs &amp; Foundries</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>65.34999999999999</v>
+        <v>65.45</v>
       </c>
       <c r="D87" t="inlineStr">
         <is>
@@ -3640,25 +3891,28 @@
       <c r="E87" t="n">
         <v>85</v>
       </c>
+      <c r="F87" t="inlineStr"/>
       <c r="G87" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H87" t="inlineStr"/>
+      <c r="J87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>ORCL</t>
+          <t>UMC</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
+          <t>05 Fabs &amp; Foundries</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>65.3</v>
+        <v>65.34999999999999</v>
       </c>
       <c r="D88" t="inlineStr">
         <is>
@@ -3668,25 +3922,28 @@
       <c r="E88" t="n">
         <v>86</v>
       </c>
+      <c r="F88" t="inlineStr"/>
       <c r="G88" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H88" t="inlineStr"/>
+      <c r="J88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>GNRC</t>
+          <t>ORCL</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>01 Power Generation / Distributed / on-site power</t>
+          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>65.2</v>
+        <v>65.3</v>
       </c>
       <c r="D89" t="inlineStr">
         <is>
@@ -3696,25 +3953,28 @@
       <c r="E89" t="n">
         <v>87</v>
       </c>
+      <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H89" t="inlineStr"/>
+      <c r="J89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>NXT</t>
+          <t>GNRC</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>01 Power Generation / Solar &amp; renewables equipment (behind-the-meter DC power)</t>
+          <t>01 Power Generation / Distributed / on-site power</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>65.12</v>
+        <v>65.2</v>
       </c>
       <c r="D90" t="inlineStr">
         <is>
@@ -3724,25 +3984,28 @@
       <c r="E90" t="n">
         <v>88</v>
       </c>
+      <c r="F90" t="inlineStr"/>
       <c r="G90" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H90" t="inlineStr"/>
+      <c r="J90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>HUBB</t>
+          <t>NXT</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>01 Power Generation / Solar &amp; renewables equipment (behind-the-meter DC power)</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>64.67</v>
+        <v>65.12</v>
       </c>
       <c r="D91" t="inlineStr">
         <is>
@@ -3752,25 +4015,28 @@
       <c r="E91" t="n">
         <v>89</v>
       </c>
+      <c r="F91" t="inlineStr"/>
       <c r="G91" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H91" t="inlineStr"/>
+      <c r="J91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>MRVL</t>
+          <t>ASX</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
+          <t>04 Semiconductor Equipment &amp; Materials / OSAT &amp; advanced packaging</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>64.47</v>
+        <v>64.84999999999999</v>
       </c>
       <c r="D92" t="inlineStr">
         <is>
@@ -3780,16 +4046,19 @@
       <c r="E92" t="n">
         <v>90</v>
       </c>
+      <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H92" t="inlineStr"/>
+      <c r="J92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>ETN</t>
+          <t>HUBB</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -3798,7 +4067,7 @@
         </is>
       </c>
       <c r="C93" t="n">
-        <v>64.3</v>
+        <v>64.67</v>
       </c>
       <c r="D93" t="inlineStr">
         <is>
@@ -3808,25 +4077,28 @@
       <c r="E93" t="n">
         <v>91</v>
       </c>
+      <c r="F93" t="inlineStr"/>
       <c r="G93" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H93" t="inlineStr"/>
+      <c r="J93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>SMCI</t>
+          <t>MRVL</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling</t>
+          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>64.25</v>
+        <v>64.47</v>
       </c>
       <c r="D94" t="inlineStr">
         <is>
@@ -3836,25 +4108,28 @@
       <c r="E94" t="n">
         <v>92</v>
       </c>
+      <c r="F94" t="inlineStr"/>
       <c r="G94" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H94" t="inlineStr"/>
+      <c r="J94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>LITE</t>
+          <t>AMKR</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
+          <t>04 Semiconductor Equipment &amp; Materials / OSAT &amp; advanced packaging</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>64.17</v>
+        <v>64.31999999999999</v>
       </c>
       <c r="D95" t="inlineStr">
         <is>
@@ -3864,25 +4139,28 @@
       <c r="E95" t="n">
         <v>93</v>
       </c>
+      <c r="F95" t="inlineStr"/>
       <c r="G95" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H95" t="inlineStr"/>
+      <c r="J95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>HIVE</t>
+          <t>ETN</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>64.05</v>
+        <v>64.3</v>
       </c>
       <c r="D96" t="inlineStr">
         <is>
@@ -3892,25 +4170,28 @@
       <c r="E96" t="n">
         <v>94</v>
       </c>
+      <c r="F96" t="inlineStr"/>
       <c r="G96" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H96" t="inlineStr"/>
+      <c r="J96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>IRM</t>
+          <t>SMCI</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>63.75</v>
+        <v>64.25</v>
       </c>
       <c r="D97" t="inlineStr">
         <is>
@@ -3920,25 +4201,28 @@
       <c r="E97" t="n">
         <v>95</v>
       </c>
+      <c r="F97" t="inlineStr"/>
       <c r="G97" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H97" t="inlineStr"/>
+      <c r="J97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>SNOW</t>
+          <t>LITE</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications</t>
+          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>63.57</v>
+        <v>64.17</v>
       </c>
       <c r="D98" t="inlineStr">
         <is>
@@ -3948,25 +4232,28 @@
       <c r="E98" t="n">
         <v>96</v>
       </c>
+      <c r="F98" t="inlineStr"/>
       <c r="G98" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H98" t="inlineStr"/>
+      <c r="J98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>CMI</t>
+          <t>HIVE</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>01 Power Generation / Distributed / on-site power</t>
+          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>63.3</v>
+        <v>64.05</v>
       </c>
       <c r="D99" t="inlineStr">
         <is>
@@ -3976,25 +4263,28 @@
       <c r="E99" t="n">
         <v>97</v>
       </c>
+      <c r="F99" t="inlineStr"/>
       <c r="G99" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H99" t="inlineStr"/>
+      <c r="J99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>KLIC</t>
+          <t>IRM</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>63.17</v>
+        <v>63.75</v>
       </c>
       <c r="D100" t="inlineStr">
         <is>
@@ -4004,25 +4294,28 @@
       <c r="E100" t="n">
         <v>98</v>
       </c>
+      <c r="F100" t="inlineStr"/>
       <c r="G100" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H100" t="inlineStr"/>
+      <c r="J100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>FLEX</t>
+          <t>SNOW</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Contract manufacturing / ODMs</t>
+          <t>10 Models, Software &amp; Applications</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>63.05</v>
+        <v>63.57</v>
       </c>
       <c r="D101" t="inlineStr">
         <is>
@@ -4032,25 +4325,28 @@
       <c r="E101" t="n">
         <v>99</v>
       </c>
+      <c r="F101" t="inlineStr"/>
       <c r="G101" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H101" t="inlineStr"/>
+      <c r="J101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>KN</t>
+          <t>CMI</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>04 Semi Equip - Materials</t>
+          <t>01 Power Generation / Distributed / on-site power</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>62.7</v>
+        <v>63.3</v>
       </c>
       <c r="D102" t="inlineStr">
         <is>
@@ -4060,25 +4356,28 @@
       <c r="E102" t="n">
         <v>100</v>
       </c>
+      <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H102" t="inlineStr"/>
+      <c r="J102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>CRWV</t>
+          <t>KLIC</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>09 Cloud - Neocloud</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C103" t="n">
-        <v>62.67</v>
+        <v>63.17</v>
       </c>
       <c r="D103" t="inlineStr">
         <is>
@@ -4088,25 +4387,28 @@
       <c r="E103" t="n">
         <v>101</v>
       </c>
+      <c r="F103" t="inlineStr"/>
       <c r="G103" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H103" t="inlineStr"/>
+      <c r="J103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>SEI</t>
+          <t>FLEX</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>01 Power Generation / Distributed / on-site power</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Contract manufacturing / ODMs</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>62.55</v>
+        <v>63.05</v>
       </c>
       <c r="D104" t="inlineStr">
         <is>
@@ -4116,25 +4418,28 @@
       <c r="E104" t="n">
         <v>102</v>
       </c>
+      <c r="F104" t="inlineStr"/>
       <c r="G104" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H104" t="inlineStr"/>
+      <c r="J104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>AAPL</t>
+          <t>KN</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / Edge AI platforms</t>
+          <t>04 Semi Equip - Materials</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>62.2</v>
+        <v>62.7</v>
       </c>
       <c r="D105" t="inlineStr">
         <is>
@@ -4144,25 +4449,28 @@
       <c r="E105" t="n">
         <v>103</v>
       </c>
+      <c r="F105" t="inlineStr"/>
       <c r="G105" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H105" t="inlineStr"/>
+      <c r="J105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>NBIS</t>
+          <t>CRWV</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Neoclouds (AI-native cloud providers)</t>
+          <t>09 Cloud - Neocloud</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>61.82</v>
+        <v>62.67</v>
       </c>
       <c r="D106" t="inlineStr">
         <is>
@@ -4172,30 +4480,28 @@
       <c r="E106" t="n">
         <v>104</v>
       </c>
+      <c r="F106" t="inlineStr"/>
       <c r="G106" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="J106" t="inlineStr">
-        <is>
-          <t>Removed 2026-05-25: dropped to ✓ (65.5) after reweight. Value 7.5 penalized by higher Value weight.</t>
-        </is>
-      </c>
+      <c r="H106" t="inlineStr"/>
+      <c r="J106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>SEI</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
+          <t>01 Power Generation / Distributed / on-site power</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>61.65</v>
+        <v>62.55</v>
       </c>
       <c r="D107" t="inlineStr">
         <is>
@@ -4205,25 +4511,28 @@
       <c r="E107" t="n">
         <v>105</v>
       </c>
+      <c r="F107" t="inlineStr"/>
       <c r="G107" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H107" t="inlineStr"/>
+      <c r="J107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>CRWD</t>
+          <t>AAPL</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
+          <t>10 Models, Software &amp; Applications / Edge AI platforms</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>61.65</v>
+        <v>62.2</v>
       </c>
       <c r="D108" t="inlineStr">
         <is>
@@ -4233,25 +4542,28 @@
       <c r="E108" t="n">
         <v>106</v>
       </c>
+      <c r="F108" t="inlineStr"/>
       <c r="G108" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H108" t="inlineStr"/>
+      <c r="J108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>BWXT</t>
+          <t>NBIS</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>01 Power Generation / Nuclear-specific</t>
+          <t>09 Compute-as-a-Service / Neoclouds (AI-native cloud providers)</t>
         </is>
       </c>
       <c r="C109" t="n">
-        <v>61.58</v>
+        <v>61.82</v>
       </c>
       <c r="D109" t="inlineStr">
         <is>
@@ -4261,25 +4573,32 @@
       <c r="E109" t="n">
         <v>107</v>
       </c>
+      <c r="F109" t="inlineStr"/>
       <c r="G109" t="inlineStr">
         <is>
           <t>N</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr"/>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>Removed 2026-05-25: dropped to ✓ (65.5) after reweight. Value 7.5 penalized by higher Value weight.</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>COHR</t>
+          <t>P</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
         </is>
       </c>
       <c r="C110" t="n">
-        <v>61.55</v>
+        <v>61.65</v>
       </c>
       <c r="D110" t="inlineStr">
         <is>
@@ -4289,25 +4608,28 @@
       <c r="E110" t="n">
         <v>108</v>
       </c>
+      <c r="F110" t="inlineStr"/>
       <c r="G110" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H110" t="inlineStr"/>
+      <c r="J110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>NXPI</t>
+          <t>CRWD</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Analog &amp; embedded (auto/edge AI)</t>
+          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>61.4</v>
+        <v>61.65</v>
       </c>
       <c r="D111" t="inlineStr">
         <is>
@@ -4317,25 +4639,28 @@
       <c r="E111" t="n">
         <v>109</v>
       </c>
+      <c r="F111" t="inlineStr"/>
       <c r="G111" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H111" t="inlineStr"/>
+      <c r="J111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>MDB</t>
+          <t>BWXT</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI data layer</t>
+          <t>01 Power Generation / Nuclear-specific</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>61.32</v>
+        <v>61.58</v>
       </c>
       <c r="D112" t="inlineStr">
         <is>
@@ -4345,25 +4670,28 @@
       <c r="E112" t="n">
         <v>110</v>
       </c>
+      <c r="F112" t="inlineStr"/>
       <c r="G112" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H112" t="inlineStr"/>
+      <c r="J112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>HUT</t>
+          <t>COHR</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
+          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
         </is>
       </c>
       <c r="C113" t="n">
-        <v>61.2</v>
+        <v>61.55</v>
       </c>
       <c r="D113" t="inlineStr">
         <is>
@@ -4373,25 +4701,28 @@
       <c r="E113" t="n">
         <v>111</v>
       </c>
+      <c r="F113" t="inlineStr"/>
       <c r="G113" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H113" t="inlineStr"/>
+      <c r="J113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>ATKR</t>
+          <t>NXPI</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>06 AI Compute Silicon / Analog &amp; embedded (auto/edge AI)</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>61.15</v>
+        <v>61.4</v>
       </c>
       <c r="D114" t="inlineStr">
         <is>
@@ -4401,25 +4732,28 @@
       <c r="E114" t="n">
         <v>112</v>
       </c>
+      <c r="F114" t="inlineStr"/>
       <c r="G114" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H114" t="inlineStr"/>
+      <c r="J114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>EQIX</t>
+          <t>MDB</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>10 Models, Software &amp; Applications / AI data layer</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>61</v>
+        <v>61.32</v>
       </c>
       <c r="D115" t="inlineStr">
         <is>
@@ -4429,25 +4763,28 @@
       <c r="E115" t="n">
         <v>113</v>
       </c>
+      <c r="F115" t="inlineStr"/>
       <c r="G115" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H115" t="inlineStr"/>
+      <c r="J115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>GFS</t>
+          <t>HUT</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>05 Fabs &amp; Foundries</t>
+          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>60.7</v>
+        <v>61.2</v>
       </c>
       <c r="D116" t="inlineStr">
         <is>
@@ -4457,25 +4794,28 @@
       <c r="E116" t="n">
         <v>114</v>
       </c>
+      <c r="F116" t="inlineStr"/>
       <c r="G116" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H116" t="inlineStr"/>
+      <c r="J116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>TTMI</t>
+          <t>ATKR</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / PCB / substrates</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>60.45</v>
+        <v>61.15</v>
       </c>
       <c r="D117" t="inlineStr">
         <is>
@@ -4485,25 +4825,28 @@
       <c r="E117" t="n">
         <v>115</v>
       </c>
+      <c r="F117" t="inlineStr"/>
       <c r="G117" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H117" t="inlineStr"/>
+      <c r="J117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>DUK</t>
+          <t>EQIX</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>60.1</v>
+        <v>61</v>
       </c>
       <c r="D118" t="inlineStr">
         <is>
@@ -4513,25 +4856,28 @@
       <c r="E118" t="n">
         <v>116</v>
       </c>
+      <c r="F118" t="inlineStr"/>
       <c r="G118" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H118" t="inlineStr"/>
+      <c r="J118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>GFS</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>05 Fabs &amp; Foundries</t>
         </is>
       </c>
       <c r="C119" t="n">
-        <v>59.1</v>
+        <v>60.7</v>
       </c>
       <c r="D119" t="inlineStr">
         <is>
@@ -4541,25 +4887,28 @@
       <c r="E119" t="n">
         <v>117</v>
       </c>
+      <c r="F119" t="inlineStr"/>
       <c r="G119" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H119" t="inlineStr"/>
+      <c r="J119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>CARR</t>
+          <t>TTMI</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>04 Semiconductor Equipment &amp; Materials / PCB / substrates</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>59</v>
+        <v>60.45</v>
       </c>
       <c r="D120" t="inlineStr">
         <is>
@@ -4569,25 +4918,28 @@
       <c r="E120" t="n">
         <v>118</v>
       </c>
+      <c r="F120" t="inlineStr"/>
       <c r="G120" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H120" t="inlineStr"/>
+      <c r="J120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>QCOM</t>
+          <t>DUK</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Application processors &amp; connectivity (edge AI)</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>59</v>
+        <v>60.1</v>
       </c>
       <c r="D121" t="inlineStr">
         <is>
@@ -4597,16 +4949,19 @@
       <c r="E121" t="n">
         <v>119</v>
       </c>
+      <c r="F121" t="inlineStr"/>
       <c r="G121" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H121" t="inlineStr"/>
+      <c r="J121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>AEP</t>
+          <t>D</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -4615,7 +4970,7 @@
         </is>
       </c>
       <c r="C122" t="n">
-        <v>58.77</v>
+        <v>59.1</v>
       </c>
       <c r="D122" t="inlineStr">
         <is>
@@ -4625,25 +4980,28 @@
       <c r="E122" t="n">
         <v>120</v>
       </c>
+      <c r="F122" t="inlineStr"/>
       <c r="G122" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H122" t="inlineStr"/>
+      <c r="J122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>ON</t>
+          <t>CAMT</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Power management silicon (SiC/GaN)</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C123" t="n">
-        <v>58.52</v>
+        <v>59.05</v>
       </c>
       <c r="D123" t="inlineStr">
         <is>
@@ -4653,25 +5011,28 @@
       <c r="E123" t="n">
         <v>121</v>
       </c>
+      <c r="F123" t="inlineStr"/>
       <c r="G123" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H123" t="inlineStr"/>
+      <c r="J123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>PPL</t>
+          <t>CARR</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C124" t="n">
-        <v>58.38</v>
+        <v>59</v>
       </c>
       <c r="D124" t="inlineStr">
         <is>
@@ -4681,25 +5042,28 @@
       <c r="E124" t="n">
         <v>122</v>
       </c>
+      <c r="F124" t="inlineStr"/>
       <c r="G124" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H124" t="inlineStr"/>
+      <c r="J124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>TEM</t>
+          <t>QCOM</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI-native vertical applications</t>
+          <t>06 AI Compute Silicon / Application processors &amp; connectivity (edge AI)</t>
         </is>
       </c>
       <c r="C125" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D125" t="inlineStr">
         <is>
@@ -4709,25 +5073,28 @@
       <c r="E125" t="n">
         <v>123</v>
       </c>
+      <c r="F125" t="inlineStr"/>
       <c r="G125" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H125" t="inlineStr"/>
+      <c r="J125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>IREN</t>
+          <t>AEP</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C126" t="n">
-        <v>57.12</v>
+        <v>58.77</v>
       </c>
       <c r="D126" t="inlineStr">
         <is>
@@ -4737,25 +5104,28 @@
       <c r="E126" t="n">
         <v>124</v>
       </c>
+      <c r="F126" t="inlineStr"/>
       <c r="G126" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H126" t="inlineStr"/>
+      <c r="J126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>XEL</t>
+          <t>ON</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>06 AI Compute Silicon / Power management silicon (SiC/GaN)</t>
         </is>
       </c>
       <c r="C127" t="n">
-        <v>57.05</v>
+        <v>58.52</v>
       </c>
       <c r="D127" t="inlineStr">
         <is>
@@ -4765,25 +5135,28 @@
       <c r="E127" t="n">
         <v>125</v>
       </c>
+      <c r="F127" t="inlineStr"/>
       <c r="G127" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H127" t="inlineStr"/>
+      <c r="J127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>WYFI</t>
+          <t>PPL</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Neoclouds (AI-native cloud providers)</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C128" t="n">
-        <v>56.88</v>
+        <v>58.38</v>
       </c>
       <c r="D128" t="inlineStr">
         <is>
@@ -4793,25 +5166,28 @@
       <c r="E128" t="n">
         <v>126</v>
       </c>
+      <c r="F128" t="inlineStr"/>
       <c r="G128" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H128" t="inlineStr"/>
+      <c r="J128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>PSIX</t>
+          <t>TEM</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>01 Power Generation / Distributed / on-site power</t>
+          <t>10 Models, Software &amp; Applications / AI-native vertical applications</t>
         </is>
       </c>
       <c r="C129" t="n">
-        <v>56.35</v>
+        <v>58</v>
       </c>
       <c r="D129" t="inlineStr">
         <is>
@@ -4821,25 +5197,28 @@
       <c r="E129" t="n">
         <v>127</v>
       </c>
+      <c r="F129" t="inlineStr"/>
       <c r="G129" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H129" t="inlineStr"/>
+      <c r="J129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>ETR</t>
+          <t>ACLS</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C130" t="n">
-        <v>56.15</v>
+        <v>57.32</v>
       </c>
       <c r="D130" t="inlineStr">
         <is>
@@ -4849,25 +5228,28 @@
       <c r="E130" t="n">
         <v>128</v>
       </c>
+      <c r="F130" t="inlineStr"/>
       <c r="G130" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H130" t="inlineStr"/>
+      <c r="J130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>SO</t>
+          <t>IREN</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
         </is>
       </c>
       <c r="C131" t="n">
-        <v>55.33</v>
+        <v>57.12</v>
       </c>
       <c r="D131" t="inlineStr">
         <is>
@@ -4877,95 +5259,231 @@
       <c r="E131" t="n">
         <v>129</v>
       </c>
+      <c r="F131" t="inlineStr"/>
       <c r="G131" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H131" t="inlineStr"/>
+      <c r="J131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>APLD</t>
+          <t>XEL</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Neoclouds (AI-native cloud providers)</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C132" t="n">
-        <v>54.73</v>
+        <v>57.05</v>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="E132" t="n">
         <v>130</v>
       </c>
+      <c r="F132" t="inlineStr"/>
       <c r="G132" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H132" t="inlineStr"/>
+      <c r="J132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>WULF</t>
+          <t>COHU</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
         </is>
       </c>
       <c r="C133" t="n">
-        <v>52.94</v>
+        <v>57</v>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="E133" t="n">
         <v>131</v>
       </c>
+      <c r="F133" t="inlineStr"/>
       <c r="G133" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H133" t="inlineStr"/>
+      <c r="J133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>UCTT</t>
+          <t>WYFI</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
+          <t>09 Compute-as-a-Service / Neoclouds (AI-native cloud providers)</t>
         </is>
       </c>
       <c r="C134" t="n">
-        <v>51.62</v>
+        <v>56.88</v>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="E134" t="n">
         <v>132</v>
       </c>
+      <c r="F134" t="inlineStr"/>
       <c r="G134" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
+      <c r="H134" t="inlineStr"/>
+      <c r="J134" t="inlineStr"/>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>PSIX</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>01 Power Generation / Distributed / on-site power</t>
+        </is>
+      </c>
+      <c r="C135" t="n">
+        <v>56.35</v>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E135" t="n">
+        <v>133</v>
+      </c>
+      <c r="F135" t="inlineStr"/>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr"/>
+      <c r="J135" t="inlineStr"/>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>ETR</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+        </is>
+      </c>
+      <c r="C136" t="n">
+        <v>56.15</v>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E136" t="n">
+        <v>134</v>
+      </c>
+      <c r="F136" t="inlineStr"/>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr"/>
+      <c r="J136" t="inlineStr"/>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>TOELY</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+        </is>
+      </c>
+      <c r="C137" t="n">
+        <v>55.92</v>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E137" t="n">
+        <v>135</v>
+      </c>
+      <c r="F137" t="inlineStr"/>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr"/>
+      <c r="J137" t="inlineStr"/>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>SO</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+        </is>
+      </c>
+      <c r="C138" t="n">
+        <v>55.33</v>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E138" t="n">
+        <v>136</v>
+      </c>
+      <c r="F138" t="inlineStr"/>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr"/>
+      <c r="J138" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
data: rebalance portfolio to the new (P1+P2+P6) scores — 15 -> 13 names
First rebalance on the overhauled scoring. Immediate (--resize), approved by Dom.

- ENTER: AMZN (77.7)
- EXIT: PLTR (72.0), APP (72.6), RDDT (74.4) — crowded software/apps that fell
  below the exit line once the business-model bias was removed
- TIER re-weight: NVDA ✓✓->✓✓✓ (8.2%->12.0%), TSM ✓✓✓->✓✓ (10.3%->9.1%)

New book: NVDA 12.0, MU 12.0, TSM 9.1, CRDO 8.2, ANET 7.9, META 7.5, AVGO 6.9,
AMZN 6.8, MSFT 6.5, GOOGL 5.8, FIX 5.8, ALAB 5.8, SNDK 5.6. Model event logged
at $10k notional; score-monotonicity gate passes. Layer-06 (silicon) now 42% —
no cap active (flagged to Dom, accepted).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/00-master/portfolio.xlsx
+++ b/00-master/portfolio.xlsx
@@ -676,7 +676,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-06-29 (refresh_targets.py — hysteresis pipeline)</t>
+          <t>2026-07-02 (refresh_targets.py — hysteresis pipeline)</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J138"/>
+  <dimension ref="A1:J122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1068,7 +1068,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Target Portfolio (refreshed 2026-06-29, live Watchlist scores)</t>
+          <t>Target Portfolio (refreshed 2026-07-02, live Watchlist scores)</t>
         </is>
       </c>
     </row>
@@ -1127,16 +1127,16 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>TSM</t>
+          <t>NVDA</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>05 Fabs &amp; Foundries</t>
+          <t>06 AI Compute Silicon / GPUs / merchant accelerators</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>87.90000000000001</v>
+        <v>85.89</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -1158,7 +1158,7 @@
       </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="n">
-        <v>10.32</v>
+        <v>12</v>
       </c>
       <c r="J3" t="inlineStr"/>
     </row>
@@ -1174,7 +1174,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>86.40000000000001</v>
+        <v>85.64</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -1196,23 +1196,23 @@
       </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="n">
-        <v>10.32</v>
+        <v>12</v>
       </c>
       <c r="J4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>NVDA</t>
+          <t>TSM</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / GPUs / merchant accelerators</t>
+          <t>05 Fabs &amp; Foundries</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>84.08</v>
+        <v>82.42</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -1234,23 +1234,23 @@
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="n">
-        <v>8.23</v>
+        <v>9.109999999999999</v>
       </c>
       <c r="J5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SNDK</t>
+          <t>CRDO</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Memory (HBM is the bottleneck)</t>
+          <t>07 Optical, Networking &amp; Interconnect / Connectivity ASICs</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>80.09999999999999</v>
+        <v>80.55</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -1272,27 +1272,27 @@
       </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="n">
-        <v>6.63</v>
+        <v>8.210000000000001</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Manually excluded 2026-05-18: $1,333 share price prevents capital-efficient sizing below ~$25k. Conscious framework override (target ~$10k portfolio). | Override removed 2026-06-09: fractional shares adopted, share-price constraint obsolete (Dom decision).</t>
+          <t>Added 2026-05-25: score 78.4, ranked #4 in reweighted watchlist. Optical connectivity pure-play.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CRDO</t>
+          <t>ANET</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Connectivity ASICs</t>
+          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>80</v>
+        <v>79.84999999999999</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -1314,13 +1314,9 @@
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="n">
-        <v>6.59</v>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>Added 2026-05-25: score 78.4, ranked #4 in reweighted watchlist. Optical connectivity pure-play.</t>
-        </is>
-      </c>
+        <v>7.87</v>
+      </c>
+      <c r="J7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1334,7 +1330,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>79.5</v>
+        <v>79.14</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -1356,23 +1352,23 @@
       </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="n">
-        <v>6.39</v>
+        <v>7.52</v>
       </c>
       <c r="J8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>RDDT</t>
+          <t>AVGO</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI advertising</t>
+          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>79.40000000000001</v>
+        <v>77.88</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -1384,7 +1380,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>ENTER (score 79.4)</t>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1394,23 +1390,23 @@
       </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="n">
-        <v>6.35</v>
+        <v>6.92</v>
       </c>
       <c r="J9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>AVGO</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
+          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>79.2</v>
+        <v>77.66</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -1422,7 +1418,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>HOLD</t>
+          <t>ENTER (score 77.7)</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1432,23 +1428,23 @@
       </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="n">
-        <v>6.27</v>
+        <v>6.81</v>
       </c>
       <c r="J10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ANET</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
+          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>78.48</v>
+        <v>77.11</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -1470,14 +1466,14 @@
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="n">
-        <v>5.98</v>
+        <v>6.55</v>
       </c>
       <c r="J11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1486,7 +1482,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>78.40000000000001</v>
+        <v>75.64</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -1508,23 +1504,23 @@
       </c>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="n">
-        <v>5.95</v>
+        <v>5.83</v>
       </c>
       <c r="J12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>FIX</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>78.03</v>
+        <v>75.58</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -1546,9 +1542,13 @@
       </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="n">
-        <v>5.8</v>
-      </c>
-      <c r="J13" t="inlineStr"/>
+        <v>5.81</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Manually excluded 2026-05-18: $1,854 share price prevents reasonable position sizing below ~$50k portfolio. Conscious framework override. | Override removed 2026-06-09: fractional shares adopted, share-price constraint obsolete (Dom decision).</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1562,7 +1562,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>77.08</v>
+        <v>75.58</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -1584,23 +1584,23 @@
       </c>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="n">
-        <v>5.42</v>
+        <v>5.8</v>
       </c>
       <c r="J14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>APP</t>
+          <t>SNDK</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI advertising</t>
+          <t>06 AI Compute Silicon / Memory (HBM is the bottleneck)</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>76.90000000000001</v>
+        <v>75.11</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -1622,14 +1622,18 @@
       </c>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="n">
-        <v>5.35</v>
-      </c>
-      <c r="J15" t="inlineStr"/>
+        <v>5.58</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Manually excluded 2026-05-18: $1,333 share price prevents capital-efficient sizing below ~$25k. Conscious framework override (target ~$10k portfolio). | Override removed 2026-06-09: fractional shares adopted, share-price constraint obsolete (Dom decision).</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>FIX</t>
+          <t>EME</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1638,7 +1642,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>76.65000000000001</v>
+        <v>74.67</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -1648,39 +1652,32 @@
       <c r="E16" t="n">
         <v>14</v>
       </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>HOLD</t>
-        </is>
-      </c>
+      <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H16" t="inlineStr"/>
-      <c r="I16" t="n">
-        <v>5.25</v>
-      </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Manually excluded 2026-05-18: $1,854 share price prevents reasonable position sizing below ~$50k portfolio. Conscious framework override. | Override removed 2026-06-09: fractional shares adopted, share-price constraint obsolete (Dom decision).</t>
+          <t>Added 2026-05-25: score 75.2, DC construction, strong momentum (86.7).</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>PLTR</t>
+          <t>RDDT</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications</t>
+          <t>10 Models, Software &amp; Applications / AI advertising</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>76.40000000000001</v>
+        <v>74.45</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -1692,33 +1689,30 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>ENTER (score 76.4)</t>
+          <t>EXIT (resize, score 74.4 &lt; 74.5)</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H17" t="inlineStr"/>
-      <c r="I17" t="n">
-        <v>5.15</v>
-      </c>
       <c r="J17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ZS</t>
+          <t>VRT</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
+          <t>03 DC Infrastructure</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>75.47</v>
+        <v>73.83</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -1740,16 +1734,16 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>VRT</t>
+          <t>APP</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>03 DC Infrastructure</t>
+          <t>10 Models, Software &amp; Applications / AI advertising</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>75.3</v>
+        <v>72.56999999999999</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -1759,7 +1753,11 @@
       <c r="E19" t="n">
         <v>17</v>
       </c>
-      <c r="F19" t="inlineStr"/>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>EXIT (resize, score 72.6 &lt; 74.5)</t>
+        </is>
+      </c>
       <c r="G19" t="inlineStr">
         <is>
           <t>N</t>
@@ -1771,16 +1769,16 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>EME</t>
+          <t>PLTR</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>10 Models, Software &amp; Applications</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>74.75</v>
+        <v>72.01000000000001</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -1790,32 +1788,32 @@
       <c r="E20" t="n">
         <v>18</v>
       </c>
-      <c r="F20" t="inlineStr"/>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>EXIT (resize, score 72.0 &lt; 74.5)</t>
+        </is>
+      </c>
       <c r="G20" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
       <c r="H20" t="inlineStr"/>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>Added 2026-05-25: score 75.2, DC construction, strong momentum (86.7).</t>
-        </is>
-      </c>
+      <c r="J20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>WDAY</t>
+          <t>APH</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / Enterprise SaaS</t>
+          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>74.7</v>
+        <v>70.56</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -1837,16 +1835,16 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>EQT</t>
+          <t>VST</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
+          <t>01 Power Generation / Independent Power Producers (IPPs)</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>74.65000000000001</v>
+        <v>70.3</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -1868,16 +1866,16 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>WDC</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / GPUs / merchant accelerators</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>74.58</v>
+        <v>70.17</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -1894,29 +1892,25 @@
         </is>
       </c>
       <c r="H23" t="inlineStr"/>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>Removed 2026-05-25: score 74.1 fell below natural 17-name cutoff (ARM 74.2). First name out.</t>
-        </is>
-      </c>
+      <c r="J23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>ADSK</t>
+          <t>TER</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / Design &amp; engineering software</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>74.25</v>
+        <v>69.84</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>✓✓</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="E24" t="n">
@@ -1934,20 +1928,20 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>KEYS</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>74.08</v>
+        <v>69.79000000000001</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>✓✓</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="E25" t="n">
@@ -1960,29 +1954,25 @@
         </is>
       </c>
       <c r="H25" t="inlineStr"/>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>Added 2026-05-22 as substitute for CTRA (delisted). Pure score-driven pick: next-best ✓✓ at 75.62, same Layer 1 NG E&amp;P sub-category — preserves natural gas thesis concentration.</t>
-        </is>
-      </c>
+      <c r="J25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>AMZN</t>
+          <t>NTAP</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>73.3</v>
+        <v>69.67</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>✓✓</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="E26" t="n">
@@ -2000,20 +1990,20 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>KEYS</t>
+          <t>CIEN</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
+          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>73.22</v>
+        <v>69.47</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>✓✓</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="E27" t="n">
@@ -2031,20 +2021,20 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>TER</t>
+          <t>EQT</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>73.05</v>
+        <v>69.34999999999999</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>✓✓</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="E28" t="n">
@@ -2062,20 +2052,20 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>HTHIY</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>72.8</v>
+        <v>69.34</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>✓✓</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="E29" t="n">
@@ -2088,29 +2078,25 @@
         </is>
       </c>
       <c r="H29" t="inlineStr"/>
-      <c r="J29" t="inlineStr">
-        <is>
-          <t>Added 2026-05-25: score 74.8, Quality 97, PEG 0.8. Enterprise SaaS with AI exposure.</t>
-        </is>
-      </c>
+      <c r="J29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>RRC</t>
+          <t>FN</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
+          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>72.75</v>
+        <v>68.70999999999999</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>✓✓</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="E30" t="n">
@@ -2128,20 +2114,20 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>STX</t>
+          <t>ARM</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
+          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>72.75</v>
+        <v>68.63</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>✓✓</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="E31" t="n">
@@ -2159,20 +2145,20 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>PANW</t>
+          <t>RMBS</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
+          <t>06 AI Compute Silicon / Memory (HBM is the bottleneck)</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>72.65000000000001</v>
+        <v>68.51000000000001</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>✓✓</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="E32" t="n">
@@ -2190,20 +2176,20 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>HTHIY</t>
+          <t>ORCL</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>72.05</v>
+        <v>68.19</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>✓✓</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="E33" t="n">
@@ -2221,20 +2207,20 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>LSCC</t>
+          <t>GLW</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Programmable logic</t>
+          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>71.98</v>
+        <v>68.02</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>✓✓</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="E34" t="n">
@@ -2252,55 +2238,55 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>WDC</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
+          <t>06 AI Compute Silicon / GPUs / merchant accelerators</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>71.62</v>
+        <v>67.83</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>✓✓</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="E35" t="n">
         <v>33</v>
       </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>EXIT (resize, score 71.6 &lt; 74.5)</t>
-        </is>
-      </c>
+      <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
       <c r="H35" t="inlineStr"/>
-      <c r="J35" t="inlineStr"/>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Removed 2026-05-25: score 74.1 fell below natural 17-name cutoff (ARM 74.2). First name out.</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>PLAB</t>
+          <t>DELL</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>71.59999999999999</v>
+        <v>67.75</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>✓✓</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="E36" t="n">
@@ -2318,20 +2304,20 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>DELL</t>
+          <t>TT</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>71.59999999999999</v>
+        <v>67.52</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>✓✓</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="E37" t="n">
@@ -2349,20 +2335,20 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>CIEN</t>
+          <t>AR</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
+          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>71.45</v>
+        <v>67.41</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>✓✓</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="E38" t="n">
@@ -2375,25 +2361,29 @@
         </is>
       </c>
       <c r="H38" t="inlineStr"/>
-      <c r="J38" t="inlineStr"/>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>Added 2026-05-22 as substitute for CTRA (delisted). Pure score-driven pick: next-best ✓✓ at 75.62, same Layer 1 NG E&amp;P sub-category — preserves natural gas thesis concentration.</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>EXE</t>
+          <t>CCJ</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
+          <t>01 Power Generation / Nuclear-specific</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>71.22</v>
+        <v>67.27</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>✓✓</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="E39" t="n">
@@ -2411,20 +2401,20 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>ARM</t>
+          <t>ADSK</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
+          <t>10 Models, Software &amp; Applications / Design &amp; engineering software</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>71.15000000000001</v>
+        <v>67.23999999999999</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>✓✓</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="E40" t="n">
@@ -2442,20 +2432,20 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>VST</t>
+          <t>EXE</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>01 Power Generation / Independent Power Producers (IPPs)</t>
+          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>71.05</v>
+        <v>67.16</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>✓✓</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="E41" t="n">
@@ -2473,20 +2463,20 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>DDOG</t>
+          <t>ABBNY</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI observability &amp; infrastructure software</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>71</v>
+        <v>67.03</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>✓✓</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="E42" t="n">
@@ -2499,29 +2489,25 @@
         </is>
       </c>
       <c r="H42" t="inlineStr"/>
-      <c r="J42" t="inlineStr">
-        <is>
-          <t>Added 2026-05-25: score 75.4, Quality 100, PEG 0.7. Beats 4 existing portfolio names.</t>
-        </is>
-      </c>
+      <c r="J42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>APH</t>
+          <t>DLR</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>70.92</v>
+        <v>66.97</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>✓✓</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="E43" t="n">
@@ -2539,20 +2525,20 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>FN</t>
+          <t>STX</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>70.09999999999999</v>
+        <v>66.88</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>✓✓</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="E44" t="n">
@@ -2570,16 +2556,16 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>PWR</t>
+          <t>SNPS</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>69.95</v>
+        <v>66.83</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
@@ -2601,16 +2587,16 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>ASML</t>
+          <t>PLAB</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>69.95</v>
+        <v>66.48</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -2632,16 +2618,16 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>PATH</t>
+          <t>RRC</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI-powered automation</t>
+          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>69.90000000000001</v>
+        <v>66.39</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -2663,16 +2649,16 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>MOD</t>
+          <t>KLAC</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>69.7</v>
+        <v>66.14</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -2694,16 +2680,16 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>LRCX</t>
+          <t>CSCO</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>69.45</v>
+        <v>66.11</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
@@ -2725,16 +2711,16 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>NOW</t>
+          <t>POWL</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>69.45</v>
+        <v>66.08</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
@@ -2756,16 +2742,16 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>MPWR</t>
+          <t>CDNS</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Power management silicon</t>
+          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>69.40000000000001</v>
+        <v>66.06999999999999</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
@@ -2787,16 +2773,16 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>ADI</t>
+          <t>LRCX</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Analog &amp; mixed-signal (signal chain + power)</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>69.40000000000001</v>
+        <v>65.88</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
@@ -2818,16 +2804,16 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>GLW</t>
+          <t>SBGSY</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>69.25</v>
+        <v>65.52</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
@@ -2849,7 +2835,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>ABBNY</t>
+          <t>PWR</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2858,7 +2844,7 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>69</v>
+        <v>65.38</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
@@ -2880,16 +2866,16 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>CCJ</t>
+          <t>MOD</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>01 Power Generation / Nuclear-specific</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>68.92</v>
+        <v>65.17</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
@@ -2911,16 +2897,16 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>INTU</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / Financial software</t>
+          <t>01 Power - Distributed</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>68.63</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
@@ -2942,16 +2928,16 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>KLAC</t>
+          <t>ADI</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>06 AI Compute Silicon / Analog &amp; mixed-signal (signal chain + power)</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>68.5</v>
+        <v>65.08</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
@@ -2973,16 +2959,16 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>CDNS</t>
+          <t>ETN</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>68.45</v>
+        <v>65.06999999999999</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
@@ -3004,16 +2990,16 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>FTNT</t>
+          <t>LSCC</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
+          <t>06 AI Compute Silicon / Programmable logic</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>68.25</v>
+        <v>65</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
@@ -3035,16 +3021,16 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>NVT</t>
+          <t>CRWV</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>09 Cloud - Neocloud</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>68.15000000000001</v>
+        <v>64.91</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
@@ -3066,16 +3052,16 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>TLN</t>
+          <t>ONTO</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>01 Power Generation / Independent Power Producers (IPPs)</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>68.08</v>
+        <v>64.88</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
@@ -3097,16 +3083,16 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>CSCO</t>
+          <t>ASML</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>68</v>
+        <v>64.88</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
@@ -3128,16 +3114,16 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>FORM</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
+          <t>10 Models, Software &amp; Applications</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>67.92</v>
+        <v>64.83</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
@@ -3154,21 +3140,25 @@
         </is>
       </c>
       <c r="H63" t="inlineStr"/>
-      <c r="J63" t="inlineStr"/>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>Added 2026-05-25: score 74.8, Quality 97, PEG 0.8. Enterprise SaaS with AI exposure.</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>TT</t>
+          <t>BESIY</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>67.83</v>
+        <v>64.83</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
@@ -3190,7 +3180,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>DLR</t>
+          <t>JCI</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -3199,7 +3189,7 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>67.8</v>
+        <v>64.81999999999999</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
@@ -3221,16 +3211,16 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>AEIS</t>
+          <t>HIVE</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
+          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>67.72</v>
+        <v>64.75</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
@@ -3252,16 +3242,16 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>NEE</t>
+          <t>HUBB</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>67.67</v>
+        <v>64.65000000000001</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
@@ -3283,16 +3273,16 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>POWL</t>
+          <t>TSEM</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>05 Fabs &amp; Foundries</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>67.34999999999999</v>
+        <v>64.20999999999999</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
@@ -3314,16 +3304,16 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>AAON</t>
+          <t>AEIS</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>67.25</v>
+        <v>64.14</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
@@ -3345,16 +3335,16 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>TXN</t>
+          <t>AAON</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Analog &amp; embedded (power management)</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>67.09999999999999</v>
+        <v>63.96</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
@@ -3376,16 +3366,16 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>AMAT</t>
+          <t>NBIS</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>09 Compute-as-a-Service / Neoclouds (AI-native cloud providers)</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>67.05</v>
+        <v>63.88</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
@@ -3402,21 +3392,25 @@
         </is>
       </c>
       <c r="H71" t="inlineStr"/>
-      <c r="J71" t="inlineStr"/>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>Removed 2026-05-25: dropped to ✓ (65.5) after reweight. Value 7.5 penalized by higher Value weight.</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>MTZ</t>
+          <t>NEE</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>67</v>
+        <v>63.75</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
@@ -3438,16 +3432,16 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>RMBS</t>
+          <t>MKSI</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Memory (HBM is the bottleneck)</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>66.92</v>
+        <v>63.75</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
@@ -3469,16 +3463,16 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>ONTO</t>
+          <t>DDOG</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>10 Models, Software &amp; Applications / AI observability &amp; infrastructure software</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>66.72</v>
+        <v>63.6</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
@@ -3495,21 +3489,25 @@
         </is>
       </c>
       <c r="H74" t="inlineStr"/>
-      <c r="J74" t="inlineStr"/>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>Added 2026-05-25: score 75.4, Quality 100, PEG 0.7. Beats 4 existing portfolio names.</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>JCI</t>
+          <t>WDAY</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>10 Models, Software &amp; Applications / Enterprise SaaS</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>66.5</v>
+        <v>63.51</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
@@ -3531,16 +3529,16 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>HPE</t>
+          <t>AMAT</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>66.47</v>
+        <v>63.45</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
@@ -3562,16 +3560,16 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>MKSI</t>
+          <t>GEV</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
+          <t>02 Grid Equipment</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>66.45</v>
+        <v>63.43</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
@@ -3593,16 +3591,16 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>ADBE</t>
+          <t>NVT</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / Creative &amp; design software</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>66.33</v>
+        <v>63.32</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
@@ -3624,16 +3622,16 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>CEG</t>
+          <t>PANW</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>01 Power - IPP / Nuclear</t>
+          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>66.28</v>
+        <v>63.21</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
@@ -3655,7 +3653,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>TSEM</t>
+          <t>UMC</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -3664,7 +3662,7 @@
         </is>
       </c>
       <c r="C80" t="n">
-        <v>66.09999999999999</v>
+        <v>63.17</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
@@ -3686,16 +3684,16 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>BESIY</t>
+          <t>TLN</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>01 Power Generation / Independent Power Producers (IPPs)</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>66.09999999999999</v>
+        <v>62.9</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
@@ -3717,16 +3715,16 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>CEG</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>01 Power - Distributed</t>
+          <t>01 Power - IPP / Nuclear</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>66.05</v>
+        <v>62.8</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
@@ -3748,16 +3746,16 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>SBGSY</t>
+          <t>LITE</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>66</v>
+        <v>62.67</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
@@ -3779,16 +3777,16 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>SNPS</t>
+          <t>HUT</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
+          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>65.55</v>
+        <v>62.62</v>
       </c>
       <c r="D84" t="inlineStr">
         <is>
@@ -3810,16 +3808,16 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>TEL</t>
+          <t>FORM</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>65.53</v>
+        <v>62.37</v>
       </c>
       <c r="D85" t="inlineStr">
         <is>
@@ -3841,16 +3839,16 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>GEV</t>
+          <t>ENTG</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>02 Grid Equipment</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>65.5</v>
+        <v>62.27</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
@@ -3872,16 +3870,16 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>ENTG</t>
+          <t>MPWR</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
+          <t>06 AI Compute Silicon / Power management silicon</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>65.45</v>
+        <v>62.18</v>
       </c>
       <c r="D87" t="inlineStr">
         <is>
@@ -3903,16 +3901,16 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>UMC</t>
+          <t>ADBE</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>05 Fabs &amp; Foundries</t>
+          <t>10 Models, Software &amp; Applications / Creative &amp; design software</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>65.34999999999999</v>
+        <v>62.05</v>
       </c>
       <c r="D88" t="inlineStr">
         <is>
@@ -3934,16 +3932,16 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>ORCL</t>
+          <t>HPE</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>65.3</v>
+        <v>62</v>
       </c>
       <c r="D89" t="inlineStr">
         <is>
@@ -3965,7 +3963,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>GNRC</t>
+          <t>CMI</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -3974,7 +3972,7 @@
         </is>
       </c>
       <c r="C90" t="n">
-        <v>65.2</v>
+        <v>61.6</v>
       </c>
       <c r="D90" t="inlineStr">
         <is>
@@ -3996,16 +3994,16 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>NXT</t>
+          <t>NOW</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>01 Power Generation / Solar &amp; renewables equipment (behind-the-meter DC power)</t>
+          <t>10 Models, Software &amp; Applications</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>65.12</v>
+        <v>61.59</v>
       </c>
       <c r="D91" t="inlineStr">
         <is>
@@ -4027,16 +4025,16 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>ASX</t>
+          <t>NXT</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / OSAT &amp; advanced packaging</t>
+          <t>01 Power Generation / Solar &amp; renewables equipment (behind-the-meter DC power)</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>64.84999999999999</v>
+        <v>61.54</v>
       </c>
       <c r="D92" t="inlineStr">
         <is>
@@ -4058,16 +4056,16 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>HUBB</t>
+          <t>COHR</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>64.67</v>
+        <v>61.51</v>
       </c>
       <c r="D93" t="inlineStr">
         <is>
@@ -4089,16 +4087,16 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>MRVL</t>
+          <t>ZS</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
+          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>64.47</v>
+        <v>61.4</v>
       </c>
       <c r="D94" t="inlineStr">
         <is>
@@ -4120,16 +4118,16 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>AMKR</t>
+          <t>INTU</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / OSAT &amp; advanced packaging</t>
+          <t>10 Models, Software &amp; Applications / Financial software</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>64.31999999999999</v>
+        <v>61.37</v>
       </c>
       <c r="D95" t="inlineStr">
         <is>
@@ -4151,7 +4149,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>ETN</t>
+          <t>MTZ</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -4160,7 +4158,7 @@
         </is>
       </c>
       <c r="C96" t="n">
-        <v>64.3</v>
+        <v>61.04</v>
       </c>
       <c r="D96" t="inlineStr">
         <is>
@@ -4182,16 +4180,16 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>SMCI</t>
+          <t>IRM</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>64.25</v>
+        <v>60.96</v>
       </c>
       <c r="D97" t="inlineStr">
         <is>
@@ -4213,16 +4211,16 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>LITE</t>
+          <t>SMCI</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>64.17</v>
+        <v>60.73</v>
       </c>
       <c r="D98" t="inlineStr">
         <is>
@@ -4244,16 +4242,16 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>HIVE</t>
+          <t>TXN</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
+          <t>06 AI Compute Silicon / Analog &amp; embedded (power management)</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>64.05</v>
+        <v>60.59</v>
       </c>
       <c r="D99" t="inlineStr">
         <is>
@@ -4275,16 +4273,16 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>IRM</t>
+          <t>TEL</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>63.75</v>
+        <v>60.55</v>
       </c>
       <c r="D100" t="inlineStr">
         <is>
@@ -4306,16 +4304,16 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>SNOW</t>
+          <t>ASX</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications</t>
+          <t>04 Semiconductor Equipment &amp; Materials / OSAT &amp; advanced packaging</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>63.57</v>
+        <v>60.46</v>
       </c>
       <c r="D101" t="inlineStr">
         <is>
@@ -4337,16 +4335,16 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>CMI</t>
+          <t>PATH</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>01 Power Generation / Distributed / on-site power</t>
+          <t>10 Models, Software &amp; Applications / AI-powered automation</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>63.3</v>
+        <v>60.04</v>
       </c>
       <c r="D102" t="inlineStr">
         <is>
@@ -4368,16 +4366,16 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>KLIC</t>
+          <t>GNRC</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>01 Power Generation / Distributed / on-site power</t>
         </is>
       </c>
       <c r="C103" t="n">
-        <v>63.17</v>
+        <v>59.98</v>
       </c>
       <c r="D103" t="inlineStr">
         <is>
@@ -4399,16 +4397,16 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>FLEX</t>
+          <t>BWXT</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Contract manufacturing / ODMs</t>
+          <t>01 Power Generation / Nuclear-specific</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>63.05</v>
+        <v>59.95</v>
       </c>
       <c r="D104" t="inlineStr">
         <is>
@@ -4430,16 +4428,16 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>KN</t>
+          <t>KLIC</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>04 Semi Equip - Materials</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>62.7</v>
+        <v>59.44</v>
       </c>
       <c r="D105" t="inlineStr">
         <is>
@@ -4461,16 +4459,16 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>CRWV</t>
+          <t>AMKR</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>09 Cloud - Neocloud</t>
+          <t>04 Semiconductor Equipment &amp; Materials / OSAT &amp; advanced packaging</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>62.67</v>
+        <v>59.15</v>
       </c>
       <c r="D106" t="inlineStr">
         <is>
@@ -4492,16 +4490,16 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>SEI</t>
+          <t>GFS</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>01 Power Generation / Distributed / on-site power</t>
+          <t>05 Fabs &amp; Foundries</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>62.55</v>
+        <v>59.05</v>
       </c>
       <c r="D107" t="inlineStr">
         <is>
@@ -4523,16 +4521,16 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>AAPL</t>
+          <t>FLEX</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / Edge AI platforms</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Contract manufacturing / ODMs</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>62.2</v>
+        <v>58.83</v>
       </c>
       <c r="D108" t="inlineStr">
         <is>
@@ -4554,16 +4552,16 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>NBIS</t>
+          <t>IREN</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Neoclouds (AI-native cloud providers)</t>
+          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
         </is>
       </c>
       <c r="C109" t="n">
-        <v>61.82</v>
+        <v>58.78</v>
       </c>
       <c r="D109" t="inlineStr">
         <is>
@@ -4580,25 +4578,21 @@
         </is>
       </c>
       <c r="H109" t="inlineStr"/>
-      <c r="J109" t="inlineStr">
-        <is>
-          <t>Removed 2026-05-25: dropped to ✓ (65.5) after reweight. Value 7.5 penalized by higher Value weight.</t>
-        </is>
-      </c>
+      <c r="J109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>FTNT</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
+          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
         </is>
       </c>
       <c r="C110" t="n">
-        <v>61.65</v>
+        <v>58.62</v>
       </c>
       <c r="D110" t="inlineStr">
         <is>
@@ -4620,16 +4614,16 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>CRWD</t>
+          <t>TTMI</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
+          <t>04 Semiconductor Equipment &amp; Materials / PCB / substrates</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>61.65</v>
+        <v>58.26</v>
       </c>
       <c r="D111" t="inlineStr">
         <is>
@@ -4651,16 +4645,16 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>BWXT</t>
+          <t>KN</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>01 Power Generation / Nuclear-specific</t>
+          <t>04 Semi Equip - Materials</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>61.58</v>
+        <v>58.22</v>
       </c>
       <c r="D112" t="inlineStr">
         <is>
@@ -4682,16 +4676,16 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>COHR</t>
+          <t>CARR</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C113" t="n">
-        <v>61.55</v>
+        <v>57.92</v>
       </c>
       <c r="D113" t="inlineStr">
         <is>
@@ -4713,16 +4707,16 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>NXPI</t>
+          <t>DUK</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Analog &amp; embedded (auto/edge AI)</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>61.4</v>
+        <v>57.67</v>
       </c>
       <c r="D114" t="inlineStr">
         <is>
@@ -4744,16 +4738,16 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>MDB</t>
+          <t>EQIX</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI data layer</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>61.32</v>
+        <v>57.57</v>
       </c>
       <c r="D115" t="inlineStr">
         <is>
@@ -4775,16 +4769,16 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>HUT</t>
+          <t>MRVL</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
+          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>61.2</v>
+        <v>57.37</v>
       </c>
       <c r="D116" t="inlineStr">
         <is>
@@ -4806,16 +4800,16 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>ATKR</t>
+          <t>SEI</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>01 Power Generation / Distributed / on-site power</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>61.15</v>
+        <v>57.09</v>
       </c>
       <c r="D117" t="inlineStr">
         <is>
@@ -4837,16 +4831,16 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>EQIX</t>
+          <t>CAMT</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>61</v>
+        <v>56.96</v>
       </c>
       <c r="D118" t="inlineStr">
         <is>
@@ -4868,16 +4862,16 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>GFS</t>
+          <t>AEP</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>05 Fabs &amp; Foundries</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C119" t="n">
-        <v>60.7</v>
+        <v>56.23</v>
       </c>
       <c r="D119" t="inlineStr">
         <is>
@@ -4899,16 +4893,16 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>TTMI</t>
+          <t>P</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / PCB / substrates</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>60.45</v>
+        <v>56.23</v>
       </c>
       <c r="D120" t="inlineStr">
         <is>
@@ -4930,16 +4924,16 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>DUK</t>
+          <t>WYFI</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>09 Compute-as-a-Service / Neoclouds (AI-native cloud providers)</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>60.1</v>
+        <v>55.62</v>
       </c>
       <c r="D121" t="inlineStr">
         <is>
@@ -4961,16 +4955,16 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>ATKR</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>59.1</v>
+        <v>55.03</v>
       </c>
       <c r="D122" t="inlineStr">
         <is>
@@ -4988,502 +4982,6 @@
       </c>
       <c r="H122" t="inlineStr"/>
       <c r="J122" t="inlineStr"/>
-    </row>
-    <row r="123">
-      <c r="A123" t="inlineStr">
-        <is>
-          <t>CAMT</t>
-        </is>
-      </c>
-      <c r="B123" t="inlineStr">
-        <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
-        </is>
-      </c>
-      <c r="C123" t="n">
-        <v>59.05</v>
-      </c>
-      <c r="D123" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E123" t="n">
-        <v>121</v>
-      </c>
-      <c r="F123" t="inlineStr"/>
-      <c r="G123" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H123" t="inlineStr"/>
-      <c r="J123" t="inlineStr"/>
-    </row>
-    <row r="124">
-      <c r="A124" t="inlineStr">
-        <is>
-          <t>CARR</t>
-        </is>
-      </c>
-      <c r="B124" t="inlineStr">
-        <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
-        </is>
-      </c>
-      <c r="C124" t="n">
-        <v>59</v>
-      </c>
-      <c r="D124" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E124" t="n">
-        <v>122</v>
-      </c>
-      <c r="F124" t="inlineStr"/>
-      <c r="G124" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H124" t="inlineStr"/>
-      <c r="J124" t="inlineStr"/>
-    </row>
-    <row r="125">
-      <c r="A125" t="inlineStr">
-        <is>
-          <t>QCOM</t>
-        </is>
-      </c>
-      <c r="B125" t="inlineStr">
-        <is>
-          <t>06 AI Compute Silicon / Application processors &amp; connectivity (edge AI)</t>
-        </is>
-      </c>
-      <c r="C125" t="n">
-        <v>59</v>
-      </c>
-      <c r="D125" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E125" t="n">
-        <v>123</v>
-      </c>
-      <c r="F125" t="inlineStr"/>
-      <c r="G125" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H125" t="inlineStr"/>
-      <c r="J125" t="inlineStr"/>
-    </row>
-    <row r="126">
-      <c r="A126" t="inlineStr">
-        <is>
-          <t>AEP</t>
-        </is>
-      </c>
-      <c r="B126" t="inlineStr">
-        <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
-        </is>
-      </c>
-      <c r="C126" t="n">
-        <v>58.77</v>
-      </c>
-      <c r="D126" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E126" t="n">
-        <v>124</v>
-      </c>
-      <c r="F126" t="inlineStr"/>
-      <c r="G126" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H126" t="inlineStr"/>
-      <c r="J126" t="inlineStr"/>
-    </row>
-    <row r="127">
-      <c r="A127" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="B127" t="inlineStr">
-        <is>
-          <t>06 AI Compute Silicon / Power management silicon (SiC/GaN)</t>
-        </is>
-      </c>
-      <c r="C127" t="n">
-        <v>58.52</v>
-      </c>
-      <c r="D127" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E127" t="n">
-        <v>125</v>
-      </c>
-      <c r="F127" t="inlineStr"/>
-      <c r="G127" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H127" t="inlineStr"/>
-      <c r="J127" t="inlineStr"/>
-    </row>
-    <row r="128">
-      <c r="A128" t="inlineStr">
-        <is>
-          <t>PPL</t>
-        </is>
-      </c>
-      <c r="B128" t="inlineStr">
-        <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
-        </is>
-      </c>
-      <c r="C128" t="n">
-        <v>58.38</v>
-      </c>
-      <c r="D128" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E128" t="n">
-        <v>126</v>
-      </c>
-      <c r="F128" t="inlineStr"/>
-      <c r="G128" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H128" t="inlineStr"/>
-      <c r="J128" t="inlineStr"/>
-    </row>
-    <row r="129">
-      <c r="A129" t="inlineStr">
-        <is>
-          <t>TEM</t>
-        </is>
-      </c>
-      <c r="B129" t="inlineStr">
-        <is>
-          <t>10 Models, Software &amp; Applications / AI-native vertical applications</t>
-        </is>
-      </c>
-      <c r="C129" t="n">
-        <v>58</v>
-      </c>
-      <c r="D129" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E129" t="n">
-        <v>127</v>
-      </c>
-      <c r="F129" t="inlineStr"/>
-      <c r="G129" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H129" t="inlineStr"/>
-      <c r="J129" t="inlineStr"/>
-    </row>
-    <row r="130">
-      <c r="A130" t="inlineStr">
-        <is>
-          <t>ACLS</t>
-        </is>
-      </c>
-      <c r="B130" t="inlineStr">
-        <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
-        </is>
-      </c>
-      <c r="C130" t="n">
-        <v>57.32</v>
-      </c>
-      <c r="D130" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E130" t="n">
-        <v>128</v>
-      </c>
-      <c r="F130" t="inlineStr"/>
-      <c r="G130" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H130" t="inlineStr"/>
-      <c r="J130" t="inlineStr"/>
-    </row>
-    <row r="131">
-      <c r="A131" t="inlineStr">
-        <is>
-          <t>IREN</t>
-        </is>
-      </c>
-      <c r="B131" t="inlineStr">
-        <is>
-          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
-        </is>
-      </c>
-      <c r="C131" t="n">
-        <v>57.12</v>
-      </c>
-      <c r="D131" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E131" t="n">
-        <v>129</v>
-      </c>
-      <c r="F131" t="inlineStr"/>
-      <c r="G131" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H131" t="inlineStr"/>
-      <c r="J131" t="inlineStr"/>
-    </row>
-    <row r="132">
-      <c r="A132" t="inlineStr">
-        <is>
-          <t>XEL</t>
-        </is>
-      </c>
-      <c r="B132" t="inlineStr">
-        <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
-        </is>
-      </c>
-      <c r="C132" t="n">
-        <v>57.05</v>
-      </c>
-      <c r="D132" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E132" t="n">
-        <v>130</v>
-      </c>
-      <c r="F132" t="inlineStr"/>
-      <c r="G132" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H132" t="inlineStr"/>
-      <c r="J132" t="inlineStr"/>
-    </row>
-    <row r="133">
-      <c r="A133" t="inlineStr">
-        <is>
-          <t>COHU</t>
-        </is>
-      </c>
-      <c r="B133" t="inlineStr">
-        <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
-        </is>
-      </c>
-      <c r="C133" t="n">
-        <v>57</v>
-      </c>
-      <c r="D133" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E133" t="n">
-        <v>131</v>
-      </c>
-      <c r="F133" t="inlineStr"/>
-      <c r="G133" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H133" t="inlineStr"/>
-      <c r="J133" t="inlineStr"/>
-    </row>
-    <row r="134">
-      <c r="A134" t="inlineStr">
-        <is>
-          <t>WYFI</t>
-        </is>
-      </c>
-      <c r="B134" t="inlineStr">
-        <is>
-          <t>09 Compute-as-a-Service / Neoclouds (AI-native cloud providers)</t>
-        </is>
-      </c>
-      <c r="C134" t="n">
-        <v>56.88</v>
-      </c>
-      <c r="D134" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E134" t="n">
-        <v>132</v>
-      </c>
-      <c r="F134" t="inlineStr"/>
-      <c r="G134" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H134" t="inlineStr"/>
-      <c r="J134" t="inlineStr"/>
-    </row>
-    <row r="135">
-      <c r="A135" t="inlineStr">
-        <is>
-          <t>PSIX</t>
-        </is>
-      </c>
-      <c r="B135" t="inlineStr">
-        <is>
-          <t>01 Power Generation / Distributed / on-site power</t>
-        </is>
-      </c>
-      <c r="C135" t="n">
-        <v>56.35</v>
-      </c>
-      <c r="D135" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E135" t="n">
-        <v>133</v>
-      </c>
-      <c r="F135" t="inlineStr"/>
-      <c r="G135" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H135" t="inlineStr"/>
-      <c r="J135" t="inlineStr"/>
-    </row>
-    <row r="136">
-      <c r="A136" t="inlineStr">
-        <is>
-          <t>ETR</t>
-        </is>
-      </c>
-      <c r="B136" t="inlineStr">
-        <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
-        </is>
-      </c>
-      <c r="C136" t="n">
-        <v>56.15</v>
-      </c>
-      <c r="D136" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E136" t="n">
-        <v>134</v>
-      </c>
-      <c r="F136" t="inlineStr"/>
-      <c r="G136" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H136" t="inlineStr"/>
-      <c r="J136" t="inlineStr"/>
-    </row>
-    <row r="137">
-      <c r="A137" t="inlineStr">
-        <is>
-          <t>TOELY</t>
-        </is>
-      </c>
-      <c r="B137" t="inlineStr">
-        <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
-        </is>
-      </c>
-      <c r="C137" t="n">
-        <v>55.92</v>
-      </c>
-      <c r="D137" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E137" t="n">
-        <v>135</v>
-      </c>
-      <c r="F137" t="inlineStr"/>
-      <c r="G137" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H137" t="inlineStr"/>
-      <c r="J137" t="inlineStr"/>
-    </row>
-    <row r="138">
-      <c r="A138" t="inlineStr">
-        <is>
-          <t>SO</t>
-        </is>
-      </c>
-      <c r="B138" t="inlineStr">
-        <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
-        </is>
-      </c>
-      <c r="C138" t="n">
-        <v>55.33</v>
-      </c>
-      <c r="D138" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="E138" t="n">
-        <v>136</v>
-      </c>
-      <c r="F138" t="inlineStr"/>
-      <c r="G138" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="H138" t="inlineStr"/>
-      <c r="J138" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
chore(data): full objective refresh 2026-07-16 (173 names) after AI selloff
- refresh_objective_inputs.py all: Value/Quality/Growth inputs + 50DMA %
  rewritten for every Watchlist row; EPS YoY >=300% withheld per rule 15
  (13 names pending filing verification), documented blanks preserved
- refresh_reverse_dcf.py: EV/FCF refreshed (112 with value, 61 blank)
- recalc --sync: cohort-relative J/O resynced; NVDA tier crossing
  85.1 (3-check) -> 84.4 (2-check) fired freeze-safe rebalance -- membership
  unchanged (12 holds, no entry/exit band crossings), NVDA 12.0% -> 11.8%
- cohort map non-null counts updated (ABBNY EV/EBITDA blanked: no
  yfinance EBITDA; ASML ND/EBITDA likewise) -- no pct/abs eligibility flips
- gates: portfolio sizing, reweight gate, cohort drift, site privacy all pass

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/00-master/portfolio.xlsx
+++ b/00-master/portfolio.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Sizing Rules" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Targets" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sizing Rules" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Targets" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -676,7 +676,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-07-02 (refresh_targets.py — hysteresis pipeline)</t>
+          <t>2026-07-16 (refresh_targets.py — hysteresis pipeline)</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J123"/>
+  <dimension ref="A1:J124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1068,7 +1068,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Target Portfolio (refreshed 2026-07-02, live Watchlist scores)</t>
+          <t>Target Portfolio (refreshed 2026-07-16, live Watchlist scores)</t>
         </is>
       </c>
     </row>
@@ -1136,11 +1136,11 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>85.06</v>
+        <v>84.39</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>✓✓✓</t>
+          <t>✓✓</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -1158,23 +1158,23 @@
       </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="n">
-        <v>12</v>
+        <v>11.76</v>
       </c>
       <c r="J3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>MU</t>
+          <t>TSM</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>06 Silicon - Memory</t>
+          <t>05 Fabs &amp; Foundries</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>84.81</v>
+        <v>82.25</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -1196,23 +1196,23 @@
       </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="n">
-        <v>11.46</v>
+        <v>10.55</v>
       </c>
       <c r="J4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>TSM</t>
+          <t>MU</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>05 Fabs &amp; Foundries</t>
+          <t>06 Silicon - Memory</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>82.42</v>
+        <v>80.64</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -1234,23 +1234,23 @@
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="n">
-        <v>10.17</v>
+        <v>9.640000000000001</v>
       </c>
       <c r="J5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ANET</t>
+          <t>CRDO</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
+          <t>07 Optical, Networking &amp; Interconnect / Connectivity ASICs</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>79.34999999999999</v>
+        <v>79.72</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -1272,9 +1272,13 @@
       </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="n">
-        <v>8.51</v>
-      </c>
-      <c r="J6" t="inlineStr"/>
+        <v>9.119999999999999</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Added 2026-05-25: score 78.4, ranked #4 in reweighted watchlist. Optical connectivity pure-play.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1288,7 +1292,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>79.14</v>
+        <v>78.3</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -1310,23 +1314,23 @@
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="n">
-        <v>8.4</v>
+        <v>8.32</v>
       </c>
       <c r="J7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CRDO</t>
+          <t>ANET</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Connectivity ASICs</t>
+          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>78.22</v>
+        <v>78.23999999999999</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -1348,13 +1352,9 @@
       </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="n">
-        <v>7.9</v>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>Added 2026-05-25: score 78.4, ranked #4 in reweighted watchlist. Optical connectivity pure-play.</t>
-        </is>
-      </c>
+        <v>8.289999999999999</v>
+      </c>
+      <c r="J8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1368,7 +1368,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>77.88</v>
+        <v>77.05</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -1390,7 +1390,7 @@
       </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="n">
-        <v>7.72</v>
+        <v>7.61</v>
       </c>
       <c r="J9" t="inlineStr"/>
     </row>
@@ -1406,7 +1406,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>77.66</v>
+        <v>76.86</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -1428,23 +1428,23 @@
       </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="n">
-        <v>7.6</v>
+        <v>7.51</v>
       </c>
       <c r="J10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>SNDK</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
+          <t>06 AI Compute Silicon / Memory (HBM is the bottleneck)</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>77.11</v>
+        <v>76.11</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -1466,14 +1466,18 @@
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="n">
-        <v>7.31</v>
-      </c>
-      <c r="J11" t="inlineStr"/>
+        <v>7.09</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Manually excluded 2026-05-18: $1,333 share price prevents capital-efficient sizing below ~$25k. Conscious framework override (target ~$10k portfolio). | Override removed 2026-06-09: fractional shares adopted, share-price constraint obsolete (Dom decision).</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1482,7 +1486,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>75.64</v>
+        <v>75.95</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -1504,23 +1508,23 @@
       </c>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="n">
-        <v>6.51</v>
+        <v>6.99</v>
       </c>
       <c r="J12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>SNDK</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Memory (HBM is the bottleneck)</t>
+          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>75.11</v>
+        <v>75.26000000000001</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -1542,18 +1546,14 @@
       </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="n">
-        <v>6.23</v>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>Manually excluded 2026-05-18: $1,333 share price prevents capital-efficient sizing below ~$25k. Conscious framework override (target ~$10k portfolio). | Override removed 2026-06-09: fractional shares adopted, share-price constraint obsolete (Dom decision).</t>
-        </is>
-      </c>
+        <v>6.6</v>
+      </c>
+      <c r="J13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>FIX</t>
+          <t>EME</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1562,7 +1562,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>75.08</v>
+        <v>75.09</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -1572,30 +1572,23 @@
       <c r="E14" t="n">
         <v>12</v>
       </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>HOLD</t>
-        </is>
-      </c>
+      <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H14" t="inlineStr"/>
-      <c r="I14" t="n">
-        <v>6.21</v>
-      </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Manually excluded 2026-05-18: $1,854 share price prevents reasonable position sizing below ~$50k portfolio. Conscious framework override. | Override removed 2026-06-09: fractional shares adopted, share-price constraint obsolete (Dom decision).</t>
+          <t>Added 2026-05-25: score 75.2, DC construction, strong momentum (86.7).</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>EME</t>
+          <t>FIX</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1604,7 +1597,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>74.67</v>
+        <v>75.08</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -1614,16 +1607,23 @@
       <c r="E15" t="n">
         <v>13</v>
       </c>
-      <c r="F15" t="inlineStr"/>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>HOLD</t>
+        </is>
+      </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H15" t="inlineStr"/>
+      <c r="I15" t="n">
+        <v>6.5</v>
+      </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Added 2026-05-25: score 75.2, DC construction, strong momentum (86.7).</t>
+          <t>Manually excluded 2026-05-18: $1,854 share price prevents reasonable position sizing below ~$50k portfolio. Conscious framework override. | Override removed 2026-06-09: fractional shares adopted, share-price constraint obsolete (Dom decision).</t>
         </is>
       </c>
     </row>
@@ -1639,7 +1639,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>73.83</v>
+        <v>73.58</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -1661,16 +1661,16 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>RDDT</t>
+          <t>ALAB</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI advertising</t>
+          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>73.62</v>
+        <v>73.25</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -1692,16 +1692,16 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ALAB</t>
+          <t>APP</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
+          <t>10 Models, Software &amp; Applications / AI advertising</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>72.75</v>
+        <v>72.70999999999999</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -1711,11 +1711,7 @@
       <c r="E18" t="n">
         <v>16</v>
       </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>EXIT (resize, score 72.7 &lt; 74.5)</t>
-        </is>
-      </c>
+      <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
           <t>N</t>
@@ -1727,7 +1723,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>APP</t>
+          <t>RDDT</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1736,7 +1732,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>72.56999999999999</v>
+        <v>72.54000000000001</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -1758,16 +1754,16 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>PLTR</t>
+          <t>TER</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>71.01000000000001</v>
+        <v>71.7</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -1798,7 +1794,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>70.56</v>
+        <v>70.78</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -1820,16 +1816,16 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>EQT</t>
+          <t>WDC</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>70.43000000000001</v>
+        <v>70.77</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -1860,7 +1856,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>70.40000000000001</v>
+        <v>70.65000000000001</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -1882,16 +1878,16 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>WDC</t>
+          <t>EQT</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
+          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>70.17</v>
+        <v>70.33</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -1913,16 +1909,16 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>TER</t>
+          <t>PLTR</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>10 Models, Software &amp; Applications</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>70.08</v>
+        <v>70.22</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -1953,11 +1949,11 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>70.01000000000001</v>
+        <v>69.54000000000001</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>✓✓</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="E26" t="n">
@@ -1984,7 +1980,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>69.67</v>
+        <v>69.25</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -2006,16 +2002,16 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>CIEN</t>
+          <t>AR</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
+          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>69.47</v>
+        <v>69.23</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -2032,21 +2028,25 @@
         </is>
       </c>
       <c r="H28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>Added 2026-05-22 as substitute for CTRA (delisted). Pure score-driven pick: next-best ✓✓ at 75.62, same Layer 1 NG E&amp;P sub-category — preserves natural gas thesis concentration.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>HTHIY</t>
+          <t>CIEN</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>69.25</v>
+        <v>69.22</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -2068,16 +2068,16 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>FN</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
+          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>69.23</v>
+        <v>69.17</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
@@ -2094,25 +2094,21 @@
         </is>
       </c>
       <c r="H30" t="inlineStr"/>
-      <c r="J30" t="inlineStr">
-        <is>
-          <t>Added 2026-05-22 as substitute for CTRA (delisted). Pure score-driven pick: next-best ✓✓ at 75.62, same Layer 1 NG E&amp;P sub-category — preserves natural gas thesis concentration.</t>
-        </is>
-      </c>
+      <c r="J30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>FN</t>
+          <t>ARM</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
+          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>68.70999999999999</v>
+        <v>69.12</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -2134,16 +2130,16 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>ARM</t>
+          <t>ORCL</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
+          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>68.62</v>
+        <v>69.09</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -2174,7 +2170,7 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>68.51000000000001</v>
+        <v>68.73</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -2196,16 +2192,16 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>ORCL</t>
+          <t>GLW</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
+          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>68.19</v>
+        <v>68.52</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -2227,16 +2223,16 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>GLW</t>
+          <t>DELL</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>68.02</v>
+        <v>68.25</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
@@ -2258,16 +2254,16 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>AMD</t>
+          <t>HTHIY</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / GPUs / merchant accelerators</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>67.83</v>
+        <v>68.23</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
@@ -2284,25 +2280,21 @@
         </is>
       </c>
       <c r="H36" t="inlineStr"/>
-      <c r="J36" t="inlineStr">
-        <is>
-          <t>Removed 2026-05-25: score 74.1 fell below natural 17-name cutoff (ARM 74.2). First name out.</t>
-        </is>
-      </c>
+      <c r="J36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>DELL</t>
+          <t>TT</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>67.75</v>
+        <v>67.53</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
@@ -2324,12 +2316,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>TT</t>
+          <t>RRC</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -2355,16 +2347,16 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>RRC</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
+          <t>06 AI Compute Silicon / GPUs / merchant accelerators</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>67.45</v>
+        <v>67.48999999999999</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -2381,21 +2373,25 @@
         </is>
       </c>
       <c r="H39" t="inlineStr"/>
-      <c r="J39" t="inlineStr"/>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>Removed 2026-05-25: score 74.1 fell below natural 17-name cutoff (ARM 74.2). First name out.</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>ADSK</t>
+          <t>CSCO</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / Design &amp; engineering software</t>
+          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>67.23999999999999</v>
+        <v>67.42</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -2417,16 +2413,16 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>EXE</t>
+          <t>STX</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>67.20999999999999</v>
+        <v>67.38</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -2448,16 +2444,16 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>SNPS</t>
+          <t>EXE</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
+          <t>01 Power Generation / Natural gas E&amp;P (powering gas turbines for data centers)</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>67.01000000000001</v>
+        <v>67.20999999999999</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
@@ -2479,16 +2475,16 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>DLR</t>
+          <t>LRCX</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>66.97</v>
+        <v>66.98999999999999</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
@@ -2510,16 +2506,16 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>STX</t>
+          <t>PLAB</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>66.88</v>
+        <v>66.86</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -2541,16 +2537,16 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>PLAB</t>
+          <t>ADSK</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
+          <t>10 Models, Software &amp; Applications / Design &amp; engineering software</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>66.56999999999999</v>
+        <v>66.8</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
@@ -2572,7 +2568,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>ABBNY</t>
+          <t>POWL</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2581,7 +2577,7 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>66.45999999999999</v>
+        <v>66.7</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -2603,16 +2599,16 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>KLAC</t>
+          <t>SNPS</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>66.27</v>
+        <v>66.64</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -2634,16 +2630,16 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>ASML</t>
+          <t>DLR</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>66.16</v>
+        <v>66.61</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -2665,16 +2661,16 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>CSCO</t>
+          <t>MOD</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>66.11</v>
+        <v>66.61</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
@@ -2696,16 +2692,16 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>LRCX</t>
+          <t>HIVE</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>66.09</v>
+        <v>66.25</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
@@ -2727,16 +2723,16 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>CDNS</t>
+          <t>SBGSY</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>66.09</v>
+        <v>66.14</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
@@ -2758,16 +2754,16 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>POWL</t>
+          <t>ONTO</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>65.55</v>
+        <v>66.04000000000001</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
@@ -2789,7 +2785,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>BESIY</t>
+          <t>KLAC</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2798,7 +2794,7 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>65.33</v>
+        <v>66.02</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
@@ -2820,16 +2816,16 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>MOD</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>01 Power - Distributed</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>65.17</v>
+        <v>65.87</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
@@ -2851,16 +2847,16 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>SBGSY</t>
+          <t>CDNS</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>04 Semiconductor Equipment &amp; Materials / EDA &amp; IP</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>65.09</v>
+        <v>65.79000000000001</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
@@ -2882,16 +2878,16 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>ADI</t>
+          <t>AEIS</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Analog &amp; mixed-signal (signal chain + power)</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>65.08</v>
+        <v>65.65000000000001</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
@@ -2913,16 +2909,16 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>ONTO</t>
+          <t>LSCC</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>06 AI Compute Silicon / Programmable logic</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>65.06999999999999</v>
+        <v>65.33</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
@@ -2944,16 +2940,16 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>PWR</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>01 Power - Distributed</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>65.03</v>
+        <v>65.23</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
@@ -2975,16 +2971,16 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>LSCC</t>
+          <t>BESIY</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Programmable logic</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>65</v>
+        <v>65.08</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
@@ -3006,16 +3002,16 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>CRWV</t>
+          <t>HOOD</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>09 Cloud - Neocloud</t>
+          <t>10 Models, Software &amp; Applications / Consumer fintech (AI adopter)</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>64.91</v>
+        <v>65.05</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
@@ -3037,16 +3033,16 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>PWR</t>
+          <t>CRWV</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>09 Cloud - Neocloud</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>64.84</v>
+        <v>65.03</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
@@ -3068,16 +3064,16 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>CRM</t>
+          <t>ADI</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications</t>
+          <t>06 AI Compute Silicon / Analog &amp; mixed-signal (signal chain + power)</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>64.83</v>
+        <v>65</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
@@ -3094,11 +3090,7 @@
         </is>
       </c>
       <c r="H62" t="inlineStr"/>
-      <c r="J62" t="inlineStr">
-        <is>
-          <t>Added 2026-05-25: score 74.8, Quality 97, PEG 0.8. Enterprise SaaS with AI exposure.</t>
-        </is>
-      </c>
+      <c r="J62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -3134,16 +3126,16 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>HIVE</t>
+          <t>HUBB</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>64.75</v>
+        <v>64.38</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
@@ -3174,7 +3166,7 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>64.68000000000001</v>
+        <v>64.31</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
@@ -3196,16 +3188,16 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>TSEM</t>
+          <t>CRM</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>05 Fabs &amp; Foundries</t>
+          <t>10 Models, Software &amp; Applications</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>64.20999999999999</v>
+        <v>64.29000000000001</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
@@ -3222,12 +3214,16 @@
         </is>
       </c>
       <c r="H66" t="inlineStr"/>
-      <c r="J66" t="inlineStr"/>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>Added 2026-05-25: score 74.8, Quality 97, PEG 0.8. Enterprise SaaS with AI exposure.</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>AEIS</t>
+          <t>MKSI</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -3236,7 +3232,7 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>64.14</v>
+        <v>64.28</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
@@ -3258,16 +3254,16 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>AAON</t>
+          <t>NBIS</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>09 Compute-as-a-Service / Neoclouds (AI-native cloud providers)</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>63.96</v>
+        <v>64.12</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
@@ -3284,21 +3280,25 @@
         </is>
       </c>
       <c r="H68" t="inlineStr"/>
-      <c r="J68" t="inlineStr"/>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>Removed 2026-05-25: dropped to ✓ (65.5) after reweight. Value 7.5 penalized by higher Value weight.</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>MKSI</t>
+          <t>ETN</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>63.91</v>
+        <v>64.06999999999999</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
@@ -3320,16 +3320,16 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>HUBB</t>
+          <t>TSEM</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>05 Fabs &amp; Foundries</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>63.88</v>
+        <v>63.96</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
@@ -3351,16 +3351,16 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>NBIS</t>
+          <t>AAON</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Neoclouds (AI-native cloud providers)</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>63.88</v>
+        <v>63.82</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
@@ -3377,25 +3377,21 @@
         </is>
       </c>
       <c r="H71" t="inlineStr"/>
-      <c r="J71" t="inlineStr">
-        <is>
-          <t>Removed 2026-05-25: dropped to ✓ (65.5) after reweight. Value 7.5 penalized by higher Value weight.</t>
-        </is>
-      </c>
+      <c r="J71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>NEE</t>
+          <t>DDOG</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>10 Models, Software &amp; Applications / AI observability &amp; infrastructure software</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>63.85</v>
+        <v>63.51</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
@@ -3412,21 +3408,25 @@
         </is>
       </c>
       <c r="H72" t="inlineStr"/>
-      <c r="J72" t="inlineStr"/>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>Added 2026-05-25: score 75.4, Quality 100, PEG 0.7. Beats 4 existing portfolio names.</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>ETN</t>
+          <t>ENTG</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>63.82</v>
+        <v>63.3</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
@@ -3457,7 +3457,7 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>63.6</v>
+        <v>63.25</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
@@ -3479,16 +3479,16 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>DDOG</t>
+          <t>NVT</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI observability &amp; infrastructure software</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>63.6</v>
+        <v>63.2</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
@@ -3505,11 +3505,7 @@
         </is>
       </c>
       <c r="H75" t="inlineStr"/>
-      <c r="J75" t="inlineStr">
-        <is>
-          <t>Added 2026-05-25: score 75.4, Quality 100, PEG 0.7. Beats 4 existing portfolio names.</t>
-        </is>
-      </c>
+      <c r="J75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -3523,7 +3519,7 @@
         </is>
       </c>
       <c r="C76" t="n">
-        <v>63.51</v>
+        <v>63.14</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
@@ -3545,16 +3541,16 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>PANW</t>
+          <t>TLN</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
+          <t>01 Power Generation / Independent Power Producers (IPPs)</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>63.21</v>
+        <v>63.12</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
@@ -3576,16 +3572,16 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>UMC</t>
+          <t>COHR</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>05 Fabs &amp; Foundries</t>
+          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>63.17</v>
+        <v>63.09</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
@@ -3607,16 +3603,16 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>TLN</t>
+          <t>FORM</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>01 Power Generation / Independent Power Producers (IPPs)</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>63.12</v>
+        <v>63.04</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
@@ -3638,12 +3634,12 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>GEV</t>
+          <t>NEE</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>02 Grid Equipment</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -3669,16 +3665,16 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>CEG</t>
+          <t>LITE</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>01 Power - IPP / Nuclear</t>
+          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>62.85</v>
+        <v>63.02</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
@@ -3700,16 +3696,16 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>LITE</t>
+          <t>PANW</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
+          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>62.67</v>
+        <v>62.94</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
@@ -3731,16 +3727,16 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>NVT</t>
+          <t>CEG</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>01 Power - IPP / Nuclear</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>62.64</v>
+        <v>62.85</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
@@ -3762,16 +3758,16 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>HUT</t>
+          <t>GEV</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
+          <t>02 Grid Equipment</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>62.62</v>
+        <v>62.77</v>
       </c>
       <c r="D84" t="inlineStr">
         <is>
@@ -3793,16 +3789,16 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>FORM</t>
+          <t>UMC</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
+          <t>05 Fabs &amp; Foundries</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>62.61</v>
+        <v>62.62</v>
       </c>
       <c r="D85" t="inlineStr">
         <is>
@@ -3824,16 +3820,16 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>ENTG</t>
+          <t>CMI</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
+          <t>01 Power Generation / Distributed / on-site power</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>62.46</v>
+        <v>62.48</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
@@ -3855,16 +3851,16 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>MPWR</t>
+          <t>ABBNY</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Power management silicon</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>62.18</v>
+        <v>62.2</v>
       </c>
       <c r="D87" t="inlineStr">
         <is>
@@ -3886,16 +3882,16 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>ADBE</t>
+          <t>NXT</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / Creative &amp; design software</t>
+          <t>01 Power Generation / Solar &amp; renewables equipment (behind-the-meter DC power)</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>62.05</v>
+        <v>62.1</v>
       </c>
       <c r="D88" t="inlineStr">
         <is>
@@ -3917,16 +3913,16 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>HPE</t>
+          <t>MPWR</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling</t>
+          <t>06 AI Compute Silicon / Power management silicon</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>62</v>
+        <v>62.05</v>
       </c>
       <c r="D89" t="inlineStr">
         <is>
@@ -3948,16 +3944,16 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>NXT</t>
+          <t>GNRC</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>01 Power Generation / Solar &amp; renewables equipment (behind-the-meter DC power)</t>
+          <t>01 Power Generation / Distributed / on-site power</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>61.75</v>
+        <v>62.02</v>
       </c>
       <c r="D90" t="inlineStr">
         <is>
@@ -3979,16 +3975,16 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>CMI</t>
+          <t>HUT</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>01 Power Generation / Distributed / on-site power</t>
+          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>61.75</v>
+        <v>62</v>
       </c>
       <c r="D91" t="inlineStr">
         <is>
@@ -4010,16 +4006,16 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>NOW</t>
+          <t>ASML</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>61.59</v>
+        <v>61.84</v>
       </c>
       <c r="D92" t="inlineStr">
         <is>
@@ -4041,16 +4037,16 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>COHR</t>
+          <t>HPE</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>61.51</v>
+        <v>61.78</v>
       </c>
       <c r="D93" t="inlineStr">
         <is>
@@ -4072,16 +4068,16 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>INTU</t>
+          <t>GFS</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / Financial software</t>
+          <t>05 Fabs &amp; Foundries</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>61.37</v>
+        <v>61.75</v>
       </c>
       <c r="D94" t="inlineStr">
         <is>
@@ -4103,16 +4099,16 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>ZS</t>
+          <t>NOW</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
+          <t>10 Models, Software &amp; Applications</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>61</v>
+        <v>61.54</v>
       </c>
       <c r="D95" t="inlineStr">
         <is>
@@ -4143,7 +4139,7 @@
         </is>
       </c>
       <c r="C96" t="n">
-        <v>60.96</v>
+        <v>61.33</v>
       </c>
       <c r="D96" t="inlineStr">
         <is>
@@ -4165,16 +4161,16 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>SMCI</t>
+          <t>TTMI</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling</t>
+          <t>04 Semiconductor Equipment &amp; Materials / PCB / substrates</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>60.73</v>
+        <v>61.27</v>
       </c>
       <c r="D97" t="inlineStr">
         <is>
@@ -4196,16 +4192,16 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>TXN</t>
+          <t>SMCI</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Analog &amp; embedded (power management)</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>60.59</v>
+        <v>61.23</v>
       </c>
       <c r="D98" t="inlineStr">
         <is>
@@ -4227,16 +4223,16 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>TEL</t>
+          <t>ADBE</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
+          <t>10 Models, Software &amp; Applications / Creative &amp; design software</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>60.55</v>
+        <v>61.2</v>
       </c>
       <c r="D99" t="inlineStr">
         <is>
@@ -4258,16 +4254,16 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>TOELY</t>
+          <t>INTU</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>10 Models, Software &amp; Applications / Financial software</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>60.5</v>
+        <v>60.97</v>
       </c>
       <c r="D100" t="inlineStr">
         <is>
@@ -4289,16 +4285,16 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>MTZ</t>
+          <t>TXN</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>06 AI Compute Silicon / Analog &amp; embedded (power management)</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>60.37</v>
+        <v>60.75</v>
       </c>
       <c r="D101" t="inlineStr">
         <is>
@@ -4320,16 +4316,16 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>GNRC</t>
+          <t>MTZ</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>01 Power Generation / Distributed / on-site power</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>60.16</v>
+        <v>60.74</v>
       </c>
       <c r="D102" t="inlineStr">
         <is>
@@ -4351,16 +4347,16 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>BWXT</t>
+          <t>TEL</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>01 Power Generation / Nuclear-specific</t>
+          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
         </is>
       </c>
       <c r="C103" t="n">
-        <v>60.16</v>
+        <v>60.55</v>
       </c>
       <c r="D103" t="inlineStr">
         <is>
@@ -4382,16 +4378,16 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>PATH</t>
+          <t>KLIC</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI-powered automation</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>60.04</v>
+        <v>60.4</v>
       </c>
       <c r="D104" t="inlineStr">
         <is>
@@ -4413,16 +4409,16 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>KLIC</t>
+          <t>FLEX</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Contract manufacturing / ODMs</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>59.67</v>
+        <v>60.25</v>
       </c>
       <c r="D105" t="inlineStr">
         <is>
@@ -4444,16 +4440,16 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>AMKR</t>
+          <t>ZS</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / OSAT &amp; advanced packaging</t>
+          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>59.35</v>
+        <v>60.05</v>
       </c>
       <c r="D106" t="inlineStr">
         <is>
@@ -4475,16 +4471,16 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>GFS</t>
+          <t>AMKR</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>05 Fabs &amp; Foundries</t>
+          <t>04 Semiconductor Equipment &amp; Materials / OSAT &amp; advanced packaging</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>59.05</v>
+        <v>59.81</v>
       </c>
       <c r="D107" t="inlineStr">
         <is>
@@ -4506,16 +4502,16 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>FLEX</t>
+          <t>PATH</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Contract manufacturing / ODMs</t>
+          <t>10 Models, Software &amp; Applications / AI-powered automation</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>58.83</v>
+        <v>59.79</v>
       </c>
       <c r="D108" t="inlineStr">
         <is>
@@ -4537,16 +4533,16 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>IREN</t>
+          <t>BWXT</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
+          <t>01 Power Generation / Nuclear-specific</t>
         </is>
       </c>
       <c r="C109" t="n">
-        <v>58.78</v>
+        <v>59.78</v>
       </c>
       <c r="D109" t="inlineStr">
         <is>
@@ -4568,16 +4564,16 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>FTNT</t>
+          <t>MRVL</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
+          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
         </is>
       </c>
       <c r="C110" t="n">
-        <v>58.62</v>
+        <v>59.44</v>
       </c>
       <c r="D110" t="inlineStr">
         <is>
@@ -4599,16 +4595,16 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>TTMI</t>
+          <t>TOELY</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / PCB / substrates</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>58.24</v>
+        <v>59.26</v>
       </c>
       <c r="D111" t="inlineStr">
         <is>
@@ -4630,16 +4626,16 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>KN</t>
+          <t>IREN</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>04 Semi Equip - Materials</t>
+          <t>09 Compute-as-a-Service / Bitcoin miners pivoting to AI hosting</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>58.24</v>
+        <v>59.16</v>
       </c>
       <c r="D112" t="inlineStr">
         <is>
@@ -4661,16 +4657,16 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>CARR</t>
+          <t>ASX</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>04 Semiconductor Equipment &amp; Materials / OSAT &amp; advanced packaging</t>
         </is>
       </c>
       <c r="C113" t="n">
-        <v>57.92</v>
+        <v>58.59</v>
       </c>
       <c r="D113" t="inlineStr">
         <is>
@@ -4692,16 +4688,16 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>ASX</t>
+          <t>KN</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / OSAT &amp; advanced packaging</t>
+          <t>04 Semi Equip - Materials</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>57.8</v>
+        <v>58.37</v>
       </c>
       <c r="D114" t="inlineStr">
         <is>
@@ -4732,7 +4728,7 @@
         </is>
       </c>
       <c r="C115" t="n">
-        <v>57.74</v>
+        <v>58.1</v>
       </c>
       <c r="D115" t="inlineStr">
         <is>
@@ -4754,7 +4750,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>EQIX</t>
+          <t>CARR</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -4763,7 +4759,7 @@
         </is>
       </c>
       <c r="C116" t="n">
-        <v>57.57</v>
+        <v>57.92</v>
       </c>
       <c r="D116" t="inlineStr">
         <is>
@@ -4785,16 +4781,16 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>MRVL</t>
+          <t>SEI</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
+          <t>01 Power Generation / Distributed / on-site power</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>57.37</v>
+        <v>57.89</v>
       </c>
       <c r="D117" t="inlineStr">
         <is>
@@ -4816,16 +4812,16 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>SEI</t>
+          <t>EQIX</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>01 Power Generation / Distributed / on-site power</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>57.29</v>
+        <v>57.81</v>
       </c>
       <c r="D118" t="inlineStr">
         <is>
@@ -4847,16 +4843,16 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>CAMT</t>
+          <t>FTNT</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>10 Models, Software &amp; Applications / AI cybersecurity</t>
         </is>
       </c>
       <c r="C119" t="n">
-        <v>57.04</v>
+        <v>57.54</v>
       </c>
       <c r="D119" t="inlineStr">
         <is>
@@ -4878,16 +4874,16 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>AEP</t>
+          <t>CAMT</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>56.32</v>
+        <v>56.82</v>
       </c>
       <c r="D120" t="inlineStr">
         <is>
@@ -4909,16 +4905,16 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>P</t>
+          <t>WYFI</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
+          <t>09 Compute-as-a-Service / Neoclouds (AI-native cloud providers)</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>56.23</v>
+        <v>56.62</v>
       </c>
       <c r="D121" t="inlineStr">
         <is>
@@ -4940,16 +4936,16 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>WYFI</t>
+          <t>AEP</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Neoclouds (AI-native cloud providers)</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>55.62</v>
+        <v>56.43</v>
       </c>
       <c r="D122" t="inlineStr">
         <is>
@@ -4980,7 +4976,7 @@
         </is>
       </c>
       <c r="C123" t="n">
-        <v>55.39</v>
+        <v>56.19</v>
       </c>
       <c r="D123" t="inlineStr">
         <is>
@@ -4998,6 +4994,37 @@
       </c>
       <c r="H123" t="inlineStr"/>
       <c r="J123" t="inlineStr"/>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Storage infrastructure</t>
+        </is>
+      </c>
+      <c r="C124" t="n">
+        <v>55.73</v>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="E124" t="n">
+        <v>122</v>
+      </c>
+      <c r="F124" t="inlineStr"/>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr"/>
+      <c r="J124" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
feat(v2): APPLY migration — inverse-vol sizing + rank selection live (Dom-approved, spec A3)
One sizing_migration_invvol event (2026-08-07, $10,169): 13→16 positions
(+VRT +RDDT +ALAB via rank form), inverse-vol weights (GMED 9.3% top,
SNDK 3.0% floor-bound). Shadow bands + EW_ROSTER now logging; series and
site data rebuilt. Tests pinned to legacy modes for hermeticity.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/00-master/portfolio.xlsx
+++ b/00-master/portfolio.xlsx
@@ -676,7 +676,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-08-03 (refresh_targets.py — hysteresis pipeline)</t>
+          <t>2026-08-07 (refresh_targets.py — hysteresis pipeline)</t>
         </is>
       </c>
     </row>
@@ -939,7 +939,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -1068,7 +1068,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Target Portfolio (refreshed 2026-08-03, live Watchlist scores)</t>
+          <t>Target Portfolio (refreshed 2026-08-07, live Watchlist scores)</t>
         </is>
       </c>
     </row>
@@ -1136,7 +1136,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>84.33</v>
+        <v>84.02</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -1158,7 +1158,7 @@
       </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="n">
-        <v>10.83</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="J3" t="inlineStr"/>
     </row>
@@ -1196,7 +1196,7 @@
       </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="n">
-        <v>9.77</v>
+        <v>6.13</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
@@ -1238,7 +1238,7 @@
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="n">
-        <v>9.75</v>
+        <v>7.57</v>
       </c>
       <c r="J5" t="inlineStr"/>
     </row>
@@ -1254,7 +1254,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>80.69</v>
+        <v>80.76000000000001</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -1276,7 +1276,7 @@
       </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="n">
-        <v>8.93</v>
+        <v>3.37</v>
       </c>
       <c r="J6" t="inlineStr"/>
     </row>
@@ -1314,7 +1314,7 @@
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="n">
-        <v>8.42</v>
+        <v>3.65</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -1325,16 +1325,16 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ANET</t>
+          <t>SNDK</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
+          <t>06 AI Compute Silicon / Memory (HBM is the bottleneck)</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>78.23999999999999</v>
+        <v>79.05</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -1356,23 +1356,27 @@
       </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="n">
-        <v>7.65</v>
-      </c>
-      <c r="J8" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Manually excluded 2026-05-18: $1,333 share price prevents capital-efficient sizing below ~$25k. Conscious framework override (target ~$10k portfolio). | Override removed 2026-06-09: fractional shares adopted, share-price constraint obsolete (Dom decision).</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>ANET</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
+          <t>07 Optical, Networking &amp; Interconnect / Networking systems</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>77.78</v>
+        <v>78.81</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -1394,23 +1398,23 @@
       </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="n">
-        <v>7.41</v>
+        <v>6.4</v>
       </c>
       <c r="J9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>AVGO</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
+          <t>09 Compute-as-a-Service / Hyperscalers (public-cloud AI revenue)</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>77.16</v>
+        <v>77.78</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -1432,23 +1436,23 @@
       </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="n">
-        <v>7.09</v>
+        <v>8.1</v>
       </c>
       <c r="J10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>GMED</t>
+          <t>AVGO</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
+          <t>06 AI Compute Silicon / Custom silicon / ASIC designers</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>76.61</v>
+        <v>77.16</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -1460,7 +1464,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>ENTER (score 76.6)</t>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1470,23 +1474,23 @@
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="n">
-        <v>6.8</v>
+        <v>6.97</v>
       </c>
       <c r="J11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>SNDK</t>
+          <t>GMED</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Memory (HBM is the bottleneck)</t>
+          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>76.34</v>
+        <v>76.61</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -1508,13 +1512,9 @@
       </c>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="n">
-        <v>6.66</v>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>Manually excluded 2026-05-18: $1,333 share price prevents capital-efficient sizing below ~$25k. Conscious framework override (target ~$10k portfolio). | Override removed 2026-06-09: fractional shares adopted, share-price constraint obsolete (Dom decision).</t>
-        </is>
-      </c>
+        <v>9.32</v>
+      </c>
+      <c r="J12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1528,7 +1528,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>74.79000000000001</v>
+        <v>75.54000000000001</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -1550,7 +1550,7 @@
       </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="n">
-        <v>5.85</v>
+        <v>6.93</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
@@ -1582,7 +1582,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>ENTER (score 74.6)</t>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1592,7 +1592,7 @@
       </c>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="n">
-        <v>5.76</v>
+        <v>8.609999999999999</v>
       </c>
       <c r="J14" t="inlineStr"/>
     </row>
@@ -1618,13 +1618,20 @@
       <c r="E15" t="n">
         <v>13</v>
       </c>
-      <c r="F15" t="inlineStr"/>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>ENTER (rank 13, score 74.1)</t>
+        </is>
+      </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H15" t="inlineStr"/>
+      <c r="I15" t="n">
+        <v>5.07</v>
+      </c>
       <c r="J15" t="inlineStr"/>
     </row>
     <row r="16">
@@ -1649,13 +1656,20 @@
       <c r="E16" t="n">
         <v>14</v>
       </c>
-      <c r="F16" t="inlineStr"/>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>ENTER (rank 14, score 73.4)</t>
+        </is>
+      </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H16" t="inlineStr"/>
+      <c r="I16" t="n">
+        <v>4.45</v>
+      </c>
       <c r="J16" t="inlineStr"/>
     </row>
     <row r="17">
@@ -1680,13 +1694,20 @@
       <c r="E17" t="n">
         <v>15</v>
       </c>
-      <c r="F17" t="inlineStr"/>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>ENTER (rank 15, score 73.3)</t>
+        </is>
+      </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="H17" t="inlineStr"/>
+      <c r="I17" t="n">
+        <v>3.14</v>
+      </c>
       <c r="J17" t="inlineStr"/>
     </row>
     <row r="18">
@@ -1723,7 +1744,7 @@
       </c>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="n">
-        <v>5.06</v>
+        <v>8.1</v>
       </c>
       <c r="J18" t="inlineStr"/>
     </row>
@@ -1749,11 +1770,7 @@
       <c r="E19" t="n">
         <v>17</v>
       </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>EXIT (pending since 2026-08-02, confirmed)</t>
-        </is>
-      </c>
+      <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
           <t>N</t>
@@ -1815,11 +1832,7 @@
       <c r="E21" t="n">
         <v>19</v>
       </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>EXIT (pending since 2026-08-02, confirmed)</t>
-        </is>
-      </c>
+      <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
           <t>N</t>
@@ -1871,7 +1884,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>70.78</v>
+        <v>71.06</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -2393,16 +2406,16 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>RMBS</t>
+          <t>GLW</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Memory (HBM is the bottleneck)</t>
+          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>68.55</v>
+        <v>68.52</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -2424,16 +2437,16 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>GLW</t>
+          <t>DELL</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>68.52</v>
+        <v>68.25</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -2455,16 +2468,16 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>DELL</t>
+          <t>HTHIY</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>68.25</v>
+        <v>68.23</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
@@ -2486,16 +2499,16 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>HTHIY</t>
+          <t>RMBS</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>06 AI Compute Silicon / Memory (HBM is the bottleneck)</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>68.23</v>
+        <v>68.18000000000001</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
@@ -2526,7 +2539,7 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>67.8</v>
+        <v>68.02</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -3327,16 +3340,16 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>ADI</t>
+          <t>JCI</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Analog &amp; mixed-signal (signal chain + power)</t>
+          <t>03 Data Center Construction, REITs &amp; Cooling</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>65</v>
+        <v>64.81999999999999</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
@@ -3358,16 +3371,16 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>JCI</t>
+          <t>CRWV</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>03 Data Center Construction, REITs &amp; Cooling</t>
+          <t>09 Cloud - Neocloud</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>64.81999999999999</v>
+        <v>64.78</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
@@ -3389,16 +3402,16 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>CRWV</t>
+          <t>HUBB</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>09 Cloud - Neocloud</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>64.78</v>
+        <v>64.38</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
@@ -3420,16 +3433,16 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>HUBB</t>
+          <t>ADI</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>06 AI Compute Silicon / Analog &amp; mixed-signal (signal chain + power)</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>64.38</v>
+        <v>64.31999999999999</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
@@ -3742,16 +3755,16 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>ENTG</t>
+          <t>LITE</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
+          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>63.3</v>
+        <v>63.35</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
@@ -3773,16 +3786,16 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>AMAT</t>
+          <t>ENTG</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Materials &amp; consumables</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>63.25</v>
+        <v>63.3</v>
       </c>
       <c r="D84" t="inlineStr">
         <is>
@@ -3804,16 +3817,16 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>NVT</t>
+          <t>AMAT</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>02 Grid &amp; Power Equipment</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>63.2</v>
+        <v>63.25</v>
       </c>
       <c r="D85" t="inlineStr">
         <is>
@@ -3835,16 +3848,16 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2252.HK</t>
+          <t>NVT</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
+          <t>02 Grid &amp; Power Equipment</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>63.15</v>
+        <v>63.2</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
@@ -3866,16 +3879,16 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>UMC</t>
+          <t>2252.HK</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>05 Fabs &amp; Foundries</t>
+          <t>11 Robotics &amp; Physical AI / Surgical &amp; medical robotics</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>63.12</v>
+        <v>63.15</v>
       </c>
       <c r="D87" t="inlineStr">
         <is>
@@ -3897,12 +3910,12 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>TLN</t>
+          <t>UMC</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>01 Power Generation / Independent Power Producers (IPPs)</t>
+          <t>05 Fabs &amp; Foundries</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -3928,16 +3941,16 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>COHR</t>
+          <t>TLN</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
+          <t>01 Power Generation / Independent Power Producers (IPPs)</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>63.09</v>
+        <v>63.12</v>
       </c>
       <c r="D89" t="inlineStr">
         <is>
@@ -3959,16 +3972,16 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>FORM</t>
+          <t>COHR</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
+          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>63.04</v>
+        <v>63.09</v>
       </c>
       <c r="D90" t="inlineStr">
         <is>
@@ -3990,16 +4003,16 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>NEE</t>
+          <t>FORM</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Test &amp; measurement</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>63.03</v>
+        <v>63.04</v>
       </c>
       <c r="D91" t="inlineStr">
         <is>
@@ -4021,16 +4034,16 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>LITE</t>
+          <t>NEE</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Optical components &amp; transceivers</t>
+          <t>01 Power Generation / Regulated utilities (data-center geographic exposure)</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>63.02</v>
+        <v>63.03</v>
       </c>
       <c r="D92" t="inlineStr">
         <is>
@@ -4889,16 +4902,16 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>TXN</t>
+          <t>INTU</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>06 AI Compute Silicon / Analog &amp; embedded (power management)</t>
+          <t>10 Models, Software &amp; Applications / Financial software</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>60.73</v>
+        <v>60.64</v>
       </c>
       <c r="D120" t="inlineStr">
         <is>
@@ -4920,16 +4933,16 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>INTU</t>
+          <t>TEL</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>10 Models, Software &amp; Applications / Financial software</t>
+          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>60.64</v>
+        <v>60.55</v>
       </c>
       <c r="D121" t="inlineStr">
         <is>
@@ -4951,16 +4964,16 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>TEL</t>
+          <t>SYM</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>07 Optical, Networking &amp; Interconnect / Cabling &amp; physical layer</t>
+          <t>11 Robotics &amp; Physical AI / Warehouse &amp; logistics automation</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>60.55</v>
+        <v>60.43</v>
       </c>
       <c r="D122" t="inlineStr">
         <is>
@@ -4982,16 +4995,16 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>SYM</t>
+          <t>KLIC</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>11 Robotics &amp; Physical AI / Warehouse &amp; logistics automation</t>
+          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
         </is>
       </c>
       <c r="C123" t="n">
-        <v>60.43</v>
+        <v>60.4</v>
       </c>
       <c r="D123" t="inlineStr">
         <is>
@@ -5013,16 +5026,16 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>KLIC</t>
+          <t>FLEX</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>04 Semiconductor Equipment &amp; Materials / Equipment</t>
+          <t>08 Servers, Systems &amp; Liquid Cooling / Contract manufacturing / ODMs</t>
         </is>
       </c>
       <c r="C124" t="n">
-        <v>60.4</v>
+        <v>60.25</v>
       </c>
       <c r="D124" t="inlineStr">
         <is>
@@ -5044,16 +5057,16 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>FLEX</t>
+          <t>TXN</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>08 Servers, Systems &amp; Liquid Cooling / Contract manufacturing / ODMs</t>
+          <t>06 AI Compute Silicon / Analog &amp; embedded (power management)</t>
         </is>
       </c>
       <c r="C125" t="n">
-        <v>60.25</v>
+        <v>60.2</v>
       </c>
       <c r="D125" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
rebalance: exit 6861.T (untradable), 16→15 names, weights renormalized
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/00-master/portfolio.xlsx
+++ b/00-master/portfolio.xlsx
@@ -676,7 +676,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-08-07 (refresh_targets.py — hysteresis pipeline)</t>
+          <t>2026-08-11 (refresh_targets.py — hysteresis pipeline)</t>
         </is>
       </c>
     </row>
@@ -1068,7 +1068,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Target Portfolio (refreshed 2026-08-07, live Watchlist scores)</t>
+          <t>Target Portfolio (refreshed 2026-08-11, live Watchlist scores)</t>
         </is>
       </c>
     </row>
@@ -1158,7 +1158,7 @@
       </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="n">
-        <v>9.199999999999999</v>
+        <v>10.23</v>
       </c>
       <c r="J3" t="inlineStr"/>
     </row>
@@ -1196,7 +1196,7 @@
       </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="n">
-        <v>6.13</v>
+        <v>6.7</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
@@ -1238,7 +1238,7 @@
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="n">
-        <v>7.57</v>
+        <v>8.41</v>
       </c>
       <c r="J5" t="inlineStr"/>
     </row>
@@ -1276,7 +1276,7 @@
       </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="n">
-        <v>3.37</v>
+        <v>3.7</v>
       </c>
       <c r="J6" t="inlineStr"/>
     </row>
@@ -1314,7 +1314,7 @@
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="n">
-        <v>3.65</v>
+        <v>3.98</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -1356,7 +1356,7 @@
       </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="n">
-        <v>3</v>
+        <v>3.04</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
       </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="n">
-        <v>6.4</v>
+        <v>7.06</v>
       </c>
       <c r="J9" t="inlineStr"/>
     </row>
@@ -1436,7 +1436,7 @@
       </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="n">
-        <v>8.1</v>
+        <v>8.859999999999999</v>
       </c>
       <c r="J10" t="inlineStr"/>
     </row>
@@ -1474,7 +1474,7 @@
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="n">
-        <v>6.97</v>
+        <v>7.76</v>
       </c>
       <c r="J11" t="inlineStr"/>
     </row>
@@ -1512,7 +1512,7 @@
       </c>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="n">
-        <v>9.32</v>
+        <v>9.960000000000001</v>
       </c>
       <c r="J12" t="inlineStr"/>
     </row>
@@ -1550,7 +1550,7 @@
       </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="n">
-        <v>6.93</v>
+        <v>7.58</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
@@ -1577,23 +1577,17 @@
           <t>✓✓</t>
         </is>
       </c>
-      <c r="E14" t="n">
-        <v>12</v>
-      </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>HOLD</t>
+          <t>EXIT (untradable)</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="H14" t="inlineStr"/>
-      <c r="I14" t="n">
-        <v>8.609999999999999</v>
-      </c>
       <c r="J14" t="inlineStr"/>
     </row>
     <row r="15">
@@ -1616,11 +1610,11 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>ENTER (rank 13, score 74.1)</t>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1630,7 +1624,7 @@
       </c>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="n">
-        <v>5.07</v>
+        <v>5.51</v>
       </c>
       <c r="J15" t="inlineStr"/>
     </row>
@@ -1654,11 +1648,11 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>ENTER (rank 14, score 73.4)</t>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1668,7 +1662,7 @@
       </c>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="n">
-        <v>4.45</v>
+        <v>4.84</v>
       </c>
       <c r="J16" t="inlineStr"/>
     </row>
@@ -1692,11 +1686,11 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>ENTER (rank 15, score 73.3)</t>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1706,7 +1700,7 @@
       </c>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="n">
-        <v>3.14</v>
+        <v>3.45</v>
       </c>
       <c r="J17" t="inlineStr"/>
     </row>
@@ -1730,7 +1724,7 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -1744,7 +1738,7 @@
       </c>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="n">
-        <v>8.1</v>
+        <v>8.9</v>
       </c>
       <c r="J18" t="inlineStr"/>
     </row>
@@ -1768,7 +1762,7 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
@@ -1799,7 +1793,7 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
@@ -1830,7 +1824,7 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
@@ -1861,7 +1855,7 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
@@ -1892,7 +1886,7 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
@@ -1923,7 +1917,7 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
@@ -1954,7 +1948,7 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
@@ -1985,7 +1979,7 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
@@ -2016,7 +2010,7 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
@@ -2047,7 +2041,7 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr">
@@ -2078,7 +2072,7 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr">
@@ -2108,9 +2102,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="E30" t="n">
-        <v>28</v>
-      </c>
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr">
         <is>
@@ -2140,7 +2131,7 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr">
@@ -2171,7 +2162,7 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr">
@@ -2202,7 +2193,7 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr">
@@ -2237,7 +2228,7 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr">
@@ -2268,7 +2259,7 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr">
@@ -2299,7 +2290,7 @@
         </is>
       </c>
       <c r="E36" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="F36" t="inlineStr"/>
       <c r="G36" t="inlineStr">
@@ -2330,7 +2321,7 @@
         </is>
       </c>
       <c r="E37" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr">
@@ -2361,7 +2352,7 @@
         </is>
       </c>
       <c r="E38" t="n">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr">
@@ -2391,9 +2382,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="E39" t="n">
-        <v>37</v>
-      </c>
       <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr">
         <is>
@@ -2423,7 +2411,7 @@
         </is>
       </c>
       <c r="E40" t="n">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr">
@@ -2454,7 +2442,7 @@
         </is>
       </c>
       <c r="E41" t="n">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="F41" t="inlineStr"/>
       <c r="G41" t="inlineStr">
@@ -2485,7 +2473,7 @@
         </is>
       </c>
       <c r="E42" t="n">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr">
@@ -2516,7 +2504,7 @@
         </is>
       </c>
       <c r="E43" t="n">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="inlineStr">
@@ -2547,7 +2535,7 @@
         </is>
       </c>
       <c r="E44" t="n">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="F44" t="inlineStr"/>
       <c r="G44" t="inlineStr">
@@ -2582,7 +2570,7 @@
         </is>
       </c>
       <c r="E45" t="n">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr">
@@ -2613,7 +2601,7 @@
         </is>
       </c>
       <c r="E46" t="n">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr">
@@ -2644,7 +2632,7 @@
         </is>
       </c>
       <c r="E47" t="n">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr">
@@ -2675,7 +2663,7 @@
         </is>
       </c>
       <c r="E48" t="n">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr">
@@ -2705,9 +2693,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="E49" t="n">
-        <v>47</v>
-      </c>
       <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr">
         <is>
@@ -2737,7 +2722,7 @@
         </is>
       </c>
       <c r="E50" t="n">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr">
@@ -2768,7 +2753,7 @@
         </is>
       </c>
       <c r="E51" t="n">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr">
@@ -2799,7 +2784,7 @@
         </is>
       </c>
       <c r="E52" t="n">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr">
@@ -2830,7 +2815,7 @@
         </is>
       </c>
       <c r="E53" t="n">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr">
@@ -2861,7 +2846,7 @@
         </is>
       </c>
       <c r="E54" t="n">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr">
@@ -2892,7 +2877,7 @@
         </is>
       </c>
       <c r="E55" t="n">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="F55" t="inlineStr"/>
       <c r="G55" t="inlineStr">
@@ -2923,7 +2908,7 @@
         </is>
       </c>
       <c r="E56" t="n">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr">
@@ -2954,7 +2939,7 @@
         </is>
       </c>
       <c r="E57" t="n">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr">
@@ -2985,7 +2970,7 @@
         </is>
       </c>
       <c r="E58" t="n">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr">
@@ -3016,7 +3001,7 @@
         </is>
       </c>
       <c r="E59" t="n">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr">
@@ -3047,7 +3032,7 @@
         </is>
       </c>
       <c r="E60" t="n">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr">
@@ -3078,7 +3063,7 @@
         </is>
       </c>
       <c r="E61" t="n">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr">
@@ -3109,7 +3094,7 @@
         </is>
       </c>
       <c r="E62" t="n">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="F62" t="inlineStr"/>
       <c r="G62" t="inlineStr">
@@ -3140,7 +3125,7 @@
         </is>
       </c>
       <c r="E63" t="n">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr">
@@ -3171,7 +3156,7 @@
         </is>
       </c>
       <c r="E64" t="n">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="F64" t="inlineStr"/>
       <c r="G64" t="inlineStr">
@@ -3201,9 +3186,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="E65" t="n">
-        <v>63</v>
-      </c>
       <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr">
         <is>
@@ -3233,7 +3215,7 @@
         </is>
       </c>
       <c r="E66" t="n">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr">
@@ -3264,7 +3246,7 @@
         </is>
       </c>
       <c r="E67" t="n">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="F67" t="inlineStr"/>
       <c r="G67" t="inlineStr">
@@ -3295,7 +3277,7 @@
         </is>
       </c>
       <c r="E68" t="n">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="F68" t="inlineStr"/>
       <c r="G68" t="inlineStr">
@@ -3326,7 +3308,7 @@
         </is>
       </c>
       <c r="E69" t="n">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="F69" t="inlineStr"/>
       <c r="G69" t="inlineStr">
@@ -3357,7 +3339,7 @@
         </is>
       </c>
       <c r="E70" t="n">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr">
@@ -3388,7 +3370,7 @@
         </is>
       </c>
       <c r="E71" t="n">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="F71" t="inlineStr"/>
       <c r="G71" t="inlineStr">
@@ -3419,7 +3401,7 @@
         </is>
       </c>
       <c r="E72" t="n">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr">
@@ -3450,7 +3432,7 @@
         </is>
       </c>
       <c r="E73" t="n">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="F73" t="inlineStr"/>
       <c r="G73" t="inlineStr">
@@ -3481,7 +3463,7 @@
         </is>
       </c>
       <c r="E74" t="n">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr">
@@ -3512,7 +3494,7 @@
         </is>
       </c>
       <c r="E75" t="n">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="F75" t="inlineStr"/>
       <c r="G75" t="inlineStr">
@@ -3547,7 +3529,7 @@
         </is>
       </c>
       <c r="E76" t="n">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="F76" t="inlineStr"/>
       <c r="G76" t="inlineStr">
@@ -3578,7 +3560,7 @@
         </is>
       </c>
       <c r="E77" t="n">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="F77" t="inlineStr"/>
       <c r="G77" t="inlineStr">
@@ -3613,7 +3595,7 @@
         </is>
       </c>
       <c r="E78" t="n">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="F78" t="inlineStr"/>
       <c r="G78" t="inlineStr">
@@ -3644,7 +3626,7 @@
         </is>
       </c>
       <c r="E79" t="n">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="F79" t="inlineStr"/>
       <c r="G79" t="inlineStr">
@@ -3675,7 +3657,7 @@
         </is>
       </c>
       <c r="E80" t="n">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="F80" t="inlineStr"/>
       <c r="G80" t="inlineStr">
@@ -3706,7 +3688,7 @@
         </is>
       </c>
       <c r="E81" t="n">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="F81" t="inlineStr"/>
       <c r="G81" t="inlineStr">
@@ -3741,7 +3723,7 @@
         </is>
       </c>
       <c r="E82" t="n">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="F82" t="inlineStr"/>
       <c r="G82" t="inlineStr">
@@ -3772,7 +3754,7 @@
         </is>
       </c>
       <c r="E83" t="n">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="F83" t="inlineStr"/>
       <c r="G83" t="inlineStr">
@@ -3803,7 +3785,7 @@
         </is>
       </c>
       <c r="E84" t="n">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="F84" t="inlineStr"/>
       <c r="G84" t="inlineStr">
@@ -3834,7 +3816,7 @@
         </is>
       </c>
       <c r="E85" t="n">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="F85" t="inlineStr"/>
       <c r="G85" t="inlineStr">
@@ -3865,7 +3847,7 @@
         </is>
       </c>
       <c r="E86" t="n">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="F86" t="inlineStr"/>
       <c r="G86" t="inlineStr">
@@ -3895,9 +3877,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="E87" t="n">
-        <v>85</v>
-      </c>
       <c r="F87" t="inlineStr"/>
       <c r="G87" t="inlineStr">
         <is>
@@ -3927,7 +3906,7 @@
         </is>
       </c>
       <c r="E88" t="n">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="F88" t="inlineStr"/>
       <c r="G88" t="inlineStr">
@@ -3958,7 +3937,7 @@
         </is>
       </c>
       <c r="E89" t="n">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr">
@@ -3989,7 +3968,7 @@
         </is>
       </c>
       <c r="E90" t="n">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="F90" t="inlineStr"/>
       <c r="G90" t="inlineStr">
@@ -4020,7 +3999,7 @@
         </is>
       </c>
       <c r="E91" t="n">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="F91" t="inlineStr"/>
       <c r="G91" t="inlineStr">
@@ -4051,7 +4030,7 @@
         </is>
       </c>
       <c r="E92" t="n">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr">
@@ -4082,7 +4061,7 @@
         </is>
       </c>
       <c r="E93" t="n">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="F93" t="inlineStr"/>
       <c r="G93" t="inlineStr">
@@ -4113,7 +4092,7 @@
         </is>
       </c>
       <c r="E94" t="n">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="F94" t="inlineStr"/>
       <c r="G94" t="inlineStr">
@@ -4144,7 +4123,7 @@
         </is>
       </c>
       <c r="E95" t="n">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="F95" t="inlineStr"/>
       <c r="G95" t="inlineStr">
@@ -4175,7 +4154,7 @@
         </is>
       </c>
       <c r="E96" t="n">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="F96" t="inlineStr"/>
       <c r="G96" t="inlineStr">
@@ -4205,9 +4184,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="E97" t="n">
-        <v>95</v>
-      </c>
       <c r="F97" t="inlineStr"/>
       <c r="G97" t="inlineStr">
         <is>
@@ -4237,7 +4213,7 @@
         </is>
       </c>
       <c r="E98" t="n">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="F98" t="inlineStr"/>
       <c r="G98" t="inlineStr">
@@ -4268,7 +4244,7 @@
         </is>
       </c>
       <c r="E99" t="n">
-        <v>97</v>
+        <v>90</v>
       </c>
       <c r="F99" t="inlineStr"/>
       <c r="G99" t="inlineStr">
@@ -4299,7 +4275,7 @@
         </is>
       </c>
       <c r="E100" t="n">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="F100" t="inlineStr"/>
       <c r="G100" t="inlineStr">
@@ -4330,7 +4306,7 @@
         </is>
       </c>
       <c r="E101" t="n">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="F101" t="inlineStr"/>
       <c r="G101" t="inlineStr">
@@ -4361,7 +4337,7 @@
         </is>
       </c>
       <c r="E102" t="n">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr">
@@ -4392,7 +4368,7 @@
         </is>
       </c>
       <c r="E103" t="n">
-        <v>101</v>
+        <v>94</v>
       </c>
       <c r="F103" t="inlineStr"/>
       <c r="G103" t="inlineStr">
@@ -4423,7 +4399,7 @@
         </is>
       </c>
       <c r="E104" t="n">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="F104" t="inlineStr"/>
       <c r="G104" t="inlineStr">
@@ -4454,7 +4430,7 @@
         </is>
       </c>
       <c r="E105" t="n">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="F105" t="inlineStr"/>
       <c r="G105" t="inlineStr">
@@ -4485,7 +4461,7 @@
         </is>
       </c>
       <c r="E106" t="n">
-        <v>104</v>
+        <v>97</v>
       </c>
       <c r="F106" t="inlineStr"/>
       <c r="G106" t="inlineStr">
@@ -4516,7 +4492,7 @@
         </is>
       </c>
       <c r="E107" t="n">
-        <v>105</v>
+        <v>98</v>
       </c>
       <c r="F107" t="inlineStr"/>
       <c r="G107" t="inlineStr">
@@ -4547,7 +4523,7 @@
         </is>
       </c>
       <c r="E108" t="n">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="F108" t="inlineStr"/>
       <c r="G108" t="inlineStr">
@@ -4578,7 +4554,7 @@
         </is>
       </c>
       <c r="E109" t="n">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="F109" t="inlineStr"/>
       <c r="G109" t="inlineStr">
@@ -4609,7 +4585,7 @@
         </is>
       </c>
       <c r="E110" t="n">
-        <v>108</v>
+        <v>101</v>
       </c>
       <c r="F110" t="inlineStr"/>
       <c r="G110" t="inlineStr">
@@ -4640,7 +4616,7 @@
         </is>
       </c>
       <c r="E111" t="n">
-        <v>109</v>
+        <v>102</v>
       </c>
       <c r="F111" t="inlineStr"/>
       <c r="G111" t="inlineStr">
@@ -4671,7 +4647,7 @@
         </is>
       </c>
       <c r="E112" t="n">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="F112" t="inlineStr"/>
       <c r="G112" t="inlineStr">
@@ -4701,9 +4677,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="E113" t="n">
-        <v>111</v>
-      </c>
       <c r="F113" t="inlineStr"/>
       <c r="G113" t="inlineStr">
         <is>
@@ -4733,7 +4706,7 @@
         </is>
       </c>
       <c r="E114" t="n">
-        <v>112</v>
+        <v>104</v>
       </c>
       <c r="F114" t="inlineStr"/>
       <c r="G114" t="inlineStr">
@@ -4764,7 +4737,7 @@
         </is>
       </c>
       <c r="E115" t="n">
-        <v>113</v>
+        <v>105</v>
       </c>
       <c r="F115" t="inlineStr"/>
       <c r="G115" t="inlineStr">
@@ -4795,7 +4768,7 @@
         </is>
       </c>
       <c r="E116" t="n">
-        <v>114</v>
+        <v>106</v>
       </c>
       <c r="F116" t="inlineStr"/>
       <c r="G116" t="inlineStr">
@@ -4826,7 +4799,7 @@
         </is>
       </c>
       <c r="E117" t="n">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="F117" t="inlineStr"/>
       <c r="G117" t="inlineStr">
@@ -4857,7 +4830,7 @@
         </is>
       </c>
       <c r="E118" t="n">
-        <v>116</v>
+        <v>108</v>
       </c>
       <c r="F118" t="inlineStr"/>
       <c r="G118" t="inlineStr">
@@ -4888,7 +4861,7 @@
         </is>
       </c>
       <c r="E119" t="n">
-        <v>117</v>
+        <v>109</v>
       </c>
       <c r="F119" t="inlineStr"/>
       <c r="G119" t="inlineStr">
@@ -4919,7 +4892,7 @@
         </is>
       </c>
       <c r="E120" t="n">
-        <v>118</v>
+        <v>110</v>
       </c>
       <c r="F120" t="inlineStr"/>
       <c r="G120" t="inlineStr">
@@ -4950,7 +4923,7 @@
         </is>
       </c>
       <c r="E121" t="n">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="F121" t="inlineStr"/>
       <c r="G121" t="inlineStr">
@@ -4981,7 +4954,7 @@
         </is>
       </c>
       <c r="E122" t="n">
-        <v>120</v>
+        <v>112</v>
       </c>
       <c r="F122" t="inlineStr"/>
       <c r="G122" t="inlineStr">
@@ -5012,7 +4985,7 @@
         </is>
       </c>
       <c r="E123" t="n">
-        <v>121</v>
+        <v>113</v>
       </c>
       <c r="F123" t="inlineStr"/>
       <c r="G123" t="inlineStr">
@@ -5043,7 +5016,7 @@
         </is>
       </c>
       <c r="E124" t="n">
-        <v>122</v>
+        <v>114</v>
       </c>
       <c r="F124" t="inlineStr"/>
       <c r="G124" t="inlineStr">
@@ -5074,7 +5047,7 @@
         </is>
       </c>
       <c r="E125" t="n">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="F125" t="inlineStr"/>
       <c r="G125" t="inlineStr">
@@ -5105,7 +5078,7 @@
         </is>
       </c>
       <c r="E126" t="n">
-        <v>124</v>
+        <v>116</v>
       </c>
       <c r="F126" t="inlineStr"/>
       <c r="G126" t="inlineStr">
@@ -5136,7 +5109,7 @@
         </is>
       </c>
       <c r="E127" t="n">
-        <v>125</v>
+        <v>117</v>
       </c>
       <c r="F127" t="inlineStr"/>
       <c r="G127" t="inlineStr">
@@ -5167,7 +5140,7 @@
         </is>
       </c>
       <c r="E128" t="n">
-        <v>126</v>
+        <v>118</v>
       </c>
       <c r="F128" t="inlineStr"/>
       <c r="G128" t="inlineStr">
@@ -5198,7 +5171,7 @@
         </is>
       </c>
       <c r="E129" t="n">
-        <v>127</v>
+        <v>119</v>
       </c>
       <c r="F129" t="inlineStr"/>
       <c r="G129" t="inlineStr">
@@ -5229,7 +5202,7 @@
         </is>
       </c>
       <c r="E130" t="n">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="F130" t="inlineStr"/>
       <c r="G130" t="inlineStr">
@@ -5259,9 +5232,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="E131" t="n">
-        <v>129</v>
-      </c>
       <c r="F131" t="inlineStr"/>
       <c r="G131" t="inlineStr">
         <is>
@@ -5291,7 +5261,7 @@
         </is>
       </c>
       <c r="E132" t="n">
-        <v>130</v>
+        <v>121</v>
       </c>
       <c r="F132" t="inlineStr"/>
       <c r="G132" t="inlineStr">
@@ -5322,7 +5292,7 @@
         </is>
       </c>
       <c r="E133" t="n">
-        <v>131</v>
+        <v>122</v>
       </c>
       <c r="F133" t="inlineStr"/>
       <c r="G133" t="inlineStr">
@@ -5353,7 +5323,7 @@
         </is>
       </c>
       <c r="E134" t="n">
-        <v>132</v>
+        <v>123</v>
       </c>
       <c r="F134" t="inlineStr"/>
       <c r="G134" t="inlineStr">
@@ -5383,9 +5353,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="E135" t="n">
-        <v>133</v>
-      </c>
       <c r="F135" t="inlineStr"/>
       <c r="G135" t="inlineStr">
         <is>
@@ -5415,7 +5382,7 @@
         </is>
       </c>
       <c r="E136" t="n">
-        <v>134</v>
+        <v>124</v>
       </c>
       <c r="F136" t="inlineStr"/>
       <c r="G136" t="inlineStr">
@@ -5446,7 +5413,7 @@
         </is>
       </c>
       <c r="E137" t="n">
-        <v>135</v>
+        <v>125</v>
       </c>
       <c r="F137" t="inlineStr"/>
       <c r="G137" t="inlineStr">
@@ -5477,7 +5444,7 @@
         </is>
       </c>
       <c r="E138" t="n">
-        <v>136</v>
+        <v>126</v>
       </c>
       <c r="F138" t="inlineStr"/>
       <c r="G138" t="inlineStr">
@@ -5508,7 +5475,7 @@
         </is>
       </c>
       <c r="E139" t="n">
-        <v>137</v>
+        <v>127</v>
       </c>
       <c r="F139" t="inlineStr"/>
       <c r="G139" t="inlineStr">
@@ -5538,9 +5505,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="E140" t="n">
-        <v>138</v>
-      </c>
       <c r="F140" t="inlineStr"/>
       <c r="G140" t="inlineStr">
         <is>
@@ -5569,9 +5533,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="E141" t="n">
-        <v>139</v>
-      </c>
       <c r="F141" t="inlineStr"/>
       <c r="G141" t="inlineStr">
         <is>
@@ -5601,7 +5562,7 @@
         </is>
       </c>
       <c r="E142" t="n">
-        <v>140</v>
+        <v>128</v>
       </c>
       <c r="F142" t="inlineStr"/>
       <c r="G142" t="inlineStr">
@@ -5632,7 +5593,7 @@
         </is>
       </c>
       <c r="E143" t="n">
-        <v>141</v>
+        <v>129</v>
       </c>
       <c r="F143" t="inlineStr"/>
       <c r="G143" t="inlineStr">
@@ -5663,7 +5624,7 @@
         </is>
       </c>
       <c r="E144" t="n">
-        <v>142</v>
+        <v>130</v>
       </c>
       <c r="F144" t="inlineStr"/>
       <c r="G144" t="inlineStr">
@@ -5694,7 +5655,7 @@
         </is>
       </c>
       <c r="E145" t="n">
-        <v>143</v>
+        <v>131</v>
       </c>
       <c r="F145" t="inlineStr"/>
       <c r="G145" t="inlineStr">
@@ -5725,7 +5686,7 @@
         </is>
       </c>
       <c r="E146" t="n">
-        <v>144</v>
+        <v>132</v>
       </c>
       <c r="F146" t="inlineStr"/>
       <c r="G146" t="inlineStr">
@@ -5756,7 +5717,7 @@
         </is>
       </c>
       <c r="E147" t="n">
-        <v>145</v>
+        <v>133</v>
       </c>
       <c r="F147" t="inlineStr"/>
       <c r="G147" t="inlineStr">
@@ -5787,7 +5748,7 @@
         </is>
       </c>
       <c r="E148" t="n">
-        <v>146</v>
+        <v>134</v>
       </c>
       <c r="F148" t="inlineStr"/>
       <c r="G148" t="inlineStr">
@@ -5818,7 +5779,7 @@
         </is>
       </c>
       <c r="E149" t="n">
-        <v>147</v>
+        <v>135</v>
       </c>
       <c r="F149" t="inlineStr"/>
       <c r="G149" t="inlineStr">
@@ -5849,7 +5810,7 @@
         </is>
       </c>
       <c r="E150" t="n">
-        <v>148</v>
+        <v>136</v>
       </c>
       <c r="F150" t="inlineStr"/>
       <c r="G150" t="inlineStr">
@@ -5879,9 +5840,6 @@
           <t>✓</t>
         </is>
       </c>
-      <c r="E151" t="n">
-        <v>149</v>
-      </c>
       <c r="F151" t="inlineStr"/>
       <c r="G151" t="inlineStr">
         <is>
@@ -5911,7 +5869,7 @@
         </is>
       </c>
       <c r="E152" t="n">
-        <v>150</v>
+        <v>137</v>
       </c>
       <c r="F152" t="inlineStr"/>
       <c r="G152" t="inlineStr">
@@ -5942,7 +5900,7 @@
         </is>
       </c>
       <c r="E153" t="n">
-        <v>151</v>
+        <v>138</v>
       </c>
       <c r="F153" t="inlineStr"/>
       <c r="G153" t="inlineStr">
@@ -5973,7 +5931,7 @@
         </is>
       </c>
       <c r="E154" t="n">
-        <v>152</v>
+        <v>139</v>
       </c>
       <c r="F154" t="inlineStr"/>
       <c r="G154" t="inlineStr">
@@ -6004,7 +5962,7 @@
         </is>
       </c>
       <c r="E155" t="n">
-        <v>153</v>
+        <v>140</v>
       </c>
       <c r="F155" t="inlineStr"/>
       <c r="G155" t="inlineStr">

</xml_diff>

<commit_message>
migrate(rule 33): sizing flipped to equal weight — sizing_migration_equal event 2026-09-07
- portfolio-config.json sizing.mode: inverse_vol -> equal
- performance-config.json: methodology seam stamped; INVVOL_ROSTER shadow
  seeded/re-targeted (16 names); one sizing_migration_equal event that
  same-day-absorbs the +NTAP membership event (reason string records it)
- Targets: 16 names @ 6.25%; one-way turnover ~15.8% of book
- ticket generated under tracking/live/ (gitignored); the unexecuted NTAP
  entry ticket was superseded by it

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/00-master/portfolio.xlsx
+++ b/00-master/portfolio.xlsx
@@ -1158,7 +1158,7 @@
       </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="n">
-        <v>8.83</v>
+        <v>6.25</v>
       </c>
       <c r="J3" t="inlineStr"/>
     </row>
@@ -1196,7 +1196,7 @@
       </c>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="n">
-        <v>5.7</v>
+        <v>6.25</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
@@ -1238,7 +1238,7 @@
       </c>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="n">
-        <v>7.89</v>
+        <v>6.25</v>
       </c>
       <c r="J5" t="inlineStr"/>
     </row>
@@ -1276,7 +1276,7 @@
       </c>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="n">
-        <v>3.27</v>
+        <v>6.25</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -1318,7 +1318,7 @@
       </c>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="n">
-        <v>8.23</v>
+        <v>6.25</v>
       </c>
       <c r="J7" t="inlineStr"/>
     </row>
@@ -1356,7 +1356,7 @@
       </c>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="n">
-        <v>6.28</v>
+        <v>6.25</v>
       </c>
       <c r="J8" t="inlineStr"/>
     </row>
@@ -1394,7 +1394,7 @@
       </c>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="n">
-        <v>3</v>
+        <v>6.25</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
@@ -1436,7 +1436,7 @@
       </c>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="n">
-        <v>3.66</v>
+        <v>6.25</v>
       </c>
       <c r="J10" t="inlineStr"/>
     </row>
@@ -1474,7 +1474,7 @@
       </c>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="n">
-        <v>8.16</v>
+        <v>6.25</v>
       </c>
       <c r="J11" t="inlineStr"/>
     </row>
@@ -1512,7 +1512,7 @@
       </c>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="n">
-        <v>9.19</v>
+        <v>6.25</v>
       </c>
       <c r="J12" t="inlineStr"/>
     </row>
@@ -1550,7 +1550,7 @@
       </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="n">
-        <v>6.49</v>
+        <v>6.25</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
@@ -1592,7 +1592,7 @@
       </c>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="n">
-        <v>3.36</v>
+        <v>6.25</v>
       </c>
       <c r="J14" t="inlineStr"/>
     </row>
@@ -1658,7 +1658,7 @@
       </c>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="n">
-        <v>4.83</v>
+        <v>6.25</v>
       </c>
       <c r="J16" t="inlineStr"/>
     </row>
@@ -1696,7 +1696,7 @@
       </c>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="n">
-        <v>4.11</v>
+        <v>6.25</v>
       </c>
       <c r="J17" t="inlineStr"/>
     </row>
@@ -1724,7 +1724,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>ENTER (rank 15, score 73.0)</t>
+          <t>HOLD</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1734,7 +1734,7 @@
       </c>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="n">
-        <v>9.17</v>
+        <v>6.25</v>
       </c>
       <c r="J18" t="inlineStr"/>
     </row>
@@ -1803,7 +1803,7 @@
       </c>
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="n">
-        <v>7.82</v>
+        <v>6.25</v>
       </c>
       <c r="J20" t="inlineStr"/>
     </row>

</xml_diff>